<commit_message>
Setup React Query (TanStack Query v5)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA916CA-73AE-434A-91C9-68BF893BB97B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CE2CEA-A456-4531-B8E1-1EC8ACF52B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21504" yWindow="84" windowWidth="17280" windowHeight="8880" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -2680,13 +2680,13 @@
     <t>Elimina prenotazioni Completate con DataPrenotazione &gt; 6 mesi fa</t>
   </si>
   <si>
-    <t>Aggiornato: 18/05/2026</t>
-  </si>
-  <si>
-    <t>Aggiornato: 18/05/2026  ·  Percorso: Backend → Frontend React/TS → Mobile React Native</t>
-  </si>
-  <si>
     <t>Parziale</t>
+  </si>
+  <si>
+    <t>Aggiornato: 20/05/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 20/05/2026  ·  Percorso: Backend → Frontend React/TS → Mobile React Native</t>
   </si>
 </sst>
 </file>
@@ -3016,6 +3016,12 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3045,12 +3051,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3366,36 +3366,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
-        <v>882</v>
-      </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+      <c r="A2" s="29" t="s">
+        <v>883</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="31" t="s">
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="32"/>
-      <c r="F4" s="33"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="35"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3560,24 +3560,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="33"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="35"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3605,14 +3605,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4555,13 +4555,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4905,11 +4905,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5175,14 +5175,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5266,40 +5266,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
-        <v>883</v>
-      </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="A2" s="29" t="s">
+        <v>884</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="33"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="35"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5622,16 +5622,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="33"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="35"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5854,16 +5854,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="35" t="s">
+      <c r="A35" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="33"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="35"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -5901,7 +5901,7 @@
       <c r="E37" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F37" s="39" t="s">
+      <c r="F37" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -5921,8 +5921,8 @@
       <c r="E38" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="F38" s="40" t="s">
-        <v>884</v>
+      <c r="F38" s="28" t="s">
+        <v>882</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -5941,8 +5941,8 @@
       <c r="E39" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="F39" s="40" t="s">
-        <v>884</v>
+      <c r="F39" s="28" t="s">
+        <v>882</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6021,8 +6021,8 @@
       <c r="E43" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="F43" s="40" t="s">
-        <v>884</v>
+      <c r="F43" s="28" t="s">
+        <v>882</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6046,16 +6046,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="32"/>
-      <c r="E46" s="32"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
-      <c r="H46" s="33"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="35"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6118,16 +6118,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="34" t="s">
+      <c r="A51" s="36" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="32"/>
-      <c r="C51" s="32"/>
-      <c r="D51" s="32"/>
-      <c r="E51" s="32"/>
-      <c r="F51" s="32"/>
-      <c r="G51" s="32"/>
-      <c r="H51" s="33"/>
+      <c r="B51" s="34"/>
+      <c r="C51" s="34"/>
+      <c r="D51" s="34"/>
+      <c r="E51" s="34"/>
+      <c r="F51" s="34"/>
+      <c r="G51" s="34"/>
+      <c r="H51" s="35"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6332,24 +6332,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="40" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="33"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6437,14 +6437,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="36" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="33"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="35"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6532,14 +6532,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="33" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="33"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="35"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -6661,14 +6661,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="33" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="33"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="35"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -6798,26 +6798,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="36" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="33"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="35"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7113,24 +7113,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="33" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="33"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7315,14 +7315,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="40" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="33"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="35"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7423,14 +7423,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="36" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="33"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="35"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7526,14 +7526,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7710,14 +7710,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8320,13 +8320,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8723,13 +8723,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
Login page + AuthContext + useAuth hook
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CE2CEA-A456-4531-B8E1-1EC8ACF52B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B368E2-F994-4CB8-832C-DFDFAFA8CE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -5921,8 +5921,8 @@
       <c r="E38" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="F38" s="28" t="s">
-        <v>882</v>
+      <c r="F38" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Step 8 - Layout shell con sidebar, header e route annidate
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B368E2-F994-4CB8-832C-DFDFAFA8CE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71A770B-3611-4DF9-A9C4-D089FABD886E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19896" yWindow="2232" windowWidth="17280" windowHeight="8880" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="884">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2680,13 +2680,10 @@
     <t>Elimina prenotazioni Completate con DataPrenotazione &gt; 6 mesi fa</t>
   </si>
   <si>
-    <t>Parziale</t>
-  </si>
-  <si>
-    <t>Aggiornato: 20/05/2026</t>
-  </si>
-  <si>
     <t>Aggiornato: 20/05/2026  ·  Percorso: Backend → Frontend React/TS → Mobile React Native</t>
+  </si>
+  <si>
+    <t>Aggiornato: 22/05/2026</t>
   </si>
 </sst>
 </file>
@@ -2782,7 +2779,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2880,12 +2877,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -2938,7 +2929,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3017,9 +3008,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3366,36 +3354,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="28" t="s">
         <v>883</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="33" t="s">
+      <c r="B4" s="33"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="34"/>
-      <c r="F4" s="35"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="34"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3560,24 +3548,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="35"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="34"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3605,14 +3593,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4555,13 +4543,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4905,11 +4893,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5175,14 +5163,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5266,40 +5254,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
-        <v>884</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="A2" s="28" t="s">
+        <v>882</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="35"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="34"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5622,16 +5610,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="35"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="34"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5854,16 +5842,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="37" t="s">
+      <c r="A35" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="35"/>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="34"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -5941,8 +5929,8 @@
       <c r="E39" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="F39" s="28" t="s">
-        <v>882</v>
+      <c r="F39" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6021,8 +6009,8 @@
       <c r="E43" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="F43" s="28" t="s">
-        <v>882</v>
+      <c r="F43" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6046,16 +6034,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="37" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="35"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="33"/>
+      <c r="H46" s="34"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6118,16 +6106,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="36" t="s">
+      <c r="A51" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="34"/>
-      <c r="C51" s="34"/>
-      <c r="D51" s="34"/>
-      <c r="E51" s="34"/>
-      <c r="F51" s="34"/>
-      <c r="G51" s="34"/>
-      <c r="H51" s="35"/>
+      <c r="B51" s="33"/>
+      <c r="C51" s="33"/>
+      <c r="D51" s="33"/>
+      <c r="E51" s="33"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="33"/>
+      <c r="H51" s="34"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6332,24 +6320,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="39" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="35"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="34"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6437,14 +6425,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="35" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="34"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6532,14 +6520,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="32" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="35"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="34"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -6661,14 +6649,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="32" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="35"/>
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="34"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -6798,26 +6786,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="35" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="34"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7113,24 +7101,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="32" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="35"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="34"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7315,14 +7303,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="40" t="s">
+      <c r="A18" s="39" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="35"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="34"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7423,14 +7411,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="35" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="35"/>
+      <c r="B27" s="33"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="34"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7526,14 +7514,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7710,14 +7698,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8320,13 +8308,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8723,13 +8711,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
Step 9 - Pagina Dashboard con KPI giornalieri e settimanali
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71A770B-3611-4DF9-A9C4-D089FABD886E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0149DBC9-E05B-4DD3-9160-B98324972867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19896" yWindow="2232" windowWidth="17280" windowHeight="8880" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22128" yWindow="924" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -2683,7 +2683,7 @@
     <t>Aggiornato: 20/05/2026  ·  Percorso: Backend → Frontend React/TS → Mobile React Native</t>
   </si>
   <si>
-    <t>Aggiornato: 22/05/2026</t>
+    <t>Aggiornato: 26/05/2026</t>
   </si>
 </sst>
 </file>
@@ -5949,8 +5949,8 @@
       <c r="E40" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="F40" s="23" t="s">
-        <v>147</v>
+      <c r="F40" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
WIP - CRUD Zone lista + hook + tipi (bottoni da collegare)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0149DBC9-E05B-4DD3-9160-B98324972867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8410B2F1-E80F-4004-B335-E82819F0D8F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-22128" yWindow="924" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="885">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2684,6 +2684,9 @@
   </si>
   <si>
     <t>Aggiornato: 26/05/2026</t>
+  </si>
+  <si>
+    <t>In corso</t>
   </si>
 </sst>
 </file>
@@ -2779,7 +2782,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2877,6 +2880,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9CEBFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -2929,7 +2938,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3039,6 +3048,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5989,8 +6001,8 @@
       <c r="E42" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="F42" s="23" t="s">
-        <v>147</v>
+      <c r="F42" s="40" t="s">
+        <v>884</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
CRUD Zone completo (lista + modal create/edit + delete)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8410B2F1-E80F-4004-B335-E82819F0D8F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF370E78-163D-4D7D-AC2D-EF98291AB8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-22128" yWindow="924" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2683,10 +2683,10 @@
     <t>Aggiornato: 20/05/2026  ·  Percorso: Backend → Frontend React/TS → Mobile React Native</t>
   </si>
   <si>
-    <t>Aggiornato: 26/05/2026</t>
-  </si>
-  <si>
     <t>In corso</t>
+  </si>
+  <si>
+    <t>Aggiornato: 27/05/2026</t>
   </si>
 </sst>
 </file>
@@ -3019,6 +3019,9 @@
     <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3048,9 +3051,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3366,36 +3366,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
-        <v>883</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
+      <c r="A2" s="29" t="s">
+        <v>884</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="32" t="s">
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="33"/>
-      <c r="F4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="35"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3560,24 +3560,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="33"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="34"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="35"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3605,14 +3605,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4555,13 +4555,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4905,11 +4905,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5175,14 +5175,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5266,40 +5266,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>882</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="34"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="35"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5622,16 +5622,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="32" t="s">
+      <c r="A22" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="34"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="35"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5854,16 +5854,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="36" t="s">
+      <c r="A35" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="33"/>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="35"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6001,8 +6001,8 @@
       <c r="E42" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="F42" s="40" t="s">
-        <v>884</v>
+      <c r="F42" s="28" t="s">
+        <v>883</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6046,16 +6046,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="37" t="s">
+      <c r="A46" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="33"/>
-      <c r="C46" s="33"/>
-      <c r="D46" s="33"/>
-      <c r="E46" s="33"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="33"/>
-      <c r="H46" s="34"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="35"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6118,16 +6118,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="35" t="s">
+      <c r="A51" s="36" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="33"/>
-      <c r="C51" s="33"/>
-      <c r="D51" s="33"/>
-      <c r="E51" s="33"/>
-      <c r="F51" s="33"/>
-      <c r="G51" s="33"/>
-      <c r="H51" s="34"/>
+      <c r="B51" s="34"/>
+      <c r="C51" s="34"/>
+      <c r="D51" s="34"/>
+      <c r="E51" s="34"/>
+      <c r="F51" s="34"/>
+      <c r="G51" s="34"/>
+      <c r="H51" s="35"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6332,24 +6332,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="40" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="34"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6437,14 +6437,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="36" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="33"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="34"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="35"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6532,14 +6532,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="33" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="34"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="35"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -6661,14 +6661,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="33" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="34"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="35"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -6798,26 +6798,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="36" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="34"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="35"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7113,24 +7113,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="33" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="34"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7315,14 +7315,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="39" t="s">
+      <c r="A18" s="40" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="34"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="35"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7423,14 +7423,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="36" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="34"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="35"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7526,14 +7526,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7710,14 +7710,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8320,13 +8320,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8723,13 +8723,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
aggiorna documenti progetto + gitignore + puntatore   submodule backend
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF370E78-163D-4D7D-AC2D-EF98291AB8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247ACF57-85EF-41E3-B99A-798902BEBE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22128" yWindow="924" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="30960" windowHeight="12120" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: chiude sessione 12/08 - stato repo, tracker e permessi Claude Code
Aggiorna CLAUDE.md con il resoconto finale della sessione di manutenzione
(pulizia repo, CI, lint frontend) e allinea il tracker Excel di conseguenza.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Personale\GestoraProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247ACF57-85EF-41E3-B99A-798902BEBE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9316D934-6D02-4DDE-A60B-332ACD1A3E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="30960" windowHeight="12120" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="901">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2680,13 +2680,61 @@
     <t>Elimina prenotazioni Completate con DataPrenotazione &gt; 6 mesi fa</t>
   </si>
   <si>
-    <t>Aggiornato: 20/05/2026  ·  Percorso: Backend → Frontend React/TS → Mobile React Native</t>
-  </si>
-  <si>
     <t>In corso</t>
   </si>
   <si>
-    <t>Aggiornato: 27/05/2026</t>
+    <t>Aggiornato: 12/08/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 12/08/2026  ·  Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>SESSIONE 12/08/2026 - Manutenzione repo e config Claude Code</t>
+  </si>
+  <si>
+    <t>Cosa e' stato fatto</t>
+  </si>
+  <si>
+    <t>Da fare</t>
+  </si>
+  <si>
+    <t>Igiene repo</t>
+  </si>
+  <si>
+    <t>Fix CLAUDE.md area (file rinominati, mai caricati in cascata), rimosso tracker duplicato Gestora_Piano_Operativo.xlsx e GUIDA_CRUD_FRONTEND.md, ristretto .gitignore (.claude/ ora tracciato)</t>
+  </si>
+  <si>
+    <t>Git hygiene</t>
+  </si>
+  <si>
+    <t>CI GitHub Actions</t>
+  </si>
+  <si>
+    <t>Fix indentazione YAML nei 3 workflow (invalidi), rimosso claude-code-review.yml (richiede secret non configurato per costo)</t>
+  </si>
+  <si>
+    <t>GitHub Actions</t>
+  </si>
+  <si>
+    <t>Lint frontend</t>
+  </si>
+  <si>
+    <t>Risolti 30 problemi lint emersi dalla prima CI: 21 any -&gt; AxiosError tipizzato, 3 violazioni fast-refresh, 4 dipendenze reset mancanti</t>
+  </si>
+  <si>
+    <t>ESLint + TypeScript</t>
+  </si>
+  <si>
+    <t>FIX-004 riformulato</t>
+  </si>
+  <si>
+    <t>Backlog ridefinito in BACKEND_FIX_TODO.md dopo lettura codice (problemi A/B/C), aggiunti CACHE-001 e AUDIT-001, ridimensionato SEC-001</t>
+  </si>
+  <si>
+    <t>Analisi codice</t>
+  </si>
+  <si>
+    <t>12/08/2026</t>
   </si>
 </sst>
 </file>
@@ -2782,7 +2830,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2886,6 +2934,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -2938,7 +2992,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3022,6 +3076,8 @@
     <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3052,6 +3108,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -3366,36 +3423,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
-        <v>884</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="A2" s="31" t="s">
+        <v>883</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="33" t="s">
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="34"/>
-      <c r="F4" s="35"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="37"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3560,24 +3617,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="35"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="37"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3605,14 +3662,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4555,13 +4612,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4905,11 +4962,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5175,14 +5232,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5254,7 +5311,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5266,40 +5323,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
-        <v>882</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="A2" s="31" t="s">
+        <v>884</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="37"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5622,16 +5679,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="35"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="37"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5854,16 +5911,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="37" t="s">
+      <c r="A35" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="35"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="37"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6002,7 +6059,7 @@
         <v>166</v>
       </c>
       <c r="F42" s="28" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -6046,16 +6103,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="35"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="36"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="37"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6118,16 +6175,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="36" t="s">
+      <c r="A51" s="38" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="34"/>
-      <c r="C51" s="34"/>
-      <c r="D51" s="34"/>
-      <c r="E51" s="34"/>
-      <c r="F51" s="34"/>
-      <c r="G51" s="34"/>
-      <c r="H51" s="35"/>
+      <c r="B51" s="36"/>
+      <c r="C51" s="36"/>
+      <c r="D51" s="36"/>
+      <c r="E51" s="36"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="36"/>
+      <c r="H51" s="37"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6272,7 +6329,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="26" t="s">
         <v>219</v>
       </c>
@@ -6283,7 +6340,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="26" t="s">
         <v>219</v>
       </c>
@@ -6294,7 +6351,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="26" t="s">
         <v>219</v>
       </c>
@@ -6303,6 +6360,111 @@
       </c>
       <c r="C67" s="26" t="s">
         <v>225</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>44</v>
+      </c>
+      <c r="B70" t="s">
+        <v>45</v>
+      </c>
+      <c r="C70" t="s">
+        <v>886</v>
+      </c>
+      <c r="D70" t="s">
+        <v>47</v>
+      </c>
+      <c r="E70" t="s">
+        <v>48</v>
+      </c>
+      <c r="F70" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>1</v>
+      </c>
+      <c r="B71" t="s">
+        <v>888</v>
+      </c>
+      <c r="C71" t="s">
+        <v>889</v>
+      </c>
+      <c r="D71" t="s">
+        <v>890</v>
+      </c>
+      <c r="E71" s="43" t="s">
+        <v>900</v>
+      </c>
+      <c r="F71" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>2</v>
+      </c>
+      <c r="B72" t="s">
+        <v>891</v>
+      </c>
+      <c r="C72" t="s">
+        <v>892</v>
+      </c>
+      <c r="D72" t="s">
+        <v>893</v>
+      </c>
+      <c r="E72" s="43" t="s">
+        <v>900</v>
+      </c>
+      <c r="F72" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>3</v>
+      </c>
+      <c r="B73" t="s">
+        <v>894</v>
+      </c>
+      <c r="C73" t="s">
+        <v>895</v>
+      </c>
+      <c r="D73" t="s">
+        <v>896</v>
+      </c>
+      <c r="E73" s="43" t="s">
+        <v>900</v>
+      </c>
+      <c r="F73" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>4</v>
+      </c>
+      <c r="B74" t="s">
+        <v>897</v>
+      </c>
+      <c r="C74" t="s">
+        <v>898</v>
+      </c>
+      <c r="D74" t="s">
+        <v>899</v>
+      </c>
+      <c r="E74" s="43" t="s">
+        <v>900</v>
+      </c>
+      <c r="F74" s="30" t="s">
+        <v>887</v>
       </c>
     </row>
   </sheetData>
@@ -6332,24 +6494,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="42" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6437,14 +6599,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="38" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6532,14 +6694,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="35" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="35"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="37"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -6661,14 +6823,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="35" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="35"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="37"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -6798,26 +6960,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="38" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="37"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7113,24 +7275,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="35" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7315,14 +7477,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="40" t="s">
+      <c r="A18" s="42" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="35"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="37"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7423,14 +7585,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="38" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="35"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="37"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7526,14 +7688,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7710,14 +7872,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8320,13 +8482,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8723,13 +8885,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
docs: chiude FASE 1 del piano di rilascio nel tracker
Sposta FIX-004, CACHE-001, FIX-001 e NAMING-001 in "Fix completate" in
BACKEND_FIX_TODO.md, aggiorna lo stato sessione in CLAUDE.md e il tracker
Excel (Dashboard, Appunti e Step, Fix e Bug) con il resoconto dei tre blocchi
di fix committati in questa sessione.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9316D934-6D02-4DDE-A60B-332ACD1A3E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E90697C5-32A3-4292-A2CA-63FF9E36FB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="901">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="912">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2683,12 +2683,6 @@
     <t>In corso</t>
   </si>
   <si>
-    <t>Aggiornato: 12/08/2026</t>
-  </si>
-  <si>
-    <t>Aggiornato: 12/08/2026  ·  Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
     <t>SESSIONE 12/08/2026 - Manutenzione repo e config Claude Code</t>
   </si>
   <si>
@@ -2735,6 +2729,45 @@
   </si>
   <si>
     <t>12/08/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 13/08/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 13/08/2026  ·  Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>FASE 1 PIANO DI RILASCIO - Fix backend (sessione 13/08/2026)</t>
+  </si>
+  <si>
+    <t># | Modulo | Cosa e' stato fatto | Pattern / Tecnologia | Data | Stato</t>
+  </si>
+  <si>
+    <t>FasciaOrariaService</t>
+  </si>
+  <si>
+    <t>FIX-004 A/B/C: guard sovrapposizione condiviso su Add/Update/UpdateStato, esteso a fasce disattivate; TryParse validato. CACHE-001: invalidazione fasce_giorno_n su tutte le scritture.</t>
+  </si>
+  <si>
+    <t>xUnit + Moq + MockQueryable.Moq</t>
+  </si>
+  <si>
+    <t>13/08/2026</t>
+  </si>
+  <si>
+    <t>PostazioneService</t>
+  </si>
+  <si>
+    <t>Verifica pattern cache: trovato e corretto stesso buco CACHE-001 in AssociaPostazioneAZonaAsync (PostazioniAttive non invalidata).</t>
+  </si>
+  <si>
+    <t>FIX-001: UpdateAsync(PostazioneUpdateDTO) non validava esistenza zona (AddAsync si'). Aggiunta validazione.</t>
+  </si>
+  <si>
+    <t>PrenotazioneDTO1.cs</t>
+  </si>
+  <si>
+    <t>NAMING-001: rinominato in PrenotazioneCreateDTO.cs (allineato nome file/classe).</t>
   </si>
 </sst>
 </file>
@@ -2992,7 +3025,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3078,6 +3111,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3108,7 +3142,9 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -3423,36 +3459,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
-        <v>883</v>
-      </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="A2" s="32" t="s">
+        <v>899</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="35" t="s">
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="36"/>
-      <c r="F4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="38"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3617,24 +3653,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="37"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="38"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3662,14 +3698,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4612,13 +4648,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4962,11 +4998,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5232,14 +5268,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5311,7 +5347,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5323,40 +5359,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
-        <v>884</v>
-      </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="A2" s="32" t="s">
+        <v>900</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="37"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5679,16 +5715,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5911,16 +5947,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="39" t="s">
+      <c r="A35" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="36"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="36"/>
-      <c r="G35" s="36"/>
-      <c r="H35" s="37"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="38"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6103,16 +6139,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="40" t="s">
+      <c r="A46" s="41" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="36"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="36"/>
-      <c r="E46" s="36"/>
-      <c r="F46" s="36"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="37"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="38"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6175,16 +6211,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="36"/>
-      <c r="C51" s="36"/>
-      <c r="D51" s="36"/>
-      <c r="E51" s="36"/>
-      <c r="F51" s="36"/>
-      <c r="G51" s="36"/>
-      <c r="H51" s="37"/>
+      <c r="B51" s="37"/>
+      <c r="C51" s="37"/>
+      <c r="D51" s="37"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="37"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="38"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6364,7 +6400,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -6375,7 +6411,7 @@
         <v>45</v>
       </c>
       <c r="C70" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="D70" t="s">
         <v>47</v>
@@ -6392,16 +6428,16 @@
         <v>1</v>
       </c>
       <c r="B71" t="s">
+        <v>886</v>
+      </c>
+      <c r="C71" t="s">
+        <v>887</v>
+      </c>
+      <c r="D71" t="s">
         <v>888</v>
       </c>
-      <c r="C71" t="s">
-        <v>889</v>
-      </c>
-      <c r="D71" t="s">
-        <v>890</v>
-      </c>
-      <c r="E71" s="43" t="s">
-        <v>900</v>
+      <c r="E71" s="31" t="s">
+        <v>898</v>
       </c>
       <c r="F71" s="29" t="s">
         <v>6</v>
@@ -6412,16 +6448,16 @@
         <v>2</v>
       </c>
       <c r="B72" t="s">
+        <v>889</v>
+      </c>
+      <c r="C72" t="s">
+        <v>890</v>
+      </c>
+      <c r="D72" t="s">
         <v>891</v>
       </c>
-      <c r="C72" t="s">
-        <v>892</v>
-      </c>
-      <c r="D72" t="s">
-        <v>893</v>
-      </c>
-      <c r="E72" s="43" t="s">
-        <v>900</v>
+      <c r="E72" s="31" t="s">
+        <v>898</v>
       </c>
       <c r="F72" s="29" t="s">
         <v>6</v>
@@ -6432,16 +6468,16 @@
         <v>3</v>
       </c>
       <c r="B73" t="s">
+        <v>892</v>
+      </c>
+      <c r="C73" t="s">
+        <v>893</v>
+      </c>
+      <c r="D73" t="s">
         <v>894</v>
       </c>
-      <c r="C73" t="s">
-        <v>895</v>
-      </c>
-      <c r="D73" t="s">
-        <v>896</v>
-      </c>
-      <c r="E73" s="43" t="s">
-        <v>900</v>
+      <c r="E73" s="31" t="s">
+        <v>898</v>
       </c>
       <c r="F73" s="29" t="s">
         <v>6</v>
@@ -6452,19 +6488,109 @@
         <v>4</v>
       </c>
       <c r="B74" t="s">
+        <v>895</v>
+      </c>
+      <c r="C74" t="s">
+        <v>896</v>
+      </c>
+      <c r="D74" t="s">
         <v>897</v>
       </c>
-      <c r="C74" t="s">
+      <c r="E74" s="31" t="s">
         <v>898</v>
       </c>
-      <c r="D74" t="s">
-        <v>899</v>
-      </c>
-      <c r="E74" s="43" t="s">
-        <v>900</v>
-      </c>
       <c r="F74" s="30" t="s">
-        <v>887</v>
+        <v>885</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>1</v>
+      </c>
+      <c r="B78" t="s">
+        <v>903</v>
+      </c>
+      <c r="C78" t="s">
+        <v>904</v>
+      </c>
+      <c r="D78" t="s">
+        <v>905</v>
+      </c>
+      <c r="E78" t="s">
+        <v>906</v>
+      </c>
+      <c r="F78" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>2</v>
+      </c>
+      <c r="B79" t="s">
+        <v>907</v>
+      </c>
+      <c r="C79" t="s">
+        <v>908</v>
+      </c>
+      <c r="D79" t="s">
+        <v>73</v>
+      </c>
+      <c r="E79" t="s">
+        <v>906</v>
+      </c>
+      <c r="F79" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>3</v>
+      </c>
+      <c r="B80" t="s">
+        <v>907</v>
+      </c>
+      <c r="C80" t="s">
+        <v>909</v>
+      </c>
+      <c r="D80" t="s">
+        <v>86</v>
+      </c>
+      <c r="E80" t="s">
+        <v>906</v>
+      </c>
+      <c r="F80" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>4</v>
+      </c>
+      <c r="B81" t="s">
+        <v>910</v>
+      </c>
+      <c r="C81" t="s">
+        <v>911</v>
+      </c>
+      <c r="D81" t="s">
+        <v>888</v>
+      </c>
+      <c r="E81" t="s">
+        <v>906</v>
+      </c>
+      <c r="F81" s="29" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -6494,24 +6620,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="43" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6599,14 +6725,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="39" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="36"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="37"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="38"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6694,14 +6820,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -6823,14 +6949,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="35" t="s">
+      <c r="A26" s="36" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="36"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="37"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="38"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -6960,26 +7086,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="39" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="37"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7275,24 +7401,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="36" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7477,14 +7603,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="43" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7552,8 +7678,8 @@
       <c r="C23" s="14" t="s">
         <v>394</v>
       </c>
-      <c r="D23" s="25" t="s">
-        <v>186</v>
+      <c r="D23" s="44" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7585,14 +7711,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="38" t="s">
+      <c r="A27" s="39" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="37"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="38"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7688,14 +7814,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7872,14 +7998,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8482,13 +8608,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8885,13 +9011,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
docs: chiude SEC-001, aggiunge Utilities.txt con note pratiche
Utilities.txt: nuovo file di appunti in root progetto per note pratiche
non legate allo stato di avanzamento (percorsi, comandi) — a partire dal
percorso e dai comandi per recuperare/modificare i secrets User Secrets.

BACKEND_FIX_TODO.md, CLAUDE.md, tracker: SEC-001 spostato in "Fix completate",
FASE 1 del piano di rilascio ora completamente chiusa (nessun fix aperto
tranne AUDIT-001, rimandato post-v1.0 per decisione architetturale).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E90697C5-32A3-4292-A2CA-63FF9E36FB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E97F76E-C259-4EFC-ADE2-0CB03EA88ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="913">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2764,10 +2764,13 @@
     <t>FIX-001: UpdateAsync(PostazioneUpdateDTO) non validava esistenza zona (AddAsync si'). Aggiunta validazione.</t>
   </si>
   <si>
-    <t>PrenotazioneDTO1.cs</t>
-  </si>
-  <si>
-    <t>NAMING-001: rinominato in PrenotazioneCreateDTO.cs (allineato nome file/classe).</t>
+    <t>SEC-001 (User Secrets)</t>
+  </si>
+  <si>
+    <t>Segreti dev migrati da appsettings.Development.json a dotnet user-secrets. Guidato Fabio passo passo, verificato con build/avvio/login. UserSecretsId committato. Store e comandi documentati in Utilities.txt.</t>
+  </si>
+  <si>
+    <t>dotnet user-secrets</t>
   </si>
 </sst>
 </file>
@@ -3112,6 +3115,9 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3141,9 +3147,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3459,36 +3462,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>899</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="36" t="s">
+      <c r="B4" s="38"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="39"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3653,24 +3656,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="38"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3698,14 +3701,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4648,13 +4651,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4998,11 +5001,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5268,14 +5271,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5359,40 +5362,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>900</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="38"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="39"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5715,16 +5718,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="39"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5947,16 +5950,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="40" t="s">
+      <c r="A35" s="41" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="37"/>
-      <c r="H35" s="38"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="39"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6139,16 +6142,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="41" t="s">
+      <c r="A46" s="42" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="37"/>
-      <c r="C46" s="37"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="37"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="37"/>
-      <c r="H46" s="38"/>
+      <c r="B46" s="38"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="38"/>
+      <c r="G46" s="38"/>
+      <c r="H46" s="39"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6211,16 +6214,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="39" t="s">
+      <c r="A51" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="37"/>
-      <c r="C51" s="37"/>
-      <c r="D51" s="37"/>
-      <c r="E51" s="37"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="38"/>
+      <c r="B51" s="38"/>
+      <c r="C51" s="38"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="38"/>
+      <c r="F51" s="38"/>
+      <c r="G51" s="38"/>
+      <c r="H51" s="39"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6575,7 +6578,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B81" t="s">
         <v>910</v>
@@ -6584,7 +6587,7 @@
         <v>911</v>
       </c>
       <c r="D81" t="s">
-        <v>888</v>
+        <v>912</v>
       </c>
       <c r="E81" t="s">
         <v>906</v>
@@ -6620,24 +6623,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="44" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="38"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="39"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6725,14 +6728,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="40" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="38"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6820,14 +6823,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="38"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="39"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -6949,14 +6952,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="36" t="s">
+      <c r="A26" s="37" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="38"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="39"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -7086,26 +7089,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="40" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="38"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7401,24 +7404,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="37" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="38"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="39"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7603,14 +7606,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="44" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="38"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="39"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7678,7 +7681,7 @@
       <c r="C23" s="14" t="s">
         <v>394</v>
       </c>
-      <c r="D23" s="44" t="s">
+      <c r="D23" s="32" t="s">
         <v>6</v>
       </c>
     </row>
@@ -7711,14 +7714,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="39" t="s">
+      <c r="A27" s="40" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="38"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="39"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7814,14 +7817,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7998,14 +8001,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8608,13 +8611,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9011,13 +9014,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
docs: chiude FASE 2 del piano di rilascio nel tracker
Aggiorna CLAUDE.md e tracker con l'esito della verifica manuale Swagger/curl
sui fix di sessione (FIX-004, CACHE-001, FIX-001, CORS) e con il resoconto
del bug multi-ruolo emerso e risolto durante la fase, non pianificato in
origine.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E97F76E-C259-4EFC-ADE2-0CB03EA88ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{949E5CDE-64C7-4907-AF61-9E20DE195038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="922">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2771,6 +2771,33 @@
   </si>
   <si>
     <t>dotnet user-secrets</t>
+  </si>
+  <si>
+    <t>RBAC-001</t>
+  </si>
+  <si>
+    <t>Ridefinito perimetro Staff/Cliente con Fabio (verifica riga per riga di tutti gli Authorize). Staff: lettura completa, scrittura senza delete-prenotazione. Cliente: tolti update/annulla prenotazione (serve regola cutoff, RBAC-002).</t>
+  </si>
+  <si>
+    <t>GestoraWebApi.Auth.Roles</t>
+  </si>
+  <si>
+    <t>Fix multi-ruolo frontend</t>
+  </si>
+  <si>
+    <t>Bug: AuthUser.role stringa singola non gestiva utenti con piu ruoli (JWT serializza come array). Fix: roles string[], normalizeRoles(), ProtectedRoute/AppLayout/PrenotazionePage/LoginPage aggiornati.</t>
+  </si>
+  <si>
+    <t>React + TypeScript</t>
+  </si>
+  <si>
+    <t>FASE 2 Piano Rilascio</t>
+  </si>
+  <si>
+    <t>dotnet test verde (28/28) + verifica manuale Swagger/curl: FIX-004 A/B/C, CACHE-001, FIX-001, CORS. Tutti confermati con token Admin reale.</t>
+  </si>
+  <si>
+    <t>curl + Swagger</t>
   </si>
 </sst>
 </file>
@@ -5350,7 +5377,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -6593,6 +6620,66 @@
         <v>906</v>
       </c>
       <c r="F81" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>6</v>
+      </c>
+      <c r="B86" t="s">
+        <v>913</v>
+      </c>
+      <c r="C86" t="s">
+        <v>914</v>
+      </c>
+      <c r="D86" t="s">
+        <v>915</v>
+      </c>
+      <c r="E86" t="s">
+        <v>906</v>
+      </c>
+      <c r="F86" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>7</v>
+      </c>
+      <c r="B87" t="s">
+        <v>916</v>
+      </c>
+      <c r="C87" t="s">
+        <v>917</v>
+      </c>
+      <c r="D87" t="s">
+        <v>918</v>
+      </c>
+      <c r="E87" t="s">
+        <v>906</v>
+      </c>
+      <c r="F87" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>8</v>
+      </c>
+      <c r="B88" t="s">
+        <v>919</v>
+      </c>
+      <c r="C88" t="s">
+        <v>920</v>
+      </c>
+      <c r="D88" t="s">
+        <v>921</v>
+      </c>
+      <c r="E88" t="s">
+        <v>906</v>
+      </c>
+      <c r="F88" s="29" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: registra la decisione di non bloccare il rilascio sul debito residuo
Deciso con Fabio il 13/08/2026: RBAC-002 (cutoff self-service Cliente),
AUDIT-001 (tracciabilità utente) e un secondo caso di NAMING-001 (file
FasciaOrariaController.cs vs classe FasceOrarieController) non bloccano
Fase 3+ del piano di rilascio — nessuno dei tre tocca il percorso di
produzione. Spostati in una sezione dedicata "Backlog post-v1.0" in
BACKEND_FIX_TODO.md, da riprendere dopo il rilascio.

Allineati CLAUDE.md, PIANO_RILASCIO.md e tracker con la decisione. Corretto
anche uno stato stale nel tracker (FIX-004 riformulato segnato "Da fare"
nonostante fosse già stato completato in un commit precedente).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{949E5CDE-64C7-4907-AF61-9E20DE195038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4AD433-7058-4DD9-8507-57C2BE16B975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1578" uniqueCount="923">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2689,9 +2689,6 @@
     <t>Cosa e' stato fatto</t>
   </si>
   <si>
-    <t>Da fare</t>
-  </si>
-  <si>
     <t>Igiene repo</t>
   </si>
   <si>
@@ -2798,6 +2795,12 @@
   </si>
   <si>
     <t>curl + Swagger</t>
+  </si>
+  <si>
+    <t>Debito tecnico residuo (RBAC-002 cutoff Cliente, AUDIT-001 tracciabilita, NAMING-001-residuo) non blocca il rilascio</t>
+  </si>
+  <si>
+    <t>Evitare scope-creep sul deploy: nessuno dei tre tocca il percorso di produzione. Spostati in Backlog post-v1.0 in BACKEND_FIX_TODO.md, si affrontano dopo la Fase 8.</t>
   </si>
 </sst>
 </file>
@@ -2893,7 +2896,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2997,12 +3000,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -3055,7 +3052,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3140,7 +3137,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3489,36 +3485,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
-        <v>899</v>
-      </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
+      <c r="A2" s="32" t="s">
+        <v>898</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="37" t="s">
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="38"/>
-      <c r="F4" s="39"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="38"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3683,24 +3679,24 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="40" t="s">
+      <c r="A15" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="39"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="38"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3728,14 +3724,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>655</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4678,13 +4674,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>768</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5028,11 +5024,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>821</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5298,14 +5294,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>867</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5377,7 +5373,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5389,40 +5385,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
-        <v>900</v>
-      </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
+      <c r="A2" s="32" t="s">
+        <v>899</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="39"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5745,16 +5741,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="39"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -5977,16 +5973,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="41" t="s">
+      <c r="A35" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="38"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="38"/>
-      <c r="F35" s="38"/>
-      <c r="G35" s="38"/>
-      <c r="H35" s="39"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="38"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6169,16 +6165,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="41" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="38"/>
-      <c r="C46" s="38"/>
-      <c r="D46" s="38"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="38"/>
-      <c r="G46" s="38"/>
-      <c r="H46" s="39"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="37"/>
+      <c r="E46" s="37"/>
+      <c r="F46" s="37"/>
+      <c r="G46" s="37"/>
+      <c r="H46" s="38"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6241,16 +6237,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="40" t="s">
+      <c r="A51" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="B51" s="38"/>
-      <c r="C51" s="38"/>
-      <c r="D51" s="38"/>
-      <c r="E51" s="38"/>
-      <c r="F51" s="38"/>
-      <c r="G51" s="38"/>
-      <c r="H51" s="39"/>
+      <c r="B51" s="37"/>
+      <c r="C51" s="37"/>
+      <c r="D51" s="37"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="37"/>
+      <c r="G51" s="37"/>
+      <c r="H51" s="38"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6428,66 +6424,57 @@
         <v>225</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>883</v>
+    <row r="68" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="26" t="s">
+        <v>905</v>
+      </c>
+      <c r="B68" s="26" t="s">
+        <v>921</v>
+      </c>
+      <c r="C68" s="26" t="s">
+        <v>922</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
         <v>44</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B71" t="s">
         <v>45</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C71" t="s">
         <v>884</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D71" t="s">
         <v>47</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E71" t="s">
         <v>48</v>
       </c>
-      <c r="F70" t="s">
+      <c r="F71" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71">
-        <v>1</v>
-      </c>
-      <c r="B71" t="s">
-        <v>886</v>
-      </c>
-      <c r="C71" t="s">
-        <v>887</v>
-      </c>
-      <c r="D71" t="s">
-        <v>888</v>
-      </c>
-      <c r="E71" s="31" t="s">
-        <v>898</v>
-      </c>
-      <c r="F71" s="29" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B72" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="C72" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
       <c r="D72" t="s">
-        <v>891</v>
-      </c>
-      <c r="E72" s="31" t="s">
-        <v>898</v>
+        <v>887</v>
+      </c>
+      <c r="E72" s="30" t="s">
+        <v>897</v>
       </c>
       <c r="F72" s="29" t="s">
         <v>6</v>
@@ -6495,19 +6482,19 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B73" t="s">
-        <v>892</v>
+        <v>888</v>
       </c>
       <c r="C73" t="s">
-        <v>893</v>
+        <v>889</v>
       </c>
       <c r="D73" t="s">
-        <v>894</v>
-      </c>
-      <c r="E73" s="31" t="s">
-        <v>898</v>
+        <v>890</v>
+      </c>
+      <c r="E73" s="30" t="s">
+        <v>897</v>
       </c>
       <c r="F73" s="29" t="s">
         <v>6</v>
@@ -6515,69 +6502,69 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
+        <v>3</v>
+      </c>
+      <c r="B74" t="s">
+        <v>891</v>
+      </c>
+      <c r="C74" t="s">
+        <v>892</v>
+      </c>
+      <c r="D74" t="s">
+        <v>893</v>
+      </c>
+      <c r="E74" s="30" t="s">
+        <v>897</v>
+      </c>
+      <c r="F74" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75">
         <v>4</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B75" t="s">
+        <v>894</v>
+      </c>
+      <c r="C75" t="s">
         <v>895</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D75" t="s">
         <v>896</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E75" s="30" t="s">
         <v>897</v>
       </c>
-      <c r="E74" s="31" t="s">
-        <v>898</v>
-      </c>
-      <c r="F74" s="30" t="s">
-        <v>885</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>901</v>
+      <c r="F75" s="29" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78">
-        <v>1</v>
-      </c>
-      <c r="B78" t="s">
-        <v>903</v>
-      </c>
-      <c r="C78" t="s">
-        <v>904</v>
-      </c>
-      <c r="D78" t="s">
-        <v>905</v>
-      </c>
-      <c r="E78" t="s">
-        <v>906</v>
-      </c>
-      <c r="F78" s="29" t="s">
-        <v>6</v>
+      <c r="A78" t="s">
+        <v>901</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B79" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="C79" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="D79" t="s">
-        <v>73</v>
+        <v>904</v>
       </c>
       <c r="E79" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="F79" s="29" t="s">
         <v>6</v>
@@ -6585,19 +6572,19 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B80" t="s">
+        <v>906</v>
+      </c>
+      <c r="C80" t="s">
         <v>907</v>
       </c>
-      <c r="C80" t="s">
-        <v>909</v>
-      </c>
       <c r="D80" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="E80" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="F80" s="29" t="s">
         <v>6</v>
@@ -6605,59 +6592,59 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
+        <v>3</v>
+      </c>
+      <c r="B81" t="s">
+        <v>906</v>
+      </c>
+      <c r="C81" t="s">
+        <v>908</v>
+      </c>
+      <c r="D81" t="s">
+        <v>86</v>
+      </c>
+      <c r="E81" t="s">
+        <v>905</v>
+      </c>
+      <c r="F81" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82">
         <v>5</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B82" t="s">
+        <v>909</v>
+      </c>
+      <c r="C82" t="s">
         <v>910</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D82" t="s">
         <v>911</v>
       </c>
-      <c r="D81" t="s">
-        <v>912</v>
-      </c>
-      <c r="E81" t="s">
-        <v>906</v>
-      </c>
-      <c r="F81" s="29" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86">
-        <v>6</v>
-      </c>
-      <c r="B86" t="s">
-        <v>913</v>
-      </c>
-      <c r="C86" t="s">
-        <v>914</v>
-      </c>
-      <c r="D86" t="s">
-        <v>915</v>
-      </c>
-      <c r="E86" t="s">
-        <v>906</v>
-      </c>
-      <c r="F86" s="29" t="s">
+      <c r="E82" t="s">
+        <v>905</v>
+      </c>
+      <c r="F82" s="29" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B87" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="C87" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="D87" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="E87" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="F87" s="29" t="s">
         <v>6</v>
@@ -6665,21 +6652,41 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88">
+        <v>7</v>
+      </c>
+      <c r="B88" t="s">
+        <v>915</v>
+      </c>
+      <c r="C88" t="s">
+        <v>916</v>
+      </c>
+      <c r="D88" t="s">
+        <v>917</v>
+      </c>
+      <c r="E88" t="s">
+        <v>905</v>
+      </c>
+      <c r="F88" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89">
         <v>8</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B89" t="s">
+        <v>918</v>
+      </c>
+      <c r="C89" t="s">
         <v>919</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D89" t="s">
         <v>920</v>
       </c>
-      <c r="D88" t="s">
-        <v>921</v>
-      </c>
-      <c r="E88" t="s">
-        <v>906</v>
-      </c>
-      <c r="F88" s="29" t="s">
+      <c r="E89" t="s">
+        <v>905</v>
+      </c>
+      <c r="F89" s="29" t="s">
         <v>6</v>
       </c>
     </row>
@@ -6710,24 +6717,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="43" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="39"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -6815,14 +6822,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="39" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="39"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="38"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6910,14 +6917,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -7039,14 +7046,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="37" t="s">
+      <c r="A26" s="36" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="39"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="38"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -7176,26 +7183,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="39" t="s">
         <v>296</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="39"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7491,24 +7498,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="36" t="s">
         <v>355</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="39"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7693,14 +7700,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
+      <c r="A18" s="43" t="s">
         <v>387</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -7768,7 +7775,7 @@
       <c r="C23" s="14" t="s">
         <v>394</v>
       </c>
-      <c r="D23" s="32" t="s">
+      <c r="D23" s="31" t="s">
         <v>6</v>
       </c>
     </row>
@@ -7801,14 +7808,14 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="39" t="s">
         <v>400</v>
       </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="39"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="38"/>
     </row>
     <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
@@ -7904,14 +7911,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>412</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8088,14 +8095,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8698,13 +8705,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>511</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9101,13 +9108,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
docs: chiude FASE 4 del piano di rilascio (backend verificato in produzione)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AADF87-2EDD-4BF9-BD76-C09CA3FD86E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E3859A-5F82-492F-9EA9-11AC62A7B496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="963">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1689" uniqueCount="978">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2791,9 +2791,6 @@
     <t>Evitare scope-creep sul deploy: nessuno dei tre tocca il percorso di produzione. Spostati in Backlog post-v1.0 in BACKEND_FIX_TODO.md, si affrontano dopo la Fase 8.</t>
   </si>
   <si>
-    <t>Aggiornato: 14/08/2026</t>
-  </si>
-  <si>
     <t>Deploy Backend</t>
   </si>
   <si>
@@ -2809,12 +2806,6 @@
     <t>Railway + GitHub Actions</t>
   </si>
   <si>
-    <t>Frontend completato. Deploy: backend su Railway OK (14/08/26), frontend Vercel da fare</t>
-  </si>
-  <si>
-    <t>Aggiornato: 14/08/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
     <t>14/08/2026</t>
   </si>
   <si>
@@ -2893,9 +2884,6 @@
     <t>FIX-007 - 404 su lista vuota</t>
   </si>
   <si>
-    <t>Sei endpoint restituiscono 404 invece di 200 con array vuoto quando non ci sono dati. Stesso anti-pattern di FIX-003, corretto solo sulle fasce orarie. Si manifesta sempre su un database di produzione appena creato. Trovato il 14/08/2026 verificando il deploy Railway. Da valutare in Fase 5.</t>
-  </si>
-  <si>
     <t>Da fare</t>
   </si>
   <si>
@@ -2921,13 +2909,70 @@
   </si>
   <si>
     <t>200 List&lt;PrenotazioneDTO&gt; filtrate su UserId dal JWT</t>
+  </si>
+  <si>
+    <t>Aggiornato: 25/08/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 25/08/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>FASE 4 PIANO DI RILASCIO - Verifica backend in produzione (sessione 25/08/2026)</t>
+  </si>
+  <si>
+    <t>Riallineamento repo</t>
+  </si>
+  <si>
+    <t>dev era avanti di 2 commit non mergiati su main (chiusura Fase 3); .gitignore aveva .vs/ scritto come commento invece di regola attiva, causando errori di commit/push su file di lock in uso. Merge dev-&gt;main (PR #3) e main-&gt;dev, .gitignore corretto in .vs/.</t>
+  </si>
+  <si>
+    <t>Git flow + GitHub PR</t>
+  </si>
+  <si>
+    <t>25/08/2026</t>
+  </si>
+  <si>
+    <t>Verifica endpoint Zona</t>
+  </si>
+  <si>
+    <t>GET get-all-zone con token Admin su DB di produzione vuoto -&gt; 404 Nessuna zona trovata. Comportamento noto e gia' tracciato, vedi FIX-007.</t>
+  </si>
+  <si>
+    <t>Postman + token JWT</t>
+  </si>
+  <si>
+    <t>Verifica endpoint FasceOrarie</t>
+  </si>
+  <si>
+    <t>GET fasce-attive con token Admin su DB vuoto -&gt; 200 OK con []. Conferma che FIX-003 tiene anche in produzione.</t>
+  </si>
+  <si>
+    <t>Verifica endpoint Dashboard</t>
+  </si>
+  <si>
+    <t>GET giornaliera con token Admin su DB vuoto -&gt; 200 OK con tutti i contatori a zero. L'aggregato non soffre dell'anti-pattern di FIX-007.</t>
+  </si>
+  <si>
+    <t>Log Railway</t>
+  </si>
+  <si>
+    <t>Controllati i log del servizio .NET su Railway durante le chiamate di verifica: nessuna eccezione, nessun errore.</t>
+  </si>
+  <si>
+    <t>Railway Deploy Logs</t>
+  </si>
+  <si>
+    <t>Frontend completato. Deploy: backend su Railway OK (14/08/26), verificato in produzione (Fase 4, 25/08/26). Frontend Vercel da fare.</t>
+  </si>
+  <si>
+    <t>Sei endpoint restituiscono 404 invece di 200 con array vuoto quando non ci sono dati. Stesso anti-pattern di FIX-003, corretto solo sulle fasce orarie. Si manifesta sempre su un database di produzione appena creato. Trovato il 14/08/2026 verificando il deploy Railway. Riconfermato in Fase 4 (25/08/2026): comportamento invariato. Da decidere in Fase 5 se e come sistemarlo prima di collegare il frontend.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3014,6 +3059,14 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="20">
@@ -3167,7 +3220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3262,6 +3315,7 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3606,36 +3660,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="34" t="s">
-        <v>919</v>
-      </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
+      <c r="A2" s="35" t="s">
+        <v>959</v>
+      </c>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="38" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="39"/>
-      <c r="F4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="41"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3804,34 +3858,34 @@
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
       <c r="D14" s="1" t="s">
+        <v>919</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>920</v>
       </c>
-      <c r="E14" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>921</v>
-      </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="41" t="s">
+      <c r="A15" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="41"/>
     </row>
     <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3859,14 +3913,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>653</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4516,7 +4570,7 @@
         <v>678</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>693</v>
@@ -4525,7 +4579,7 @@
         <v>443</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4676,7 +4730,7 @@
         <v>678</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>861</v>
@@ -4685,7 +4739,7 @@
         <v>443</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4850,22 +4904,22 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="B52" t="s">
         <v>678</v>
       </c>
       <c r="C52" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="D52" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="E52" t="s">
         <v>443</v>
       </c>
       <c r="F52" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
     </row>
   </sheetData>
@@ -4889,13 +4943,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>766</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5239,11 +5293,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>819</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5509,14 +5563,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>865</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5588,7 +5642,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5600,40 +5654,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="34" t="s">
-        <v>926</v>
-      </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
+      <c r="A2" s="35" t="s">
+        <v>960</v>
+      </c>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -5956,16 +6010,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="40"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="41"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -6188,16 +6242,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="42" t="s">
+      <c r="A35" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="39"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="40"/>
+      <c r="B35" s="40"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="40"/>
+      <c r="G35" s="40"/>
+      <c r="H35" s="41"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6380,16 +6434,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="44" t="s">
         <v>178</v>
       </c>
-      <c r="B46" s="39"/>
-      <c r="C46" s="39"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="39"/>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="40"/>
+      <c r="B46" s="40"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="40"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="40"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="41"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6452,16 +6506,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="41" t="s">
+      <c r="A51" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="B51" s="39"/>
-      <c r="C51" s="39"/>
-      <c r="D51" s="39"/>
-      <c r="E51" s="39"/>
-      <c r="F51" s="39"/>
-      <c r="G51" s="39"/>
-      <c r="H51" s="40"/>
+      <c r="B51" s="40"/>
+      <c r="C51" s="40"/>
+      <c r="D51" s="40"/>
+      <c r="E51" s="40"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="41"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6652,24 +6706,24 @@
     </row>
     <row r="69" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="25" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="B69" s="25" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C69" s="25" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="25" t="s">
+        <v>924</v>
+      </c>
+      <c r="B70" s="25" t="s">
         <v>927</v>
       </c>
-      <c r="B70" s="25" t="s">
-        <v>930</v>
-      </c>
       <c r="C70" s="25" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -6929,7 +6983,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="E93" s="28"/>
       <c r="F93" s="27"/>
@@ -6959,16 +7013,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="C95" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="D95" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="E95" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F95" s="27" t="s">
         <v>6</v>
@@ -6979,16 +7033,16 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
-        <v>936</v>
+        <v>933</v>
       </c>
       <c r="C96" t="s">
-        <v>937</v>
+        <v>934</v>
       </c>
       <c r="D96" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="E96" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F96" s="27" t="s">
         <v>6</v>
@@ -6999,16 +7053,16 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="C97" t="s">
-        <v>940</v>
+        <v>937</v>
       </c>
       <c r="D97" t="s">
-        <v>941</v>
+        <v>938</v>
       </c>
       <c r="E97" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F97" s="27" t="s">
         <v>6</v>
@@ -7019,16 +7073,16 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>942</v>
+        <v>939</v>
       </c>
       <c r="C98" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
       <c r="D98" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="E98" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F98" s="27" t="s">
         <v>6</v>
@@ -7039,16 +7093,16 @@
         <v>5</v>
       </c>
       <c r="B99" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="C99" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
       <c r="D99" t="s">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="E99" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F99" s="27" t="s">
         <v>6</v>
@@ -7059,18 +7113,143 @@
         <v>6</v>
       </c>
       <c r="B100" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="C100" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="D100" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
       <c r="E100" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="F100" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="34" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>44</v>
+      </c>
+      <c r="B103" t="s">
+        <v>45</v>
+      </c>
+      <c r="C103" t="s">
+        <v>882</v>
+      </c>
+      <c r="D103" t="s">
+        <v>47</v>
+      </c>
+      <c r="E103" t="s">
+        <v>48</v>
+      </c>
+      <c r="F103" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104">
+        <v>1</v>
+      </c>
+      <c r="B104" t="s">
+        <v>962</v>
+      </c>
+      <c r="C104" t="s">
+        <v>963</v>
+      </c>
+      <c r="D104" t="s">
+        <v>964</v>
+      </c>
+      <c r="E104" t="s">
+        <v>965</v>
+      </c>
+      <c r="F104" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>2</v>
+      </c>
+      <c r="B105" t="s">
+        <v>966</v>
+      </c>
+      <c r="C105" t="s">
+        <v>967</v>
+      </c>
+      <c r="D105" t="s">
+        <v>968</v>
+      </c>
+      <c r="E105" t="s">
+        <v>965</v>
+      </c>
+      <c r="F105" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>3</v>
+      </c>
+      <c r="B106" t="s">
+        <v>969</v>
+      </c>
+      <c r="C106" t="s">
+        <v>970</v>
+      </c>
+      <c r="D106" t="s">
+        <v>968</v>
+      </c>
+      <c r="E106" t="s">
+        <v>965</v>
+      </c>
+      <c r="F106" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <v>4</v>
+      </c>
+      <c r="B107" t="s">
+        <v>971</v>
+      </c>
+      <c r="C107" t="s">
+        <v>972</v>
+      </c>
+      <c r="D107" t="s">
+        <v>968</v>
+      </c>
+      <c r="E107" t="s">
+        <v>965</v>
+      </c>
+      <c r="F107" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108">
+        <v>5</v>
+      </c>
+      <c r="B108" t="s">
+        <v>973</v>
+      </c>
+      <c r="C108" t="s">
+        <v>974</v>
+      </c>
+      <c r="D108" t="s">
+        <v>975</v>
+      </c>
+      <c r="E108" t="s">
+        <v>965</v>
+      </c>
+      <c r="F108" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -7101,24 +7280,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="46" t="s">
         <v>226</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="41"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7206,14 +7385,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="42" t="s">
         <v>246</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="41"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -7301,14 +7480,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="39" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="40"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="41"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -7430,14 +7609,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="39" t="s">
         <v>284</v>
       </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="40"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="41"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -7546,13 +7725,13 @@
         <v>285</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>921</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>922</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="D33" s="2" t="s">
         <v>923</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>924</v>
       </c>
       <c r="E33" s="30" t="s">
         <v>6</v>
@@ -7584,26 +7763,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>294</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="42" t="s">
         <v>295</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7858,7 +8037,7 @@
         <v>880</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>925</v>
+        <v>976</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7901,24 +8080,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>352</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="39" t="s">
         <v>353</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="41"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8103,14 +8282,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="45" t="s">
+      <c r="A18" s="46" t="s">
         <v>385</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="40"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="41"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -8212,27 +8391,27 @@
     </row>
     <row r="26" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>953</v>
+        <v>977</v>
       </c>
       <c r="D26" s="33" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="41" t="s">
+      <c r="A28" s="42" t="s">
         <v>398</v>
       </c>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="40"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="41"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -8328,14 +8507,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>410</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8512,14 +8691,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>433</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9122,13 +9301,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>509</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9525,13 +9704,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>588</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
docs: aggiorna stato progetto a fine Fase 7, chiude backlog pre-rilascio
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E3859A-5F82-492F-9EA9-11AC62A7B496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEFE51A-6821-4D47-8656-5CA5833F901B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1689" uniqueCount="978">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="1007">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2674,9 +2674,6 @@
     <t>Elimina prenotazioni Completate con DataPrenotazione &gt; 6 mesi fa</t>
   </si>
   <si>
-    <t>In corso</t>
-  </si>
-  <si>
     <t>SESSIONE 12/08/2026 - Manutenzione repo e config Claude Code</t>
   </si>
   <si>
@@ -2878,94 +2875,184 @@
     <t>PowerShell Invoke-RestMethod</t>
   </si>
   <si>
-    <t>Zona / Postazione / Prenotazione</t>
-  </si>
-  <si>
-    <t>FIX-007 - 404 su lista vuota</t>
+    <t>(Program.cs)</t>
+  </si>
+  <si>
+    <t>/health</t>
+  </si>
+  <si>
+    <t>Pubblico (nessuna autenticazione)</t>
+  </si>
+  <si>
+    <t>200 Healthy - usato come Healthcheck Path su Railway</t>
+  </si>
+  <si>
+    <t>/get-all-fasce</t>
+  </si>
+  <si>
+    <t>200 List&lt;FasciaOrariaDTO&gt; (attive e disattivate)</t>
+  </si>
+  <si>
+    <t>/get-mie-prenotazioni</t>
+  </si>
+  <si>
+    <t>200 List&lt;PrenotazioneDTO&gt; filtrate su UserId dal JWT</t>
+  </si>
+  <si>
+    <t>Aggiornato: 25/08/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>FASE 4 PIANO DI RILASCIO - Verifica backend in produzione (sessione 25/08/2026)</t>
+  </si>
+  <si>
+    <t>Riallineamento repo</t>
+  </si>
+  <si>
+    <t>dev era avanti di 2 commit non mergiati su main (chiusura Fase 3); .gitignore aveva .vs/ scritto come commento invece di regola attiva, causando errori di commit/push su file di lock in uso. Merge dev-&gt;main (PR #3) e main-&gt;dev, .gitignore corretto in .vs/.</t>
+  </si>
+  <si>
+    <t>Git flow + GitHub PR</t>
+  </si>
+  <si>
+    <t>25/08/2026</t>
+  </si>
+  <si>
+    <t>Verifica endpoint Zona</t>
+  </si>
+  <si>
+    <t>GET get-all-zone con token Admin su DB di produzione vuoto -&gt; 404 Nessuna zona trovata. Comportamento noto e gia' tracciato, vedi FIX-007.</t>
+  </si>
+  <si>
+    <t>Postman + token JWT</t>
+  </si>
+  <si>
+    <t>Verifica endpoint FasceOrarie</t>
+  </si>
+  <si>
+    <t>GET fasce-attive con token Admin su DB vuoto -&gt; 200 OK con []. Conferma che FIX-003 tiene anche in produzione.</t>
+  </si>
+  <si>
+    <t>Verifica endpoint Dashboard</t>
+  </si>
+  <si>
+    <t>GET giornaliera con token Admin su DB vuoto -&gt; 200 OK con tutti i contatori a zero. L'aggregato non soffre dell'anti-pattern di FIX-007.</t>
+  </si>
+  <si>
+    <t>Log Railway</t>
+  </si>
+  <si>
+    <t>Controllati i log del servizio .NET su Railway durante le chiamate di verifica: nessuna eccezione, nessun errore.</t>
+  </si>
+  <si>
+    <t>Railway Deploy Logs</t>
+  </si>
+  <si>
+    <t>Aggiornato: 27/08/2026</t>
+  </si>
+  <si>
+    <t>27-ago-26</t>
+  </si>
+  <si>
+    <t>Frontend completato e deployato: backend Railway OK (14/08), verificato in produzione (25/08), frontend Vercel deployato e testato in produzione (27/08). Bug Fase 5 (5) e Fase 7 (3) risolti. Nessun backlog residuo prima del rilascio v1.0.</t>
+  </si>
+  <si>
+    <t>FASE 5 PIANO DI RILASCIO - Fix backlog frontend/backend (sessioni 26-27/08/2026)</t>
+  </si>
+  <si>
+    <t>Checklist Fase 5</t>
+  </si>
+  <si>
+    <t>Completati i test dei ruoli Staff, Cliente, sicurezza/sessione (401 -&gt; logout automatico). Bug 1-5 di Fix Fase 5.txt diagnosticati e risolti.</t>
+  </si>
+  <si>
+    <t>Test manuale + Postman</t>
+  </si>
+  <si>
+    <t>26/08/2026</t>
+  </si>
+  <si>
+    <t>RBAC/UX Staff-Cliente</t>
+  </si>
+  <si>
+    <t>Cliente 403 su get-all-prenotazioni (endpoint sbagliato), pulsanti Staff su Zone/Postazioni/Fasce visibili quando non dovevano, vincolo una-prenotazione-al-giorno bloccava Staff/Admin su prenotazioni per conto cliente, aggiunto campo NomeCliente.</t>
+  </si>
+  <si>
+    <t>React Query + EF Core migration</t>
+  </si>
+  <si>
+    <t>Migration produzione</t>
+  </si>
+  <si>
+    <t>RimuoviVincoloIndiceAggiungiNomeCliente applicata a mano sul DB Railway via railway connect Postgres + psql, verificata con \d Prenotazioni.</t>
+  </si>
+  <si>
+    <t>EF Core Migrations + Railway CLI</t>
+  </si>
+  <si>
+    <t>Bug emersi post-fix</t>
+  </si>
+  <si>
+    <t>Filtro GetPostazioniPerZonaAsync troppo restrittivo, Fasce Orarie non filtrate per giorno in creazione prenotazione, Dashboard chiarita con sottosezioni Oggi/Questa settimana.</t>
+  </si>
+  <si>
+    <t>React Query + EF Core</t>
+  </si>
+  <si>
+    <t>Chiusura backlog Fase 5</t>
+  </si>
+  <si>
+    <t>GAP-001 (UI creazione utenti), RBAC-002 (cutoff 2h self-service Cliente), AUDIT-001 (log attivita esteso), NAMING-001-residuo (rinomina controller), DEAD-CODE-001 (filtro postazioni disponibili). dotnet test 31/31 verdi.</t>
+  </si>
+  <si>
+    <t>ASP.NET Core + React</t>
+  </si>
+  <si>
+    <t>27/08/2026</t>
+  </si>
+  <si>
+    <t>FASE 6-7 PIANO DI RILASCIO - Deploy Vercel e testing integrato (sessione 27/08/2026)</t>
+  </si>
+  <si>
+    <t>Deploy frontend Vercel</t>
+  </si>
+  <si>
+    <t>Repo collegato, root directory gestora-frontend, VITE_API_URL su Railway, deploy completato: https://gestora-project-xi.vercel.app</t>
+  </si>
+  <si>
+    <t>Vercel</t>
+  </si>
+  <si>
+    <t>CORS produzione</t>
+  </si>
+  <si>
+    <t>Aggiunta AllowedOrigins__1 su Railway con l'URL Vercel, verificato con preflight OPTIONS (Access-Control-Allow-Origin corretto).</t>
+  </si>
+  <si>
+    <t>Testing integrato</t>
+  </si>
+  <si>
+    <t>Flussi Admin/Staff/Cliente testati in produzione (Vercel+Railway+Postgres): CRUD, prenotazioni, pannello utenti, route protette.</t>
+  </si>
+  <si>
+    <t>Test manuale in produzione</t>
+  </si>
+  <si>
+    <t>Bug emersi in produzione</t>
+  </si>
+  <si>
+    <t>404 Vercel su refresh e su login fallito (mancava vercel.json rewrite + interceptor redirect su ogni 401), pulsante Annulla mancante per il Cliente dopo riapertura RBAC-002.</t>
+  </si>
+  <si>
+    <t>React Router + Axios</t>
+  </si>
+  <si>
+    <t>Fase 8 - prossimo passo</t>
+  </si>
+  <si>
+    <t>Aggiornare CLAUDE.md con URL definitivi, commit finale con tag v1.0.0, documentare credenziali Admin iniziali, aggiornare tracker con stati finali.</t>
   </si>
   <si>
     <t>Da fare</t>
-  </si>
-  <si>
-    <t>(Program.cs)</t>
-  </si>
-  <si>
-    <t>/health</t>
-  </si>
-  <si>
-    <t>Pubblico (nessuna autenticazione)</t>
-  </si>
-  <si>
-    <t>200 Healthy - usato come Healthcheck Path su Railway</t>
-  </si>
-  <si>
-    <t>/get-all-fasce</t>
-  </si>
-  <si>
-    <t>200 List&lt;FasciaOrariaDTO&gt; (attive e disattivate)</t>
-  </si>
-  <si>
-    <t>/get-mie-prenotazioni</t>
-  </si>
-  <si>
-    <t>200 List&lt;PrenotazioneDTO&gt; filtrate su UserId dal JWT</t>
-  </si>
-  <si>
-    <t>Aggiornato: 25/08/2026</t>
-  </si>
-  <si>
-    <t>Aggiornato: 25/08/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
-    <t>FASE 4 PIANO DI RILASCIO - Verifica backend in produzione (sessione 25/08/2026)</t>
-  </si>
-  <si>
-    <t>Riallineamento repo</t>
-  </si>
-  <si>
-    <t>dev era avanti di 2 commit non mergiati su main (chiusura Fase 3); .gitignore aveva .vs/ scritto come commento invece di regola attiva, causando errori di commit/push su file di lock in uso. Merge dev-&gt;main (PR #3) e main-&gt;dev, .gitignore corretto in .vs/.</t>
-  </si>
-  <si>
-    <t>Git flow + GitHub PR</t>
-  </si>
-  <si>
-    <t>25/08/2026</t>
-  </si>
-  <si>
-    <t>Verifica endpoint Zona</t>
-  </si>
-  <si>
-    <t>GET get-all-zone con token Admin su DB di produzione vuoto -&gt; 404 Nessuna zona trovata. Comportamento noto e gia' tracciato, vedi FIX-007.</t>
-  </si>
-  <si>
-    <t>Postman + token JWT</t>
-  </si>
-  <si>
-    <t>Verifica endpoint FasceOrarie</t>
-  </si>
-  <si>
-    <t>GET fasce-attive con token Admin su DB vuoto -&gt; 200 OK con []. Conferma che FIX-003 tiene anche in produzione.</t>
-  </si>
-  <si>
-    <t>Verifica endpoint Dashboard</t>
-  </si>
-  <si>
-    <t>GET giornaliera con token Admin su DB vuoto -&gt; 200 OK con tutti i contatori a zero. L'aggregato non soffre dell'anti-pattern di FIX-007.</t>
-  </si>
-  <si>
-    <t>Log Railway</t>
-  </si>
-  <si>
-    <t>Controllati i log del servizio .NET su Railway durante le chiamate di verifica: nessuna eccezione, nessun errore.</t>
-  </si>
-  <si>
-    <t>Railway Deploy Logs</t>
-  </si>
-  <si>
-    <t>Frontend completato. Deploy: backend su Railway OK (14/08/26), verificato in produzione (Fase 4, 25/08/26). Frontend Vercel da fare.</t>
-  </si>
-  <si>
-    <t>Sei endpoint restituiscono 404 invece di 200 con array vuoto quando non ci sono dati. Stesso anti-pattern di FIX-003, corretto solo sulle fasce orarie. Si manifesta sempre su un database di produzione appena creato. Trovato il 14/08/2026 verificando il deploy Railway. Riconfermato in Fase 4 (25/08/2026): comportamento invariato. Da decidere in Fase 5 se e come sistemarlo prima di collegare il frontend.</t>
   </si>
 </sst>
 </file>
@@ -3164,7 +3251,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE99C"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3220,7 +3307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3309,13 +3396,20 @@
     <xf numFmtId="15" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3346,6 +3440,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -3648,7 +3743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -3660,36 +3755,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
-        <v>959</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="A2" s="38" t="s">
+        <v>971</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="39" t="s">
+      <c r="B4" s="43"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="40"/>
-      <c r="F4" s="41"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="44"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3858,43 +3953,51 @@
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
       <c r="D14" s="1" t="s">
+        <v>918</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>919</v>
       </c>
-      <c r="E14" s="30" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>920</v>
-      </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="42" t="s">
+      <c r="A15" s="1"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="37"/>
+    </row>
+    <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="41"/>
-    </row>
-    <row r="16" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="37" t="s">
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="44"/>
+    </row>
+    <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="36"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3913,14 +4016,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>653</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4570,7 +4673,7 @@
         <v>678</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>693</v>
@@ -4579,7 +4682,7 @@
         <v>443</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4730,7 +4833,7 @@
         <v>678</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>861</v>
@@ -4739,7 +4842,7 @@
         <v>443</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4904,22 +5007,22 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="B52" t="s">
         <v>678</v>
       </c>
       <c r="C52" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="D52" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="E52" t="s">
         <v>443</v>
       </c>
       <c r="F52" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
     </row>
   </sheetData>
@@ -4943,13 +5046,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>766</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5293,11 +5396,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>819</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5563,14 +5666,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>865</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5642,7 +5745,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5654,40 +5757,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
-        <v>960</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
+      <c r="A2" s="38" t="s">
+        <v>955</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="41"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -6010,16 +6113,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="39" t="s">
+      <c r="A22" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="41"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="44"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -6242,16 +6345,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="43" t="s">
+      <c r="A35" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="40"/>
-      <c r="C35" s="40"/>
-      <c r="D35" s="40"/>
-      <c r="E35" s="40"/>
-      <c r="F35" s="40"/>
-      <c r="G35" s="40"/>
-      <c r="H35" s="41"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="44"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6429,21 +6532,21 @@
       <c r="E44" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="F44" s="32" t="s">
-        <v>880</v>
+      <c r="F44" s="26" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="44" t="s">
+      <c r="A46" s="47" t="s">
         <v>178</v>
       </c>
-      <c r="B46" s="40"/>
-      <c r="C46" s="40"/>
-      <c r="D46" s="40"/>
-      <c r="E46" s="40"/>
-      <c r="F46" s="40"/>
-      <c r="G46" s="40"/>
-      <c r="H46" s="41"/>
+      <c r="B46" s="43"/>
+      <c r="C46" s="43"/>
+      <c r="D46" s="43"/>
+      <c r="E46" s="43"/>
+      <c r="F46" s="43"/>
+      <c r="G46" s="43"/>
+      <c r="H46" s="44"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6506,16 +6609,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="42" t="s">
+      <c r="A51" s="45" t="s">
         <v>190</v>
       </c>
-      <c r="B51" s="40"/>
-      <c r="C51" s="40"/>
-      <c r="D51" s="40"/>
-      <c r="E51" s="40"/>
-      <c r="F51" s="40"/>
-      <c r="G51" s="40"/>
-      <c r="H51" s="41"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="43"/>
+      <c r="D51" s="43"/>
+      <c r="E51" s="43"/>
+      <c r="F51" s="43"/>
+      <c r="G51" s="43"/>
+      <c r="H51" s="44"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -6695,40 +6798,40 @@
     </row>
     <row r="68" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="25" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="B68" s="25" t="s">
+        <v>916</v>
+      </c>
+      <c r="C68" s="25" t="s">
         <v>917</v>
-      </c>
-      <c r="C68" s="25" t="s">
-        <v>918</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="25" t="s">
+        <v>923</v>
+      </c>
+      <c r="B69" s="25" t="s">
         <v>924</v>
       </c>
-      <c r="B69" s="25" t="s">
+      <c r="C69" s="25" t="s">
         <v>925</v>
-      </c>
-      <c r="C69" s="25" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="25" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B70" s="25" t="s">
+        <v>926</v>
+      </c>
+      <c r="C70" s="25" t="s">
         <v>927</v>
-      </c>
-      <c r="C70" s="25" t="s">
-        <v>928</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
@@ -6739,7 +6842,7 @@
         <v>45</v>
       </c>
       <c r="C73" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D73" t="s">
         <v>47</v>
@@ -6756,16 +6859,16 @@
         <v>1</v>
       </c>
       <c r="B74" t="s">
+        <v>882</v>
+      </c>
+      <c r="C74" t="s">
         <v>883</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>884</v>
       </c>
-      <c r="D74" t="s">
-        <v>885</v>
-      </c>
       <c r="E74" s="28" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="F74" s="27" t="s">
         <v>6</v>
@@ -6776,16 +6879,16 @@
         <v>2</v>
       </c>
       <c r="B75" t="s">
+        <v>885</v>
+      </c>
+      <c r="C75" t="s">
         <v>886</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>887</v>
       </c>
-      <c r="D75" t="s">
-        <v>888</v>
-      </c>
       <c r="E75" s="28" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="F75" s="27" t="s">
         <v>6</v>
@@ -6796,16 +6899,16 @@
         <v>3</v>
       </c>
       <c r="B76" t="s">
+        <v>888</v>
+      </c>
+      <c r="C76" t="s">
         <v>889</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>890</v>
       </c>
-      <c r="D76" t="s">
-        <v>891</v>
-      </c>
       <c r="E76" s="28" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="F76" s="27" t="s">
         <v>6</v>
@@ -6816,16 +6919,16 @@
         <v>4</v>
       </c>
       <c r="B77" t="s">
+        <v>891</v>
+      </c>
+      <c r="C77" t="s">
         <v>892</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>893</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" s="28" t="s">
         <v>894</v>
-      </c>
-      <c r="E77" s="28" t="s">
-        <v>895</v>
       </c>
       <c r="F77" s="27" t="s">
         <v>6</v>
@@ -6833,12 +6936,12 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
@@ -6846,16 +6949,16 @@
         <v>1</v>
       </c>
       <c r="B81" t="s">
+        <v>897</v>
+      </c>
+      <c r="C81" t="s">
         <v>898</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>899</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>900</v>
-      </c>
-      <c r="E81" t="s">
-        <v>901</v>
       </c>
       <c r="F81" s="27" t="s">
         <v>6</v>
@@ -6866,16 +6969,16 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
+        <v>901</v>
+      </c>
+      <c r="C82" t="s">
         <v>902</v>
-      </c>
-      <c r="C82" t="s">
-        <v>903</v>
       </c>
       <c r="D82" t="s">
         <v>73</v>
       </c>
       <c r="E82" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F82" s="27" t="s">
         <v>6</v>
@@ -6886,16 +6989,16 @@
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C83" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="D83" t="s">
         <v>86</v>
       </c>
       <c r="E83" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F83" s="27" t="s">
         <v>6</v>
@@ -6906,16 +7009,16 @@
         <v>5</v>
       </c>
       <c r="B84" t="s">
+        <v>904</v>
+      </c>
+      <c r="C84" t="s">
         <v>905</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>906</v>
       </c>
-      <c r="D84" t="s">
-        <v>907</v>
-      </c>
       <c r="E84" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F84" s="27" t="s">
         <v>6</v>
@@ -6926,16 +7029,16 @@
         <v>6</v>
       </c>
       <c r="B89" t="s">
+        <v>907</v>
+      </c>
+      <c r="C89" t="s">
         <v>908</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>909</v>
       </c>
-      <c r="D89" t="s">
-        <v>910</v>
-      </c>
       <c r="E89" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F89" s="27" t="s">
         <v>6</v>
@@ -6946,16 +7049,16 @@
         <v>7</v>
       </c>
       <c r="B90" t="s">
+        <v>910</v>
+      </c>
+      <c r="C90" t="s">
         <v>911</v>
       </c>
-      <c r="C90" t="s">
+      <c r="D90" t="s">
         <v>912</v>
       </c>
-      <c r="D90" t="s">
-        <v>913</v>
-      </c>
       <c r="E90" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F90" s="27" t="s">
         <v>6</v>
@@ -6966,16 +7069,16 @@
         <v>8</v>
       </c>
       <c r="B91" t="s">
+        <v>913</v>
+      </c>
+      <c r="C91" t="s">
         <v>914</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
         <v>915</v>
       </c>
-      <c r="D91" t="s">
-        <v>916</v>
-      </c>
       <c r="E91" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F91" s="27" t="s">
         <v>6</v>
@@ -6983,7 +7086,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="E93" s="28"/>
       <c r="F93" s="27"/>
@@ -6996,7 +7099,7 @@
         <v>45</v>
       </c>
       <c r="C94" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D94" t="s">
         <v>47</v>
@@ -7013,16 +7116,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
+        <v>929</v>
+      </c>
+      <c r="C95" t="s">
         <v>930</v>
       </c>
-      <c r="C95" t="s">
+      <c r="D95" t="s">
         <v>931</v>
       </c>
-      <c r="D95" t="s">
-        <v>932</v>
-      </c>
       <c r="E95" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F95" s="27" t="s">
         <v>6</v>
@@ -7033,16 +7136,16 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
+        <v>932</v>
+      </c>
+      <c r="C96" t="s">
         <v>933</v>
       </c>
-      <c r="C96" t="s">
+      <c r="D96" t="s">
         <v>934</v>
       </c>
-      <c r="D96" t="s">
-        <v>935</v>
-      </c>
       <c r="E96" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F96" s="27" t="s">
         <v>6</v>
@@ -7053,16 +7156,16 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
+        <v>935</v>
+      </c>
+      <c r="C97" t="s">
         <v>936</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>937</v>
       </c>
-      <c r="D97" t="s">
-        <v>938</v>
-      </c>
       <c r="E97" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F97" s="27" t="s">
         <v>6</v>
@@ -7073,16 +7176,16 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
+        <v>938</v>
+      </c>
+      <c r="C98" t="s">
         <v>939</v>
       </c>
-      <c r="C98" t="s">
+      <c r="D98" t="s">
         <v>940</v>
       </c>
-      <c r="D98" t="s">
-        <v>941</v>
-      </c>
       <c r="E98" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F98" s="27" t="s">
         <v>6</v>
@@ -7093,16 +7196,16 @@
         <v>5</v>
       </c>
       <c r="B99" t="s">
+        <v>941</v>
+      </c>
+      <c r="C99" t="s">
         <v>942</v>
       </c>
-      <c r="C99" t="s">
+      <c r="D99" t="s">
         <v>943</v>
       </c>
-      <c r="D99" t="s">
-        <v>944</v>
-      </c>
       <c r="E99" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F99" s="27" t="s">
         <v>6</v>
@@ -7113,24 +7216,24 @@
         <v>6</v>
       </c>
       <c r="B100" t="s">
+        <v>944</v>
+      </c>
+      <c r="C100" t="s">
         <v>945</v>
       </c>
-      <c r="C100" t="s">
+      <c r="D100" t="s">
         <v>946</v>
       </c>
-      <c r="D100" t="s">
-        <v>947</v>
-      </c>
       <c r="E100" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F100" s="27" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="34" t="s">
-        <v>961</v>
+      <c r="A102" s="32" t="s">
+        <v>956</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
@@ -7141,7 +7244,7 @@
         <v>45</v>
       </c>
       <c r="C103" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D103" t="s">
         <v>47</v>
@@ -7158,16 +7261,16 @@
         <v>1</v>
       </c>
       <c r="B104" t="s">
-        <v>962</v>
+        <v>957</v>
       </c>
       <c r="C104" t="s">
-        <v>963</v>
+        <v>958</v>
       </c>
       <c r="D104" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="E104" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="F104" s="27" t="s">
         <v>6</v>
@@ -7178,16 +7281,16 @@
         <v>2</v>
       </c>
       <c r="B105" t="s">
-        <v>966</v>
+        <v>961</v>
       </c>
       <c r="C105" t="s">
-        <v>967</v>
+        <v>962</v>
       </c>
       <c r="D105" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="E105" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="F105" s="27" t="s">
         <v>6</v>
@@ -7198,16 +7301,16 @@
         <v>3</v>
       </c>
       <c r="B106" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
       <c r="C106" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="D106" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="E106" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="F106" s="27" t="s">
         <v>6</v>
@@ -7218,16 +7321,16 @@
         <v>4</v>
       </c>
       <c r="B107" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
       <c r="C107" t="s">
-        <v>972</v>
+        <v>967</v>
       </c>
       <c r="D107" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="E107" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="F107" s="27" t="s">
         <v>6</v>
@@ -7238,19 +7341,269 @@
         <v>5</v>
       </c>
       <c r="B108" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="C108" t="s">
+        <v>969</v>
+      </c>
+      <c r="D108" t="s">
+        <v>970</v>
+      </c>
+      <c r="E108" t="s">
+        <v>960</v>
+      </c>
+      <c r="F108" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
         <v>974</v>
       </c>
-      <c r="D108" t="s">
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>44</v>
+      </c>
+      <c r="B111" t="s">
+        <v>45</v>
+      </c>
+      <c r="C111" t="s">
+        <v>881</v>
+      </c>
+      <c r="D111" t="s">
+        <v>47</v>
+      </c>
+      <c r="E111" t="s">
+        <v>48</v>
+      </c>
+      <c r="F111" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112">
+        <v>1</v>
+      </c>
+      <c r="B112" t="s">
         <v>975</v>
       </c>
-      <c r="E108" t="s">
-        <v>965</v>
-      </c>
-      <c r="F108" s="27" t="s">
-        <v>6</v>
+      <c r="C112" t="s">
+        <v>976</v>
+      </c>
+      <c r="D112" t="s">
+        <v>977</v>
+      </c>
+      <c r="E112" t="s">
+        <v>978</v>
+      </c>
+      <c r="F112" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <v>2</v>
+      </c>
+      <c r="B113" t="s">
+        <v>979</v>
+      </c>
+      <c r="C113" t="s">
+        <v>980</v>
+      </c>
+      <c r="D113" t="s">
+        <v>981</v>
+      </c>
+      <c r="E113" t="s">
+        <v>978</v>
+      </c>
+      <c r="F113" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <v>3</v>
+      </c>
+      <c r="B114" t="s">
+        <v>982</v>
+      </c>
+      <c r="C114" t="s">
+        <v>983</v>
+      </c>
+      <c r="D114" t="s">
+        <v>984</v>
+      </c>
+      <c r="E114" t="s">
+        <v>978</v>
+      </c>
+      <c r="F114" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>4</v>
+      </c>
+      <c r="B115" t="s">
+        <v>985</v>
+      </c>
+      <c r="C115" t="s">
+        <v>986</v>
+      </c>
+      <c r="D115" t="s">
+        <v>987</v>
+      </c>
+      <c r="E115" t="s">
+        <v>978</v>
+      </c>
+      <c r="F115" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <v>5</v>
+      </c>
+      <c r="B116" t="s">
+        <v>988</v>
+      </c>
+      <c r="C116" t="s">
+        <v>989</v>
+      </c>
+      <c r="D116" t="s">
+        <v>990</v>
+      </c>
+      <c r="E116" t="s">
+        <v>991</v>
+      </c>
+      <c r="F116" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>44</v>
+      </c>
+      <c r="B119" t="s">
+        <v>45</v>
+      </c>
+      <c r="C119" t="s">
+        <v>881</v>
+      </c>
+      <c r="D119" t="s">
+        <v>47</v>
+      </c>
+      <c r="E119" t="s">
+        <v>48</v>
+      </c>
+      <c r="F119" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <v>1</v>
+      </c>
+      <c r="B120" t="s">
+        <v>993</v>
+      </c>
+      <c r="C120" t="s">
+        <v>994</v>
+      </c>
+      <c r="D120" t="s">
+        <v>995</v>
+      </c>
+      <c r="E120" t="s">
+        <v>991</v>
+      </c>
+      <c r="F120" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <v>2</v>
+      </c>
+      <c r="B121" t="s">
+        <v>996</v>
+      </c>
+      <c r="C121" t="s">
+        <v>997</v>
+      </c>
+      <c r="D121" t="s">
+        <v>940</v>
+      </c>
+      <c r="E121" t="s">
+        <v>991</v>
+      </c>
+      <c r="F121" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122">
+        <v>3</v>
+      </c>
+      <c r="B122" t="s">
+        <v>998</v>
+      </c>
+      <c r="C122" t="s">
+        <v>999</v>
+      </c>
+      <c r="D122" t="s">
+        <v>1000</v>
+      </c>
+      <c r="E122" t="s">
+        <v>991</v>
+      </c>
+      <c r="F122" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A123">
+        <v>4</v>
+      </c>
+      <c r="B123" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C123" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D123" t="s">
+        <v>1003</v>
+      </c>
+      <c r="E123" t="s">
+        <v>991</v>
+      </c>
+      <c r="F123" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124">
+        <v>5</v>
+      </c>
+      <c r="B124" t="s">
+        <v>1004</v>
+      </c>
+      <c r="C124" t="s">
+        <v>1005</v>
+      </c>
+      <c r="D124" t="s">
+        <v>443</v>
+      </c>
+      <c r="E124" t="s">
+        <v>443</v>
+      </c>
+      <c r="F124" s="50" t="s">
+        <v>1006</v>
       </c>
     </row>
   </sheetData>
@@ -7269,7 +7622,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7280,24 +7633,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="49" t="s">
         <v>226</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="41"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="44"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7385,14 +7738,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="41"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="44"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -7480,14 +7833,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="42" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="41"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -7609,14 +7962,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="39" t="s">
+      <c r="A26" s="42" t="s">
         <v>284</v>
       </c>
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="41"/>
+      <c r="B26" s="43"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="44"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -7725,17 +8078,20 @@
         <v>285</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>920</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>921</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="D33" s="2" t="s">
         <v>922</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>923</v>
-      </c>
       <c r="E33" s="30" t="s">
         <v>6</v>
       </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E34" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7763,26 +8119,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>294</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="45" t="s">
         <v>295</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="41"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="44"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8032,12 +8388,12 @@
       <c r="D15" s="31">
         <v>46094</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="32" t="s">
-        <v>880</v>
-      </c>
+      <c r="E15" s="12" t="s">
+        <v>972</v>
+      </c>
+      <c r="F15" s="26"/>
       <c r="G15" s="5" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -8080,24 +8436,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>352</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="42" t="s">
         <v>353</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="41"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="44"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8282,14 +8638,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="46" t="s">
+      <c r="A18" s="49" t="s">
         <v>385</v>
       </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="41"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="44"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -8390,28 +8746,20 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
-        <v>948</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>949</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>977</v>
-      </c>
-      <c r="D26" s="33" t="s">
-        <v>950</v>
-      </c>
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="45" t="s">
         <v>398</v>
       </c>
-      <c r="B28" s="40"/>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="41"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="44"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -8507,14 +8855,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>410</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -8691,14 +9039,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>433</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9301,13 +9649,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>509</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9704,13 +10052,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="48" t="s">
         <v>588</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
add JobsController.cs + gestione docs
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEFE51A-6821-4D47-8656-5CA5833F901B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B978BCF-AED2-4B56-A86F-3442199517BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="1007">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1762" uniqueCount="1017">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2947,9 +2947,6 @@
     <t>Railway Deploy Logs</t>
   </si>
   <si>
-    <t>Aggiornato: 27/08/2026</t>
-  </si>
-  <si>
     <t>27-ago-26</t>
   </si>
   <si>
@@ -3053,6 +3050,39 @@
   </si>
   <si>
     <t>Da fare</t>
+  </si>
+  <si>
+    <t>Verificato</t>
+  </si>
+  <si>
+    <t>OK 27/08/2026 - forzato a comando via JobsController (trigger manuale) su dato di test in locale, cancellazione confermata da log</t>
+  </si>
+  <si>
+    <t>Jobs</t>
+  </si>
+  <si>
+    <t>/trigger/{jobName}</t>
+  </si>
+  <si>
+    <t>jobName (route, es. PrenotazioniCleanupJob)</t>
+  </si>
+  <si>
+    <t>202 Accepted / 404 se job non esiste - forza esecuzione immediata di un job Quartz senza attendere il cron (27/08/2026, solo locale)</t>
+  </si>
+  <si>
+    <t>Jobs Quartz</t>
+  </si>
+  <si>
+    <t>Verifica flussi automatizzati mai testati (foglio Jobs)</t>
+  </si>
+  <si>
+    <t>OK 28/08/2026 - confermato via log Railway (View Logs), scattato correttamente alle 00:00 ora italiana (02:00 UTC) su 2 prenotazioni reali, esito Completata verificato.</t>
+  </si>
+  <si>
+    <t>PrenotazioniCleanupJob verificato via trigger manuale (JobsController). PrenotazioniJob confermato 28/08/2026 via log Railway: scattato regolarmente alle 00:00 ora italiana su 2 prenotazioni reali, transizione a Completata avvenuta.</t>
+  </si>
+  <si>
+    <t>Aggiornato: 28/08/2026</t>
   </si>
 </sst>
 </file>
@@ -3410,6 +3440,7 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3440,7 +3471,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -3755,36 +3785,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>971</v>
-      </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
+      <c r="A2" s="39" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="42" t="s">
+      <c r="B4" s="44"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="43"/>
-      <c r="F4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="45"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3971,24 +4001,24 @@
       <c r="F15" s="37"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="45" t="s">
+      <c r="A16" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="44"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="45"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4005,7 +4035,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -4016,14 +4046,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>653</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5023,6 +5053,26 @@
       </c>
       <c r="F52" t="s">
         <v>950</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B53" t="s">
+        <v>661</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D53" t="s">
+        <v>673</v>
+      </c>
+      <c r="E53" t="s">
+        <v>1010</v>
+      </c>
+      <c r="F53" t="s">
+        <v>1011</v>
       </c>
     </row>
   </sheetData>
@@ -5046,13 +5096,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>766</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5396,11 +5446,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>819</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5654,7 +5704,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -5665,17 +5715,17 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="49" t="s">
         <v>865</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-    </row>
-    <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+    </row>
+    <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>866</v>
       </c>
@@ -5694,8 +5744,11 @@
       <c r="F3" s="9" t="s">
         <v>871</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="32" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>872</v>
       </c>
@@ -5714,8 +5767,11 @@
       <c r="F4" s="11" t="s">
         <v>442</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G4" s="27" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
         <v>876</v>
       </c>
@@ -5733,6 +5789,9 @@
       </c>
       <c r="F5" s="14" t="s">
         <v>442</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>1007</v>
       </c>
     </row>
   </sheetData>
@@ -5757,40 +5816,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>955</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="44"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="45"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -6113,16 +6172,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="44"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="45"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -6345,16 +6404,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="47" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="43"/>
-      <c r="C35" s="43"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="44"/>
+      <c r="B35" s="44"/>
+      <c r="C35" s="44"/>
+      <c r="D35" s="44"/>
+      <c r="E35" s="44"/>
+      <c r="F35" s="44"/>
+      <c r="G35" s="44"/>
+      <c r="H35" s="45"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -6537,16 +6596,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="47" t="s">
+      <c r="A46" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="B46" s="43"/>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="44"/>
+      <c r="B46" s="44"/>
+      <c r="C46" s="44"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="44"/>
+      <c r="F46" s="44"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="45"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -6609,16 +6668,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="45" t="s">
+      <c r="A51" s="46" t="s">
         <v>190</v>
       </c>
-      <c r="B51" s="43"/>
-      <c r="C51" s="43"/>
-      <c r="D51" s="43"/>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="43"/>
-      <c r="H51" s="44"/>
+      <c r="B51" s="44"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="44"/>
+      <c r="F51" s="44"/>
+      <c r="G51" s="44"/>
+      <c r="H51" s="45"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -7358,7 +7417,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
@@ -7386,16 +7445,16 @@
         <v>1</v>
       </c>
       <c r="B112" t="s">
+        <v>974</v>
+      </c>
+      <c r="C112" t="s">
         <v>975</v>
       </c>
-      <c r="C112" t="s">
+      <c r="D112" t="s">
         <v>976</v>
       </c>
-      <c r="D112" t="s">
+      <c r="E112" t="s">
         <v>977</v>
-      </c>
-      <c r="E112" t="s">
-        <v>978</v>
       </c>
       <c r="F112" s="27" t="s">
         <v>6</v>
@@ -7406,16 +7465,16 @@
         <v>2</v>
       </c>
       <c r="B113" t="s">
+        <v>978</v>
+      </c>
+      <c r="C113" t="s">
         <v>979</v>
       </c>
-      <c r="C113" t="s">
+      <c r="D113" t="s">
         <v>980</v>
       </c>
-      <c r="D113" t="s">
-        <v>981</v>
-      </c>
       <c r="E113" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="F113" s="27" t="s">
         <v>6</v>
@@ -7426,16 +7485,16 @@
         <v>3</v>
       </c>
       <c r="B114" t="s">
+        <v>981</v>
+      </c>
+      <c r="C114" t="s">
         <v>982</v>
       </c>
-      <c r="C114" t="s">
+      <c r="D114" t="s">
         <v>983</v>
       </c>
-      <c r="D114" t="s">
-        <v>984</v>
-      </c>
       <c r="E114" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="F114" s="27" t="s">
         <v>6</v>
@@ -7446,16 +7505,16 @@
         <v>4</v>
       </c>
       <c r="B115" t="s">
+        <v>984</v>
+      </c>
+      <c r="C115" t="s">
         <v>985</v>
       </c>
-      <c r="C115" t="s">
+      <c r="D115" t="s">
         <v>986</v>
       </c>
-      <c r="D115" t="s">
-        <v>987</v>
-      </c>
       <c r="E115" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="F115" s="27" t="s">
         <v>6</v>
@@ -7466,16 +7525,16 @@
         <v>5</v>
       </c>
       <c r="B116" t="s">
+        <v>987</v>
+      </c>
+      <c r="C116" t="s">
         <v>988</v>
       </c>
-      <c r="C116" t="s">
+      <c r="D116" t="s">
         <v>989</v>
       </c>
-      <c r="D116" t="s">
+      <c r="E116" t="s">
         <v>990</v>
-      </c>
-      <c r="E116" t="s">
-        <v>991</v>
       </c>
       <c r="F116" s="27" t="s">
         <v>6</v>
@@ -7483,7 +7542,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
@@ -7511,16 +7570,16 @@
         <v>1</v>
       </c>
       <c r="B120" t="s">
+        <v>992</v>
+      </c>
+      <c r="C120" t="s">
         <v>993</v>
       </c>
-      <c r="C120" t="s">
+      <c r="D120" t="s">
         <v>994</v>
       </c>
-      <c r="D120" t="s">
-        <v>995</v>
-      </c>
       <c r="E120" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="F120" s="27" t="s">
         <v>6</v>
@@ -7531,16 +7590,16 @@
         <v>2</v>
       </c>
       <c r="B121" t="s">
+        <v>995</v>
+      </c>
+      <c r="C121" t="s">
         <v>996</v>
-      </c>
-      <c r="C121" t="s">
-        <v>997</v>
       </c>
       <c r="D121" t="s">
         <v>940</v>
       </c>
       <c r="E121" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="F121" s="27" t="s">
         <v>6</v>
@@ -7551,16 +7610,16 @@
         <v>3</v>
       </c>
       <c r="B122" t="s">
+        <v>997</v>
+      </c>
+      <c r="C122" t="s">
         <v>998</v>
       </c>
-      <c r="C122" t="s">
+      <c r="D122" t="s">
         <v>999</v>
       </c>
-      <c r="D122" t="s">
-        <v>1000</v>
-      </c>
       <c r="E122" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="F122" s="27" t="s">
         <v>6</v>
@@ -7571,16 +7630,16 @@
         <v>4</v>
       </c>
       <c r="B123" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C123" t="s">
         <v>1001</v>
       </c>
-      <c r="C123" t="s">
+      <c r="D123" t="s">
         <v>1002</v>
       </c>
-      <c r="D123" t="s">
-        <v>1003</v>
-      </c>
       <c r="E123" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="F123" s="27" t="s">
         <v>6</v>
@@ -7591,10 +7650,10 @@
         <v>5</v>
       </c>
       <c r="B124" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C124" t="s">
         <v>1004</v>
-      </c>
-      <c r="C124" t="s">
-        <v>1005</v>
       </c>
       <c r="D124" t="s">
         <v>443</v>
@@ -7602,8 +7661,8 @@
       <c r="E124" t="s">
         <v>443</v>
       </c>
-      <c r="F124" s="50" t="s">
-        <v>1006</v>
+      <c r="F124" s="38" t="s">
+        <v>1005</v>
       </c>
     </row>
   </sheetData>
@@ -7633,24 +7692,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="50" t="s">
         <v>226</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -7738,14 +7797,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="45" t="s">
+      <c r="A10" s="46" t="s">
         <v>246</v>
       </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="44"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="45"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -7833,14 +7892,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="43" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="44"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="45"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -7962,14 +8021,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="42" t="s">
+      <c r="A26" s="43" t="s">
         <v>284</v>
       </c>
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="44"/>
+      <c r="B26" s="44"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="44"/>
+      <c r="F26" s="45"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -8119,26 +8178,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>294</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="46" t="s">
         <v>295</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="45"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8389,11 +8448,11 @@
         <v>46094</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="F15" s="26"/>
       <c r="G15" s="5" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -8426,7 +8485,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -8436,24 +8495,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>352</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="43" t="s">
         <v>353</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8638,14 +8697,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="50" t="s">
         <v>385</v>
       </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="44"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="45"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -8752,14 +8811,14 @@
       <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="45" t="s">
+      <c r="A28" s="46" t="s">
         <v>398</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="44"/>
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="45"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -8828,6 +8887,20 @@
         <v>409</v>
       </c>
       <c r="D33" s="21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1015</v>
+      </c>
+      <c r="D34" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -8855,14 +8928,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>410</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9039,14 +9112,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>433</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -9649,13 +9722,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>509</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -10052,13 +10125,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>588</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
feat: Fase 2 checkpoint 2a - rename MaxPrenotazioni -> MaxCoperti
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B978BCF-AED2-4B56-A86F-3442199517BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A21BFD-9F3D-45AF-9B6F-8C75FC256371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1762" uniqueCount="1017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1798" uniqueCount="1038">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2899,9 +2899,6 @@
     <t>200 List&lt;PrenotazioneDTO&gt; filtrate su UserId dal JWT</t>
   </si>
   <si>
-    <t>Aggiornato: 25/08/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
     <t>FASE 4 PIANO DI RILASCIO - Verifica backend in produzione (sessione 25/08/2026)</t>
   </si>
   <si>
@@ -3082,7 +3079,73 @@
     <t>PrenotazioniCleanupJob verificato via trigger manuale (JobsController). PrenotazioniJob confermato 28/08/2026 via log Railway: scattato regolarmente alle 00:00 ora italiana su 2 prenotazioni reali, transizione a Completata avvenuta.</t>
   </si>
   <si>
-    <t>Aggiornato: 28/08/2026</t>
+    <t>Aggiornato: 31/08/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 31/08/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>FASE 1 ROADMAP REVISIONE - Fondamenta di deploy (sessione 31/08/2026)</t>
+  </si>
+  <si>
+    <t>Revisione roadmap</t>
+  </si>
+  <si>
+    <t>Confronto con seconda sessione, 3 decisioni prese (bonus capienza solo tavoli da 2, vincolo una-al-giorno Cliente rimandato a v2.0), ROADMAP_REVISIONE.md riscritto con Definition of Done, procedura migration produzione, tracciabilita REV-001..REV-097</t>
+  </si>
+  <si>
+    <t>31/08/2026</t>
+  </si>
+  <si>
+    <t>Config deploy nel repo</t>
+  </si>
+  <si>
+    <t>railway.json + global.json portano build/deploy nel repository. Corretti in corsa 2 problemi emersi nel primo deploy: SDK .NET 6 invece di 9 (mancava global.json), startCommand auto-rilevato sbagliato (puntava a GestoraWebApi.Tests)</t>
+  </si>
+  <si>
+    <t>Nixpacks + Railway config-as-code</t>
+  </si>
+  <si>
+    <t>Health check + avviso migration</t>
+  </si>
+  <si>
+    <t>Health check esteso al DB (AddDbContextCheck), avviso in log all'avvio se ci sono migration non applicate, migration StatoAsEnum documentata (no-op intenzionale)</t>
+  </si>
+  <si>
+    <t>ASP.NET Core HealthChecks + EF Core</t>
+  </si>
+  <si>
+    <t>3 fix sicurezza anticipati da Fase 4</t>
+  </si>
+  <si>
+    <t>REV-008 lockout(5/15min)+rate limit login(5/min per IP), REV-009 niente piu' leak di exception.Message sulle 500, REV-013 policy password anche su reset Admin</t>
+  </si>
+  <si>
+    <t>ASP.NET Identity + RateLimiting + FluentValidation</t>
+  </si>
+  <si>
+    <t>Fase 1 chiusa</t>
+  </si>
+  <si>
+    <t>dotnet test 31/31 verdi, pacchetti allineati (EF Tools 9.0.9, rimosso Serilog.Sinks.Seq), Fabio ha tolto il build command custom su Railway e verificato GET /health -&gt; Healthy in produzione</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 1</t>
+  </si>
+  <si>
+    <t>Fondamenta di deploy (REV-008, REV-009, REV-013, REV-035, REV-036, config Railway)</t>
+  </si>
+  <si>
+    <t>Config build/deploy nel repo (railway.json+global.json), health check esteso al DB, avviso migration non applicate, lockout+rate limit login, niente leak exception.Message, policy password su reset Admin, pacchetti allineati. Verificato in produzione: /health -&gt; Healthy.</t>
+  </si>
+  <si>
+    <t>Post-v1</t>
+  </si>
+  <si>
+    <t>Fondamenta di deploy: config Railway nel repo, health check DB, sicurezza login</t>
+  </si>
+  <si>
+    <t>31-ago-26</t>
   </si>
 </sst>
 </file>
@@ -3796,7 +3859,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="39" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
@@ -5057,22 +5120,22 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B53" t="s">
         <v>661</v>
       </c>
       <c r="C53" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="D53" t="s">
         <v>673</v>
       </c>
       <c r="E53" t="s">
+        <v>1009</v>
+      </c>
+      <c r="F53" t="s">
         <v>1010</v>
-      </c>
-      <c r="F53" t="s">
-        <v>1011</v>
       </c>
     </row>
   </sheetData>
@@ -5745,7 +5808,7 @@
         <v>871</v>
       </c>
       <c r="G3" s="32" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5768,7 +5831,7 @@
         <v>442</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5791,7 +5854,7 @@
         <v>442</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
   </sheetData>
@@ -5804,7 +5867,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H132"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5829,7 +5892,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="39" t="s">
-        <v>955</v>
+        <v>1016</v>
       </c>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
@@ -7292,7 +7355,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="32" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
@@ -7320,16 +7383,16 @@
         <v>1</v>
       </c>
       <c r="B104" t="s">
+        <v>956</v>
+      </c>
+      <c r="C104" t="s">
         <v>957</v>
       </c>
-      <c r="C104" t="s">
+      <c r="D104" t="s">
         <v>958</v>
       </c>
-      <c r="D104" t="s">
+      <c r="E104" t="s">
         <v>959</v>
-      </c>
-      <c r="E104" t="s">
-        <v>960</v>
       </c>
       <c r="F104" s="27" t="s">
         <v>6</v>
@@ -7340,16 +7403,16 @@
         <v>2</v>
       </c>
       <c r="B105" t="s">
+        <v>960</v>
+      </c>
+      <c r="C105" t="s">
         <v>961</v>
       </c>
-      <c r="C105" t="s">
+      <c r="D105" t="s">
         <v>962</v>
       </c>
-      <c r="D105" t="s">
-        <v>963</v>
-      </c>
       <c r="E105" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="F105" s="27" t="s">
         <v>6</v>
@@ -7360,16 +7423,16 @@
         <v>3</v>
       </c>
       <c r="B106" t="s">
+        <v>963</v>
+      </c>
+      <c r="C106" t="s">
         <v>964</v>
       </c>
-      <c r="C106" t="s">
-        <v>965</v>
-      </c>
       <c r="D106" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="E106" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="F106" s="27" t="s">
         <v>6</v>
@@ -7380,16 +7443,16 @@
         <v>4</v>
       </c>
       <c r="B107" t="s">
+        <v>965</v>
+      </c>
+      <c r="C107" t="s">
         <v>966</v>
       </c>
-      <c r="C107" t="s">
-        <v>967</v>
-      </c>
       <c r="D107" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="E107" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="F107" s="27" t="s">
         <v>6</v>
@@ -7400,16 +7463,16 @@
         <v>5</v>
       </c>
       <c r="B108" t="s">
+        <v>967</v>
+      </c>
+      <c r="C108" t="s">
         <v>968</v>
       </c>
-      <c r="C108" t="s">
+      <c r="D108" t="s">
         <v>969</v>
       </c>
-      <c r="D108" t="s">
-        <v>970</v>
-      </c>
       <c r="E108" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="F108" s="27" t="s">
         <v>6</v>
@@ -7417,7 +7480,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
@@ -7445,16 +7508,16 @@
         <v>1</v>
       </c>
       <c r="B112" t="s">
+        <v>973</v>
+      </c>
+      <c r="C112" t="s">
         <v>974</v>
       </c>
-      <c r="C112" t="s">
+      <c r="D112" t="s">
         <v>975</v>
       </c>
-      <c r="D112" t="s">
+      <c r="E112" t="s">
         <v>976</v>
-      </c>
-      <c r="E112" t="s">
-        <v>977</v>
       </c>
       <c r="F112" s="27" t="s">
         <v>6</v>
@@ -7465,16 +7528,16 @@
         <v>2</v>
       </c>
       <c r="B113" t="s">
+        <v>977</v>
+      </c>
+      <c r="C113" t="s">
         <v>978</v>
       </c>
-      <c r="C113" t="s">
+      <c r="D113" t="s">
         <v>979</v>
       </c>
-      <c r="D113" t="s">
-        <v>980</v>
-      </c>
       <c r="E113" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="F113" s="27" t="s">
         <v>6</v>
@@ -7485,16 +7548,16 @@
         <v>3</v>
       </c>
       <c r="B114" t="s">
+        <v>980</v>
+      </c>
+      <c r="C114" t="s">
         <v>981</v>
       </c>
-      <c r="C114" t="s">
+      <c r="D114" t="s">
         <v>982</v>
       </c>
-      <c r="D114" t="s">
-        <v>983</v>
-      </c>
       <c r="E114" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="F114" s="27" t="s">
         <v>6</v>
@@ -7505,16 +7568,16 @@
         <v>4</v>
       </c>
       <c r="B115" t="s">
+        <v>983</v>
+      </c>
+      <c r="C115" t="s">
         <v>984</v>
       </c>
-      <c r="C115" t="s">
+      <c r="D115" t="s">
         <v>985</v>
       </c>
-      <c r="D115" t="s">
-        <v>986</v>
-      </c>
       <c r="E115" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="F115" s="27" t="s">
         <v>6</v>
@@ -7525,16 +7588,16 @@
         <v>5</v>
       </c>
       <c r="B116" t="s">
+        <v>986</v>
+      </c>
+      <c r="C116" t="s">
         <v>987</v>
       </c>
-      <c r="C116" t="s">
+      <c r="D116" t="s">
         <v>988</v>
       </c>
-      <c r="D116" t="s">
+      <c r="E116" t="s">
         <v>989</v>
-      </c>
-      <c r="E116" t="s">
-        <v>990</v>
       </c>
       <c r="F116" s="27" t="s">
         <v>6</v>
@@ -7542,7 +7605,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
@@ -7570,16 +7633,16 @@
         <v>1</v>
       </c>
       <c r="B120" t="s">
+        <v>991</v>
+      </c>
+      <c r="C120" t="s">
         <v>992</v>
       </c>
-      <c r="C120" t="s">
+      <c r="D120" t="s">
         <v>993</v>
       </c>
-      <c r="D120" t="s">
-        <v>994</v>
-      </c>
       <c r="E120" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="F120" s="27" t="s">
         <v>6</v>
@@ -7590,16 +7653,16 @@
         <v>2</v>
       </c>
       <c r="B121" t="s">
+        <v>994</v>
+      </c>
+      <c r="C121" t="s">
         <v>995</v>
-      </c>
-      <c r="C121" t="s">
-        <v>996</v>
       </c>
       <c r="D121" t="s">
         <v>940</v>
       </c>
       <c r="E121" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="F121" s="27" t="s">
         <v>6</v>
@@ -7610,16 +7673,16 @@
         <v>3</v>
       </c>
       <c r="B122" t="s">
+        <v>996</v>
+      </c>
+      <c r="C122" t="s">
         <v>997</v>
       </c>
-      <c r="C122" t="s">
+      <c r="D122" t="s">
         <v>998</v>
       </c>
-      <c r="D122" t="s">
-        <v>999</v>
-      </c>
       <c r="E122" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="F122" s="27" t="s">
         <v>6</v>
@@ -7630,16 +7693,16 @@
         <v>4</v>
       </c>
       <c r="B123" t="s">
+        <v>999</v>
+      </c>
+      <c r="C123" t="s">
         <v>1000</v>
       </c>
-      <c r="C123" t="s">
+      <c r="D123" t="s">
         <v>1001</v>
       </c>
-      <c r="D123" t="s">
-        <v>1002</v>
-      </c>
       <c r="E123" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="F123" s="27" t="s">
         <v>6</v>
@@ -7650,10 +7713,10 @@
         <v>5</v>
       </c>
       <c r="B124" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C124" t="s">
         <v>1003</v>
-      </c>
-      <c r="C124" t="s">
-        <v>1004</v>
       </c>
       <c r="D124" t="s">
         <v>443</v>
@@ -7662,7 +7725,114 @@
         <v>443</v>
       </c>
       <c r="F124" s="38" t="s">
-        <v>1005</v>
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>44</v>
+      </c>
+      <c r="B127" t="s">
+        <v>45</v>
+      </c>
+      <c r="C127" t="s">
+        <v>881</v>
+      </c>
+      <c r="D127" t="s">
+        <v>47</v>
+      </c>
+      <c r="E127" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A128">
+        <v>1</v>
+      </c>
+      <c r="B128" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C128" t="s">
+        <v>1019</v>
+      </c>
+      <c r="D128" t="s">
+        <v>443</v>
+      </c>
+      <c r="E128" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A129">
+        <v>2</v>
+      </c>
+      <c r="B129" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C129" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D129" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E129" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A130">
+        <v>3</v>
+      </c>
+      <c r="B130" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C130" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D130" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E130" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A131">
+        <v>4</v>
+      </c>
+      <c r="B131" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C131" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D131" t="s">
+        <v>1029</v>
+      </c>
+      <c r="E131" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A132">
+        <v>5</v>
+      </c>
+      <c r="B132" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C132" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D132" t="s">
+        <v>443</v>
+      </c>
+      <c r="E132" t="s">
+        <v>1020</v>
       </c>
     </row>
   </sheetData>
@@ -8166,7 +8336,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -8448,11 +8618,11 @@
         <v>46094</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="F15" s="26"/>
       <c r="G15" s="5" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -8472,6 +8642,26 @@
       </c>
       <c r="G16" s="8" t="s">
         <v>351</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1037</v>
+      </c>
+      <c r="E17" t="s">
+        <v>1037</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -8485,7 +8675,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -8892,15 +9082,29 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B34" t="s">
         <v>1012</v>
       </c>
-      <c r="B34" t="s">
-        <v>1013</v>
-      </c>
       <c r="C34" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="D34" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D35" s="27" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: nuovo algoritmo di assegnazione tavoli (checkpoint 2b)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A21BFD-9F3D-45AF-9B6F-8C75FC256371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC168AD0-D524-4AC1-AEC1-BA6AEBBB23E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1798" uniqueCount="1038">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1826" uniqueCount="1051">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3146,6 +3146,45 @@
   </si>
   <si>
     <t>31-ago-26</t>
+  </si>
+  <si>
+    <t>FASE 2 CHECKPOINT 2a - Rename MaxPrenotazioni -&gt; MaxCoperti (sessione 31/08/2026)</t>
+  </si>
+  <si>
+    <t>Rename backend+frontend</t>
+  </si>
+  <si>
+    <t>MaxPrenotazioni -&gt; MaxCoperti in modello, DTO, validator, mapping, service, test (backend) e tipi/form/tabella (frontend). Etichetta chiara aggiunta nel form (REV-005)</t>
+  </si>
+  <si>
+    <t>EF Core + React Hook Form</t>
+  </si>
+  <si>
+    <t>Migration + deploy Dockerfile</t>
+  </si>
+  <si>
+    <t>Migration RinominaMaxPrenotazioniInMaxCoperti (RenameColumn). Nixpacks abbandonato dopo 2 fallimenti (SDK 6 invece di 9, poi dotnet-sdk_9 assente da nixpkgs pinnato) - sostituito con Dockerfile multi-stage (REV-011)</t>
+  </si>
+  <si>
+    <t>EF Core Migrations + Docker</t>
+  </si>
+  <si>
+    <t>Applicata a mano su Railway via railway connect Postgres + psql: backup mirato tabella (\copy CSV, 7 righe) poi ALTER TABLE RENAME COLUMN. Verificato: Fasce Orarie, creazione/modifica prenotazione, Dashboard - tutto pulito</t>
+  </si>
+  <si>
+    <t>Railway CLI + psql</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 2 checkpoint 2a</t>
+  </si>
+  <si>
+    <t>Rename MaxPrenotazioni -&gt; MaxCoperti (REV-005, REV-011)</t>
+  </si>
+  <si>
+    <t>Rename completo backend+frontend, migration applicata in produzione con backup mirato, deploy passato da Nixpacks a Dockerfile dopo 2 fallimenti di build. Verificato in produzione su Fasce Orarie, Prenotazioni, Dashboard.</t>
+  </si>
+  <si>
+    <t>Rename MaxCoperti + migration produzione + Dockerfile</t>
   </si>
 </sst>
 </file>
@@ -5867,7 +5906,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H132"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7832,6 +7871,79 @@
         <v>443</v>
       </c>
       <c r="E132" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>44</v>
+      </c>
+      <c r="B135" t="s">
+        <v>45</v>
+      </c>
+      <c r="C135" t="s">
+        <v>881</v>
+      </c>
+      <c r="D135" t="s">
+        <v>47</v>
+      </c>
+      <c r="E135" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A136">
+        <v>1</v>
+      </c>
+      <c r="B136" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C136" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D136" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E136" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A137">
+        <v>2</v>
+      </c>
+      <c r="B137" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C137" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D137" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E137" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A138">
+        <v>3</v>
+      </c>
+      <c r="B138" t="s">
+        <v>980</v>
+      </c>
+      <c r="C138" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D138" t="s">
+        <v>1046</v>
+      </c>
+      <c r="E138" t="s">
         <v>1020</v>
       </c>
     </row>
@@ -8336,7 +8448,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -8664,6 +8776,26 @@
         <v>6</v>
       </c>
     </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1037</v>
+      </c>
+      <c r="E18" t="s">
+        <v>1037</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>
@@ -8675,7 +8807,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -9105,6 +9237,20 @@
         <v>1034</v>
       </c>
       <c r="D35" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1049</v>
+      </c>
+      <c r="D36" s="27" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 3 - prenotazioni simultanee, vincolo a database (REV-003/026/032)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C05CA7D-E397-4E28-953C-66E7030C4A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA07801-11FD-4D4A-B768-04A1885D0875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3072" yWindow="3072" windowWidth="17280" windowHeight="9960" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2003" uniqueCount="1137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="1150">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3376,9 +3376,6 @@
     <t>01-set-26</t>
   </si>
   <si>
-    <t>Codice completo, 57/57 test, nessuna migration. Test manuali di Fabio pendenti per chiusura Fase 2.</t>
-  </si>
-  <si>
     <t>Unificazione disponibilita/assegnazione + fix correlati (REV-001, REV-002, REV-006, REV-016, REV-024, REV-034, REV-092)</t>
   </si>
   <si>
@@ -3427,9 +3424,6 @@
     <t>Checkpoint 2c chiuso (codice)</t>
   </si>
   <si>
-    <t>Nessuna migration in tutto il 2c. dotnet test 57 su 57 verdi (erano 42), frontend tsc-build-eslint puliti. 3 commit su dev. Restano i test manuali di Fabio per la chiusura formale della Fase 2.</t>
-  </si>
-  <si>
     <t>xUnit + Vite</t>
   </si>
   <si>
@@ -3443,6 +3437,51 @@
   </si>
   <si>
     <t>/riepilogo-sala</t>
+  </si>
+  <si>
+    <t>Frontend - Prenotazioni</t>
+  </si>
+  <si>
+    <t>NEW-001: modal di modifica prenotazione</t>
+  </si>
+  <si>
+    <t>Nessun pulsante Modifica nelle prenotazioni (solo Conferma-Completa-Annulla). update-prenotazione e' capacita' solo-backend: il fix REV-002 non e' raggiungibile dall'app. Riusare PrenotazioneModal (prop prenotazione + precompilazione + mutation PUT + pulsante per stato Attiva). Da fare in Fase 6 insieme a REV-015 (stesso componente).</t>
+  </si>
+  <si>
+    <t>Pianificato (Fase 6)</t>
+  </si>
+  <si>
+    <t>NEW-002: pannello disponibilita' nel form di creazione (opzionale)</t>
+  </si>
+  <si>
+    <t>Scelti data + coperti, mostrare le fasce con semaforo, posti residui e il motivo del rifiuto (campo messaggio di check-disponibilita) invece di scoprirlo solo all'invio. NON una pagina pubblica per il cliente (esclusa dalla v1, decisione 10). Da confermare se vale lo sforzo.</t>
+  </si>
+  <si>
+    <t>Pianificato (Fase 10)</t>
+  </si>
+  <si>
+    <t>Nessuna migration in tutto il 2c. dotnet test 57 su 57 verdi (erano 42), frontend tsc-build-eslint puliti. 4 commit su dev. Tutti e 5 i test manuali di Fabio passati (2 e 3 via UI e Postman, 1-4-5 ok). FASE 2 CHIUSA.</t>
+  </si>
+  <si>
+    <t>Fase 3 - decisioni prese (impl. su Opus)</t>
+  </si>
+  <si>
+    <t>Indice A2 (unique PIENO su PostazioneId, DataPrenotazione, FasciaOrariaId; denormalizzare le 2 colonne sulla join). AnnullaPrenotazioneAsync elimina le righe join. 23505 a nuova ConflictException a 409, stringere InvalidOperationException a 409 nel middleware (anticipa REV-026). Transazione dentro CreateExecutionStrategy().ExecuteAsync. Test concorrenza: InMemory non applica gli unique index, valutare Testcontainers o spezzare il test. Migration manuale (breaking).</t>
+  </si>
+  <si>
+    <t>Pianificato</t>
+  </si>
+  <si>
+    <t>FASE 2 CHIUSA 01/09/2026: checkpoint 2c completo + tutti i 5 test manuali di Fabio passati. Nessuna migration nel 2c.</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 3</t>
+  </si>
+  <si>
+    <t>Prenotazioni simultanee: operazione atomica + unique index a DB sullo slot tavolo (denorm A2) + 23505 a 409 + test concorrenza</t>
+  </si>
+  <si>
+    <t>Decisioni prese 01/09. Implementazione su Opus. Richiede migration manuale (breaking).</t>
   </si>
 </sst>
 </file>
@@ -3546,7 +3585,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3645,6 +3684,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE9F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -3697,7 +3742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3804,6 +3849,8 @@
     <xf numFmtId="0" fontId="5" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3834,7 +3881,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -4149,36 +4196,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="42" t="s">
         <v>1106</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="44" t="s">
+      <c r="B4" s="47"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="F4" s="46"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="48"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -4365,24 +4412,24 @@
       <c r="F15" s="37"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="47" t="s">
+      <c r="A16" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="45"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="46"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="48"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="41"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4410,14 +4457,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>644</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4907,7 +4954,7 @@
         <v>669</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>684</v>
@@ -4916,7 +4963,7 @@
         <v>438</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5190,7 +5237,7 @@
         <v>733</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="E41" s="14" t="s">
         <v>691</v>
@@ -5480,13 +5527,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>1074</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6017,11 +6064,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>800</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6287,14 +6334,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>846</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6375,7 +6422,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H155"/>
+  <dimension ref="A1:H156"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -6387,40 +6434,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="42" t="s">
         <v>1110</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="48"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -6743,16 +6790,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="46"/>
+      <c r="B22" s="47"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="47"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="48"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -6975,16 +7022,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="48" t="s">
+      <c r="A35" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="B35" s="45"/>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="46"/>
+      <c r="B35" s="47"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="47"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="48"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -7167,16 +7214,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="49" t="s">
+      <c r="A46" s="51" t="s">
         <v>174</v>
       </c>
-      <c r="B46" s="45"/>
-      <c r="C46" s="45"/>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="45"/>
-      <c r="H46" s="46"/>
+      <c r="B46" s="47"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="47"/>
+      <c r="E46" s="47"/>
+      <c r="F46" s="47"/>
+      <c r="G46" s="47"/>
+      <c r="H46" s="48"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -7239,16 +7286,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="47" t="s">
+      <c r="A51" s="49" t="s">
         <v>186</v>
       </c>
-      <c r="B51" s="45"/>
-      <c r="C51" s="45"/>
-      <c r="D51" s="45"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-      <c r="G51" s="45"/>
-      <c r="H51" s="46"/>
+      <c r="B51" s="47"/>
+      <c r="C51" s="47"/>
+      <c r="D51" s="47"/>
+      <c r="E51" s="47"/>
+      <c r="F51" s="47"/>
+      <c r="G51" s="47"/>
+      <c r="H51" s="48"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -8593,7 +8640,7 @@
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
@@ -8621,16 +8668,16 @@
         <v>1</v>
       </c>
       <c r="B151" s="27" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C151" s="27" t="s">
         <v>1118</v>
       </c>
-      <c r="C151" s="27" t="s">
+      <c r="D151" s="27" t="s">
         <v>1119</v>
       </c>
-      <c r="D151" s="27" t="s">
-        <v>1120</v>
-      </c>
-      <c r="E151" s="52" t="s">
-        <v>1135</v>
+      <c r="E151" s="40" t="s">
+        <v>1133</v>
       </c>
       <c r="F151" s="27" t="s">
         <v>6</v>
@@ -8641,16 +8688,16 @@
         <v>2</v>
       </c>
       <c r="B152" s="27" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C152" s="27" t="s">
         <v>1121</v>
       </c>
-      <c r="C152" s="27" t="s">
+      <c r="D152" s="27" t="s">
         <v>1122</v>
       </c>
-      <c r="D152" s="27" t="s">
-        <v>1123</v>
-      </c>
-      <c r="E152" s="52" t="s">
-        <v>1135</v>
+      <c r="E152" s="40" t="s">
+        <v>1133</v>
       </c>
       <c r="F152" s="27" t="s">
         <v>6</v>
@@ -8661,16 +8708,16 @@
         <v>3</v>
       </c>
       <c r="B153" s="27" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C153" s="27" t="s">
         <v>1124</v>
       </c>
-      <c r="C153" s="27" t="s">
+      <c r="D153" s="27" t="s">
         <v>1125</v>
       </c>
-      <c r="D153" s="27" t="s">
-        <v>1126</v>
-      </c>
-      <c r="E153" s="52" t="s">
-        <v>1135</v>
+      <c r="E153" s="40" t="s">
+        <v>1133</v>
       </c>
       <c r="F153" s="27" t="s">
         <v>6</v>
@@ -8681,16 +8728,16 @@
         <v>4</v>
       </c>
       <c r="B154" s="27" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C154" s="27" t="s">
         <v>1127</v>
       </c>
-      <c r="C154" s="27" t="s">
+      <c r="D154" s="27" t="s">
         <v>1128</v>
       </c>
-      <c r="D154" s="27" t="s">
-        <v>1129</v>
-      </c>
-      <c r="E154" s="52" t="s">
-        <v>1135</v>
+      <c r="E154" s="40" t="s">
+        <v>1133</v>
       </c>
       <c r="F154" s="27" t="s">
         <v>6</v>
@@ -8701,19 +8748,39 @@
         <v>5</v>
       </c>
       <c r="B155" s="27" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C155" s="27" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D155" s="27" t="s">
         <v>1130</v>
       </c>
-      <c r="C155" s="27" t="s">
-        <v>1131</v>
-      </c>
-      <c r="D155" s="27" t="s">
-        <v>1132</v>
-      </c>
-      <c r="E155" s="52" t="s">
-        <v>1135</v>
+      <c r="E155" s="40" t="s">
+        <v>1133</v>
       </c>
       <c r="F155" s="27" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A156" s="41">
+        <v>6</v>
+      </c>
+      <c r="B156" s="41" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C156" s="41" t="s">
+        <v>1144</v>
+      </c>
+      <c r="D156" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="E156" s="54" t="s">
+        <v>1133</v>
+      </c>
+      <c r="F156" s="41" t="s">
+        <v>1145</v>
       </c>
     </row>
   </sheetData>
@@ -8743,24 +8810,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="53" t="s">
         <v>222</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="46"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8848,14 +8915,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="49" t="s">
         <v>242</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="46"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="48"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -8943,14 +9010,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="46" t="s">
         <v>256</v>
       </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="46"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="48"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -9072,14 +9139,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="44" t="s">
+      <c r="A26" s="46" t="s">
         <v>280</v>
       </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="46"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="48"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -9231,7 +9298,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -9243,26 +9310,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>289</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="49" t="s">
         <v>290</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="48"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -9622,7 +9689,26 @@
         <v>6</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>1114</v>
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="41" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41" t="s">
+        <v>1145</v>
+      </c>
+      <c r="G21" s="41" t="s">
+        <v>1149</v>
       </c>
     </row>
   </sheetData>
@@ -9636,7 +9722,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -9646,24 +9732,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>347</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="46" t="s">
         <v>348</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="46"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="48"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -9848,14 +9934,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="51" t="s">
+      <c r="A18" s="53" t="s">
         <v>380</v>
       </c>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="46"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="48"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -9962,14 +10048,14 @@
       <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="47" t="s">
+      <c r="A28" s="49" t="s">
         <v>393</v>
       </c>
-      <c r="B28" s="45"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="46"/>
+      <c r="B28" s="47"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="48"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -10102,13 +10188,41 @@
         <v>1111</v>
       </c>
       <c r="B38" s="27" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C38" s="27" t="s">
         <v>1115</v>
       </c>
-      <c r="C38" s="27" t="s">
-        <v>1116</v>
-      </c>
       <c r="D38" s="27" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="41" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B39" s="41" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C39" s="41" t="s">
+        <v>1137</v>
+      </c>
+      <c r="D39" s="41" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="41" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B40" s="41" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C40" s="41" t="s">
+        <v>1140</v>
+      </c>
+      <c r="D40" s="41" t="s">
+        <v>1141</v>
       </c>
     </row>
   </sheetData>
@@ -10135,14 +10249,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>405</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -10319,14 +10433,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>428</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -10929,13 +11043,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>504</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11332,13 +11446,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>583</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
Fase 3 fix + pulizia
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA07801-11FD-4D4A-B768-04A1885D0875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A3F8AA-8E9C-4991-9E4C-131A18EAF092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dashboard" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="1150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="1222">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3127,12 +3127,6 @@
     <t>CRUD + Assegnazione automatica (motore AssegnazioneTavoli)</t>
   </si>
   <si>
-    <t>42 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 42 test OK</t>
-  </si>
-  <si>
     <t>FASE 2 CHECKPOINT 2b - Nuovo algoritmo di assegnazione tavoli (sessione 31/08/2026)</t>
   </si>
   <si>
@@ -3352,21 +3346,9 @@
     <t>La somma dei posti distribuiti e sempre pari ai coperti</t>
   </si>
   <si>
-    <t>Aggiornato: 01/09/2026</t>
-  </si>
-  <si>
     <t>Unificata sul motore AssegnazioneTavoli, posti residui sul tetto MaxCoperti (checkpoint 2c)</t>
   </si>
   <si>
-    <t>57 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 57 test OK</t>
-  </si>
-  <si>
-    <t>Aggiornato: 01/09/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
     <t>Roadmap revisione - Fase 2 checkpoint 2c</t>
   </si>
   <si>
@@ -3445,9 +3427,6 @@
     <t>NEW-001: modal di modifica prenotazione</t>
   </si>
   <si>
-    <t>Nessun pulsante Modifica nelle prenotazioni (solo Conferma-Completa-Annulla). update-prenotazione e' capacita' solo-backend: il fix REV-002 non e' raggiungibile dall'app. Riusare PrenotazioneModal (prop prenotazione + precompilazione + mutation PUT + pulsante per stato Attiva). Da fare in Fase 6 insieme a REV-015 (stesso componente).</t>
-  </si>
-  <si>
     <t>Pianificato (Fase 6)</t>
   </si>
   <si>
@@ -3481,7 +3460,244 @@
     <t>Prenotazioni simultanee: operazione atomica + unique index a DB sullo slot tavolo (denorm A2) + 23505 a 409 + test concorrenza</t>
   </si>
   <si>
-    <t>Decisioni prese 01/09. Implementazione su Opus. Richiede migration manuale (breaking).</t>
+    <t>Aggiornato: 02/09/2026</t>
+  </si>
+  <si>
+    <t>70 test unitari</t>
+  </si>
+  <si>
+    <t>Testing - 70 test OK</t>
+  </si>
+  <si>
+    <t>Concorrenza prenotazioni</t>
+  </si>
+  <si>
+    <t>Unique index UX_PrenotazionePostazione_Slot + transazioni (Fase 3)</t>
+  </si>
+  <si>
+    <t>Aggiornato: 02/09/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>FASE 3 ROADMAP REVISIONE - Prenotazioni simultanee (sessione 02/09/2026)</t>
+  </si>
+  <si>
+    <t>Vincolo a database (REV-003)</t>
+  </si>
+  <si>
+    <t>PrenotazionePostazione porta la copia denormalizzata di DataPrenotazione e FasciaOrariaId; unique index PIENO UX_PrenotazionePostazione_Slot su (PostazioneId, DataPrenotazione, FasciaOrariaId). E' il database a rifiutare la seconda scrittura, non il livello di isolamento della transazione.</t>
+  </si>
+  <si>
+    <t>EF Core 9 + PostgreSQL unique index</t>
+  </si>
+  <si>
+    <t>02/09/2026</t>
+  </si>
+  <si>
+    <t>Migration scritta a mano</t>
+  </si>
+  <si>
+    <t>AggiungiSlotPrenotazionePostazione: lo scaffolding EF era inutilizzabile (riempiva le colonne con 0001-01-01 e 0, poi falliva l'indice). Ordine vincolante: colonne nullable, backfill dallo slot della prenotazione, cancellazione righe delle annullate, NOT NULL, indice.</t>
+  </si>
+  <si>
+    <t>EF Core Migrations + SQL</t>
+  </si>
+  <si>
+    <t>Operazione atomica + annullo</t>
+  </si>
+  <si>
+    <t>AddAsync, UpdateAsync e AnnullaPrenotazioneAsync dentro CreateExecutionStrategy().ExecuteAsync + transazione (helper EseguiInTransazioneAsync). In UpdateAsync i DELETE sono salvati prima degli INSERT: EF non garantisce quell'ordine in una sola SaveChanges e l'indice rifiuterebbe una modifica che riusa lo stesso tavolo. L'annullo cancella le righe join: la prenotazione annullata libera il tavolo.</t>
+  </si>
+  <si>
+    <t>EF Core execution strategy + transazioni</t>
+  </si>
+  <si>
+    <t>23505 a 409 e REV-026 completo</t>
+  </si>
+  <si>
+    <t>Nuove ConflictException e DbExceptionTranslator: la violazione dell'unique index diventa un 409 leggibile, un 23505 di altri vincoli resta 500. Convertite 37 InvalidOperationException nei 5 service (34 ConflictException, 3 NotFoundException) e rimossa la mappatura generica dal middleware: da ora il 409 e' solo ConflictException.</t>
+  </si>
+  <si>
+    <t>ExceptionMiddleware + Npgsql</t>
+  </si>
+  <si>
+    <t>REV-032 parziale</t>
+  </si>
+  <si>
+    <t>L'audit log di creazione, modifica e annullo e' entrato nella stessa transazione della scrittura che registra: se il log fallisce, l'operazione non resta scritta e non tracciata. Zone, Postazioni e Fasce restano alla Fase 7.</t>
+  </si>
+  <si>
+    <t>LogActivityService + transazioni</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>70/70 verdi (erano 57): 6 su DbExceptionTranslator (23505 riconosciuto solo sul constraint giusto) e 7 su PrenotazioniService (slot valorizzato in creazione e modifica, conflitto tradotto, righe join cancellate sull'annullo, fallimento del log che fa fallire l'operazione). Nessun test di concorrenza automatico: l'InMemory non applica gli unique index, scelto di non introdurre Testcontainers.</t>
+  </si>
+  <si>
+    <t>xUnit + Moq + MockQueryable</t>
+  </si>
+  <si>
+    <t>Migration in produzione</t>
+  </si>
+  <si>
+    <t>Backup mirato con \copy (Prenotazioni 20 righe, PrenotazioniPostazioni 33) - il servizio Postgres su Railway non ha TCP proxy pubblico, pg_dump da locale non e' possibile. Pre-check duplicati 0, cancellate 14 righe di annullate, risultato 19 righe con slot completo. Poi merge dev-&gt;main e deploy.</t>
+  </si>
+  <si>
+    <t>Test di concorrenza superato</t>
+  </si>
+  <si>
+    <t>Due POST crea-prenotazione realmente simultanee (due SendAsync su HttpClient senza attesa reciproca) su una zona di test con un solo tavolo da 2: HTTP 201 + HTTP 409 'Il tavolo e' stato appena assegnato a un'altra prenotazione'. Il controllo applicativo aveva visto il tavolo libero per entrambe: a fermare la seconda e' stato l'unique index. FASE 3 CHIUSA.</t>
+  </si>
+  <si>
+    <t>PowerShell + HttpClient</t>
+  </si>
+  <si>
+    <t>Da ricordare - BOM negli script SQL</t>
+  </si>
+  <si>
+    <t>dotnet ef migrations script genera il file con BOM UTF-8: psql lo attacca alla prima istruzione, START TRANSACTION fallisce con syntax error e tutto lo script gira in autocommit, senza rollback in caso di errore. Successo in produzione il 02/09 (esito corretto ma senza rete di sicurezza). Il file in Scripts/ e' stato ripulito e porta la nota in testa.</t>
+  </si>
+  <si>
+    <t>psql + EF Core tooling</t>
+  </si>
+  <si>
+    <t>Unique index sullo slot (tavolo + data + fascia) con colonne denormalizzate sulla join, scritture in transazione dentro l'execution strategy, violazione 23505 tradotta in 409 leggibile</t>
+  </si>
+  <si>
+    <t>EF Core + PostgreSQL + ExceptionMiddleware</t>
+  </si>
+  <si>
+    <t>02-set-26</t>
+  </si>
+  <si>
+    <t>FASE 3 CHIUSA 02/09/2026: migration applicata in produzione (19 righe finali, 14 di annullate cancellate) e test di concorrenza superato in produzione (201 + 409). Chiusi anche REV-026 completo e REV-032 parziale, anticipati dalla Fase 7. Prossimo: Fase 4 sicurezza e primo avvio.</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 4</t>
+  </si>
+  <si>
+    <t>Sicurezza e primo avvio: schermata di primo avvio al posto di seed-admin pubblico (REV-007), email fuori dai log (REV-070), 401 e 403 distinti senza logout (REV-025), campo riservato non scrivibile dal Cliente (REV-033)</t>
+  </si>
+  <si>
+    <t>Nessun task Fabio previsto. A fine fase va decisa l'eventuale release intermedia v1.0.1.</t>
+  </si>
+  <si>
+    <t>Prenotazioni simultanee (REV-003, REV-026, REV-032 parziale)</t>
+  </si>
+  <si>
+    <t>Unique index UX_PrenotazionePostazione_Slot sullo slot con DataPrenotazione e FasciaOrariaId denormalizzate sulla join; creazione, modifica e annullo in transazione dentro l'execution strategy, con i DELETE salvati prima degli INSERT; l'annullo cancella le righe join e libera il tavolo; 23505 tradotto in ConflictException a 409; 37 InvalidOperationException convertite e mappatura generica rimossa dal middleware; audit log dentro la transazione. 70/70 test. Migration applicata in produzione e test di concorrenza superato (201 + 409).</t>
+  </si>
+  <si>
+    <t>Backend - Postazioni</t>
+  </si>
+  <si>
+    <t>NEW-003 (REV-099): un tavolo usato una volta non e' piu' modificabile</t>
+  </si>
+  <si>
+    <t>PostazioneService.UpdateAsync rifiuta l'aggiornamento se HasPrenotazioniAsync trova una qualsiasi riga in PrenotazioniPostazioni, senza distinguere fra prenotazioni future e storiche: dopo la prima prenotazione completata il tavolo non si puo' piu' rinominare, spostare di zona ne' disattivare. Emerso il 02/09 provando a disattivare i tavoli per preparare il test di concorrenza. Il controllo corretto guarda solo le prenotazioni future e non annullate.</t>
+  </si>
+  <si>
+    <t>Pianificato (Fase 7)</t>
+  </si>
+  <si>
+    <t>Nessun pulsante Modifica nelle prenotazioni (solo Conferma-Completa-Annulla). update-prenotazione e' capacita' solo-backend: il fix REV-002 non e' raggiungibile dall'app. Riusare PrenotazioneModal (prop prenotazione + precompilazione + mutation PUT + pulsante per stato Attiva). Da fare in Fase 6 insieme a REV-015 (stesso componente). Riscontrato di nuovo il 02/09/2026 durante i test di Fase 3: la prova di modifica e' stata possibile solo via Swagger.</t>
+  </si>
+  <si>
+    <t>DbExceptionTranslatorTests</t>
+  </si>
+  <si>
+    <t>IsUniqueViolation_ConVincoloAtteso_RestituisceTrue</t>
+  </si>
+  <si>
+    <t>23505 sul constraint dello slot viene riconosciuto</t>
+  </si>
+  <si>
+    <t>PostgresException costruita a mano</t>
+  </si>
+  <si>
+    <t>IsUniqueViolation_SenzaNomeVincolo_RiconosceQualunque23505</t>
+  </si>
+  <si>
+    <t>Senza nome constraint riconosce ogni violazione di unicita'</t>
+  </si>
+  <si>
+    <t>IsUniqueViolation_VincoloDiverso_RestituisceFalse</t>
+  </si>
+  <si>
+    <t>Un 23505 di un altro indice non e' un conflitto di slot</t>
+  </si>
+  <si>
+    <t>IsUniqueViolation_AltroCodiceErrore_RestituisceFalse</t>
+  </si>
+  <si>
+    <t>23503 (foreign key) non viene tradotto</t>
+  </si>
+  <si>
+    <t>IsUniqueViolation_EccezioneNonPostgres_RestituisceFalse</t>
+  </si>
+  <si>
+    <t>Un'eccezione non Postgres non viene tradotta</t>
+  </si>
+  <si>
+    <t>IsUniqueViolation_Null_RestituisceFalse</t>
+  </si>
+  <si>
+    <t>Null non fa eccezione</t>
+  </si>
+  <si>
+    <t>AddAsync_ValorizzaLoSlotSulleRigheJoin</t>
+  </si>
+  <si>
+    <t>Creazione: DataPrenotazione e FasciaOrariaId scritte sulla riga join</t>
+  </si>
+  <si>
+    <t>Moq + InMemory</t>
+  </si>
+  <si>
+    <t>UpdateAsync_ValorizzaLoSlotSulleRigheJoin</t>
+  </si>
+  <si>
+    <t>Modifica: lo slot viene riscritto sulle righe nuove</t>
+  </si>
+  <si>
+    <t>AddAsync_ThrowsConflictException_QuandoIlTavoloVieneOccupatoNelFrattempo</t>
+  </si>
+  <si>
+    <t>23505 sullo slot in creazione diventa ConflictException (409)</t>
+  </si>
+  <si>
+    <t>Moq + DbUpdateException</t>
+  </si>
+  <si>
+    <t>UpdateAsync_ThrowsConflictException_QuandoIlTavoloVieneOccupatoNelFrattempo</t>
+  </si>
+  <si>
+    <t>23505 sullo slot in modifica diventa ConflictException (409)</t>
+  </si>
+  <si>
+    <t>AddAsync_NonTraduceUnaViolazioneDiAltriVincoli</t>
+  </si>
+  <si>
+    <t>Un 23505 di un altro indice resta errore interno (500)</t>
+  </si>
+  <si>
+    <t>AnnullaPrenotazioneAsync_CancellaLeRigheJoin</t>
+  </si>
+  <si>
+    <t>L'annullo marca come Deleted le righe del tavolo: lo slot si libera</t>
+  </si>
+  <si>
+    <t>Moq + InMemory ChangeTracker</t>
+  </si>
+  <si>
+    <t>AddAsync_FallisceSeLAuditLogFallisce</t>
+  </si>
+  <si>
+    <t>REV-032: il log e' nella transazione, se fallisce fallisce tutto</t>
+  </si>
+  <si>
+    <t>Moq</t>
   </si>
 </sst>
 </file>
@@ -3585,7 +3801,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3690,6 +3906,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -3742,7 +3964,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3851,6 +4073,7 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3881,7 +4104,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -4196,36 +4419,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
-        <v>1106</v>
-      </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
+      <c r="A2" s="43" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="48"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="F4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="49"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -4332,7 +4555,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>1107</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4365,10 +4588,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1108</v>
+        <v>1143</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1031</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4376,11 +4599,11 @@
         <v>33</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1032</v>
+        <v>1144</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1109</v>
+        <v>1144</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -4407,29 +4630,35 @@
       <c r="A15" s="1"/>
       <c r="B15" s="34"/>
       <c r="C15" s="33"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="37"/>
+      <c r="D15" s="35" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="37" t="s">
+        <v>1146</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="49" t="s">
+      <c r="A16" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="48"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="49"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4457,14 +4686,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>644</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4954,7 +5183,7 @@
         <v>669</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>1134</v>
+        <v>1128</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>684</v>
@@ -4963,7 +5192,7 @@
         <v>438</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>1132</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5237,7 +5466,7 @@
         <v>733</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>1131</v>
+        <v>1125</v>
       </c>
       <c r="E41" s="14" t="s">
         <v>691</v>
@@ -5516,7 +5745,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -5527,13 +5756,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
-        <v>1074</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="A1" s="53" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5795,13 +6024,13 @@
         <v>799</v>
       </c>
       <c r="B18" s="11" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>1074</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>1075</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>1077</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>6</v>
@@ -5812,13 +6041,13 @@
         <v>799</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E19" s="39" t="s">
         <v>6</v>
@@ -5829,13 +6058,13 @@
         <v>799</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>6</v>
@@ -5846,13 +6075,13 @@
         <v>799</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E21" s="39" t="s">
         <v>6</v>
@@ -5863,13 +6092,13 @@
         <v>799</v>
       </c>
       <c r="B22" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="C22" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="D22" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E22" s="27" t="s">
         <v>6</v>
@@ -5880,13 +6109,13 @@
         <v>799</v>
       </c>
       <c r="B23" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="C23" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="D23" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E23" s="27" t="s">
         <v>6</v>
@@ -5897,13 +6126,13 @@
         <v>799</v>
       </c>
       <c r="B24" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="C24" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="D24" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E24" s="27" t="s">
         <v>6</v>
@@ -5914,13 +6143,13 @@
         <v>799</v>
       </c>
       <c r="B25" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="C25" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="D25" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E25" s="27" t="s">
         <v>6</v>
@@ -5931,13 +6160,13 @@
         <v>799</v>
       </c>
       <c r="B26" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="C26" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="D26" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E26" s="27" t="s">
         <v>6</v>
@@ -5948,13 +6177,13 @@
         <v>799</v>
       </c>
       <c r="B27" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="C27" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="D27" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E27" s="27" t="s">
         <v>6</v>
@@ -5965,13 +6194,13 @@
         <v>799</v>
       </c>
       <c r="B28" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="C28" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="D28" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E28" s="27" t="s">
         <v>6</v>
@@ -5982,13 +6211,13 @@
         <v>799</v>
       </c>
       <c r="B29" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="C29" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="D29" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E29" s="27" t="s">
         <v>6</v>
@@ -5999,13 +6228,13 @@
         <v>799</v>
       </c>
       <c r="B30" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="C30" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="D30" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E30" s="27" t="s">
         <v>6</v>
@@ -6016,13 +6245,13 @@
         <v>799</v>
       </c>
       <c r="B31" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="C31" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="D31" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E31" s="27" t="s">
         <v>6</v>
@@ -6033,15 +6262,236 @@
         <v>799</v>
       </c>
       <c r="B32" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="C32" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="D32" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E32" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1192</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E33" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E34" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1196</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1197</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E35" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1198</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E36" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1200</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E37" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E38" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>777</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>777</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E40" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>777</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1209</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1210</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1211</v>
+      </c>
+      <c r="E41" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>777</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1212</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1213</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1211</v>
+      </c>
+      <c r="E42" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>777</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1214</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1215</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1211</v>
+      </c>
+      <c r="E43" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>777</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1217</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1218</v>
+      </c>
+      <c r="E44" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>777</v>
+      </c>
+      <c r="B45" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1220</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1221</v>
+      </c>
+      <c r="E45" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -6064,11 +6514,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>800</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6334,14 +6784,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>846</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6422,7 +6872,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H156"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -6434,40 +6884,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="A2" s="43" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="48"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="49"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -6790,16 +7240,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="46" t="s">
+      <c r="A22" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="48"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="49"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -7022,16 +7472,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="50" t="s">
+      <c r="A35" s="51" t="s">
         <v>135</v>
       </c>
-      <c r="B35" s="47"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="47"/>
-      <c r="E35" s="47"/>
-      <c r="F35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="48"/>
+      <c r="B35" s="48"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="49"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -7214,16 +7664,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="51" t="s">
+      <c r="A46" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="B46" s="47"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="47"/>
-      <c r="E46" s="47"/>
-      <c r="F46" s="47"/>
-      <c r="G46" s="47"/>
-      <c r="H46" s="48"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="48"/>
+      <c r="F46" s="48"/>
+      <c r="G46" s="48"/>
+      <c r="H46" s="49"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -7286,16 +7736,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="49" t="s">
+      <c r="A51" s="50" t="s">
         <v>186</v>
       </c>
-      <c r="B51" s="47"/>
-      <c r="C51" s="47"/>
-      <c r="D51" s="47"/>
-      <c r="E51" s="47"/>
-      <c r="F51" s="47"/>
-      <c r="G51" s="47"/>
-      <c r="H51" s="48"/>
+      <c r="B51" s="48"/>
+      <c r="C51" s="48"/>
+      <c r="D51" s="48"/>
+      <c r="E51" s="48"/>
+      <c r="F51" s="48"/>
+      <c r="G51" s="48"/>
+      <c r="H51" s="49"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -8495,7 +8945,7 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
@@ -8523,13 +8973,13 @@
         <v>1</v>
       </c>
       <c r="B142" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C142" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D142" t="s">
         <v>1034</v>
-      </c>
-      <c r="C142" t="s">
-        <v>1035</v>
-      </c>
-      <c r="D142" t="s">
-        <v>1036</v>
       </c>
       <c r="E142" t="s">
         <v>999</v>
@@ -8543,13 +8993,13 @@
         <v>2</v>
       </c>
       <c r="B143" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C143" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D143" t="s">
         <v>1037</v>
-      </c>
-      <c r="C143" t="s">
-        <v>1038</v>
-      </c>
-      <c r="D143" t="s">
-        <v>1039</v>
       </c>
       <c r="E143" t="s">
         <v>999</v>
@@ -8563,13 +9013,13 @@
         <v>3</v>
       </c>
       <c r="B144" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C144" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D144" t="s">
         <v>1040</v>
-      </c>
-      <c r="C144" t="s">
-        <v>1041</v>
-      </c>
-      <c r="D144" t="s">
-        <v>1042</v>
       </c>
       <c r="E144" t="s">
         <v>999</v>
@@ -8583,13 +9033,13 @@
         <v>4</v>
       </c>
       <c r="B145" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C145" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D145" t="s">
         <v>1043</v>
-      </c>
-      <c r="C145" t="s">
-        <v>1044</v>
-      </c>
-      <c r="D145" t="s">
-        <v>1045</v>
       </c>
       <c r="E145" t="s">
         <v>999</v>
@@ -8603,10 +9053,10 @@
         <v>5</v>
       </c>
       <c r="B146" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="C146" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="D146" t="s">
         <v>30</v>
@@ -8623,13 +9073,13 @@
         <v>6</v>
       </c>
       <c r="B147" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C147" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D147" t="s">
         <v>1048</v>
-      </c>
-      <c r="C147" t="s">
-        <v>1049</v>
-      </c>
-      <c r="D147" t="s">
-        <v>1050</v>
       </c>
       <c r="E147" t="s">
         <v>999</v>
@@ -8640,7 +9090,7 @@
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>1116</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
@@ -8668,16 +9118,16 @@
         <v>1</v>
       </c>
       <c r="B151" s="27" t="s">
-        <v>1117</v>
+        <v>1111</v>
       </c>
       <c r="C151" s="27" t="s">
-        <v>1118</v>
+        <v>1112</v>
       </c>
       <c r="D151" s="27" t="s">
-        <v>1119</v>
+        <v>1113</v>
       </c>
       <c r="E151" s="40" t="s">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="F151" s="27" t="s">
         <v>6</v>
@@ -8688,16 +9138,16 @@
         <v>2</v>
       </c>
       <c r="B152" s="27" t="s">
-        <v>1120</v>
+        <v>1114</v>
       </c>
       <c r="C152" s="27" t="s">
-        <v>1121</v>
+        <v>1115</v>
       </c>
       <c r="D152" s="27" t="s">
-        <v>1122</v>
+        <v>1116</v>
       </c>
       <c r="E152" s="40" t="s">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="F152" s="27" t="s">
         <v>6</v>
@@ -8708,16 +9158,16 @@
         <v>3</v>
       </c>
       <c r="B153" s="27" t="s">
-        <v>1123</v>
+        <v>1117</v>
       </c>
       <c r="C153" s="27" t="s">
-        <v>1124</v>
+        <v>1118</v>
       </c>
       <c r="D153" s="27" t="s">
-        <v>1125</v>
+        <v>1119</v>
       </c>
       <c r="E153" s="40" t="s">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="F153" s="27" t="s">
         <v>6</v>
@@ -8728,16 +9178,16 @@
         <v>4</v>
       </c>
       <c r="B154" s="27" t="s">
-        <v>1126</v>
+        <v>1120</v>
       </c>
       <c r="C154" s="27" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D154" s="27" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E154" s="40" t="s">
         <v>1127</v>
-      </c>
-      <c r="D154" s="27" t="s">
-        <v>1128</v>
-      </c>
-      <c r="E154" s="40" t="s">
-        <v>1133</v>
       </c>
       <c r="F154" s="27" t="s">
         <v>6</v>
@@ -8748,16 +9198,16 @@
         <v>5</v>
       </c>
       <c r="B155" s="27" t="s">
-        <v>1129</v>
+        <v>1123</v>
       </c>
       <c r="C155" s="27" t="s">
-        <v>1142</v>
+        <v>1135</v>
       </c>
       <c r="D155" s="27" t="s">
-        <v>1130</v>
+        <v>1124</v>
       </c>
       <c r="E155" s="40" t="s">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="F155" s="27" t="s">
         <v>6</v>
@@ -8768,19 +9218,224 @@
         <v>6</v>
       </c>
       <c r="B156" s="41" t="s">
-        <v>1143</v>
+        <v>1136</v>
       </c>
       <c r="C156" s="41" t="s">
-        <v>1144</v>
+        <v>1137</v>
       </c>
       <c r="D156" s="41" t="s">
         <v>268</v>
       </c>
-      <c r="E156" s="54" t="s">
-        <v>1133</v>
-      </c>
-      <c r="F156" s="41" t="s">
-        <v>1145</v>
+      <c r="E156" s="42" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F156" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>40</v>
+      </c>
+      <c r="B159" t="s">
+        <v>41</v>
+      </c>
+      <c r="C159" t="s">
+        <v>862</v>
+      </c>
+      <c r="D159" t="s">
+        <v>43</v>
+      </c>
+      <c r="E159" t="s">
+        <v>44</v>
+      </c>
+      <c r="F159" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A160" s="27">
+        <v>1</v>
+      </c>
+      <c r="B160" s="27" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C160" s="27" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D160" s="27" t="s">
+        <v>1151</v>
+      </c>
+      <c r="E160" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F160" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A161" s="27">
+        <v>2</v>
+      </c>
+      <c r="B161" s="27" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C161" s="27" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D161" s="27" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E161" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F161" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A162" s="27">
+        <v>3</v>
+      </c>
+      <c r="B162" s="27" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C162" s="27" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D162" s="27" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E162" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F162" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A163" s="27">
+        <v>4</v>
+      </c>
+      <c r="B163" s="27" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C163" s="27" t="s">
+        <v>1160</v>
+      </c>
+      <c r="D163" s="27" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E163" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F163" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A164" s="27">
+        <v>5</v>
+      </c>
+      <c r="B164" s="27" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C164" s="27" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D164" s="27" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E164" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F164" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A165" s="27">
+        <v>6</v>
+      </c>
+      <c r="B165" s="27" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C165" s="27" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D165" s="27" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E165" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F165" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A166" s="27">
+        <v>7</v>
+      </c>
+      <c r="B166" s="27" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C166" s="27" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D166" s="27" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E166" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F166" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A167" s="27">
+        <v>8</v>
+      </c>
+      <c r="B167" s="27" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C167" s="27" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D167" s="27" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E167" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F167" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A168" s="27">
+        <v>9</v>
+      </c>
+      <c r="B168" s="27" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C168" s="27" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D168" s="27" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E168" s="40" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F168" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -8799,7 +9454,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -8810,24 +9465,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="54" t="s">
         <v>222</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="49"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -8915,14 +9570,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="50" t="s">
         <v>242</v>
       </c>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="48"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="49"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -9010,14 +9665,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="46" t="s">
+      <c r="A17" s="47" t="s">
         <v>256</v>
       </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="47"/>
-      <c r="F17" s="48"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="49"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -9139,14 +9794,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="47" t="s">
         <v>280</v>
       </c>
-      <c r="B26" s="47"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="48"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="49"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -9224,7 +9879,7 @@
         <v>73</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>75</v>
@@ -9269,18 +9924,35 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C34" t="s">
         <v>1052</v>
       </c>
-      <c r="B34" t="s">
+      <c r="D34" t="s">
         <v>1053</v>
       </c>
-      <c r="C34" t="s">
-        <v>1054</v>
-      </c>
-      <c r="D34" t="s">
-        <v>1055</v>
-      </c>
       <c r="E34" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E35" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -9298,7 +9970,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -9310,26 +9982,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>289</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="50" t="s">
         <v>290</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="48"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="49"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -9651,10 +10323,10 @@
         <v>1014</v>
       </c>
       <c r="B19" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="C19" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="D19" t="s">
         <v>1016</v>
@@ -9666,7 +10338,7 @@
         <v>6</v>
       </c>
       <c r="G19" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -9674,22 +10346,22 @@
         <v>1014</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>1111</v>
+        <v>1105</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>1112</v>
+        <v>1106</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>1113</v>
+        <v>1107</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>1113</v>
+        <v>1107</v>
       </c>
       <c r="F20" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>1146</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -9697,18 +10369,41 @@
         <v>1014</v>
       </c>
       <c r="B21" s="41" t="s">
-        <v>1147</v>
+        <v>1140</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>1148</v>
-      </c>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41" t="s">
-        <v>1145</v>
+        <v>1141</v>
+      </c>
+      <c r="D21" s="41" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>6</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>1149</v>
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="41" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B22" s="41" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>1181</v>
+      </c>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="55" t="s">
+        <v>1138</v>
+      </c>
+      <c r="G22" s="41" t="s">
+        <v>1182</v>
       </c>
     </row>
   </sheetData>
@@ -9722,7 +10417,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -9732,24 +10427,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>347</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="47" t="s">
         <v>348</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="48"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="49"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -9934,14 +10629,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="53" t="s">
+      <c r="A18" s="54" t="s">
         <v>380</v>
       </c>
-      <c r="B18" s="47"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="47"/>
-      <c r="F18" s="48"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="49"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -10048,14 +10743,14 @@
       <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="49" t="s">
+      <c r="A28" s="50" t="s">
         <v>393</v>
       </c>
-      <c r="B28" s="47"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="48"/>
+      <c r="B28" s="48"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="48"/>
+      <c r="E28" s="48"/>
+      <c r="F28" s="49"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -10171,13 +10866,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="B37" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="C37" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="D37" s="27" t="s">
         <v>6</v>
@@ -10185,13 +10880,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="27" t="s">
-        <v>1111</v>
+        <v>1105</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>1114</v>
+        <v>1108</v>
       </c>
       <c r="C38" s="27" t="s">
-        <v>1115</v>
+        <v>1109</v>
       </c>
       <c r="D38" s="27" t="s">
         <v>6</v>
@@ -10199,30 +10894,58 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="41" t="s">
-        <v>1135</v>
+        <v>1129</v>
       </c>
       <c r="B39" s="41" t="s">
-        <v>1136</v>
+        <v>1130</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1137</v>
+        <v>1189</v>
       </c>
       <c r="D39" s="41" t="s">
-        <v>1138</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="41" t="s">
-        <v>1135</v>
+        <v>1129</v>
       </c>
       <c r="B40" s="41" t="s">
-        <v>1139</v>
+        <v>1132</v>
       </c>
       <c r="C40" s="41" t="s">
+        <v>1133</v>
+      </c>
+      <c r="D40" s="41" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="27" t="s">
         <v>1140</v>
       </c>
-      <c r="D40" s="41" t="s">
-        <v>1141</v>
+      <c r="B41" s="27" t="s">
+        <v>1183</v>
+      </c>
+      <c r="C41" s="27" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D41" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="41" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B42" s="41" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C42" s="41" t="s">
+        <v>1187</v>
+      </c>
+      <c r="D42" s="55" t="s">
+        <v>1188</v>
       </c>
     </row>
   </sheetData>
@@ -10249,14 +10972,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>405</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -10433,14 +11156,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>428</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11043,13 +11766,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>504</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11446,13 +12169,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>583</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11567,7 +12290,7 @@
         <v>603</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>604</v>
@@ -11734,13 +12457,13 @@
         <v>638</v>
       </c>
       <c r="C19" s="14" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E19" s="14" t="s">
         <v>1062</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>1063</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -11762,36 +12485,36 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C21" t="s">
         <v>1065</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>1066</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>1067</v>
-      </c>
-      <c r="D21" t="s">
-        <v>1068</v>
-      </c>
-      <c r="E21" t="s">
-        <v>1069</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="B22" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D22" t="s">
         <v>1070</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>1071</v>
-      </c>
-      <c r="D22" t="s">
-        <v>1072</v>
-      </c>
-      <c r="E22" t="s">
-        <v>1073</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: chiusura Fase 3 - stato sessione, roadmap e tracker
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A3F8AA-8E9C-4991-9E4C-131A18EAF092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A04D2F8-C169-479E-8AD3-16D0650D18FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="1222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="1223">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3547,9 +3547,6 @@
     <t>Test di concorrenza superato</t>
   </si>
   <si>
-    <t>Due POST crea-prenotazione realmente simultanee (due SendAsync su HttpClient senza attesa reciproca) su una zona di test con un solo tavolo da 2: HTTP 201 + HTTP 409 'Il tavolo e' stato appena assegnato a un'altra prenotazione'. Il controllo applicativo aveva visto il tavolo libero per entrambe: a fermare la seconda e' stato l'unique index. FASE 3 CHIUSA.</t>
-  </si>
-  <si>
     <t>PowerShell + HttpClient</t>
   </si>
   <si>
@@ -3571,9 +3568,6 @@
     <t>02-set-26</t>
   </si>
   <si>
-    <t>FASE 3 CHIUSA 02/09/2026: migration applicata in produzione (19 righe finali, 14 di annullate cancellate) e test di concorrenza superato in produzione (201 + 409). Chiusi anche REV-026 completo e REV-032 parziale, anticipati dalla Fase 7. Prossimo: Fase 4 sicurezza e primo avvio.</t>
-  </si>
-  <si>
     <t>Roadmap revisione - Fase 4</t>
   </si>
   <si>
@@ -3698,6 +3692,15 @@
   </si>
   <si>
     <t>Moq</t>
+  </si>
+  <si>
+    <t>In corso</t>
+  </si>
+  <si>
+    <t>02/09/2026: codice, migration in produzione e test di concorrenza (201+409) completati. NON ancora chiusa formalmente: mancano commit/push (DoD punto 5) e la pulizia dei dati di test in produzione (zona Test concorrenza, tavolo, prenotazioni di prova). Chiusi anche REV-026 completo e REV-032 parziale.</t>
+  </si>
+  <si>
+    <t>Due POST crea-prenotazione realmente simultanee (due SendAsync su HttpClient senza attesa reciproca) su una zona di test con un solo tavolo da 2: HTTP 201 + HTTP 409 'Il tavolo e' stato appena assegnato a un'altra prenotazione'. Il controllo applicativo aveva visto il tavolo libero per entrambe: a fermare la seconda e' stato l'unique index. Restano commit/push e pulizia dei dati di test in produzione prima della chiusura formale (DoD punto 5).</t>
   </si>
 </sst>
 </file>
@@ -4074,6 +4077,7 @@
     <xf numFmtId="49" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4104,7 +4108,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -4419,36 +4422,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>1142</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="47" t="s">
+      <c r="B4" s="49"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="50"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -4641,24 +4644,24 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="50" t="s">
+      <c r="A16" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="49"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="50"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4686,14 +4689,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>644</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5756,13 +5759,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>1072</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6276,16 +6279,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C33" t="s">
         <v>1190</v>
       </c>
-      <c r="B33" t="s">
+      <c r="D33" t="s">
         <v>1191</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1192</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1193</v>
       </c>
       <c r="E33" s="27" t="s">
         <v>6</v>
@@ -6293,16 +6296,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="B34" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="C34" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="D34" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -6310,16 +6313,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="B35" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="C35" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="D35" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -6327,16 +6330,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="B36" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="C36" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="D36" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -6344,13 +6347,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="B37" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C37" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="D37" t="s">
         <v>1075</v>
@@ -6361,13 +6364,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="B38" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="C38" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="D38" t="s">
         <v>1075</v>
@@ -6381,13 +6384,13 @@
         <v>777</v>
       </c>
       <c r="B39" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D39" t="s">
         <v>1204</v>
-      </c>
-      <c r="C39" t="s">
-        <v>1205</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1206</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -6398,13 +6401,13 @@
         <v>777</v>
       </c>
       <c r="B40" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="C40" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="D40" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -6415,13 +6418,13 @@
         <v>777</v>
       </c>
       <c r="B41" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D41" t="s">
         <v>1209</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1210</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1211</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -6432,13 +6435,13 @@
         <v>777</v>
       </c>
       <c r="B42" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
       <c r="C42" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="D42" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="E42" s="27" t="s">
         <v>6</v>
@@ -6449,13 +6452,13 @@
         <v>777</v>
       </c>
       <c r="B43" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
       <c r="C43" t="s">
-        <v>1215</v>
+        <v>1213</v>
       </c>
       <c r="D43" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>6</v>
@@ -6466,13 +6469,13 @@
         <v>777</v>
       </c>
       <c r="B44" t="s">
+        <v>1214</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1215</v>
+      </c>
+      <c r="D44" t="s">
         <v>1216</v>
-      </c>
-      <c r="C44" t="s">
-        <v>1217</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1218</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>6</v>
@@ -6483,13 +6486,13 @@
         <v>777</v>
       </c>
       <c r="B45" t="s">
+        <v>1217</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1218</v>
+      </c>
+      <c r="D45" t="s">
         <v>1219</v>
-      </c>
-      <c r="C45" t="s">
-        <v>1220</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1221</v>
       </c>
       <c r="E45" s="27" t="s">
         <v>6</v>
@@ -6514,11 +6517,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>800</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6784,14 +6787,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>846</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6884,40 +6887,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>1147</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="49"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="50"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -7240,16 +7243,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="49"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -7472,16 +7475,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="51" t="s">
+      <c r="A35" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="49"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="49"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="49"/>
+      <c r="H35" s="50"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -7664,16 +7667,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="52" t="s">
+      <c r="A46" s="53" t="s">
         <v>174</v>
       </c>
-      <c r="B46" s="48"/>
-      <c r="C46" s="48"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="48"/>
-      <c r="H46" s="49"/>
+      <c r="B46" s="49"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="49"/>
+      <c r="E46" s="49"/>
+      <c r="F46" s="49"/>
+      <c r="G46" s="49"/>
+      <c r="H46" s="50"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -7736,16 +7739,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="50" t="s">
+      <c r="A51" s="51" t="s">
         <v>186</v>
       </c>
-      <c r="B51" s="48"/>
-      <c r="C51" s="48"/>
-      <c r="D51" s="48"/>
-      <c r="E51" s="48"/>
-      <c r="F51" s="48"/>
-      <c r="G51" s="48"/>
-      <c r="H51" s="49"/>
+      <c r="B51" s="49"/>
+      <c r="C51" s="49"/>
+      <c r="D51" s="49"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="49"/>
+      <c r="G51" s="49"/>
+      <c r="H51" s="50"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -9406,10 +9409,10 @@
         <v>1170</v>
       </c>
       <c r="C167" s="27" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D167" s="27" t="s">
         <v>1171</v>
-      </c>
-      <c r="D167" s="27" t="s">
-        <v>1172</v>
       </c>
       <c r="E167" s="40" t="s">
         <v>1152</v>
@@ -9423,13 +9426,13 @@
         <v>9</v>
       </c>
       <c r="B168" s="27" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C168" s="27" t="s">
         <v>1173</v>
       </c>
-      <c r="C168" s="27" t="s">
+      <c r="D168" s="27" t="s">
         <v>1174</v>
-      </c>
-      <c r="D168" s="27" t="s">
-        <v>1175</v>
       </c>
       <c r="E168" s="40" t="s">
         <v>1152</v>
@@ -9465,24 +9468,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="55" t="s">
         <v>222</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="50"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -9570,14 +9573,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="51" t="s">
         <v>242</v>
       </c>
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="49"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="50"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -9665,14 +9668,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="48" t="s">
         <v>256</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="49"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="50"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -9794,14 +9797,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="47" t="s">
+      <c r="A26" s="48" t="s">
         <v>280</v>
       </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="49"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="50"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -9947,10 +9950,10 @@
         <v>1145</v>
       </c>
       <c r="C35" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D35" t="s">
         <v>1176</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1177</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -9982,26 +9985,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>289</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="51" t="s">
         <v>290</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="50"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -10375,16 +10378,16 @@
         <v>1141</v>
       </c>
       <c r="D21" s="41" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="E21" s="41" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F21" s="27" t="s">
-        <v>6</v>
+        <v>1177</v>
+      </c>
+      <c r="F21" s="38" t="s">
+        <v>1220</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>1179</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -10392,18 +10395,18 @@
         <v>1014</v>
       </c>
       <c r="B22" s="41" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="D22" s="41"/>
       <c r="E22" s="41"/>
-      <c r="F22" s="55" t="s">
+      <c r="F22" s="43" t="s">
         <v>1138</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
     </row>
   </sheetData>
@@ -10427,24 +10430,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>347</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="48" t="s">
         <v>348</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="50"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -10629,14 +10632,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="55" t="s">
         <v>380</v>
       </c>
-      <c r="B18" s="48"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="49"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="50"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -10743,14 +10746,14 @@
       <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="51" t="s">
         <v>393</v>
       </c>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="49"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="50"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -10900,7 +10903,7 @@
         <v>1130</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="D39" s="41" t="s">
         <v>1131</v>
@@ -10925,10 +10928,10 @@
         <v>1140</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="D41" s="27" t="s">
         <v>6</v>
@@ -10936,16 +10939,16 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="41" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B42" s="41" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C42" s="41" t="s">
         <v>1185</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="D42" s="43" t="s">
         <v>1186</v>
-      </c>
-      <c r="C42" s="41" t="s">
-        <v>1187</v>
-      </c>
-      <c r="D42" s="55" t="s">
-        <v>1188</v>
       </c>
     </row>
   </sheetData>
@@ -10972,14 +10975,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>405</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11156,14 +11159,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>428</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11766,13 +11769,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>504</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -12169,13 +12172,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>583</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
docs: chiusura Fase 3 - sicurezza repository, rotazione JWT, tracker
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A04D2F8-C169-479E-8AD3-16D0650D18FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849C9D46-754E-44C7-BD15-BDD35A506DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="1223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2211" uniqueCount="1252">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3460,9 +3460,6 @@
     <t>Prenotazioni simultanee: operazione atomica + unique index a DB sullo slot tavolo (denorm A2) + 23505 a 409 + test concorrenza</t>
   </si>
   <si>
-    <t>Aggiornato: 02/09/2026</t>
-  </si>
-  <si>
     <t>70 test unitari</t>
   </si>
   <si>
@@ -3475,9 +3472,6 @@
     <t>Unique index UX_PrenotazionePostazione_Slot + transazioni (Fase 3)</t>
   </si>
   <si>
-    <t>Aggiornato: 02/09/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
     <t>FASE 3 ROADMAP REVISIONE - Prenotazioni simultanee (sessione 02/09/2026)</t>
   </si>
   <si>
@@ -3694,13 +3688,106 @@
     <t>Moq</t>
   </si>
   <si>
-    <t>In corso</t>
-  </si>
-  <si>
-    <t>02/09/2026: codice, migration in produzione e test di concorrenza (201+409) completati. NON ancora chiusa formalmente: mancano commit/push (DoD punto 5) e la pulizia dei dati di test in produzione (zona Test concorrenza, tavolo, prenotazioni di prova). Chiusi anche REV-026 completo e REV-032 parziale.</t>
-  </si>
-  <si>
     <t>Due POST crea-prenotazione realmente simultanee (due SendAsync su HttpClient senza attesa reciproca) su una zona di test con un solo tavolo da 2: HTTP 201 + HTTP 409 'Il tavolo e' stato appena assegnato a un'altra prenotazione'. Il controllo applicativo aveva visto il tavolo libero per entrambe: a fermare la seconda e' stato l'unique index. Restano commit/push e pulizia dei dati di test in produzione prima della chiusura formale (DoD punto 5).</t>
+  </si>
+  <si>
+    <t>Aggiornato: 03/09/2026</t>
+  </si>
+  <si>
+    <t>Aggiornato: 03/09/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
+  </si>
+  <si>
+    <t>FASE 3 ROADMAP REVISIONE - Chiusura formale, sicurezza repository e credenziali (sessione 03/09/2026)</t>
+  </si>
+  <si>
+    <t>Storia Git ripulita dai backup</t>
+  </si>
+  <si>
+    <t>I tre file backup_Prenotazioni_20260902.csv, backup_PrenotazioniPostazioni_20260902.csv e backup_20260902_pre_slot.dump erano nel commit 15f98a0, gia' pushato su dev e main di un repository PUBBLICO. Storia riscritta con git-filter-repo (--invert-paths sui 3 path, 80 commit riparsati) e force push su dev (a07fda0) e main (b09e583). Verificato: nessun oggetto backup_ in git rev-list --objects --all, raw.githubusercontent su main -&gt; 404. Il commit vecchio resta raggiungibile per SHA diretto (oggetto orfano su GitHub) ma i dati sono inventati, quindi nessun ticket a GitHub Support.</t>
+  </si>
+  <si>
+    <t>git-filter-repo + force push</t>
+  </si>
+  <si>
+    <t>03/09/2026</t>
+  </si>
+  <si>
+    <t>Regole .gitignore sui backup</t>
+  </si>
+  <si>
+    <t>Aggiunte backup_*.csv, backup_*.dump e *.dump al .gitignore di root. Erano state messe per errore in GestoraWebApi/.gitignore e con spazi iniziali, che in gitignore fanno parte del pattern e rendevano le regole inefficaci. Verificato con git check-ignore prima del commit.</t>
+  </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <t>Rotazione JwtSettings__Secret</t>
+  </si>
+  <si>
+    <t>Segreto da 64 byte (512 bit) generato con RandomNumberGenerator direttamente negli appunti di Windows (mai stampato a video, mai incollato in chat) e sostituito su Railway. Dopo il redeploy: /health -&gt; Healthy e login dal frontend riuscito. Il token Admin esposto in chat il 02/09 e' invalidato.</t>
+  </si>
+  <si>
+    <t>ASP.NET Core JWT + Railway</t>
+  </si>
+  <si>
+    <t>Dati di test in produzione</t>
+  </si>
+  <si>
+    <t>Zona Test concorrenza, tavolo da 2 e prenotazione del 09/09 lasciati in produzione: la produzione resta l'ambiente di test fino a fine progetto. Rimandata una pulizia generale del database (NEW-005). Nota emersa: l'hook useDeletePrenotazione esiste nel frontend ma non e' collegato a nessun pulsante, quindi l'eliminazione passa solo da Postman (NEW-004).</t>
+  </si>
+  <si>
+    <t>Decisione di processo</t>
+  </si>
+  <si>
+    <t>Fase 3 chiusa</t>
+  </si>
+  <si>
+    <t>Codice, migration in produzione, test di concorrenza (201 + 409) e 70/70 test erano gia' completi il 02/09. Con il commit e push del lavoro residuo e la storia ripulita la Fase 3 e' chiusa formalmente (DoD punto 5). Prossimo passo: Fase 4 - sicurezza e primo avvio.</t>
+  </si>
+  <si>
+    <t>Un file rimosso da un commit resta nella storia: per toglierlo da un repository pubblico serve riscrivere la storia con git-filter-repo e fare force push</t>
+  </si>
+  <si>
+    <t>Cancellare il file e committare lo toglie dal tree corrente ma non dalla cronologia: resta scaricabile da chiunque conosca lo SHA del vecchio commit. Dopo il force push gli oggetti orfani restano comunque sui server GitHub finche' non fanno garbage collection: con dati realmente sensibili va aperto anche un ticket a GitHub Support per la purga.</t>
+  </si>
+  <si>
+    <t>La produzione resta l'ambiente di test fino a fine progetto: nessuna pulizia mirata dei dati di prova</t>
+  </si>
+  <si>
+    <t>Cancellare zona, tavolo e prenotazioni di test a ogni giro significherebbe ricrearli al giro dopo. Si accumulano e si fa una pulizia generale del database di produzione a fine progetto (NEW-005). Attenzione: le zone di test attive compaiono nelle disponibilita' reali - se danno fastidio vanno disattivate, non eliminate.</t>
+  </si>
+  <si>
+    <t>03-set-26</t>
+  </si>
+  <si>
+    <t>FASE 3 CHIUSA 03/09/2026. Codice, migration in produzione e test di concorrenza (201 + 409) completati il 02/09; chiusura formale il 03/09 con commit e push, storia Git ripulita dai backup con dati (git-filter-repo + force push su dev e main) e rotazione di JwtSettings__Secret. Chiusi anche REV-026 completo e REV-032 parziale. Dati di test lasciati in produzione per scelta (NEW-005).</t>
+  </si>
+  <si>
+    <t>Sicurezza - repository</t>
+  </si>
+  <si>
+    <t>Backup con dati delle prenotazioni in un repository pubblico (risolto)</t>
+  </si>
+  <si>
+    <t>I tre backup del 02/09 erano finiti nel commit 15f98a0, gia' pushato su dev e main di un repository pubblico. Storia riscritta con git-filter-repo e force push su entrambi i branch; regole .gitignore aggiunte per impedire che si ripeta. Dati confermati inventati: nessuna richiesta di purga a GitHub Support.</t>
+  </si>
+  <si>
+    <t>NEW-004: hook useDeletePrenotazione mai collegato all'interfaccia</t>
+  </si>
+  <si>
+    <t>usePrenotazioni.ts espone useDeletePrenotazione ma nessun componente lo usa: nel frontend esiste solo Annulla, non Elimina. Stesso schema di NEW-001 (modifica): capacita' backend non raggiungibile dall'app, l'eliminazione passa solo da Postman. Emerso il 03/09 durante la pulizia dei dati di test. Da valutare in Fase 6 insieme a NEW-001, stesso componente.</t>
+  </si>
+  <si>
+    <t>Produzione - Database</t>
+  </si>
+  <si>
+    <t>NEW-005: pulizia generale del database di produzione a fine progetto</t>
+  </si>
+  <si>
+    <t>La produzione e' usata anche come ambiente di test, quindi i dati di prova non vengono cancellati man mano (zona Test concorrenza, tavolo da 2, prenotazione del 09/09 e quanto si accumulera' nei prossimi giri). A fine progetto va fatta una pulizia generale prima della consegna. Ordine vincolante per via di NEW-003/REV-099: prima le prenotazioni, poi le postazioni, poi le zone.</t>
+  </si>
+  <si>
+    <t>Pianificato (fine progetto)</t>
   </si>
 </sst>
 </file>
@@ -3967,7 +4054,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4107,6 +4194,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4433,7 +4523,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="44" t="s">
-        <v>1142</v>
+        <v>1219</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -4591,10 +4681,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4602,11 +4692,11 @@
         <v>33</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -4634,13 +4724,13 @@
       <c r="B15" s="34"/>
       <c r="C15" s="33"/>
       <c r="D15" s="35" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="37" t="s">
         <v>1145</v>
-      </c>
-      <c r="E15" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>1146</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -6279,16 +6369,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C33" t="s">
         <v>1188</v>
       </c>
-      <c r="B33" t="s">
+      <c r="D33" t="s">
         <v>1189</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1190</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1191</v>
       </c>
       <c r="E33" s="27" t="s">
         <v>6</v>
@@ -6296,16 +6386,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="B34" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="C34" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="D34" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -6313,16 +6403,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="B35" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="C35" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="D35" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -6330,16 +6420,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="B36" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="C36" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="D36" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -6347,13 +6437,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="B37" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="C37" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="D37" t="s">
         <v>1075</v>
@@ -6364,13 +6454,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="B38" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C38" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="D38" t="s">
         <v>1075</v>
@@ -6384,13 +6474,13 @@
         <v>777</v>
       </c>
       <c r="B39" t="s">
+        <v>1200</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D39" t="s">
         <v>1202</v>
-      </c>
-      <c r="C39" t="s">
-        <v>1203</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1204</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -6401,13 +6491,13 @@
         <v>777</v>
       </c>
       <c r="B40" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="C40" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="D40" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -6418,13 +6508,13 @@
         <v>777</v>
       </c>
       <c r="B41" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1206</v>
+      </c>
+      <c r="D41" t="s">
         <v>1207</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1208</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1209</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -6435,13 +6525,13 @@
         <v>777</v>
       </c>
       <c r="B42" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="C42" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="D42" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="E42" s="27" t="s">
         <v>6</v>
@@ -6452,13 +6542,13 @@
         <v>777</v>
       </c>
       <c r="B43" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
       <c r="C43" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="D43" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>6</v>
@@ -6469,13 +6559,13 @@
         <v>777</v>
       </c>
       <c r="B44" t="s">
+        <v>1212</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1213</v>
+      </c>
+      <c r="D44" t="s">
         <v>1214</v>
-      </c>
-      <c r="C44" t="s">
-        <v>1215</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1216</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>6</v>
@@ -6486,13 +6576,13 @@
         <v>777</v>
       </c>
       <c r="B45" t="s">
+        <v>1215</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1216</v>
+      </c>
+      <c r="D45" t="s">
         <v>1217</v>
-      </c>
-      <c r="C45" t="s">
-        <v>1218</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1219</v>
       </c>
       <c r="E45" s="27" t="s">
         <v>6</v>
@@ -6875,7 +6965,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:H178"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -6900,7 +6990,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="44" t="s">
-        <v>1147</v>
+        <v>1220</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -7959,83 +8049,65 @@
         <v>908</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
+    <row r="71" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="56" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B71" s="25" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C71" s="25" t="s">
+        <v>1238</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="56" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B72" s="25" t="s">
+        <v>1239</v>
+      </c>
+      <c r="C72" s="25" t="s">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
         <v>861</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
         <v>40</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B75" t="s">
         <v>41</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C75" t="s">
         <v>862</v>
       </c>
-      <c r="D73" t="s">
+      <c r="D75" t="s">
         <v>43</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E75" t="s">
         <v>44</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F75" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74">
-        <v>1</v>
-      </c>
-      <c r="B74" t="s">
-        <v>863</v>
-      </c>
-      <c r="C74" t="s">
-        <v>864</v>
-      </c>
-      <c r="D74" t="s">
-        <v>865</v>
-      </c>
-      <c r="E74" s="28" t="s">
-        <v>875</v>
-      </c>
-      <c r="F74" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75">
-        <v>2</v>
-      </c>
-      <c r="B75" t="s">
-        <v>866</v>
-      </c>
-      <c r="C75" t="s">
-        <v>867</v>
-      </c>
-      <c r="D75" t="s">
-        <v>868</v>
-      </c>
-      <c r="E75" s="28" t="s">
-        <v>875</v>
-      </c>
-      <c r="F75" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B76" t="s">
-        <v>869</v>
+        <v>863</v>
       </c>
       <c r="C76" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
       <c r="D76" t="s">
-        <v>871</v>
+        <v>865</v>
       </c>
       <c r="E76" s="28" t="s">
         <v>875</v>
@@ -8046,16 +8118,16 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B77" t="s">
-        <v>872</v>
+        <v>866</v>
       </c>
       <c r="C77" t="s">
-        <v>873</v>
+        <v>867</v>
       </c>
       <c r="D77" t="s">
-        <v>874</v>
+        <v>868</v>
       </c>
       <c r="E77" s="28" t="s">
         <v>875</v>
@@ -8064,68 +8136,68 @@
         <v>6</v>
       </c>
     </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>3</v>
+      </c>
+      <c r="B78" t="s">
+        <v>869</v>
+      </c>
+      <c r="C78" t="s">
+        <v>870</v>
+      </c>
+      <c r="D78" t="s">
+        <v>871</v>
+      </c>
+      <c r="E78" s="28" t="s">
+        <v>875</v>
+      </c>
+      <c r="F78" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
+      <c r="A79">
+        <v>4</v>
+      </c>
+      <c r="B79" t="s">
+        <v>872</v>
+      </c>
+      <c r="C79" t="s">
+        <v>873</v>
+      </c>
+      <c r="D79" t="s">
+        <v>874</v>
+      </c>
+      <c r="E79" s="28" t="s">
+        <v>875</v>
+      </c>
+      <c r="F79" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
         <v>876</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
         <v>877</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81">
-        <v>1</v>
-      </c>
-      <c r="B81" t="s">
-        <v>878</v>
-      </c>
-      <c r="C81" t="s">
-        <v>879</v>
-      </c>
-      <c r="D81" t="s">
-        <v>880</v>
-      </c>
-      <c r="E81" t="s">
-        <v>881</v>
-      </c>
-      <c r="F81" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82">
-        <v>2</v>
-      </c>
-      <c r="B82" t="s">
-        <v>882</v>
-      </c>
-      <c r="C82" t="s">
-        <v>883</v>
-      </c>
-      <c r="D82" t="s">
-        <v>69</v>
-      </c>
-      <c r="E82" t="s">
-        <v>881</v>
-      </c>
-      <c r="F82" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B83" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="C83" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="D83" t="s">
-        <v>82</v>
+        <v>880</v>
       </c>
       <c r="E83" t="s">
         <v>881</v>
@@ -8136,16 +8208,16 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B84" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="C84" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="D84" t="s">
-        <v>887</v>
+        <v>69</v>
       </c>
       <c r="E84" t="s">
         <v>881</v>
@@ -8154,58 +8226,58 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89">
-        <v>6</v>
-      </c>
-      <c r="B89" t="s">
-        <v>888</v>
-      </c>
-      <c r="C89" t="s">
-        <v>889</v>
-      </c>
-      <c r="D89" t="s">
-        <v>890</v>
-      </c>
-      <c r="E89" t="s">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>3</v>
+      </c>
+      <c r="B85" t="s">
+        <v>882</v>
+      </c>
+      <c r="C85" t="s">
+        <v>884</v>
+      </c>
+      <c r="D85" t="s">
+        <v>82</v>
+      </c>
+      <c r="E85" t="s">
         <v>881</v>
       </c>
-      <c r="F89" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90">
-        <v>7</v>
-      </c>
-      <c r="B90" t="s">
-        <v>891</v>
-      </c>
-      <c r="C90" t="s">
-        <v>892</v>
-      </c>
-      <c r="D90" t="s">
-        <v>893</v>
-      </c>
-      <c r="E90" t="s">
+      <c r="F85" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>5</v>
+      </c>
+      <c r="B86" t="s">
+        <v>885</v>
+      </c>
+      <c r="C86" t="s">
+        <v>886</v>
+      </c>
+      <c r="D86" t="s">
+        <v>887</v>
+      </c>
+      <c r="E86" t="s">
         <v>881</v>
       </c>
-      <c r="F90" s="27" t="s">
+      <c r="F86" s="27" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B91" t="s">
-        <v>894</v>
+        <v>888</v>
       </c>
       <c r="C91" t="s">
-        <v>895</v>
+        <v>889</v>
       </c>
       <c r="D91" t="s">
-        <v>896</v>
+        <v>890</v>
       </c>
       <c r="E91" t="s">
         <v>881</v>
@@ -8214,85 +8286,85 @@
         <v>6</v>
       </c>
     </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>7</v>
+      </c>
+      <c r="B92" t="s">
+        <v>891</v>
+      </c>
+      <c r="C92" t="s">
+        <v>892</v>
+      </c>
+      <c r="D92" t="s">
+        <v>893</v>
+      </c>
+      <c r="E92" t="s">
+        <v>881</v>
+      </c>
+      <c r="F92" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
+      <c r="A93">
+        <v>8</v>
+      </c>
+      <c r="B93" t="s">
+        <v>894</v>
+      </c>
+      <c r="C93" t="s">
+        <v>895</v>
+      </c>
+      <c r="D93" t="s">
+        <v>896</v>
+      </c>
+      <c r="E93" t="s">
+        <v>881</v>
+      </c>
+      <c r="F93" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
         <v>909</v>
       </c>
-      <c r="E93" s="28"/>
-      <c r="F93" s="27"/>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
+      <c r="E95" s="28"/>
+      <c r="F95" s="27"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
         <v>40</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B96" t="s">
         <v>41</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C96" t="s">
         <v>862</v>
       </c>
-      <c r="D94" t="s">
+      <c r="D96" t="s">
         <v>43</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E96" t="s">
         <v>44</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F96" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95">
-        <v>1</v>
-      </c>
-      <c r="B95" t="s">
-        <v>910</v>
-      </c>
-      <c r="C95" t="s">
-        <v>911</v>
-      </c>
-      <c r="D95" t="s">
-        <v>912</v>
-      </c>
-      <c r="E95" t="s">
-        <v>904</v>
-      </c>
-      <c r="F95" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96">
-        <v>2</v>
-      </c>
-      <c r="B96" t="s">
-        <v>913</v>
-      </c>
-      <c r="C96" t="s">
-        <v>914</v>
-      </c>
-      <c r="D96" t="s">
-        <v>915</v>
-      </c>
-      <c r="E96" t="s">
-        <v>904</v>
-      </c>
-      <c r="F96" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B97" t="s">
-        <v>916</v>
+        <v>910</v>
       </c>
       <c r="C97" t="s">
-        <v>917</v>
+        <v>911</v>
       </c>
       <c r="D97" t="s">
-        <v>918</v>
+        <v>912</v>
       </c>
       <c r="E97" t="s">
         <v>904</v>
@@ -8303,16 +8375,16 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B98" t="s">
-        <v>919</v>
+        <v>913</v>
       </c>
       <c r="C98" t="s">
-        <v>920</v>
+        <v>914</v>
       </c>
       <c r="D98" t="s">
-        <v>921</v>
+        <v>915</v>
       </c>
       <c r="E98" t="s">
         <v>904</v>
@@ -8323,16 +8395,16 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B99" t="s">
-        <v>922</v>
+        <v>916</v>
       </c>
       <c r="C99" t="s">
-        <v>923</v>
+        <v>917</v>
       </c>
       <c r="D99" t="s">
-        <v>924</v>
+        <v>918</v>
       </c>
       <c r="E99" t="s">
         <v>904</v>
@@ -8343,16 +8415,16 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B100" t="s">
-        <v>925</v>
+        <v>919</v>
       </c>
       <c r="C100" t="s">
-        <v>926</v>
+        <v>920</v>
       </c>
       <c r="D100" t="s">
-        <v>927</v>
+        <v>921</v>
       </c>
       <c r="E100" t="s">
         <v>904</v>
@@ -8361,83 +8433,83 @@
         <v>6</v>
       </c>
     </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101">
+        <v>5</v>
+      </c>
+      <c r="B101" t="s">
+        <v>922</v>
+      </c>
+      <c r="C101" t="s">
+        <v>923</v>
+      </c>
+      <c r="D101" t="s">
+        <v>924</v>
+      </c>
+      <c r="E101" t="s">
+        <v>904</v>
+      </c>
+      <c r="F101" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="32" t="s">
+      <c r="A102">
+        <v>6</v>
+      </c>
+      <c r="B102" t="s">
+        <v>925</v>
+      </c>
+      <c r="C102" t="s">
+        <v>926</v>
+      </c>
+      <c r="D102" t="s">
+        <v>927</v>
+      </c>
+      <c r="E102" t="s">
+        <v>904</v>
+      </c>
+      <c r="F102" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="32" t="s">
         <v>936</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
         <v>40</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B105" t="s">
         <v>41</v>
       </c>
-      <c r="C103" t="s">
+      <c r="C105" t="s">
         <v>862</v>
       </c>
-      <c r="D103" t="s">
+      <c r="D105" t="s">
         <v>43</v>
       </c>
-      <c r="E103" t="s">
+      <c r="E105" t="s">
         <v>44</v>
       </c>
-      <c r="F103" t="s">
+      <c r="F105" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104">
-        <v>1</v>
-      </c>
-      <c r="B104" t="s">
-        <v>937</v>
-      </c>
-      <c r="C104" t="s">
-        <v>938</v>
-      </c>
-      <c r="D104" t="s">
-        <v>939</v>
-      </c>
-      <c r="E104" t="s">
-        <v>940</v>
-      </c>
-      <c r="F104" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105">
-        <v>2</v>
-      </c>
-      <c r="B105" t="s">
-        <v>941</v>
-      </c>
-      <c r="C105" t="s">
-        <v>942</v>
-      </c>
-      <c r="D105" t="s">
-        <v>943</v>
-      </c>
-      <c r="E105" t="s">
-        <v>940</v>
-      </c>
-      <c r="F105" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B106" t="s">
-        <v>944</v>
+        <v>937</v>
       </c>
       <c r="C106" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="D106" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="E106" t="s">
         <v>940</v>
@@ -8448,13 +8520,13 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B107" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="C107" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="D107" t="s">
         <v>943</v>
@@ -8468,16 +8540,16 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B108" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
       <c r="C108" t="s">
-        <v>949</v>
+        <v>945</v>
       </c>
       <c r="D108" t="s">
-        <v>950</v>
+        <v>943</v>
       </c>
       <c r="E108" t="s">
         <v>940</v>
@@ -8486,83 +8558,83 @@
         <v>6</v>
       </c>
     </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109">
+        <v>4</v>
+      </c>
+      <c r="B109" t="s">
+        <v>946</v>
+      </c>
+      <c r="C109" t="s">
+        <v>947</v>
+      </c>
+      <c r="D109" t="s">
+        <v>943</v>
+      </c>
+      <c r="E109" t="s">
+        <v>940</v>
+      </c>
+      <c r="F109" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" t="s">
+      <c r="A110">
+        <v>5</v>
+      </c>
+      <c r="B110" t="s">
+        <v>948</v>
+      </c>
+      <c r="C110" t="s">
+        <v>949</v>
+      </c>
+      <c r="D110" t="s">
+        <v>950</v>
+      </c>
+      <c r="E110" t="s">
+        <v>940</v>
+      </c>
+      <c r="F110" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
         <v>953</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" t="s">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
         <v>40</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B113" t="s">
         <v>41</v>
       </c>
-      <c r="C111" t="s">
+      <c r="C113" t="s">
         <v>862</v>
       </c>
-      <c r="D111" t="s">
+      <c r="D113" t="s">
         <v>43</v>
       </c>
-      <c r="E111" t="s">
+      <c r="E113" t="s">
         <v>44</v>
       </c>
-      <c r="F111" t="s">
+      <c r="F113" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112">
-        <v>1</v>
-      </c>
-      <c r="B112" t="s">
-        <v>954</v>
-      </c>
-      <c r="C112" t="s">
-        <v>955</v>
-      </c>
-      <c r="D112" t="s">
-        <v>956</v>
-      </c>
-      <c r="E112" t="s">
-        <v>957</v>
-      </c>
-      <c r="F112" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113">
-        <v>2</v>
-      </c>
-      <c r="B113" t="s">
-        <v>958</v>
-      </c>
-      <c r="C113" t="s">
-        <v>959</v>
-      </c>
-      <c r="D113" t="s">
-        <v>960</v>
-      </c>
-      <c r="E113" t="s">
-        <v>957</v>
-      </c>
-      <c r="F113" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B114" t="s">
-        <v>961</v>
+        <v>954</v>
       </c>
       <c r="C114" t="s">
-        <v>962</v>
+        <v>955</v>
       </c>
       <c r="D114" t="s">
-        <v>963</v>
+        <v>956</v>
       </c>
       <c r="E114" t="s">
         <v>957</v>
@@ -8573,16 +8645,16 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B115" t="s">
-        <v>964</v>
+        <v>958</v>
       </c>
       <c r="C115" t="s">
-        <v>965</v>
+        <v>959</v>
       </c>
       <c r="D115" t="s">
-        <v>966</v>
+        <v>960</v>
       </c>
       <c r="E115" t="s">
         <v>957</v>
@@ -8593,101 +8665,101 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116">
+        <v>3</v>
+      </c>
+      <c r="B116" t="s">
+        <v>961</v>
+      </c>
+      <c r="C116" t="s">
+        <v>962</v>
+      </c>
+      <c r="D116" t="s">
+        <v>963</v>
+      </c>
+      <c r="E116" t="s">
+        <v>957</v>
+      </c>
+      <c r="F116" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>4</v>
+      </c>
+      <c r="B117" t="s">
+        <v>964</v>
+      </c>
+      <c r="C117" t="s">
+        <v>965</v>
+      </c>
+      <c r="D117" t="s">
+        <v>966</v>
+      </c>
+      <c r="E117" t="s">
+        <v>957</v>
+      </c>
+      <c r="F117" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118">
         <v>5</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B118" t="s">
         <v>967</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C118" t="s">
         <v>968</v>
       </c>
-      <c r="D116" t="s">
+      <c r="D118" t="s">
         <v>969</v>
       </c>
-      <c r="E116" t="s">
+      <c r="E118" t="s">
         <v>970</v>
       </c>
-      <c r="F116" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
+      <c r="F118" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
         <v>971</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
         <v>40</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B121" t="s">
         <v>41</v>
       </c>
-      <c r="C119" t="s">
+      <c r="C121" t="s">
         <v>862</v>
       </c>
-      <c r="D119" t="s">
+      <c r="D121" t="s">
         <v>43</v>
       </c>
-      <c r="E119" t="s">
+      <c r="E121" t="s">
         <v>44</v>
       </c>
-      <c r="F119" t="s">
+      <c r="F121" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120">
-        <v>1</v>
-      </c>
-      <c r="B120" t="s">
-        <v>972</v>
-      </c>
-      <c r="C120" t="s">
-        <v>973</v>
-      </c>
-      <c r="D120" t="s">
-        <v>974</v>
-      </c>
-      <c r="E120" t="s">
-        <v>970</v>
-      </c>
-      <c r="F120" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121">
-        <v>2</v>
-      </c>
-      <c r="B121" t="s">
-        <v>975</v>
-      </c>
-      <c r="C121" t="s">
-        <v>976</v>
-      </c>
-      <c r="D121" t="s">
-        <v>921</v>
-      </c>
-      <c r="E121" t="s">
-        <v>970</v>
-      </c>
-      <c r="F121" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B122" t="s">
-        <v>977</v>
+        <v>972</v>
       </c>
       <c r="C122" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="D122" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
       <c r="E122" t="s">
         <v>970</v>
@@ -8698,16 +8770,16 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B123" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="C123" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="D123" t="s">
-        <v>982</v>
+        <v>921</v>
       </c>
       <c r="E123" t="s">
         <v>970</v>
@@ -8718,101 +8790,101 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124">
+        <v>3</v>
+      </c>
+      <c r="B124" t="s">
+        <v>977</v>
+      </c>
+      <c r="C124" t="s">
+        <v>978</v>
+      </c>
+      <c r="D124" t="s">
+        <v>979</v>
+      </c>
+      <c r="E124" t="s">
+        <v>970</v>
+      </c>
+      <c r="F124" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A125">
+        <v>4</v>
+      </c>
+      <c r="B125" t="s">
+        <v>980</v>
+      </c>
+      <c r="C125" t="s">
+        <v>981</v>
+      </c>
+      <c r="D125" t="s">
+        <v>982</v>
+      </c>
+      <c r="E125" t="s">
+        <v>970</v>
+      </c>
+      <c r="F125" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126">
         <v>5</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B126" t="s">
         <v>983</v>
       </c>
-      <c r="C124" t="s">
+      <c r="C126" t="s">
         <v>984</v>
       </c>
-      <c r="D124" t="s">
+      <c r="D126" t="s">
         <v>438</v>
       </c>
-      <c r="E124" t="s">
+      <c r="E126" t="s">
         <v>438</v>
       </c>
-      <c r="F124" s="38" t="s">
+      <c r="F126" s="38" t="s">
         <v>985</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
         <v>996</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
         <v>40</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B129" t="s">
         <v>41</v>
       </c>
-      <c r="C127" t="s">
+      <c r="C129" t="s">
         <v>862</v>
       </c>
-      <c r="D127" t="s">
+      <c r="D129" t="s">
         <v>43</v>
       </c>
-      <c r="E127" t="s">
+      <c r="E129" t="s">
         <v>44</v>
       </c>
-      <c r="F127" t="s">
+      <c r="F129" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128">
-        <v>1</v>
-      </c>
-      <c r="B128" t="s">
-        <v>997</v>
-      </c>
-      <c r="C128" t="s">
-        <v>998</v>
-      </c>
-      <c r="D128" t="s">
-        <v>438</v>
-      </c>
-      <c r="E128" t="s">
-        <v>999</v>
-      </c>
-      <c r="F128" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129">
-        <v>2</v>
-      </c>
-      <c r="B129" t="s">
-        <v>1000</v>
-      </c>
-      <c r="C129" t="s">
-        <v>1001</v>
-      </c>
-      <c r="D129" t="s">
-        <v>1002</v>
-      </c>
-      <c r="E129" t="s">
-        <v>999</v>
-      </c>
-      <c r="F129" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B130" t="s">
-        <v>1003</v>
+        <v>997</v>
       </c>
       <c r="C130" t="s">
-        <v>1004</v>
+        <v>998</v>
       </c>
       <c r="D130" t="s">
-        <v>1005</v>
+        <v>438</v>
       </c>
       <c r="E130" t="s">
         <v>999</v>
@@ -8823,16 +8895,16 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B131" t="s">
-        <v>1006</v>
+        <v>1000</v>
       </c>
       <c r="C131" t="s">
-        <v>1007</v>
+        <v>1001</v>
       </c>
       <c r="D131" t="s">
-        <v>1008</v>
+        <v>1002</v>
       </c>
       <c r="E131" t="s">
         <v>999</v>
@@ -8843,16 +8915,16 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B132" t="s">
-        <v>1009</v>
+        <v>1003</v>
       </c>
       <c r="C132" t="s">
-        <v>1010</v>
+        <v>1004</v>
       </c>
       <c r="D132" t="s">
-        <v>438</v>
+        <v>1005</v>
       </c>
       <c r="E132" t="s">
         <v>999</v>
@@ -8861,83 +8933,83 @@
         <v>6</v>
       </c>
     </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A133">
+        <v>4</v>
+      </c>
+      <c r="B133" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C133" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D133" t="s">
+        <v>1008</v>
+      </c>
+      <c r="E133" t="s">
+        <v>999</v>
+      </c>
+      <c r="F133" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" t="s">
+      <c r="A134">
+        <v>5</v>
+      </c>
+      <c r="B134" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C134" t="s">
+        <v>1010</v>
+      </c>
+      <c r="D134" t="s">
+        <v>438</v>
+      </c>
+      <c r="E134" t="s">
+        <v>999</v>
+      </c>
+      <c r="F134" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
         <v>1017</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" t="s">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
         <v>40</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B137" t="s">
         <v>41</v>
       </c>
-      <c r="C135" t="s">
+      <c r="C137" t="s">
         <v>862</v>
       </c>
-      <c r="D135" t="s">
+      <c r="D137" t="s">
         <v>43</v>
       </c>
-      <c r="E135" t="s">
+      <c r="E137" t="s">
         <v>44</v>
       </c>
-      <c r="F135" t="s">
+      <c r="F137" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136">
-        <v>1</v>
-      </c>
-      <c r="B136" t="s">
-        <v>1018</v>
-      </c>
-      <c r="C136" t="s">
-        <v>1019</v>
-      </c>
-      <c r="D136" t="s">
-        <v>1020</v>
-      </c>
-      <c r="E136" t="s">
-        <v>999</v>
-      </c>
-      <c r="F136" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137">
-        <v>2</v>
-      </c>
-      <c r="B137" t="s">
-        <v>1021</v>
-      </c>
-      <c r="C137" t="s">
-        <v>1022</v>
-      </c>
-      <c r="D137" t="s">
-        <v>1023</v>
-      </c>
-      <c r="E137" t="s">
-        <v>999</v>
-      </c>
-      <c r="F137" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B138" t="s">
-        <v>961</v>
+        <v>1018</v>
       </c>
       <c r="C138" t="s">
-        <v>1024</v>
+        <v>1019</v>
       </c>
       <c r="D138" t="s">
-        <v>1025</v>
+        <v>1020</v>
       </c>
       <c r="E138" t="s">
         <v>999</v>
@@ -8946,83 +9018,83 @@
         <v>6</v>
       </c>
     </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A139">
+        <v>2</v>
+      </c>
+      <c r="B139" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C139" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D139" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E139" t="s">
+        <v>999</v>
+      </c>
+      <c r="F139" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
+      <c r="A140">
+        <v>3</v>
+      </c>
+      <c r="B140" t="s">
+        <v>961</v>
+      </c>
+      <c r="C140" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D140" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E140" t="s">
+        <v>999</v>
+      </c>
+      <c r="F140" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
         <v>1031</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" t="s">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
         <v>40</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B143" t="s">
         <v>41</v>
       </c>
-      <c r="C141" t="s">
+      <c r="C143" t="s">
         <v>862</v>
       </c>
-      <c r="D141" t="s">
+      <c r="D143" t="s">
         <v>43</v>
       </c>
-      <c r="E141" t="s">
+      <c r="E143" t="s">
         <v>44</v>
       </c>
-      <c r="F141" t="s">
+      <c r="F143" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142">
-        <v>1</v>
-      </c>
-      <c r="B142" t="s">
-        <v>1032</v>
-      </c>
-      <c r="C142" t="s">
-        <v>1033</v>
-      </c>
-      <c r="D142" t="s">
-        <v>1034</v>
-      </c>
-      <c r="E142" t="s">
-        <v>999</v>
-      </c>
-      <c r="F142" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143">
-        <v>2</v>
-      </c>
-      <c r="B143" t="s">
-        <v>1035</v>
-      </c>
-      <c r="C143" t="s">
-        <v>1036</v>
-      </c>
-      <c r="D143" t="s">
-        <v>1037</v>
-      </c>
-      <c r="E143" t="s">
-        <v>999</v>
-      </c>
-      <c r="F143" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B144" t="s">
-        <v>1038</v>
+        <v>1032</v>
       </c>
       <c r="C144" t="s">
-        <v>1039</v>
+        <v>1033</v>
       </c>
       <c r="D144" t="s">
-        <v>1040</v>
+        <v>1034</v>
       </c>
       <c r="E144" t="s">
         <v>999</v>
@@ -9033,16 +9105,16 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B145" t="s">
-        <v>1041</v>
+        <v>1035</v>
       </c>
       <c r="C145" t="s">
-        <v>1042</v>
+        <v>1036</v>
       </c>
       <c r="D145" t="s">
-        <v>1043</v>
+        <v>1037</v>
       </c>
       <c r="E145" t="s">
         <v>999</v>
@@ -9053,16 +9125,16 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B146" t="s">
-        <v>1044</v>
+        <v>1038</v>
       </c>
       <c r="C146" t="s">
-        <v>1045</v>
+        <v>1039</v>
       </c>
       <c r="D146" t="s">
-        <v>30</v>
+        <v>1040</v>
       </c>
       <c r="E146" t="s">
         <v>999</v>
@@ -9073,16 +9145,16 @@
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B147" t="s">
-        <v>1046</v>
+        <v>1041</v>
       </c>
       <c r="C147" t="s">
-        <v>1047</v>
+        <v>1042</v>
       </c>
       <c r="D147" t="s">
-        <v>1048</v>
+        <v>1043</v>
       </c>
       <c r="E147" t="s">
         <v>999</v>
@@ -9091,83 +9163,83 @@
         <v>6</v>
       </c>
     </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A148">
+        <v>5</v>
+      </c>
+      <c r="B148" t="s">
+        <v>1044</v>
+      </c>
+      <c r="C148" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D148" t="s">
+        <v>30</v>
+      </c>
+      <c r="E148" t="s">
+        <v>999</v>
+      </c>
+      <c r="F148" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" t="s">
+      <c r="A149">
+        <v>6</v>
+      </c>
+      <c r="B149" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C149" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D149" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E149" t="s">
+        <v>999</v>
+      </c>
+      <c r="F149" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
         <v>1110</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A150" t="s">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
         <v>40</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B152" t="s">
         <v>41</v>
       </c>
-      <c r="C150" t="s">
+      <c r="C152" t="s">
         <v>862</v>
       </c>
-      <c r="D150" t="s">
+      <c r="D152" t="s">
         <v>43</v>
       </c>
-      <c r="E150" t="s">
+      <c r="E152" t="s">
         <v>44</v>
       </c>
-      <c r="F150" t="s">
+      <c r="F152" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A151" s="27">
-        <v>1</v>
-      </c>
-      <c r="B151" s="27" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C151" s="27" t="s">
-        <v>1112</v>
-      </c>
-      <c r="D151" s="27" t="s">
-        <v>1113</v>
-      </c>
-      <c r="E151" s="40" t="s">
-        <v>1127</v>
-      </c>
-      <c r="F151" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A152" s="27">
-        <v>2</v>
-      </c>
-      <c r="B152" s="27" t="s">
-        <v>1114</v>
-      </c>
-      <c r="C152" s="27" t="s">
-        <v>1115</v>
-      </c>
-      <c r="D152" s="27" t="s">
-        <v>1116</v>
-      </c>
-      <c r="E152" s="40" t="s">
-        <v>1127</v>
-      </c>
-      <c r="F152" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B153" s="27" t="s">
-        <v>1117</v>
+        <v>1111</v>
       </c>
       <c r="C153" s="27" t="s">
-        <v>1118</v>
+        <v>1112</v>
       </c>
       <c r="D153" s="27" t="s">
-        <v>1119</v>
+        <v>1113</v>
       </c>
       <c r="E153" s="40" t="s">
         <v>1127</v>
@@ -9178,16 +9250,16 @@
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B154" s="27" t="s">
-        <v>1120</v>
+        <v>1114</v>
       </c>
       <c r="C154" s="27" t="s">
-        <v>1121</v>
+        <v>1115</v>
       </c>
       <c r="D154" s="27" t="s">
-        <v>1122</v>
+        <v>1116</v>
       </c>
       <c r="E154" s="40" t="s">
         <v>1127</v>
@@ -9198,16 +9270,16 @@
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="27">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B155" s="27" t="s">
-        <v>1123</v>
+        <v>1117</v>
       </c>
       <c r="C155" s="27" t="s">
-        <v>1135</v>
+        <v>1118</v>
       </c>
       <c r="D155" s="27" t="s">
-        <v>1124</v>
+        <v>1119</v>
       </c>
       <c r="E155" s="40" t="s">
         <v>1127</v>
@@ -9217,105 +9289,105 @@
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A156" s="41">
-        <v>6</v>
-      </c>
-      <c r="B156" s="41" t="s">
+      <c r="A156" s="27">
+        <v>4</v>
+      </c>
+      <c r="B156" s="27" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C156" s="27" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D156" s="27" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E156" s="40" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F156" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A157" s="27">
+        <v>5</v>
+      </c>
+      <c r="B157" s="27" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C157" s="27" t="s">
+        <v>1135</v>
+      </c>
+      <c r="D157" s="27" t="s">
+        <v>1124</v>
+      </c>
+      <c r="E157" s="40" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F157" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A158" s="41">
+        <v>6</v>
+      </c>
+      <c r="B158" s="41" t="s">
         <v>1136</v>
       </c>
-      <c r="C156" s="41" t="s">
+      <c r="C158" s="41" t="s">
         <v>1137</v>
       </c>
-      <c r="D156" s="41" t="s">
+      <c r="D158" s="41" t="s">
         <v>268</v>
       </c>
-      <c r="E156" s="42" t="s">
+      <c r="E158" s="42" t="s">
         <v>1127</v>
       </c>
-      <c r="F156" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A158" t="s">
-        <v>1148</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A159" t="s">
+      <c r="F158" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
         <v>40</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B161" t="s">
         <v>41</v>
       </c>
-      <c r="C159" t="s">
+      <c r="C161" t="s">
         <v>862</v>
       </c>
-      <c r="D159" t="s">
+      <c r="D161" t="s">
         <v>43</v>
       </c>
-      <c r="E159" t="s">
+      <c r="E161" t="s">
         <v>44</v>
       </c>
-      <c r="F159" t="s">
+      <c r="F161" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A160" s="27">
-        <v>1</v>
-      </c>
-      <c r="B160" s="27" t="s">
-        <v>1149</v>
-      </c>
-      <c r="C160" s="27" t="s">
-        <v>1150</v>
-      </c>
-      <c r="D160" s="27" t="s">
-        <v>1151</v>
-      </c>
-      <c r="E160" s="40" t="s">
-        <v>1152</v>
-      </c>
-      <c r="F160" s="27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A161" s="27">
-        <v>2</v>
-      </c>
-      <c r="B161" s="27" t="s">
-        <v>1153</v>
-      </c>
-      <c r="C161" s="27" t="s">
-        <v>1154</v>
-      </c>
-      <c r="D161" s="27" t="s">
-        <v>1155</v>
-      </c>
-      <c r="E161" s="40" t="s">
-        <v>1152</v>
-      </c>
-      <c r="F161" s="27" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B162" s="27" t="s">
-        <v>1156</v>
+        <v>1147</v>
       </c>
       <c r="C162" s="27" t="s">
-        <v>1157</v>
+        <v>1148</v>
       </c>
       <c r="D162" s="27" t="s">
-        <v>1158</v>
+        <v>1149</v>
       </c>
       <c r="E162" s="40" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="F162" s="27" t="s">
         <v>6</v>
@@ -9323,19 +9395,19 @@
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B163" s="27" t="s">
-        <v>1159</v>
+        <v>1151</v>
       </c>
       <c r="C163" s="27" t="s">
-        <v>1160</v>
+        <v>1152</v>
       </c>
       <c r="D163" s="27" t="s">
-        <v>1161</v>
+        <v>1153</v>
       </c>
       <c r="E163" s="40" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="F163" s="27" t="s">
         <v>6</v>
@@ -9343,19 +9415,19 @@
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="27">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B164" s="27" t="s">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="C164" s="27" t="s">
-        <v>1163</v>
+        <v>1155</v>
       </c>
       <c r="D164" s="27" t="s">
-        <v>1164</v>
+        <v>1156</v>
       </c>
       <c r="E164" s="40" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="F164" s="27" t="s">
         <v>6</v>
@@ -9363,19 +9435,19 @@
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="27">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B165" s="27" t="s">
-        <v>1165</v>
+        <v>1157</v>
       </c>
       <c r="C165" s="27" t="s">
-        <v>1166</v>
+        <v>1158</v>
       </c>
       <c r="D165" s="27" t="s">
-        <v>1167</v>
+        <v>1159</v>
       </c>
       <c r="E165" s="40" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="F165" s="27" t="s">
         <v>6</v>
@@ -9383,19 +9455,19 @@
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="27">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B166" s="27" t="s">
-        <v>1168</v>
+        <v>1160</v>
       </c>
       <c r="C166" s="27" t="s">
-        <v>1169</v>
+        <v>1161</v>
       </c>
       <c r="D166" s="27" t="s">
-        <v>1025</v>
+        <v>1162</v>
       </c>
       <c r="E166" s="40" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="F166" s="27" t="s">
         <v>6</v>
@@ -9403,19 +9475,19 @@
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="27">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B167" s="27" t="s">
-        <v>1170</v>
+        <v>1163</v>
       </c>
       <c r="C167" s="27" t="s">
-        <v>1222</v>
+        <v>1164</v>
       </c>
       <c r="D167" s="27" t="s">
-        <v>1171</v>
+        <v>1165</v>
       </c>
       <c r="E167" s="40" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="F167" s="27" t="s">
         <v>6</v>
@@ -9423,21 +9495,186 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="27">
+        <v>7</v>
+      </c>
+      <c r="B168" s="27" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C168" s="27" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D168" s="27" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E168" s="40" t="s">
+        <v>1150</v>
+      </c>
+      <c r="F168" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A169" s="27">
+        <v>8</v>
+      </c>
+      <c r="B169" s="27" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C169" s="27" t="s">
+        <v>1218</v>
+      </c>
+      <c r="D169" s="27" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E169" s="40" t="s">
+        <v>1150</v>
+      </c>
+      <c r="F169" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A170" s="27">
         <v>9</v>
       </c>
-      <c r="B168" s="27" t="s">
+      <c r="B170" s="27" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C170" s="27" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D170" s="27" t="s">
         <v>1172</v>
       </c>
-      <c r="C168" s="27" t="s">
-        <v>1173</v>
-      </c>
-      <c r="D168" s="27" t="s">
-        <v>1174</v>
-      </c>
-      <c r="E168" s="40" t="s">
-        <v>1152</v>
-      </c>
-      <c r="F168" s="27" t="s">
+      <c r="E170" s="40" t="s">
+        <v>1150</v>
+      </c>
+      <c r="F170" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>40</v>
+      </c>
+      <c r="B173" t="s">
+        <v>41</v>
+      </c>
+      <c r="C173" t="s">
+        <v>862</v>
+      </c>
+      <c r="D173" t="s">
+        <v>43</v>
+      </c>
+      <c r="E173" t="s">
+        <v>44</v>
+      </c>
+      <c r="F173" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A174" s="27">
+        <v>1</v>
+      </c>
+      <c r="B174" s="27" t="s">
+        <v>1222</v>
+      </c>
+      <c r="C174" s="27" t="s">
+        <v>1223</v>
+      </c>
+      <c r="D174" s="27" t="s">
+        <v>1224</v>
+      </c>
+      <c r="E174" s="40" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F174" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A175" s="27">
+        <v>2</v>
+      </c>
+      <c r="B175" s="27" t="s">
+        <v>1226</v>
+      </c>
+      <c r="C175" s="27" t="s">
+        <v>1227</v>
+      </c>
+      <c r="D175" s="27" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E175" s="40" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F175" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A176" s="27">
+        <v>3</v>
+      </c>
+      <c r="B176" s="27" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C176" s="27" t="s">
+        <v>1230</v>
+      </c>
+      <c r="D176" s="27" t="s">
+        <v>1231</v>
+      </c>
+      <c r="E176" s="40" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F176" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A177" s="27">
+        <v>4</v>
+      </c>
+      <c r="B177" s="27" t="s">
+        <v>1232</v>
+      </c>
+      <c r="C177" s="27" t="s">
+        <v>1233</v>
+      </c>
+      <c r="D177" s="27" t="s">
+        <v>1234</v>
+      </c>
+      <c r="E177" s="40" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F177" s="43" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A178" s="27">
+        <v>5</v>
+      </c>
+      <c r="B178" s="27" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C178" s="27" t="s">
+        <v>1236</v>
+      </c>
+      <c r="D178" s="27" t="s">
+        <v>438</v>
+      </c>
+      <c r="E178" s="40" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F178" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -9947,13 +10184,13 @@
         <v>1050</v>
       </c>
       <c r="B35" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="C35" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="D35" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -10378,16 +10615,16 @@
         <v>1141</v>
       </c>
       <c r="D21" s="41" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="E21" s="41" t="s">
-        <v>1177</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>1220</v>
+        <v>1241</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>6</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>1221</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -10395,10 +10632,10 @@
         <v>1014</v>
       </c>
       <c r="B22" s="41" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="C22" s="41" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="D22" s="41"/>
       <c r="E22" s="41"/>
@@ -10406,7 +10643,7 @@
         <v>1138</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
     </row>
   </sheetData>
@@ -10420,7 +10657,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -10903,7 +11140,7 @@
         <v>1130</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="D39" s="41" t="s">
         <v>1131</v>
@@ -10928,10 +11165,10 @@
         <v>1140</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="D41" s="27" t="s">
         <v>6</v>
@@ -10939,16 +11176,58 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="41" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B42" s="41" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C42" s="41" t="s">
         <v>1183</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="D42" s="43" t="s">
         <v>1184</v>
       </c>
-      <c r="C42" s="41" t="s">
-        <v>1185</v>
-      </c>
-      <c r="D42" s="43" t="s">
-        <v>1186</v>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="41" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B43" s="41" t="s">
+        <v>1244</v>
+      </c>
+      <c r="C43" s="41" t="s">
+        <v>1245</v>
+      </c>
+      <c r="D43" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="41" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B44" s="41" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C44" s="41" t="s">
+        <v>1247</v>
+      </c>
+      <c r="D44" s="43" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="41" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B45" s="41" t="s">
+        <v>1249</v>
+      </c>
+      <c r="C45" s="41" t="s">
+        <v>1250</v>
+      </c>
+      <c r="D45" s="43" t="s">
+        <v>1251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: chiusura Fase 4 e rilascio v1.0.1 - CLAUDE.md, roadmap e tracker aggiornati
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5709AF6-F77C-418B-AC97-A9C6712096D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A98A4F0-2D9F-4141-86AF-7B3D086734D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2280" uniqueCount="1286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2292" uniqueCount="1293">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -2719,9 +2719,6 @@
     <t>Deploy Backend</t>
   </si>
   <si>
-    <t>Railway — PostgreSQL + .NET, health check /health</t>
-  </si>
-  <si>
     <t>Deploy backend Railway</t>
   </si>
   <si>
@@ -3890,6 +3887,30 @@
   </si>
   <si>
     <t>200 / 409 se l'installazione e' gia' configurata / 400 validazione - REV-007, sostituisce seed-admin</t>
+  </si>
+  <si>
+    <t>RILASCIO v1.0.1</t>
+  </si>
+  <si>
+    <t>Merge dev -&gt; main in fast-forward (main era antenato diretto di dev, nessun conflitto possibile): commit 66e7f5c, tag v1.0.1 pubblicato su GitHub sulla punta di main. Railway e Vercel ridistribuiti sul push. Nessuna migration, quindi nessun backup ne' finestra di manutenzione: deploy di solo codice. Verificato in produzione: /health Healthy, /api/Setup/stato setupCompletato true, POST seed-admin 404. Con questo le Fasi 1-4 sono in produzione. Il merge ha portato anche 094d146 (Fase 3 fix + pulizia), rimasto su dev: solo correzione di accenti in un messaggio, nessun buco funzionale.</t>
+  </si>
+  <si>
+    <t>Git + Railway + Vercel</t>
+  </si>
+  <si>
+    <t>Rilascio</t>
+  </si>
+  <si>
+    <t>v1.0.1</t>
+  </si>
+  <si>
+    <t>Merge dev -&gt; main delle Fasi 1-4 con tag v1.0.1</t>
+  </si>
+  <si>
+    <t>Fast-forward, commit 66e7f5c. Nessuna migration. Verificato in produzione: /health Healthy, /api/Setup/stato setupCompletato true, seed-admin 404. Railway e Vercel ridistribuiti sul push.</t>
+  </si>
+  <si>
+    <t>Railway - PostgreSQL + .NET, health check /health - in produzione v1.0.1 (03/09/2026)</t>
   </si>
 </sst>
 </file>
@@ -4625,7 +4646,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="B2" s="46"/>
       <c r="C2" s="46"/>
@@ -4660,7 +4681,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4696,7 +4717,7 @@
         <v>6</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4750,7 +4771,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4783,10 +4804,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4794,11 +4815,11 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -4818,7 +4839,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>895</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4826,13 +4847,13 @@
       <c r="B15" s="34"/>
       <c r="C15" s="33"/>
       <c r="D15" s="35" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="37" t="s">
         <v>1136</v>
-      </c>
-      <c r="E15" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>1137</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5092,13 +5113,13 @@
     </row>
     <row r="13" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="B13" t="s">
         <v>665</v>
       </c>
       <c r="C13" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="D13" t="s">
         <v>653</v>
@@ -5107,27 +5128,27 @@
         <v>437</v>
       </c>
       <c r="F13" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="B14" t="s">
         <v>651</v>
       </c>
       <c r="C14" t="s">
+        <v>1282</v>
+      </c>
+      <c r="D14" t="s">
         <v>1283</v>
-      </c>
-      <c r="D14" t="s">
-        <v>1284</v>
       </c>
       <c r="E14" t="s">
         <v>654</v>
       </c>
       <c r="F14" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5398,7 +5419,7 @@
         <v>665</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>680</v>
@@ -5407,7 +5428,7 @@
         <v>437</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5578,7 +5599,7 @@
         <v>665</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>680</v>
@@ -5587,7 +5608,7 @@
         <v>437</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5681,13 +5702,13 @@
         <v>729</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>687</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5738,7 +5759,7 @@
         <v>665</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>837</v>
@@ -5747,7 +5768,7 @@
         <v>437</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5912,42 +5933,42 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B54" t="s">
         <v>665</v>
       </c>
       <c r="C54" t="s">
+        <v>923</v>
+      </c>
+      <c r="D54" t="s">
         <v>924</v>
-      </c>
-      <c r="D54" t="s">
-        <v>925</v>
       </c>
       <c r="E54" t="s">
         <v>437</v>
       </c>
       <c r="F54" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B55" t="s">
         <v>651</v>
       </c>
       <c r="C55" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="D55" t="s">
         <v>660</v>
       </c>
       <c r="E55" t="s">
+        <v>984</v>
+      </c>
+      <c r="F55" t="s">
         <v>985</v>
-      </c>
-      <c r="F55" t="s">
-        <v>986</v>
       </c>
     </row>
   </sheetData>
@@ -5972,7 +5993,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="55" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -6239,13 +6260,13 @@
         <v>794</v>
       </c>
       <c r="B18" s="11" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C18" s="11" t="s">
         <v>1067</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="D18" s="11" t="s">
         <v>1068</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>1069</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>6</v>
@@ -6256,13 +6277,13 @@
         <v>794</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>1070</v>
       </c>
-      <c r="C19" s="14" t="s">
-        <v>1071</v>
-      </c>
       <c r="D19" s="14" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E19" s="39" t="s">
         <v>6</v>
@@ -6273,13 +6294,13 @@
         <v>794</v>
       </c>
       <c r="B20" s="11" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>1072</v>
       </c>
-      <c r="C20" s="11" t="s">
-        <v>1073</v>
-      </c>
       <c r="D20" s="11" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>6</v>
@@ -6290,13 +6311,13 @@
         <v>794</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C21" s="14" t="s">
         <v>1074</v>
       </c>
-      <c r="C21" s="14" t="s">
-        <v>1075</v>
-      </c>
       <c r="D21" s="14" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E21" s="39" t="s">
         <v>6</v>
@@ -6307,13 +6328,13 @@
         <v>794</v>
       </c>
       <c r="B22" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C22" t="s">
         <v>1076</v>
       </c>
-      <c r="C22" t="s">
-        <v>1077</v>
-      </c>
       <c r="D22" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E22" s="27" t="s">
         <v>6</v>
@@ -6324,13 +6345,13 @@
         <v>794</v>
       </c>
       <c r="B23" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C23" t="s">
         <v>1078</v>
       </c>
-      <c r="C23" t="s">
-        <v>1079</v>
-      </c>
       <c r="D23" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E23" s="27" t="s">
         <v>6</v>
@@ -6341,13 +6362,13 @@
         <v>794</v>
       </c>
       <c r="B24" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C24" t="s">
         <v>1080</v>
       </c>
-      <c r="C24" t="s">
-        <v>1081</v>
-      </c>
       <c r="D24" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E24" s="27" t="s">
         <v>6</v>
@@ -6358,13 +6379,13 @@
         <v>794</v>
       </c>
       <c r="B25" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C25" t="s">
         <v>1082</v>
       </c>
-      <c r="C25" t="s">
-        <v>1083</v>
-      </c>
       <c r="D25" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E25" s="27" t="s">
         <v>6</v>
@@ -6375,13 +6396,13 @@
         <v>794</v>
       </c>
       <c r="B26" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C26" t="s">
         <v>1084</v>
       </c>
-      <c r="C26" t="s">
-        <v>1085</v>
-      </c>
       <c r="D26" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E26" s="27" t="s">
         <v>6</v>
@@ -6392,13 +6413,13 @@
         <v>794</v>
       </c>
       <c r="B27" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C27" t="s">
         <v>1086</v>
       </c>
-      <c r="C27" t="s">
-        <v>1087</v>
-      </c>
       <c r="D27" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E27" s="27" t="s">
         <v>6</v>
@@ -6409,13 +6430,13 @@
         <v>794</v>
       </c>
       <c r="B28" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C28" t="s">
         <v>1088</v>
       </c>
-      <c r="C28" t="s">
-        <v>1089</v>
-      </c>
       <c r="D28" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E28" s="27" t="s">
         <v>6</v>
@@ -6426,13 +6447,13 @@
         <v>794</v>
       </c>
       <c r="B29" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C29" t="s">
         <v>1090</v>
       </c>
-      <c r="C29" t="s">
-        <v>1091</v>
-      </c>
       <c r="D29" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E29" s="27" t="s">
         <v>6</v>
@@ -6443,13 +6464,13 @@
         <v>794</v>
       </c>
       <c r="B30" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C30" t="s">
         <v>1092</v>
       </c>
-      <c r="C30" t="s">
-        <v>1093</v>
-      </c>
       <c r="D30" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E30" s="27" t="s">
         <v>6</v>
@@ -6460,13 +6481,13 @@
         <v>794</v>
       </c>
       <c r="B31" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C31" t="s">
         <v>1094</v>
       </c>
-      <c r="C31" t="s">
-        <v>1095</v>
-      </c>
       <c r="D31" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E31" s="27" t="s">
         <v>6</v>
@@ -6477,13 +6498,13 @@
         <v>794</v>
       </c>
       <c r="B32" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C32" t="s">
         <v>1096</v>
       </c>
-      <c r="C32" t="s">
-        <v>1097</v>
-      </c>
       <c r="D32" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E32" s="27" t="s">
         <v>6</v>
@@ -6491,16 +6512,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B33" t="s">
         <v>1177</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>1178</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>1179</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1180</v>
       </c>
       <c r="E33" s="27" t="s">
         <v>6</v>
@@ -6508,16 +6529,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B34" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C34" t="s">
         <v>1181</v>
       </c>
-      <c r="C34" t="s">
-        <v>1182</v>
-      </c>
       <c r="D34" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -6525,16 +6546,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B35" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C35" t="s">
         <v>1183</v>
       </c>
-      <c r="C35" t="s">
-        <v>1184</v>
-      </c>
       <c r="D35" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -6542,16 +6563,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B36" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C36" t="s">
         <v>1185</v>
       </c>
-      <c r="C36" t="s">
-        <v>1186</v>
-      </c>
       <c r="D36" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -6559,16 +6580,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B37" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C37" t="s">
         <v>1187</v>
       </c>
-      <c r="C37" t="s">
-        <v>1188</v>
-      </c>
       <c r="D37" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E37" s="27" t="s">
         <v>6</v>
@@ -6576,16 +6597,16 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B38" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C38" t="s">
         <v>1189</v>
       </c>
-      <c r="C38" t="s">
-        <v>1190</v>
-      </c>
       <c r="D38" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E38" s="27" t="s">
         <v>6</v>
@@ -6596,13 +6617,13 @@
         <v>772</v>
       </c>
       <c r="B39" t="s">
+        <v>1190</v>
+      </c>
+      <c r="C39" t="s">
         <v>1191</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>1192</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1193</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -6613,13 +6634,13 @@
         <v>772</v>
       </c>
       <c r="B40" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C40" t="s">
         <v>1194</v>
       </c>
-      <c r="C40" t="s">
-        <v>1195</v>
-      </c>
       <c r="D40" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -6630,13 +6651,13 @@
         <v>772</v>
       </c>
       <c r="B41" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C41" t="s">
         <v>1196</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>1197</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1198</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -6647,13 +6668,13 @@
         <v>772</v>
       </c>
       <c r="B42" t="s">
+        <v>1198</v>
+      </c>
+      <c r="C42" t="s">
         <v>1199</v>
       </c>
-      <c r="C42" t="s">
-        <v>1200</v>
-      </c>
       <c r="D42" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="E42" s="27" t="s">
         <v>6</v>
@@ -6664,13 +6685,13 @@
         <v>772</v>
       </c>
       <c r="B43" t="s">
+        <v>1200</v>
+      </c>
+      <c r="C43" t="s">
         <v>1201</v>
       </c>
-      <c r="C43" t="s">
-        <v>1202</v>
-      </c>
       <c r="D43" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>6</v>
@@ -6681,13 +6702,13 @@
         <v>772</v>
       </c>
       <c r="B44" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C44" t="s">
         <v>1203</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>1204</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1205</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>6</v>
@@ -6698,13 +6719,13 @@
         <v>772</v>
       </c>
       <c r="B45" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C45" t="s">
         <v>1206</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>1207</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1208</v>
       </c>
       <c r="E45" s="27" t="s">
         <v>6</v>
@@ -7028,7 +7049,7 @@
         <v>847</v>
       </c>
       <c r="G3" s="32" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7051,7 +7072,7 @@
         <v>436</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7074,7 +7095,7 @@
         <v>436</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
   </sheetData>
@@ -7087,7 +7108,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H190"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7112,7 +7133,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="B2" s="46"/>
       <c r="C2" s="46"/>
@@ -8151,46 +8172,46 @@
     </row>
     <row r="69" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="25" t="s">
+        <v>898</v>
+      </c>
+      <c r="B69" s="25" t="s">
         <v>899</v>
       </c>
-      <c r="B69" s="25" t="s">
+      <c r="C69" s="25" t="s">
         <v>900</v>
-      </c>
-      <c r="C69" s="25" t="s">
-        <v>901</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="25" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B70" s="25" t="s">
+        <v>901</v>
+      </c>
+      <c r="C70" s="25" t="s">
         <v>902</v>
-      </c>
-      <c r="C70" s="25" t="s">
-        <v>903</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="44" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="B71" s="25" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C71" s="25" t="s">
         <v>1228</v>
-      </c>
-      <c r="C71" s="25" t="s">
-        <v>1229</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="44" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="B72" s="25" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C72" s="25" t="s">
         <v>1230</v>
-      </c>
-      <c r="C72" s="25" t="s">
-        <v>1231</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -8450,7 +8471,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="E95" s="28"/>
       <c r="F95" s="27"/>
@@ -8480,16 +8501,16 @@
         <v>1</v>
       </c>
       <c r="B97" t="s">
+        <v>904</v>
+      </c>
+      <c r="C97" t="s">
         <v>905</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>906</v>
       </c>
-      <c r="D97" t="s">
-        <v>907</v>
-      </c>
       <c r="E97" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F97" s="27" t="s">
         <v>6</v>
@@ -8500,16 +8521,16 @@
         <v>2</v>
       </c>
       <c r="B98" t="s">
+        <v>907</v>
+      </c>
+      <c r="C98" t="s">
         <v>908</v>
       </c>
-      <c r="C98" t="s">
+      <c r="D98" t="s">
         <v>909</v>
       </c>
-      <c r="D98" t="s">
-        <v>910</v>
-      </c>
       <c r="E98" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F98" s="27" t="s">
         <v>6</v>
@@ -8520,16 +8541,16 @@
         <v>3</v>
       </c>
       <c r="B99" t="s">
+        <v>910</v>
+      </c>
+      <c r="C99" t="s">
         <v>911</v>
       </c>
-      <c r="C99" t="s">
+      <c r="D99" t="s">
         <v>912</v>
       </c>
-      <c r="D99" t="s">
-        <v>913</v>
-      </c>
       <c r="E99" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F99" s="27" t="s">
         <v>6</v>
@@ -8540,16 +8561,16 @@
         <v>4</v>
       </c>
       <c r="B100" t="s">
+        <v>913</v>
+      </c>
+      <c r="C100" t="s">
         <v>914</v>
       </c>
-      <c r="C100" t="s">
+      <c r="D100" t="s">
         <v>915</v>
       </c>
-      <c r="D100" t="s">
-        <v>916</v>
-      </c>
       <c r="E100" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F100" s="27" t="s">
         <v>6</v>
@@ -8560,16 +8581,16 @@
         <v>5</v>
       </c>
       <c r="B101" t="s">
+        <v>916</v>
+      </c>
+      <c r="C101" t="s">
         <v>917</v>
       </c>
-      <c r="C101" t="s">
+      <c r="D101" t="s">
         <v>918</v>
       </c>
-      <c r="D101" t="s">
-        <v>919</v>
-      </c>
       <c r="E101" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F101" s="27" t="s">
         <v>6</v>
@@ -8580,16 +8601,16 @@
         <v>6</v>
       </c>
       <c r="B102" t="s">
+        <v>919</v>
+      </c>
+      <c r="C102" t="s">
         <v>920</v>
       </c>
-      <c r="C102" t="s">
+      <c r="D102" t="s">
         <v>921</v>
       </c>
-      <c r="D102" t="s">
-        <v>922</v>
-      </c>
       <c r="E102" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F102" s="27" t="s">
         <v>6</v>
@@ -8597,7 +8618,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="32" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
@@ -8625,16 +8646,16 @@
         <v>1</v>
       </c>
       <c r="B106" t="s">
+        <v>931</v>
+      </c>
+      <c r="C106" t="s">
         <v>932</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
         <v>933</v>
       </c>
-      <c r="D106" t="s">
+      <c r="E106" t="s">
         <v>934</v>
-      </c>
-      <c r="E106" t="s">
-        <v>935</v>
       </c>
       <c r="F106" s="27" t="s">
         <v>6</v>
@@ -8645,16 +8666,16 @@
         <v>2</v>
       </c>
       <c r="B107" t="s">
+        <v>935</v>
+      </c>
+      <c r="C107" t="s">
         <v>936</v>
       </c>
-      <c r="C107" t="s">
+      <c r="D107" t="s">
         <v>937</v>
       </c>
-      <c r="D107" t="s">
-        <v>938</v>
-      </c>
       <c r="E107" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F107" s="27" t="s">
         <v>6</v>
@@ -8665,16 +8686,16 @@
         <v>3</v>
       </c>
       <c r="B108" t="s">
+        <v>938</v>
+      </c>
+      <c r="C108" t="s">
         <v>939</v>
       </c>
-      <c r="C108" t="s">
-        <v>940</v>
-      </c>
       <c r="D108" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E108" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F108" s="27" t="s">
         <v>6</v>
@@ -8685,16 +8706,16 @@
         <v>4</v>
       </c>
       <c r="B109" t="s">
+        <v>940</v>
+      </c>
+      <c r="C109" t="s">
         <v>941</v>
       </c>
-      <c r="C109" t="s">
-        <v>942</v>
-      </c>
       <c r="D109" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E109" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F109" s="27" t="s">
         <v>6</v>
@@ -8705,16 +8726,16 @@
         <v>5</v>
       </c>
       <c r="B110" t="s">
+        <v>942</v>
+      </c>
+      <c r="C110" t="s">
         <v>943</v>
       </c>
-      <c r="C110" t="s">
+      <c r="D110" t="s">
         <v>944</v>
       </c>
-      <c r="D110" t="s">
-        <v>945</v>
-      </c>
       <c r="E110" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F110" s="27" t="s">
         <v>6</v>
@@ -8722,7 +8743,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
@@ -8750,16 +8771,16 @@
         <v>1</v>
       </c>
       <c r="B114" t="s">
+        <v>948</v>
+      </c>
+      <c r="C114" t="s">
         <v>949</v>
       </c>
-      <c r="C114" t="s">
+      <c r="D114" t="s">
         <v>950</v>
       </c>
-      <c r="D114" t="s">
+      <c r="E114" t="s">
         <v>951</v>
-      </c>
-      <c r="E114" t="s">
-        <v>952</v>
       </c>
       <c r="F114" s="27" t="s">
         <v>6</v>
@@ -8770,16 +8791,16 @@
         <v>2</v>
       </c>
       <c r="B115" t="s">
+        <v>952</v>
+      </c>
+      <c r="C115" t="s">
         <v>953</v>
       </c>
-      <c r="C115" t="s">
+      <c r="D115" t="s">
         <v>954</v>
       </c>
-      <c r="D115" t="s">
-        <v>955</v>
-      </c>
       <c r="E115" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="F115" s="27" t="s">
         <v>6</v>
@@ -8790,16 +8811,16 @@
         <v>3</v>
       </c>
       <c r="B116" t="s">
+        <v>955</v>
+      </c>
+      <c r="C116" t="s">
         <v>956</v>
       </c>
-      <c r="C116" t="s">
+      <c r="D116" t="s">
         <v>957</v>
       </c>
-      <c r="D116" t="s">
-        <v>958</v>
-      </c>
       <c r="E116" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="F116" s="27" t="s">
         <v>6</v>
@@ -8810,16 +8831,16 @@
         <v>4</v>
       </c>
       <c r="B117" t="s">
+        <v>958</v>
+      </c>
+      <c r="C117" t="s">
         <v>959</v>
       </c>
-      <c r="C117" t="s">
+      <c r="D117" t="s">
         <v>960</v>
       </c>
-      <c r="D117" t="s">
-        <v>961</v>
-      </c>
       <c r="E117" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="F117" s="27" t="s">
         <v>6</v>
@@ -8830,16 +8851,16 @@
         <v>5</v>
       </c>
       <c r="B118" t="s">
+        <v>961</v>
+      </c>
+      <c r="C118" t="s">
         <v>962</v>
       </c>
-      <c r="C118" t="s">
+      <c r="D118" t="s">
         <v>963</v>
       </c>
-      <c r="D118" t="s">
+      <c r="E118" t="s">
         <v>964</v>
-      </c>
-      <c r="E118" t="s">
-        <v>965</v>
       </c>
       <c r="F118" s="27" t="s">
         <v>6</v>
@@ -8847,7 +8868,7 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
@@ -8875,16 +8896,16 @@
         <v>1</v>
       </c>
       <c r="B122" t="s">
+        <v>966</v>
+      </c>
+      <c r="C122" t="s">
         <v>967</v>
       </c>
-      <c r="C122" t="s">
+      <c r="D122" t="s">
         <v>968</v>
       </c>
-      <c r="D122" t="s">
-        <v>969</v>
-      </c>
       <c r="E122" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="F122" s="27" t="s">
         <v>6</v>
@@ -8895,16 +8916,16 @@
         <v>2</v>
       </c>
       <c r="B123" t="s">
+        <v>969</v>
+      </c>
+      <c r="C123" t="s">
         <v>970</v>
       </c>
-      <c r="C123" t="s">
-        <v>971</v>
-      </c>
       <c r="D123" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="E123" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="F123" s="27" t="s">
         <v>6</v>
@@ -8915,16 +8936,16 @@
         <v>3</v>
       </c>
       <c r="B124" t="s">
+        <v>971</v>
+      </c>
+      <c r="C124" t="s">
         <v>972</v>
       </c>
-      <c r="C124" t="s">
+      <c r="D124" t="s">
         <v>973</v>
       </c>
-      <c r="D124" t="s">
-        <v>974</v>
-      </c>
       <c r="E124" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="F124" s="27" t="s">
         <v>6</v>
@@ -8935,16 +8956,16 @@
         <v>4</v>
       </c>
       <c r="B125" t="s">
+        <v>974</v>
+      </c>
+      <c r="C125" t="s">
         <v>975</v>
       </c>
-      <c r="C125" t="s">
+      <c r="D125" t="s">
         <v>976</v>
       </c>
-      <c r="D125" t="s">
-        <v>977</v>
-      </c>
       <c r="E125" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="F125" s="27" t="s">
         <v>6</v>
@@ -8955,10 +8976,10 @@
         <v>5</v>
       </c>
       <c r="B126" t="s">
+        <v>977</v>
+      </c>
+      <c r="C126" t="s">
         <v>978</v>
-      </c>
-      <c r="C126" t="s">
-        <v>979</v>
       </c>
       <c r="D126" t="s">
         <v>437</v>
@@ -8967,12 +8988,12 @@
         <v>437</v>
       </c>
       <c r="F126" s="38" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
@@ -9000,16 +9021,16 @@
         <v>1</v>
       </c>
       <c r="B130" t="s">
+        <v>991</v>
+      </c>
+      <c r="C130" t="s">
         <v>992</v>
-      </c>
-      <c r="C130" t="s">
-        <v>993</v>
       </c>
       <c r="D130" t="s">
         <v>437</v>
       </c>
       <c r="E130" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F130" s="27" t="s">
         <v>6</v>
@@ -9020,16 +9041,16 @@
         <v>2</v>
       </c>
       <c r="B131" t="s">
+        <v>994</v>
+      </c>
+      <c r="C131" t="s">
         <v>995</v>
       </c>
-      <c r="C131" t="s">
+      <c r="D131" t="s">
         <v>996</v>
       </c>
-      <c r="D131" t="s">
-        <v>997</v>
-      </c>
       <c r="E131" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F131" s="27" t="s">
         <v>6</v>
@@ -9040,16 +9061,16 @@
         <v>3</v>
       </c>
       <c r="B132" t="s">
+        <v>997</v>
+      </c>
+      <c r="C132" t="s">
         <v>998</v>
       </c>
-      <c r="C132" t="s">
+      <c r="D132" t="s">
         <v>999</v>
       </c>
-      <c r="D132" t="s">
-        <v>1000</v>
-      </c>
       <c r="E132" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F132" s="27" t="s">
         <v>6</v>
@@ -9060,16 +9081,16 @@
         <v>4</v>
       </c>
       <c r="B133" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C133" t="s">
         <v>1001</v>
       </c>
-      <c r="C133" t="s">
+      <c r="D133" t="s">
         <v>1002</v>
       </c>
-      <c r="D133" t="s">
-        <v>1003</v>
-      </c>
       <c r="E133" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F133" s="27" t="s">
         <v>6</v>
@@ -9080,16 +9101,16 @@
         <v>5</v>
       </c>
       <c r="B134" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C134" t="s">
         <v>1004</v>
-      </c>
-      <c r="C134" t="s">
-        <v>1005</v>
       </c>
       <c r="D134" t="s">
         <v>437</v>
       </c>
       <c r="E134" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F134" s="27" t="s">
         <v>6</v>
@@ -9097,7 +9118,7 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
@@ -9125,16 +9146,16 @@
         <v>1</v>
       </c>
       <c r="B138" t="s">
+        <v>1012</v>
+      </c>
+      <c r="C138" t="s">
         <v>1013</v>
       </c>
-      <c r="C138" t="s">
+      <c r="D138" t="s">
         <v>1014</v>
       </c>
-      <c r="D138" t="s">
-        <v>1015</v>
-      </c>
       <c r="E138" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F138" s="27" t="s">
         <v>6</v>
@@ -9145,16 +9166,16 @@
         <v>2</v>
       </c>
       <c r="B139" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C139" t="s">
         <v>1016</v>
       </c>
-      <c r="C139" t="s">
+      <c r="D139" t="s">
         <v>1017</v>
       </c>
-      <c r="D139" t="s">
-        <v>1018</v>
-      </c>
       <c r="E139" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F139" s="27" t="s">
         <v>6</v>
@@ -9165,16 +9186,16 @@
         <v>3</v>
       </c>
       <c r="B140" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="C140" t="s">
+        <v>1018</v>
+      </c>
+      <c r="D140" t="s">
         <v>1019</v>
       </c>
-      <c r="D140" t="s">
-        <v>1020</v>
-      </c>
       <c r="E140" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F140" s="27" t="s">
         <v>6</v>
@@ -9182,7 +9203,7 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
@@ -9210,16 +9231,16 @@
         <v>1</v>
       </c>
       <c r="B144" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C144" t="s">
         <v>1027</v>
       </c>
-      <c r="C144" t="s">
+      <c r="D144" t="s">
         <v>1028</v>
       </c>
-      <c r="D144" t="s">
-        <v>1029</v>
-      </c>
       <c r="E144" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F144" s="27" t="s">
         <v>6</v>
@@ -9230,16 +9251,16 @@
         <v>2</v>
       </c>
       <c r="B145" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C145" t="s">
         <v>1030</v>
       </c>
-      <c r="C145" t="s">
+      <c r="D145" t="s">
         <v>1031</v>
       </c>
-      <c r="D145" t="s">
-        <v>1032</v>
-      </c>
       <c r="E145" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F145" s="27" t="s">
         <v>6</v>
@@ -9250,16 +9271,16 @@
         <v>3</v>
       </c>
       <c r="B146" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C146" t="s">
         <v>1033</v>
       </c>
-      <c r="C146" t="s">
+      <c r="D146" t="s">
         <v>1034</v>
       </c>
-      <c r="D146" t="s">
-        <v>1035</v>
-      </c>
       <c r="E146" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F146" s="27" t="s">
         <v>6</v>
@@ -9270,16 +9291,16 @@
         <v>4</v>
       </c>
       <c r="B147" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C147" t="s">
         <v>1036</v>
       </c>
-      <c r="C147" t="s">
+      <c r="D147" t="s">
         <v>1037</v>
       </c>
-      <c r="D147" t="s">
-        <v>1038</v>
-      </c>
       <c r="E147" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F147" s="27" t="s">
         <v>6</v>
@@ -9290,16 +9311,16 @@
         <v>5</v>
       </c>
       <c r="B148" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C148" t="s">
         <v>1039</v>
-      </c>
-      <c r="C148" t="s">
-        <v>1040</v>
       </c>
       <c r="D148" t="s">
         <v>29</v>
       </c>
       <c r="E148" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F148" s="27" t="s">
         <v>6</v>
@@ -9310,16 +9331,16 @@
         <v>6</v>
       </c>
       <c r="B149" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C149" t="s">
         <v>1041</v>
       </c>
-      <c r="C149" t="s">
+      <c r="D149" t="s">
         <v>1042</v>
       </c>
-      <c r="D149" t="s">
-        <v>1043</v>
-      </c>
       <c r="E149" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="F149" s="27" t="s">
         <v>6</v>
@@ -9327,7 +9348,7 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
@@ -9355,16 +9376,16 @@
         <v>1</v>
       </c>
       <c r="B153" s="27" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C153" s="27" t="s">
         <v>1105</v>
       </c>
-      <c r="C153" s="27" t="s">
+      <c r="D153" s="27" t="s">
         <v>1106</v>
       </c>
-      <c r="D153" s="27" t="s">
-        <v>1107</v>
-      </c>
       <c r="E153" s="40" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="F153" s="27" t="s">
         <v>6</v>
@@ -9375,16 +9396,16 @@
         <v>2</v>
       </c>
       <c r="B154" s="27" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C154" s="27" t="s">
         <v>1108</v>
       </c>
-      <c r="C154" s="27" t="s">
+      <c r="D154" s="27" t="s">
         <v>1109</v>
       </c>
-      <c r="D154" s="27" t="s">
-        <v>1110</v>
-      </c>
       <c r="E154" s="40" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="F154" s="27" t="s">
         <v>6</v>
@@ -9395,16 +9416,16 @@
         <v>3</v>
       </c>
       <c r="B155" s="27" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C155" s="27" t="s">
         <v>1111</v>
       </c>
-      <c r="C155" s="27" t="s">
+      <c r="D155" s="27" t="s">
         <v>1112</v>
       </c>
-      <c r="D155" s="27" t="s">
-        <v>1113</v>
-      </c>
       <c r="E155" s="40" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="F155" s="27" t="s">
         <v>6</v>
@@ -9415,16 +9436,16 @@
         <v>4</v>
       </c>
       <c r="B156" s="27" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C156" s="27" t="s">
         <v>1114</v>
       </c>
-      <c r="C156" s="27" t="s">
+      <c r="D156" s="27" t="s">
         <v>1115</v>
       </c>
-      <c r="D156" s="27" t="s">
-        <v>1116</v>
-      </c>
       <c r="E156" s="40" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="F156" s="27" t="s">
         <v>6</v>
@@ -9435,16 +9456,16 @@
         <v>5</v>
       </c>
       <c r="B157" s="27" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C157" s="27" t="s">
+        <v>1128</v>
+      </c>
+      <c r="D157" s="27" t="s">
         <v>1117</v>
       </c>
-      <c r="C157" s="27" t="s">
-        <v>1129</v>
-      </c>
-      <c r="D157" s="27" t="s">
-        <v>1118</v>
-      </c>
       <c r="E157" s="40" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="F157" s="27" t="s">
         <v>6</v>
@@ -9455,16 +9476,16 @@
         <v>6</v>
       </c>
       <c r="B158" s="41" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C158" s="41" t="s">
         <v>1130</v>
-      </c>
-      <c r="C158" s="41" t="s">
-        <v>1131</v>
       </c>
       <c r="D158" s="41" t="s">
         <v>267</v>
       </c>
       <c r="E158" s="42" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="F158" s="27" t="s">
         <v>6</v>
@@ -9472,7 +9493,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
@@ -9500,16 +9521,16 @@
         <v>1</v>
       </c>
       <c r="B162" s="27" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C162" s="27" t="s">
         <v>1139</v>
       </c>
-      <c r="C162" s="27" t="s">
+      <c r="D162" s="27" t="s">
         <v>1140</v>
       </c>
-      <c r="D162" s="27" t="s">
+      <c r="E162" s="40" t="s">
         <v>1141</v>
-      </c>
-      <c r="E162" s="40" t="s">
-        <v>1142</v>
       </c>
       <c r="F162" s="27" t="s">
         <v>6</v>
@@ -9520,16 +9541,16 @@
         <v>2</v>
       </c>
       <c r="B163" s="27" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C163" s="27" t="s">
         <v>1143</v>
       </c>
-      <c r="C163" s="27" t="s">
+      <c r="D163" s="27" t="s">
         <v>1144</v>
       </c>
-      <c r="D163" s="27" t="s">
-        <v>1145</v>
-      </c>
       <c r="E163" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F163" s="27" t="s">
         <v>6</v>
@@ -9540,16 +9561,16 @@
         <v>3</v>
       </c>
       <c r="B164" s="27" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C164" s="27" t="s">
         <v>1146</v>
       </c>
-      <c r="C164" s="27" t="s">
+      <c r="D164" s="27" t="s">
         <v>1147</v>
       </c>
-      <c r="D164" s="27" t="s">
-        <v>1148</v>
-      </c>
       <c r="E164" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F164" s="27" t="s">
         <v>6</v>
@@ -9560,16 +9581,16 @@
         <v>4</v>
       </c>
       <c r="B165" s="27" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C165" s="27" t="s">
         <v>1149</v>
       </c>
-      <c r="C165" s="27" t="s">
+      <c r="D165" s="27" t="s">
         <v>1150</v>
       </c>
-      <c r="D165" s="27" t="s">
-        <v>1151</v>
-      </c>
       <c r="E165" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F165" s="27" t="s">
         <v>6</v>
@@ -9580,16 +9601,16 @@
         <v>5</v>
       </c>
       <c r="B166" s="27" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C166" s="27" t="s">
         <v>1152</v>
       </c>
-      <c r="C166" s="27" t="s">
+      <c r="D166" s="27" t="s">
         <v>1153</v>
       </c>
-      <c r="D166" s="27" t="s">
-        <v>1154</v>
-      </c>
       <c r="E166" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F166" s="27" t="s">
         <v>6</v>
@@ -9600,16 +9621,16 @@
         <v>6</v>
       </c>
       <c r="B167" s="27" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C167" s="27" t="s">
         <v>1155</v>
       </c>
-      <c r="C167" s="27" t="s">
+      <c r="D167" s="27" t="s">
         <v>1156</v>
       </c>
-      <c r="D167" s="27" t="s">
-        <v>1157</v>
-      </c>
       <c r="E167" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F167" s="27" t="s">
         <v>6</v>
@@ -9620,16 +9641,16 @@
         <v>7</v>
       </c>
       <c r="B168" s="27" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C168" s="27" t="s">
         <v>1158</v>
       </c>
-      <c r="C168" s="27" t="s">
-        <v>1159</v>
-      </c>
       <c r="D168" s="27" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="E168" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F168" s="27" t="s">
         <v>6</v>
@@ -9640,16 +9661,16 @@
         <v>8</v>
       </c>
       <c r="B169" s="27" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C169" s="27" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D169" s="27" t="s">
         <v>1160</v>
       </c>
-      <c r="C169" s="27" t="s">
-        <v>1209</v>
-      </c>
-      <c r="D169" s="27" t="s">
-        <v>1161</v>
-      </c>
       <c r="E169" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F169" s="27" t="s">
         <v>6</v>
@@ -9660,16 +9681,16 @@
         <v>9</v>
       </c>
       <c r="B170" s="27" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C170" s="27" t="s">
         <v>1162</v>
       </c>
-      <c r="C170" s="27" t="s">
+      <c r="D170" s="27" t="s">
         <v>1163</v>
       </c>
-      <c r="D170" s="27" t="s">
-        <v>1164</v>
-      </c>
       <c r="E170" s="40" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="F170" s="27" t="s">
         <v>6</v>
@@ -9677,7 +9698,7 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
@@ -9705,16 +9726,16 @@
         <v>1</v>
       </c>
       <c r="B174" s="27" t="s">
+        <v>1212</v>
+      </c>
+      <c r="C174" s="27" t="s">
         <v>1213</v>
       </c>
-      <c r="C174" s="27" t="s">
+      <c r="D174" s="27" t="s">
         <v>1214</v>
       </c>
-      <c r="D174" s="27" t="s">
+      <c r="E174" s="40" t="s">
         <v>1215</v>
-      </c>
-      <c r="E174" s="40" t="s">
-        <v>1216</v>
       </c>
       <c r="F174" s="27" t="s">
         <v>6</v>
@@ -9725,16 +9746,16 @@
         <v>2</v>
       </c>
       <c r="B175" s="27" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C175" s="27" t="s">
         <v>1217</v>
       </c>
-      <c r="C175" s="27" t="s">
+      <c r="D175" s="27" t="s">
         <v>1218</v>
       </c>
-      <c r="D175" s="27" t="s">
-        <v>1219</v>
-      </c>
       <c r="E175" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F175" s="27" t="s">
         <v>6</v>
@@ -9745,16 +9766,16 @@
         <v>3</v>
       </c>
       <c r="B176" s="27" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C176" s="27" t="s">
         <v>1220</v>
       </c>
-      <c r="C176" s="27" t="s">
+      <c r="D176" s="27" t="s">
         <v>1221</v>
       </c>
-      <c r="D176" s="27" t="s">
-        <v>1222</v>
-      </c>
       <c r="E176" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F176" s="27" t="s">
         <v>6</v>
@@ -9765,19 +9786,19 @@
         <v>4</v>
       </c>
       <c r="B177" s="27" t="s">
+        <v>1222</v>
+      </c>
+      <c r="C177" s="27" t="s">
         <v>1223</v>
       </c>
-      <c r="C177" s="27" t="s">
+      <c r="D177" s="27" t="s">
         <v>1224</v>
       </c>
-      <c r="D177" s="27" t="s">
-        <v>1225</v>
-      </c>
       <c r="E177" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F177" s="43" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
@@ -9785,16 +9806,16 @@
         <v>5</v>
       </c>
       <c r="B178" s="27" t="s">
+        <v>1225</v>
+      </c>
+      <c r="C178" s="27" t="s">
         <v>1226</v>
-      </c>
-      <c r="C178" s="27" t="s">
-        <v>1227</v>
       </c>
       <c r="D178" s="27" t="s">
         <v>437</v>
       </c>
       <c r="E178" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F178" s="27" t="s">
         <v>6</v>
@@ -9802,7 +9823,7 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -9830,16 +9851,16 @@
         <v>1</v>
       </c>
       <c r="B182" s="27" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C182" s="27" t="s">
         <v>1247</v>
       </c>
-      <c r="C182" s="27" t="s">
+      <c r="D182" s="27" t="s">
         <v>1248</v>
       </c>
-      <c r="D182" s="27" t="s">
-        <v>1249</v>
-      </c>
       <c r="E182" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F182" s="27" t="s">
         <v>6</v>
@@ -9850,16 +9871,16 @@
         <v>2</v>
       </c>
       <c r="B183" s="27" t="s">
+        <v>1249</v>
+      </c>
+      <c r="C183" s="27" t="s">
         <v>1250</v>
       </c>
-      <c r="C183" s="27" t="s">
+      <c r="D183" s="27" t="s">
         <v>1251</v>
       </c>
-      <c r="D183" s="27" t="s">
-        <v>1252</v>
-      </c>
       <c r="E183" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F183" s="27" t="s">
         <v>6</v>
@@ -9870,16 +9891,16 @@
         <v>3</v>
       </c>
       <c r="B184" s="27" t="s">
+        <v>1252</v>
+      </c>
+      <c r="C184" s="27" t="s">
         <v>1253</v>
       </c>
-      <c r="C184" s="27" t="s">
+      <c r="D184" s="27" t="s">
         <v>1254</v>
       </c>
-      <c r="D184" s="27" t="s">
-        <v>1255</v>
-      </c>
       <c r="E184" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F184" s="27" t="s">
         <v>6</v>
@@ -9890,16 +9911,16 @@
         <v>4</v>
       </c>
       <c r="B185" s="27" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C185" s="27" t="s">
         <v>1256</v>
-      </c>
-      <c r="C185" s="27" t="s">
-        <v>1257</v>
       </c>
       <c r="D185" s="27" t="s">
         <v>401</v>
       </c>
       <c r="E185" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F185" s="27" t="s">
         <v>6</v>
@@ -9910,16 +9931,16 @@
         <v>5</v>
       </c>
       <c r="B186" s="27" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C186" s="27" t="s">
         <v>1258</v>
       </c>
-      <c r="C186" s="27" t="s">
+      <c r="D186" s="27" t="s">
         <v>1259</v>
       </c>
-      <c r="D186" s="27" t="s">
-        <v>1260</v>
-      </c>
       <c r="E186" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F186" s="27" t="s">
         <v>6</v>
@@ -9930,16 +9951,16 @@
         <v>6</v>
       </c>
       <c r="B187" s="27" t="s">
+        <v>1260</v>
+      </c>
+      <c r="C187" s="27" t="s">
         <v>1261</v>
       </c>
-      <c r="C187" s="27" t="s">
+      <c r="D187" s="27" t="s">
         <v>1262</v>
       </c>
-      <c r="D187" s="27" t="s">
-        <v>1263</v>
-      </c>
       <c r="E187" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F187" s="27" t="s">
         <v>6</v>
@@ -9950,19 +9971,19 @@
         <v>7</v>
       </c>
       <c r="B188" s="27" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C188" s="27" t="s">
         <v>1264</v>
-      </c>
-      <c r="C188" s="27" t="s">
-        <v>1265</v>
       </c>
       <c r="D188" s="27" t="s">
         <v>22</v>
       </c>
       <c r="E188" s="40" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F188" s="43" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
@@ -9970,19 +9991,39 @@
         <v>8</v>
       </c>
       <c r="B189" s="27" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C189" s="27" t="s">
+        <v>1286</v>
+      </c>
+      <c r="D189" s="27" t="s">
+        <v>1287</v>
+      </c>
+      <c r="E189" s="40" t="s">
+        <v>1215</v>
+      </c>
+      <c r="F189" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A190" s="27">
+        <v>9</v>
+      </c>
+      <c r="B190" s="27" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C190" s="27" t="s">
         <v>1266</v>
       </c>
-      <c r="C189" s="27" t="s">
+      <c r="D190" s="27" t="s">
         <v>1267</v>
       </c>
-      <c r="D189" s="27" t="s">
-        <v>1268</v>
-      </c>
-      <c r="E189" s="40" t="s">
+      <c r="E190" s="40" t="s">
         <v>437</v>
       </c>
-      <c r="F189" s="38" t="s">
-        <v>980</v>
+      <c r="F190" s="38" t="s">
+        <v>979</v>
       </c>
     </row>
   </sheetData>
@@ -10426,7 +10467,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -10457,13 +10498,13 @@
         <v>280</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>896</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="D33" s="2" t="s">
         <v>897</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>898</v>
       </c>
       <c r="E33" s="30" t="s">
         <v>6</v>
@@ -10471,16 +10512,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B34" t="s">
         <v>1044</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>1045</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>1046</v>
-      </c>
-      <c r="D34" t="s">
-        <v>1047</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -10488,16 +10529,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B35" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="C35" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D35" t="s">
         <v>1165</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1166</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -10505,16 +10546,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B36" t="s">
+        <v>1268</v>
+      </c>
+      <c r="C36" t="s">
         <v>1269</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>1270</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1271</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -10534,7 +10575,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -10816,11 +10857,11 @@
         <v>46094</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="F15" s="26"/>
       <c r="G15" s="5" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -10844,19 +10885,19 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C17" t="s">
         <v>1009</v>
       </c>
-      <c r="B17" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>1010</v>
       </c>
-      <c r="D17" t="s">
-        <v>1011</v>
-      </c>
       <c r="E17" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="F17" s="27" t="s">
         <v>6</v>
@@ -10864,19 +10905,19 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B18" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="C18" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="D18" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="E18" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="F18" s="27" t="s">
         <v>6</v>
@@ -10884,113 +10925,136 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B19" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C19" t="s">
         <v>1048</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E19" t="s">
+        <v>1010</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G19" t="s">
         <v>1049</v>
-      </c>
-      <c r="D19" t="s">
-        <v>1011</v>
-      </c>
-      <c r="E19" t="s">
-        <v>1011</v>
-      </c>
-      <c r="F19" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="G19" t="s">
-        <v>1050</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="27" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B20" s="27" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C20" s="27" t="s">
         <v>1099</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="D20" s="27" t="s">
         <v>1100</v>
       </c>
-      <c r="D20" s="27" t="s">
-        <v>1101</v>
-      </c>
       <c r="E20" s="27" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="F20" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="41" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B21" s="41" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C21" s="41" t="s">
         <v>1134</v>
       </c>
-      <c r="C21" s="41" t="s">
-        <v>1135</v>
-      </c>
       <c r="D21" s="41" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="E21" s="41" t="s">
+        <v>1231</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="41" t="s">
         <v>1232</v>
-      </c>
-      <c r="F21" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="G21" s="41" t="s">
-        <v>1233</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="41" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B22" s="41" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C22" s="41" t="s">
         <v>1168</v>
       </c>
-      <c r="C22" s="41" t="s">
-        <v>1169</v>
-      </c>
       <c r="D22" s="41" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="E22" s="41" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="F22" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="41" t="s">
-        <v>1009</v>
+        <v>1288</v>
       </c>
       <c r="B23" s="41" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>1290</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>1231</v>
+      </c>
+      <c r="E23" s="41" t="s">
+        <v>1231</v>
+      </c>
+      <c r="F23" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G23" s="41" t="s">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="41" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B24" s="41" t="s">
+        <v>1273</v>
+      </c>
+      <c r="C24" s="41" t="s">
         <v>1274</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="43" t="s">
+        <v>1131</v>
+      </c>
+      <c r="G24" s="41" t="s">
         <v>1275</v>
-      </c>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="43" t="s">
-        <v>1132</v>
-      </c>
-      <c r="G23" s="41" t="s">
-        <v>1276</v>
       </c>
     </row>
   </sheetData>
@@ -11411,13 +11475,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>986</v>
+      </c>
+      <c r="B34" t="s">
         <v>987</v>
       </c>
-      <c r="B34" t="s">
-        <v>988</v>
-      </c>
       <c r="C34" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="D34" s="27" t="s">
         <v>6</v>
@@ -11425,13 +11489,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B35" t="s">
         <v>1006</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>1007</v>
-      </c>
-      <c r="C35" t="s">
-        <v>1008</v>
       </c>
       <c r="D35" s="27" t="s">
         <v>6</v>
@@ -11439,13 +11503,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B36" t="s">
         <v>1021</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>1022</v>
-      </c>
-      <c r="C36" t="s">
-        <v>1023</v>
       </c>
       <c r="D36" s="27" t="s">
         <v>6</v>
@@ -11453,13 +11517,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B37" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C37" t="s">
         <v>1051</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1052</v>
       </c>
       <c r="D37" s="27" t="s">
         <v>6</v>
@@ -11467,13 +11531,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="27" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B38" s="27" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C38" s="27" t="s">
         <v>1102</v>
-      </c>
-      <c r="C38" s="27" t="s">
-        <v>1103</v>
       </c>
       <c r="D38" s="27" t="s">
         <v>6</v>
@@ -11481,41 +11545,41 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="41" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B39" s="41" t="s">
         <v>1123</v>
       </c>
-      <c r="B39" s="41" t="s">
+      <c r="C39" s="41" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D39" s="41" t="s">
         <v>1124</v>
-      </c>
-      <c r="C39" s="41" t="s">
-        <v>1176</v>
-      </c>
-      <c r="D39" s="41" t="s">
-        <v>1125</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="41" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B40" s="41" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C40" s="41" t="s">
         <v>1126</v>
       </c>
-      <c r="C40" s="41" t="s">
+      <c r="D40" s="41" t="s">
         <v>1127</v>
-      </c>
-      <c r="D40" s="41" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="27" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="B41" s="27" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C41" s="27" t="s">
         <v>1170</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>1171</v>
       </c>
       <c r="D41" s="27" t="s">
         <v>6</v>
@@ -11523,27 +11587,27 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="41" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B42" s="41" t="s">
         <v>1172</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="C42" s="41" t="s">
         <v>1173</v>
       </c>
-      <c r="C42" s="41" t="s">
+      <c r="D42" s="43" t="s">
         <v>1174</v>
-      </c>
-      <c r="D42" s="43" t="s">
-        <v>1175</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="41" t="s">
+        <v>1233</v>
+      </c>
+      <c r="B43" s="41" t="s">
         <v>1234</v>
       </c>
-      <c r="B43" s="41" t="s">
+      <c r="C43" s="41" t="s">
         <v>1235</v>
-      </c>
-      <c r="C43" s="41" t="s">
-        <v>1236</v>
       </c>
       <c r="D43" s="27" t="s">
         <v>6</v>
@@ -11551,41 +11615,41 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="41" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B44" s="41" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C44" s="41" t="s">
         <v>1237</v>
       </c>
-      <c r="C44" s="41" t="s">
-        <v>1238</v>
-      </c>
       <c r="D44" s="43" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="41" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B45" s="41" t="s">
         <v>1239</v>
       </c>
-      <c r="B45" s="41" t="s">
+      <c r="C45" s="41" t="s">
         <v>1240</v>
       </c>
-      <c r="C45" s="41" t="s">
+      <c r="D45" s="43" t="s">
         <v>1241</v>
-      </c>
-      <c r="D45" s="43" t="s">
-        <v>1242</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="27" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B46" s="27" t="s">
+        <v>1276</v>
+      </c>
+      <c r="C46" s="27" t="s">
         <v>1277</v>
-      </c>
-      <c r="C46" s="27" t="s">
-        <v>1278</v>
       </c>
       <c r="D46" s="27" t="s">
         <v>6</v>
@@ -12933,7 +12997,7 @@
         <v>602</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>603</v>
@@ -13100,13 +13164,13 @@
         <v>637</v>
       </c>
       <c r="C19" s="14" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>1054</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="E19" s="14" t="s">
         <v>1055</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>1056</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13128,36 +13192,36 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B21" t="s">
         <v>1057</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>1058</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>1059</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>1060</v>
-      </c>
-      <c r="E21" t="s">
-        <v>1061</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B22" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C22" t="s">
         <v>1062</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>1063</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>1064</v>
-      </c>
-      <c r="E22" t="s">
-        <v>1065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Fase 5 - test del backend (REV-051, REV-052, REV-053, REV-054)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A98A4F0-2D9F-4141-86AF-7B3D086734D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DE6127-D849-4D69-9BAD-35FD7861990C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2292" uniqueCount="1293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2330" uniqueCount="1310">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3229,9 +3229,6 @@
     <t>Alimenta NumeroPosti (REV-001)</t>
   </si>
   <si>
-    <t>TEST UNITARI - xUnit + Moq  (Totale: 42 test  |  Tutti OK)</t>
-  </si>
-  <si>
     <t>CalcolaCapienza_TavoloSingolo_NessunBonus</t>
   </si>
   <si>
@@ -3763,12 +3760,6 @@
     <t>Login, Register, Token JWT - primo avvio via /api/Setup (REV-007), seed-admin rimosso</t>
   </si>
   <si>
-    <t>74 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 74 test OK</t>
-  </si>
-  <si>
     <t>FASE 4 ROADMAP REVISIONE - Sicurezza e primo avvio (sessione 03/09/2026)</t>
   </si>
   <si>
@@ -3832,9 +3823,6 @@
     <t>Prossimo passo - Fase 5</t>
   </si>
   <si>
-    <t>Test del backend: copertura del flusso di prenotazione, oggi non toccato dai test verdi (REV-051 creazione e modifica, REV-052 assegnazione reale del tavolo, REV-053 disponibilita' dashboard e ruoli, REV-054 job notturni). A fine Fase 4 va decisa l'eventuale release intermedia v1.0.1.</t>
-  </si>
-  <si>
     <t>xUnit</t>
   </si>
   <si>
@@ -3847,9 +3835,6 @@
     <t>ASP.NET Core + Identity + React</t>
   </si>
   <si>
-    <t>74 test unitari con xUnit + Moq</t>
-  </si>
-  <si>
     <t>FASE 4 CHIUSA 03/09/2026. Schermata di primo avvio al posto di seed-admin pubblico (REV-007, backend + frontend), ForbiddenException a 403 senza logout (REV-025), NomeCliente riservato a Staff e Admin (REV-033), email fuori dai log di accesso (REV-070). Nessuna migration. Test 74/74. Primo avvio verificato end-to-end su DB locale ricreato da zero. Resta da decidere l'eventuale release intermedia v1.0.1.</t>
   </si>
   <si>
@@ -3859,9 +3844,6 @@
     <t>Test del backend: copertura del flusso di prenotazione (REV-051, REV-052, REV-053, REV-054)</t>
   </si>
   <si>
-    <t>Oggi i test verdi non toccano la creazione di una prenotazione ne' l'assegnazione reale del tavolo. Nessun task Fabio previsto.</t>
-  </si>
-  <si>
     <t>Sicurezza e primo avvio (REV-007, REV-025, REV-033, REV-070)</t>
   </si>
   <si>
@@ -3911,6 +3893,75 @@
   </si>
   <si>
     <t>Railway - PostgreSQL + .NET, health check /health - in produzione v1.0.1 (03/09/2026)</t>
+  </si>
+  <si>
+    <t>165 test unitari</t>
+  </si>
+  <si>
+    <t>Testing - 165 test OK</t>
+  </si>
+  <si>
+    <t>Test del backend: copertura del flusso di prenotazione (REV-051 creazione e modifica, REV-052 assegnazione reale del tavolo, REV-053 disponibilita' dashboard e ruoli, REV-054 job notturni). La release intermedia v1.0.1 e' stata decisa e fatta lo stesso giorno (vedi riga precedente).</t>
+  </si>
+  <si>
+    <t>FASE 5 ROADMAP REVISIONE - Test del backend (sessione 03/09/2026)</t>
+  </si>
+  <si>
+    <t>REV-052 - assegnazione reale del tavolo</t>
+  </si>
+  <si>
+    <t>Il vecchio PostazioneAssignmentServiceTests testava solo il motore puro AssegnazioneTavoli (rinominato in AssegnazioneTavoliTests, contenuto invariato). Ricreato da zero un nuovo PostazioneAssignmentServiceTests (16 test) sul metodo davvero usato in produzione, AssegnaPostazioneDisponibileAsync: filtro zone disattivate (REV-024), zona preferita, slot gia' occupati, distribuzione coperti sull'unione (REV-001).</t>
+  </si>
+  <si>
+    <t>REV-051 - creazione e modifica prenotazione</t>
+  </si>
+  <si>
+    <t>+45 test in PrenotazioniServiceTests: tetto MaxCoperti della fascia, giorno/stato fascia, zona preferita, limite una prenotazione al giorno (solo self-service), preavviso minimo 2h in modifica, contenuto scritto da AddAsync/UpdateAsync incluso NumeroPosti (rimasto a 0 fino al checkpoint 2b senza che nessun test se ne accorgesse).</t>
+  </si>
+  <si>
+    <t>REV-054 - job notturni</t>
+  </si>
+  <si>
+    <t>13 test sulla logica dei job (AutomaticCompletPrenotazioniAsync, AutomaticDeletePrenotazioniAsync) con orologio fisso, piu' nuovo JobsNotturniTests sui gusci Quartz veri: un'eccezione del service non deve uscire dal job, altrimenti Quartz la tratta da misfire.</t>
+  </si>
+  <si>
+    <t>xUnit + Moq + Quartz</t>
+  </si>
+  <si>
+    <t>REV-053 - disponibilita, dashboard, ruoli</t>
+  </si>
+  <si>
+    <t>DashboardServiceTests 1 a 17 test, +3 su DisponibilitaService, +7 sul validator, +6 sui ruoli (Admin testato per la prima volta, prima solo Staff), nuovo PrenotazioniRepositoryTests (filtro annullate e giorno/fascia, prima verificato solo dai mock).</t>
+  </si>
+  <si>
+    <t>Fase 5 chiusa - verifiche</t>
+  </si>
+  <si>
+    <t>dotnet test 165/165 (erano 74), dotnet build 0 errori/0 warning. Controllo di qualita': rotti temporaneamente due punti del codice (filtro zone disattivate, limite giornaliero) e verificato che solo i test attesi fallissero, poi ripristinato - nessun falso verde. Nessuna migration, nessuna azione richiesta a Fabio (fase solo di test automatici).</t>
+  </si>
+  <si>
+    <t>Prossimo passo - Fase 6</t>
+  </si>
+  <si>
+    <t>Bug del frontend: schermata bianca (REV-014), scelta zona non collegata al form (REV-015), modal di modifica prenotazione mancante (NEW-001), verifica dashboard su fuso orario lato client (REV-016), errore esplicito su indirizzo server mancante (REV-017), scadenza sessione pulita (REV-025).</t>
+  </si>
+  <si>
+    <t>React 19</t>
+  </si>
+  <si>
+    <t>165 test unitari con xUnit + Moq</t>
+  </si>
+  <si>
+    <t>FASE 5 CHIUSA 03/09/2026. dotnet test 165/165 (erano 74): REV-052 assegnazione reale del tavolo (era coperto solo il motore puro), REV-051 creazione/modifica prenotazione, REV-054 job notturni, REV-053 disponibilita/dashboard/ruoli. Nessuna migration, nessuna azione richiesta a Fabio.</t>
+  </si>
+  <si>
+    <t>Test del backend (REV-051, REV-052, REV-053, REV-054)</t>
+  </si>
+  <si>
+    <t>PostazioneAssignmentServiceTests ricreato sul metodo reale AssegnaPostazioneDisponibileAsync (16 test), motore puro rinominato in AssegnazioneTavoliTests; +45 test su creazione/modifica prenotazione in PrenotazioniServiceTests; +13 test sui job notturni + nuovo JobsNotturniTests sui gusci Quartz; DashboardServiceTests 1-&gt;17, +3 DisponibilitaService, +7 validator, +6 ruoli (Admin testato per la prima volta), nuovo PrenotazioniRepositoryTests. Controllo di qualita': mutazioni temporanee sul codice per verificare che i test nuovi sappiano davvero fallire. dotnet test 165/165 (erano 74), dotnet build pulita. Nessuna migration.</t>
+  </si>
+  <si>
+    <t>TEST UNITARI - xUnit + Moq  (Totale: 165 test  |  Tutti OK  |  elenco dettagliato fermo alla Fase 2b/42 test - da Fase 3 in poi il riepilogo per fase e' in ROADMAP_REVISIONE.md e nel foglio Appunti e Step)</t>
   </si>
 </sst>
 </file>
@@ -4177,7 +4228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4291,6 +4342,7 @@
     <xf numFmtId="49" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4635,36 +4687,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
-        <v>1209</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="A2" s="46" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="49" t="s">
+      <c r="B4" s="51"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="52"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -4681,7 +4733,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4771,7 +4823,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4804,10 +4856,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1243</v>
+        <v>1287</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1243</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4815,11 +4867,11 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1244</v>
+        <v>1288</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1244</v>
+        <v>1288</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -4839,7 +4891,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>1292</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4847,34 +4899,34 @@
       <c r="B15" s="34"/>
       <c r="C15" s="33"/>
       <c r="D15" s="35" t="s">
+        <v>1134</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="37" t="s">
         <v>1135</v>
       </c>
-      <c r="E15" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>1136</v>
-      </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="50"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="51"/>
+      <c r="B16" s="51"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="51"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="52"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4902,14 +4954,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>643</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5113,13 +5165,13 @@
     </row>
     <row r="13" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1279</v>
+        <v>1273</v>
       </c>
       <c r="B13" t="s">
         <v>665</v>
       </c>
       <c r="C13" t="s">
-        <v>1280</v>
+        <v>1274</v>
       </c>
       <c r="D13" t="s">
         <v>653</v>
@@ -5128,27 +5180,27 @@
         <v>437</v>
       </c>
       <c r="F13" t="s">
-        <v>1281</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>1279</v>
+        <v>1273</v>
       </c>
       <c r="B14" t="s">
         <v>651</v>
       </c>
       <c r="C14" t="s">
-        <v>1282</v>
+        <v>1276</v>
       </c>
       <c r="D14" t="s">
-        <v>1283</v>
+        <v>1277</v>
       </c>
       <c r="E14" t="s">
         <v>654</v>
       </c>
       <c r="F14" t="s">
-        <v>1284</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5419,7 +5471,7 @@
         <v>665</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>680</v>
@@ -5428,7 +5480,7 @@
         <v>437</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5702,13 +5754,13 @@
         <v>729</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>687</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>1278</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5992,13 +6044,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
-        <v>1065</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
+      <c r="A1" s="56" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6260,13 +6312,13 @@
         <v>794</v>
       </c>
       <c r="B18" s="11" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C18" s="11" t="s">
         <v>1066</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="D18" s="11" t="s">
         <v>1067</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>1068</v>
       </c>
       <c r="E18" s="39" t="s">
         <v>6</v>
@@ -6277,13 +6329,13 @@
         <v>794</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>1069</v>
       </c>
-      <c r="C19" s="14" t="s">
-        <v>1070</v>
-      </c>
       <c r="D19" s="14" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E19" s="39" t="s">
         <v>6</v>
@@ -6294,13 +6346,13 @@
         <v>794</v>
       </c>
       <c r="B20" s="11" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>1071</v>
       </c>
-      <c r="C20" s="11" t="s">
-        <v>1072</v>
-      </c>
       <c r="D20" s="11" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E20" s="39" t="s">
         <v>6</v>
@@ -6311,13 +6363,13 @@
         <v>794</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C21" s="14" t="s">
         <v>1073</v>
       </c>
-      <c r="C21" s="14" t="s">
-        <v>1074</v>
-      </c>
       <c r="D21" s="14" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E21" s="39" t="s">
         <v>6</v>
@@ -6328,13 +6380,13 @@
         <v>794</v>
       </c>
       <c r="B22" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C22" t="s">
         <v>1075</v>
       </c>
-      <c r="C22" t="s">
-        <v>1076</v>
-      </c>
       <c r="D22" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E22" s="27" t="s">
         <v>6</v>
@@ -6345,13 +6397,13 @@
         <v>794</v>
       </c>
       <c r="B23" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C23" t="s">
         <v>1077</v>
       </c>
-      <c r="C23" t="s">
-        <v>1078</v>
-      </c>
       <c r="D23" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E23" s="27" t="s">
         <v>6</v>
@@ -6362,13 +6414,13 @@
         <v>794</v>
       </c>
       <c r="B24" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C24" t="s">
         <v>1079</v>
       </c>
-      <c r="C24" t="s">
-        <v>1080</v>
-      </c>
       <c r="D24" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E24" s="27" t="s">
         <v>6</v>
@@ -6379,13 +6431,13 @@
         <v>794</v>
       </c>
       <c r="B25" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C25" t="s">
         <v>1081</v>
       </c>
-      <c r="C25" t="s">
-        <v>1082</v>
-      </c>
       <c r="D25" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E25" s="27" t="s">
         <v>6</v>
@@ -6396,13 +6448,13 @@
         <v>794</v>
       </c>
       <c r="B26" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C26" t="s">
         <v>1083</v>
       </c>
-      <c r="C26" t="s">
-        <v>1084</v>
-      </c>
       <c r="D26" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E26" s="27" t="s">
         <v>6</v>
@@ -6413,13 +6465,13 @@
         <v>794</v>
       </c>
       <c r="B27" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C27" t="s">
         <v>1085</v>
       </c>
-      <c r="C27" t="s">
-        <v>1086</v>
-      </c>
       <c r="D27" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E27" s="27" t="s">
         <v>6</v>
@@ -6430,13 +6482,13 @@
         <v>794</v>
       </c>
       <c r="B28" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C28" t="s">
         <v>1087</v>
       </c>
-      <c r="C28" t="s">
-        <v>1088</v>
-      </c>
       <c r="D28" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E28" s="27" t="s">
         <v>6</v>
@@ -6447,13 +6499,13 @@
         <v>794</v>
       </c>
       <c r="B29" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C29" t="s">
         <v>1089</v>
       </c>
-      <c r="C29" t="s">
-        <v>1090</v>
-      </c>
       <c r="D29" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E29" s="27" t="s">
         <v>6</v>
@@ -6464,13 +6516,13 @@
         <v>794</v>
       </c>
       <c r="B30" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C30" t="s">
         <v>1091</v>
       </c>
-      <c r="C30" t="s">
-        <v>1092</v>
-      </c>
       <c r="D30" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E30" s="27" t="s">
         <v>6</v>
@@ -6481,13 +6533,13 @@
         <v>794</v>
       </c>
       <c r="B31" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C31" t="s">
         <v>1093</v>
       </c>
-      <c r="C31" t="s">
-        <v>1094</v>
-      </c>
       <c r="D31" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E31" s="27" t="s">
         <v>6</v>
@@ -6498,13 +6550,13 @@
         <v>794</v>
       </c>
       <c r="B32" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C32" t="s">
         <v>1095</v>
       </c>
-      <c r="C32" t="s">
-        <v>1096</v>
-      </c>
       <c r="D32" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E32" s="27" t="s">
         <v>6</v>
@@ -6512,16 +6564,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B33" t="s">
         <v>1176</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>1177</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>1178</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1179</v>
       </c>
       <c r="E33" s="27" t="s">
         <v>6</v>
@@ -6529,16 +6581,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B34" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C34" t="s">
         <v>1180</v>
       </c>
-      <c r="C34" t="s">
-        <v>1181</v>
-      </c>
       <c r="D34" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -6546,16 +6598,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B35" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C35" t="s">
         <v>1182</v>
       </c>
-      <c r="C35" t="s">
-        <v>1183</v>
-      </c>
       <c r="D35" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -6563,16 +6615,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B36" t="s">
+        <v>1183</v>
+      </c>
+      <c r="C36" t="s">
         <v>1184</v>
       </c>
-      <c r="C36" t="s">
-        <v>1185</v>
-      </c>
       <c r="D36" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -6580,16 +6632,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B37" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C37" t="s">
         <v>1186</v>
       </c>
-      <c r="C37" t="s">
-        <v>1187</v>
-      </c>
       <c r="D37" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E37" s="27" t="s">
         <v>6</v>
@@ -6597,16 +6649,16 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B38" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C38" t="s">
         <v>1188</v>
       </c>
-      <c r="C38" t="s">
-        <v>1189</v>
-      </c>
       <c r="D38" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E38" s="27" t="s">
         <v>6</v>
@@ -6617,13 +6669,13 @@
         <v>772</v>
       </c>
       <c r="B39" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C39" t="s">
         <v>1190</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>1191</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1192</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -6634,13 +6686,13 @@
         <v>772</v>
       </c>
       <c r="B40" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C40" t="s">
         <v>1193</v>
       </c>
-      <c r="C40" t="s">
-        <v>1194</v>
-      </c>
       <c r="D40" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -6651,13 +6703,13 @@
         <v>772</v>
       </c>
       <c r="B41" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C41" t="s">
         <v>1195</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>1196</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1197</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -6668,13 +6720,13 @@
         <v>772</v>
       </c>
       <c r="B42" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C42" t="s">
         <v>1198</v>
       </c>
-      <c r="C42" t="s">
-        <v>1199</v>
-      </c>
       <c r="D42" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="E42" s="27" t="s">
         <v>6</v>
@@ -6685,13 +6737,13 @@
         <v>772</v>
       </c>
       <c r="B43" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C43" t="s">
         <v>1200</v>
       </c>
-      <c r="C43" t="s">
-        <v>1201</v>
-      </c>
       <c r="D43" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>6</v>
@@ -6702,13 +6754,13 @@
         <v>772</v>
       </c>
       <c r="B44" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C44" t="s">
         <v>1202</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>1203</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1204</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>6</v>
@@ -6719,13 +6771,13 @@
         <v>772</v>
       </c>
       <c r="B45" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C45" t="s">
         <v>1205</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>1206</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1207</v>
       </c>
       <c r="E45" s="27" t="s">
         <v>6</v>
@@ -6750,11 +6802,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>795</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7020,14 +7072,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>841</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7108,7 +7160,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7120,40 +7172,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
-        <v>1210</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
+      <c r="A2" s="46" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="51"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="52"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -7476,16 +7528,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="49" t="s">
+      <c r="A22" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="50"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="51"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="51"/>
+      <c r="H22" s="52"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -7708,16 +7760,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="53" t="s">
+      <c r="A35" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="B35" s="50"/>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="51"/>
+      <c r="B35" s="51"/>
+      <c r="C35" s="51"/>
+      <c r="D35" s="51"/>
+      <c r="E35" s="51"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="51"/>
+      <c r="H35" s="52"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -7900,16 +7952,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="54" t="s">
+      <c r="A46" s="55" t="s">
         <v>173</v>
       </c>
-      <c r="B46" s="50"/>
-      <c r="C46" s="50"/>
-      <c r="D46" s="50"/>
-      <c r="E46" s="50"/>
-      <c r="F46" s="50"/>
-      <c r="G46" s="50"/>
-      <c r="H46" s="51"/>
+      <c r="B46" s="51"/>
+      <c r="C46" s="51"/>
+      <c r="D46" s="51"/>
+      <c r="E46" s="51"/>
+      <c r="F46" s="51"/>
+      <c r="G46" s="51"/>
+      <c r="H46" s="52"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -7972,16 +8024,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="52" t="s">
+      <c r="A51" s="53" t="s">
         <v>185</v>
       </c>
-      <c r="B51" s="50"/>
-      <c r="C51" s="50"/>
-      <c r="D51" s="50"/>
-      <c r="E51" s="50"/>
-      <c r="F51" s="50"/>
-      <c r="G51" s="50"/>
-      <c r="H51" s="51"/>
+      <c r="B51" s="51"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="51"/>
+      <c r="E51" s="51"/>
+      <c r="F51" s="51"/>
+      <c r="G51" s="51"/>
+      <c r="H51" s="52"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -8194,24 +8246,24 @@
     </row>
     <row r="71" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="44" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="B71" s="25" t="s">
+        <v>1226</v>
+      </c>
+      <c r="C71" s="25" t="s">
         <v>1227</v>
-      </c>
-      <c r="C71" s="25" t="s">
-        <v>1228</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="44" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="B72" s="25" t="s">
+        <v>1228</v>
+      </c>
+      <c r="C72" s="25" t="s">
         <v>1229</v>
-      </c>
-      <c r="C72" s="25" t="s">
-        <v>1230</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -9348,7 +9400,7 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
@@ -9376,16 +9428,16 @@
         <v>1</v>
       </c>
       <c r="B153" s="27" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C153" s="27" t="s">
         <v>1104</v>
       </c>
-      <c r="C153" s="27" t="s">
+      <c r="D153" s="27" t="s">
         <v>1105</v>
       </c>
-      <c r="D153" s="27" t="s">
-        <v>1106</v>
-      </c>
       <c r="E153" s="40" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="F153" s="27" t="s">
         <v>6</v>
@@ -9396,16 +9448,16 @@
         <v>2</v>
       </c>
       <c r="B154" s="27" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C154" s="27" t="s">
         <v>1107</v>
       </c>
-      <c r="C154" s="27" t="s">
+      <c r="D154" s="27" t="s">
         <v>1108</v>
       </c>
-      <c r="D154" s="27" t="s">
-        <v>1109</v>
-      </c>
       <c r="E154" s="40" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="F154" s="27" t="s">
         <v>6</v>
@@ -9416,16 +9468,16 @@
         <v>3</v>
       </c>
       <c r="B155" s="27" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C155" s="27" t="s">
         <v>1110</v>
       </c>
-      <c r="C155" s="27" t="s">
+      <c r="D155" s="27" t="s">
         <v>1111</v>
       </c>
-      <c r="D155" s="27" t="s">
-        <v>1112</v>
-      </c>
       <c r="E155" s="40" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="F155" s="27" t="s">
         <v>6</v>
@@ -9436,16 +9488,16 @@
         <v>4</v>
       </c>
       <c r="B156" s="27" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C156" s="27" t="s">
         <v>1113</v>
       </c>
-      <c r="C156" s="27" t="s">
+      <c r="D156" s="27" t="s">
         <v>1114</v>
       </c>
-      <c r="D156" s="27" t="s">
-        <v>1115</v>
-      </c>
       <c r="E156" s="40" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="F156" s="27" t="s">
         <v>6</v>
@@ -9456,16 +9508,16 @@
         <v>5</v>
       </c>
       <c r="B157" s="27" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C157" s="27" t="s">
+        <v>1127</v>
+      </c>
+      <c r="D157" s="27" t="s">
         <v>1116</v>
       </c>
-      <c r="C157" s="27" t="s">
-        <v>1128</v>
-      </c>
-      <c r="D157" s="27" t="s">
-        <v>1117</v>
-      </c>
       <c r="E157" s="40" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="F157" s="27" t="s">
         <v>6</v>
@@ -9476,16 +9528,16 @@
         <v>6</v>
       </c>
       <c r="B158" s="41" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C158" s="41" t="s">
         <v>1129</v>
-      </c>
-      <c r="C158" s="41" t="s">
-        <v>1130</v>
       </c>
       <c r="D158" s="41" t="s">
         <v>267</v>
       </c>
       <c r="E158" s="42" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="F158" s="27" t="s">
         <v>6</v>
@@ -9493,7 +9545,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
@@ -9521,16 +9573,16 @@
         <v>1</v>
       </c>
       <c r="B162" s="27" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C162" s="27" t="s">
         <v>1138</v>
       </c>
-      <c r="C162" s="27" t="s">
+      <c r="D162" s="27" t="s">
         <v>1139</v>
       </c>
-      <c r="D162" s="27" t="s">
+      <c r="E162" s="40" t="s">
         <v>1140</v>
-      </c>
-      <c r="E162" s="40" t="s">
-        <v>1141</v>
       </c>
       <c r="F162" s="27" t="s">
         <v>6</v>
@@ -9541,16 +9593,16 @@
         <v>2</v>
       </c>
       <c r="B163" s="27" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C163" s="27" t="s">
         <v>1142</v>
       </c>
-      <c r="C163" s="27" t="s">
+      <c r="D163" s="27" t="s">
         <v>1143</v>
       </c>
-      <c r="D163" s="27" t="s">
-        <v>1144</v>
-      </c>
       <c r="E163" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F163" s="27" t="s">
         <v>6</v>
@@ -9561,16 +9613,16 @@
         <v>3</v>
       </c>
       <c r="B164" s="27" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C164" s="27" t="s">
         <v>1145</v>
       </c>
-      <c r="C164" s="27" t="s">
+      <c r="D164" s="27" t="s">
         <v>1146</v>
       </c>
-      <c r="D164" s="27" t="s">
-        <v>1147</v>
-      </c>
       <c r="E164" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F164" s="27" t="s">
         <v>6</v>
@@ -9581,16 +9633,16 @@
         <v>4</v>
       </c>
       <c r="B165" s="27" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C165" s="27" t="s">
         <v>1148</v>
       </c>
-      <c r="C165" s="27" t="s">
+      <c r="D165" s="27" t="s">
         <v>1149</v>
       </c>
-      <c r="D165" s="27" t="s">
-        <v>1150</v>
-      </c>
       <c r="E165" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F165" s="27" t="s">
         <v>6</v>
@@ -9601,16 +9653,16 @@
         <v>5</v>
       </c>
       <c r="B166" s="27" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C166" s="27" t="s">
         <v>1151</v>
       </c>
-      <c r="C166" s="27" t="s">
+      <c r="D166" s="27" t="s">
         <v>1152</v>
       </c>
-      <c r="D166" s="27" t="s">
-        <v>1153</v>
-      </c>
       <c r="E166" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F166" s="27" t="s">
         <v>6</v>
@@ -9621,16 +9673,16 @@
         <v>6</v>
       </c>
       <c r="B167" s="27" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C167" s="27" t="s">
         <v>1154</v>
       </c>
-      <c r="C167" s="27" t="s">
+      <c r="D167" s="27" t="s">
         <v>1155</v>
       </c>
-      <c r="D167" s="27" t="s">
-        <v>1156</v>
-      </c>
       <c r="E167" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F167" s="27" t="s">
         <v>6</v>
@@ -9641,16 +9693,16 @@
         <v>7</v>
       </c>
       <c r="B168" s="27" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C168" s="27" t="s">
         <v>1157</v>
-      </c>
-      <c r="C168" s="27" t="s">
-        <v>1158</v>
       </c>
       <c r="D168" s="27" t="s">
         <v>1019</v>
       </c>
       <c r="E168" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F168" s="27" t="s">
         <v>6</v>
@@ -9661,16 +9713,16 @@
         <v>8</v>
       </c>
       <c r="B169" s="27" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C169" s="27" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D169" s="27" t="s">
         <v>1159</v>
       </c>
-      <c r="C169" s="27" t="s">
-        <v>1208</v>
-      </c>
-      <c r="D169" s="27" t="s">
-        <v>1160</v>
-      </c>
       <c r="E169" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F169" s="27" t="s">
         <v>6</v>
@@ -9681,16 +9733,16 @@
         <v>9</v>
       </c>
       <c r="B170" s="27" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C170" s="27" t="s">
         <v>1161</v>
       </c>
-      <c r="C170" s="27" t="s">
+      <c r="D170" s="27" t="s">
         <v>1162</v>
       </c>
-      <c r="D170" s="27" t="s">
-        <v>1163</v>
-      </c>
       <c r="E170" s="40" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="F170" s="27" t="s">
         <v>6</v>
@@ -9698,7 +9750,7 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
@@ -9726,16 +9778,16 @@
         <v>1</v>
       </c>
       <c r="B174" s="27" t="s">
+        <v>1211</v>
+      </c>
+      <c r="C174" s="27" t="s">
         <v>1212</v>
       </c>
-      <c r="C174" s="27" t="s">
+      <c r="D174" s="27" t="s">
         <v>1213</v>
       </c>
-      <c r="D174" s="27" t="s">
+      <c r="E174" s="40" t="s">
         <v>1214</v>
-      </c>
-      <c r="E174" s="40" t="s">
-        <v>1215</v>
       </c>
       <c r="F174" s="27" t="s">
         <v>6</v>
@@ -9746,16 +9798,16 @@
         <v>2</v>
       </c>
       <c r="B175" s="27" t="s">
+        <v>1215</v>
+      </c>
+      <c r="C175" s="27" t="s">
         <v>1216</v>
       </c>
-      <c r="C175" s="27" t="s">
+      <c r="D175" s="27" t="s">
         <v>1217</v>
       </c>
-      <c r="D175" s="27" t="s">
-        <v>1218</v>
-      </c>
       <c r="E175" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F175" s="27" t="s">
         <v>6</v>
@@ -9766,16 +9818,16 @@
         <v>3</v>
       </c>
       <c r="B176" s="27" t="s">
+        <v>1218</v>
+      </c>
+      <c r="C176" s="27" t="s">
         <v>1219</v>
       </c>
-      <c r="C176" s="27" t="s">
+      <c r="D176" s="27" t="s">
         <v>1220</v>
       </c>
-      <c r="D176" s="27" t="s">
-        <v>1221</v>
-      </c>
       <c r="E176" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F176" s="27" t="s">
         <v>6</v>
@@ -9786,19 +9838,19 @@
         <v>4</v>
       </c>
       <c r="B177" s="27" t="s">
+        <v>1221</v>
+      </c>
+      <c r="C177" s="27" t="s">
         <v>1222</v>
       </c>
-      <c r="C177" s="27" t="s">
+      <c r="D177" s="27" t="s">
         <v>1223</v>
       </c>
-      <c r="D177" s="27" t="s">
-        <v>1224</v>
-      </c>
       <c r="E177" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F177" s="43" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
@@ -9806,16 +9858,16 @@
         <v>5</v>
       </c>
       <c r="B178" s="27" t="s">
+        <v>1224</v>
+      </c>
+      <c r="C178" s="27" t="s">
         <v>1225</v>
-      </c>
-      <c r="C178" s="27" t="s">
-        <v>1226</v>
       </c>
       <c r="D178" s="27" t="s">
         <v>437</v>
       </c>
       <c r="E178" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F178" s="27" t="s">
         <v>6</v>
@@ -9823,7 +9875,7 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>1245</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -9851,16 +9903,16 @@
         <v>1</v>
       </c>
       <c r="B182" s="27" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="C182" s="27" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="D182" s="27" t="s">
-        <v>1248</v>
+        <v>1245</v>
       </c>
       <c r="E182" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F182" s="27" t="s">
         <v>6</v>
@@ -9871,16 +9923,16 @@
         <v>2</v>
       </c>
       <c r="B183" s="27" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="C183" s="27" t="s">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="D183" s="27" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="E183" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F183" s="27" t="s">
         <v>6</v>
@@ -9891,16 +9943,16 @@
         <v>3</v>
       </c>
       <c r="B184" s="27" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="C184" s="27" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="D184" s="27" t="s">
-        <v>1254</v>
+        <v>1251</v>
       </c>
       <c r="E184" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F184" s="27" t="s">
         <v>6</v>
@@ -9911,16 +9963,16 @@
         <v>4</v>
       </c>
       <c r="B185" s="27" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="C185" s="27" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="D185" s="27" t="s">
         <v>401</v>
       </c>
       <c r="E185" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F185" s="27" t="s">
         <v>6</v>
@@ -9931,16 +9983,16 @@
         <v>5</v>
       </c>
       <c r="B186" s="27" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="C186" s="27" t="s">
-        <v>1258</v>
+        <v>1255</v>
       </c>
       <c r="D186" s="27" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
       <c r="E186" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F186" s="27" t="s">
         <v>6</v>
@@ -9951,16 +10003,16 @@
         <v>6</v>
       </c>
       <c r="B187" s="27" t="s">
-        <v>1260</v>
+        <v>1257</v>
       </c>
       <c r="C187" s="27" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="D187" s="27" t="s">
-        <v>1262</v>
+        <v>1259</v>
       </c>
       <c r="E187" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F187" s="27" t="s">
         <v>6</v>
@@ -9971,19 +10023,19 @@
         <v>7</v>
       </c>
       <c r="B188" s="27" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="C188" s="27" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="D188" s="27" t="s">
         <v>22</v>
       </c>
       <c r="E188" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F188" s="43" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
@@ -9991,16 +10043,16 @@
         <v>8</v>
       </c>
       <c r="B189" s="27" t="s">
-        <v>1285</v>
+        <v>1279</v>
       </c>
       <c r="C189" s="27" t="s">
-        <v>1286</v>
+        <v>1280</v>
       </c>
       <c r="D189" s="27" t="s">
-        <v>1287</v>
+        <v>1281</v>
       </c>
       <c r="E189" s="40" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F189" s="27" t="s">
         <v>6</v>
@@ -10011,18 +10063,163 @@
         <v>9</v>
       </c>
       <c r="B190" s="27" t="s">
-        <v>1265</v>
+        <v>1262</v>
       </c>
       <c r="C190" s="27" t="s">
-        <v>1266</v>
+        <v>1289</v>
       </c>
       <c r="D190" s="27" t="s">
-        <v>1267</v>
+        <v>1263</v>
       </c>
       <c r="E190" s="40" t="s">
         <v>437</v>
       </c>
-      <c r="F190" s="38" t="s">
+      <c r="F190" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B191" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>39</v>
+      </c>
+      <c r="B192" t="s">
+        <v>40</v>
+      </c>
+      <c r="C192" t="s">
+        <v>857</v>
+      </c>
+      <c r="D192" t="s">
+        <v>42</v>
+      </c>
+      <c r="E192" t="s">
+        <v>43</v>
+      </c>
+      <c r="F192" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A193">
+        <v>1</v>
+      </c>
+      <c r="B193" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C193" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D193" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E193" s="45">
+        <v>46090</v>
+      </c>
+      <c r="F193" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A194">
+        <v>2</v>
+      </c>
+      <c r="B194" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C194" t="s">
+        <v>1294</v>
+      </c>
+      <c r="D194" t="s">
+        <v>74</v>
+      </c>
+      <c r="E194" s="45">
+        <v>46090</v>
+      </c>
+      <c r="F194" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A195">
+        <v>3</v>
+      </c>
+      <c r="B195" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C195" t="s">
+        <v>1296</v>
+      </c>
+      <c r="D195" t="s">
+        <v>1297</v>
+      </c>
+      <c r="E195" s="45">
+        <v>46090</v>
+      </c>
+      <c r="F195" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A196">
+        <v>4</v>
+      </c>
+      <c r="B196" t="s">
+        <v>1298</v>
+      </c>
+      <c r="C196" t="s">
+        <v>1299</v>
+      </c>
+      <c r="D196" t="s">
+        <v>74</v>
+      </c>
+      <c r="E196" s="45">
+        <v>46090</v>
+      </c>
+      <c r="F196" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A197">
+        <v>5</v>
+      </c>
+      <c r="B197" t="s">
+        <v>1300</v>
+      </c>
+      <c r="C197" t="s">
+        <v>1301</v>
+      </c>
+      <c r="D197" t="s">
+        <v>1259</v>
+      </c>
+      <c r="E197" s="45">
+        <v>46090</v>
+      </c>
+      <c r="F197" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A198">
+        <v>6</v>
+      </c>
+      <c r="B198" t="s">
+        <v>1302</v>
+      </c>
+      <c r="C198" t="s">
+        <v>1303</v>
+      </c>
+      <c r="D198" t="s">
+        <v>1304</v>
+      </c>
+      <c r="E198" t="s">
+        <v>437</v>
+      </c>
+      <c r="F198" s="38" t="s">
         <v>979</v>
       </c>
     </row>
@@ -10053,24 +10250,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="57" t="s">
         <v>221</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="51"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="52"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -10158,14 +10355,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="53" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="50"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="51"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="52"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -10253,14 +10450,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="49" t="s">
+      <c r="A17" s="50" t="s">
         <v>255</v>
       </c>
-      <c r="B17" s="50"/>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="51"/>
+      <c r="B17" s="51"/>
+      <c r="C17" s="51"/>
+      <c r="D17" s="51"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="52"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -10382,14 +10579,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="49" t="s">
+      <c r="A26" s="50" t="s">
         <v>279</v>
       </c>
-      <c r="B26" s="50"/>
-      <c r="C26" s="50"/>
-      <c r="D26" s="50"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="51"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="52"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -10467,7 +10664,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1271</v>
+        <v>1305</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -10532,13 +10729,13 @@
         <v>1043</v>
       </c>
       <c r="B35" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="C35" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D35" t="s">
         <v>1164</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1165</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -10549,13 +10746,13 @@
         <v>1043</v>
       </c>
       <c r="B36" t="s">
-        <v>1268</v>
+        <v>1264</v>
       </c>
       <c r="C36" t="s">
-        <v>1269</v>
+        <v>1265</v>
       </c>
       <c r="D36" t="s">
-        <v>1270</v>
+        <v>1266</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -10587,26 +10784,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="53" t="s">
         <v>289</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="51"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="52"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -10951,22 +11148,22 @@
         <v>1008</v>
       </c>
       <c r="B20" s="27" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C20" s="27" t="s">
         <v>1098</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="D20" s="27" t="s">
         <v>1099</v>
       </c>
-      <c r="D20" s="27" t="s">
-        <v>1100</v>
-      </c>
       <c r="E20" s="27" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="F20" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -10974,22 +11171,22 @@
         <v>1008</v>
       </c>
       <c r="B21" s="41" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C21" s="41" t="s">
         <v>1133</v>
       </c>
-      <c r="C21" s="41" t="s">
-        <v>1134</v>
-      </c>
       <c r="D21" s="41" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="E21" s="41" t="s">
+        <v>1230</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="41" t="s">
         <v>1231</v>
-      </c>
-      <c r="F21" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="G21" s="41" t="s">
-        <v>1232</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -10997,45 +11194,45 @@
         <v>1008</v>
       </c>
       <c r="B22" s="41" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C22" s="41" t="s">
         <v>1167</v>
       </c>
-      <c r="C22" s="41" t="s">
-        <v>1168</v>
-      </c>
       <c r="D22" s="41" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="E22" s="41" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="F22" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1272</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="41" t="s">
-        <v>1288</v>
+        <v>1282</v>
       </c>
       <c r="B23" s="41" t="s">
-        <v>1289</v>
+        <v>1283</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>1290</v>
+        <v>1284</v>
       </c>
       <c r="D23" s="41" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="E23" s="41" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="F23" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G23" s="41" t="s">
-        <v>1291</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -11043,18 +11240,22 @@
         <v>1008</v>
       </c>
       <c r="B24" s="41" t="s">
-        <v>1273</v>
+        <v>1268</v>
       </c>
       <c r="C24" s="41" t="s">
-        <v>1274</v>
-      </c>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="43" t="s">
-        <v>1131</v>
+        <v>1269</v>
+      </c>
+      <c r="D24" s="41" t="s">
+        <v>1230</v>
+      </c>
+      <c r="E24" s="41" t="s">
+        <v>1230</v>
+      </c>
+      <c r="F24" s="27" t="s">
+        <v>6</v>
       </c>
       <c r="G24" s="41" t="s">
-        <v>1275</v>
+        <v>1306</v>
       </c>
     </row>
   </sheetData>
@@ -11068,7 +11269,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -11078,24 +11279,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>346</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="50" t="s">
         <v>347</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="51"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="52"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -11280,14 +11481,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="56" t="s">
+      <c r="A18" s="57" t="s">
         <v>379</v>
       </c>
-      <c r="B18" s="50"/>
-      <c r="C18" s="50"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="51"/>
+      <c r="B18" s="51"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="52"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -11394,14 +11595,14 @@
       <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="52" t="s">
+      <c r="A28" s="53" t="s">
         <v>392</v>
       </c>
-      <c r="B28" s="50"/>
-      <c r="C28" s="50"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="50"/>
-      <c r="F28" s="51"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="52"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -11531,13 +11732,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="27" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B38" s="27" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C38" s="27" t="s">
         <v>1101</v>
-      </c>
-      <c r="C38" s="27" t="s">
-        <v>1102</v>
       </c>
       <c r="D38" s="27" t="s">
         <v>6</v>
@@ -11545,41 +11746,41 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="41" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B39" s="41" t="s">
         <v>1122</v>
       </c>
-      <c r="B39" s="41" t="s">
+      <c r="C39" s="41" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D39" s="41" t="s">
         <v>1123</v>
-      </c>
-      <c r="C39" s="41" t="s">
-        <v>1175</v>
-      </c>
-      <c r="D39" s="41" t="s">
-        <v>1124</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="41" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B40" s="41" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C40" s="41" t="s">
         <v>1125</v>
       </c>
-      <c r="C40" s="41" t="s">
+      <c r="D40" s="41" t="s">
         <v>1126</v>
-      </c>
-      <c r="D40" s="41" t="s">
-        <v>1127</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="27" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="B41" s="27" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C41" s="27" t="s">
         <v>1169</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>1170</v>
       </c>
       <c r="D41" s="27" t="s">
         <v>6</v>
@@ -11587,27 +11788,27 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="41" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B42" s="41" t="s">
         <v>1171</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="C42" s="41" t="s">
         <v>1172</v>
       </c>
-      <c r="C42" s="41" t="s">
+      <c r="D42" s="43" t="s">
         <v>1173</v>
-      </c>
-      <c r="D42" s="43" t="s">
-        <v>1174</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="41" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B43" s="41" t="s">
         <v>1233</v>
       </c>
-      <c r="B43" s="41" t="s">
+      <c r="C43" s="41" t="s">
         <v>1234</v>
-      </c>
-      <c r="C43" s="41" t="s">
-        <v>1235</v>
       </c>
       <c r="D43" s="27" t="s">
         <v>6</v>
@@ -11615,43 +11816,57 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="41" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B44" s="41" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C44" s="41" t="s">
         <v>1236</v>
       </c>
-      <c r="C44" s="41" t="s">
-        <v>1237</v>
-      </c>
       <c r="D44" s="43" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="41" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B45" s="41" t="s">
         <v>1238</v>
       </c>
-      <c r="B45" s="41" t="s">
+      <c r="C45" s="41" t="s">
         <v>1239</v>
       </c>
-      <c r="C45" s="41" t="s">
+      <c r="D45" s="43" t="s">
         <v>1240</v>
-      </c>
-      <c r="D45" s="43" t="s">
-        <v>1241</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="27" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>1276</v>
+        <v>1270</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>1277</v>
+        <v>1271</v>
       </c>
       <c r="D46" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1308</v>
+      </c>
+      <c r="D47" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -11679,14 +11894,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>404</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -11863,14 +12078,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>427</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -12473,13 +12688,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>503</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -12876,13 +13091,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="56" t="s">
         <v>582</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
feat: Fase 6 - bug del frontend (REV-014, REV-015, REV-016, REV-017, REV-025, NEW-001, NEW-004)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DE6127-D849-4D69-9BAD-35FD7861990C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ECFA5CE-5A8F-4DA2-A227-AAB39471C163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2330" uniqueCount="1310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2408" uniqueCount="1361">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3403,9 +3403,6 @@
     <t>NEW-001: modal di modifica prenotazione</t>
   </si>
   <si>
-    <t>Pianificato (Fase 6)</t>
-  </si>
-  <si>
     <t>NEW-002: pannello disponibilita' nel form di creazione (opzionale)</t>
   </si>
   <si>
@@ -3556,9 +3553,6 @@
     <t>Pianificato (Fase 7)</t>
   </si>
   <si>
-    <t>Nessun pulsante Modifica nelle prenotazioni (solo Conferma-Completa-Annulla). update-prenotazione e' capacita' solo-backend: il fix REV-002 non e' raggiungibile dall'app. Riusare PrenotazioneModal (prop prenotazione + precompilazione + mutation PUT + pulsante per stato Attiva). Da fare in Fase 6 insieme a REV-015 (stesso componente). Riscontrato di nuovo il 02/09/2026 durante i test di Fase 3: la prova di modifica e' stata possibile solo via Swagger.</t>
-  </si>
-  <si>
     <t>DbExceptionTranslatorTests</t>
   </si>
   <si>
@@ -3658,12 +3652,6 @@
     <t>Due POST crea-prenotazione realmente simultanee (due SendAsync su HttpClient senza attesa reciproca) su una zona di test con un solo tavolo da 2: HTTP 201 + HTTP 409 'Il tavolo e' stato appena assegnato a un'altra prenotazione'. Il controllo applicativo aveva visto il tavolo libero per entrambe: a fermare la seconda e' stato l'unique index. Restano commit/push e pulizia dei dati di test in produzione prima della chiusura formale (DoD punto 5).</t>
   </si>
   <si>
-    <t>Aggiornato: 03/09/2026</t>
-  </si>
-  <si>
-    <t>Aggiornato: 03/09/2026 - Percorso: Backend -&gt; Frontend React/TS -&gt; Mobile React Native</t>
-  </si>
-  <si>
     <t>FASE 3 ROADMAP REVISIONE - Chiusura formale, sicurezza repository e credenziali (sessione 03/09/2026)</t>
   </si>
   <si>
@@ -3742,9 +3730,6 @@
     <t>NEW-004: hook useDeletePrenotazione mai collegato all'interfaccia</t>
   </si>
   <si>
-    <t>usePrenotazioni.ts espone useDeletePrenotazione ma nessun componente lo usa: nel frontend esiste solo Annulla, non Elimina. Stesso schema di NEW-001 (modifica): capacita' backend non raggiungibile dall'app, l'eliminazione passa solo da Postman. Emerso il 03/09 durante la pulizia dei dati di test. Da valutare in Fase 6 insieme a NEW-001, stesso componente.</t>
-  </si>
-  <si>
     <t>Produzione - Database</t>
   </si>
   <si>
@@ -3895,12 +3880,6 @@
     <t>Railway - PostgreSQL + .NET, health check /health - in produzione v1.0.1 (03/09/2026)</t>
   </si>
   <si>
-    <t>165 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 165 test OK</t>
-  </si>
-  <si>
     <t>Test del backend: copertura del flusso di prenotazione (REV-051 creazione e modifica, REV-052 assegnazione reale del tavolo, REV-053 disponibilita' dashboard e ruoli, REV-054 job notturni). La release intermedia v1.0.1 e' stata decisa e fatta lo stesso giorno (vedi riga precedente).</t>
   </si>
   <si>
@@ -3937,9 +3916,6 @@
     <t>Fase 5 chiusa - verifiche</t>
   </si>
   <si>
-    <t>dotnet test 165/165 (erano 74), dotnet build 0 errori/0 warning. Controllo di qualita': rotti temporaneamente due punti del codice (filtro zone disattivate, limite giornaliero) e verificato che solo i test attesi fallissero, poi ripristinato - nessun falso verde. Nessuna migration, nessuna azione richiesta a Fabio (fase solo di test automatici).</t>
-  </si>
-  <si>
     <t>Prossimo passo - Fase 6</t>
   </si>
   <si>
@@ -3949,9 +3925,6 @@
     <t>React 19</t>
   </si>
   <si>
-    <t>165 test unitari con xUnit + Moq</t>
-  </si>
-  <si>
     <t>FASE 5 CHIUSA 03/09/2026. dotnet test 165/165 (erano 74): REV-052 assegnazione reale del tavolo (era coperto solo il motore puro), REV-051 creazione/modifica prenotazione, REV-054 job notturni, REV-053 disponibilita/dashboard/ruoli. Nessuna migration, nessuna azione richiesta a Fabio.</t>
   </si>
   <si>
@@ -3962,6 +3935,186 @@
   </si>
   <si>
     <t>TEST UNITARI - xUnit + Moq  (Totale: 165 test  |  Tutti OK  |  elenco dettagliato fermo alla Fase 2b/42 test - da Fase 3 in poi il riepilogo per fase e' in ROADMAP_REVISIONE.md e nel foglio Appunti e Step)</t>
+  </si>
+  <si>
+    <t>In corso</t>
+  </si>
+  <si>
+    <t>FASE 6 ROADMAP REVISIONE - Bug del frontend (sessione 04/09/2026)</t>
+  </si>
+  <si>
+    <t>REV-017 - indirizzo del server mancante</t>
+  </si>
+  <si>
+    <t>lib/axios.ts si ferma all'avvio con un messaggio esplicito se VITE_API_URL non e' impostata. Prima baseURL restava undefined e Axios chiamava URL relativi: le richieste finivano sull'host del frontend, che risponde con l'HTML della SPA, e l'utente vedeva errori di parsing incomprensibili invece della causa vera (variabile di deploy non configurata).</t>
+  </si>
+  <si>
+    <t>Axios + variabili Vite</t>
+  </si>
+  <si>
+    <t>REV-014 - schermata bianca</t>
+  </si>
+  <si>
+    <t>AuthContext decodificava il token con JSON.parse(atob(...)) senza protezione, dentro l'inizializzatore di useState del provider che avvolge l'intero router: un token troncato in localStorage faceva esplodere il primo render e nemmeno /login era raggiungibile. Ora il token illeggibile viene scartato e ripulito (si riparte anonimi), incluso quello gia' scaduto via claim exp. Aggiunto un ErrorBoundary sopra AuthProvider come rete di sicurezza, con Ricarica e Torna al login. Rimossa anche la seconda decodifica non protetta che stava in LoginPage: ora login() restituisce l'utente gia' decodificato.</t>
+  </si>
+  <si>
+    <t>React 19 + JWT + Error Boundary</t>
+  </si>
+  <si>
+    <t>REV-025 - scadenza sessione pulita</t>
+  </si>
+  <si>
+    <t>Su 401 con token presente l'interceptor faceva window.location.href = '/login': ricaricamento a pagina intera, nessun messaggio, sembrava un crash. Nuovo lib/session.ts come ponte fra l'interceptor (che vive fuori da React) e i componenti; AppLayout si registra e reagisce con logout, queryClient.clear(), toast 'Sessione scaduta' e navigazione senza reload. Il redirect duro resta solo come fallback se nessuno e' in ascolto. Il logout manuale ora svuota anch'esso la cache delle query.</t>
+  </si>
+  <si>
+    <t>Axios interceptor + React Query</t>
+  </si>
+  <si>
+    <t>REV-016 - dashboard e fuso orario lato client</t>
+  </si>
+  <si>
+    <t>Non era solo da verificare: il bug era vivo. DashboardPage calcolava sia la data di oggi sia il lunedi' corrente con toISOString(), cioe' in UTC, quindi fra mezzanotte e le due mostrava la giornata precedente e il lunedi' scivolava a domenica - proprio cio' che IClock.TodayInRome aveva risolto lato backend. Nuovo lib/date.ts con oggiInItalia() e lunediSettimanaCorrenteInItalia(), fuso Europe/Rome fissato nel codice (il locale e' del ristorante, non del dispositivo di chi guarda).</t>
+  </si>
+  <si>
+    <t>Intl.DateTimeFormat + Europe/Rome</t>
+  </si>
+  <si>
+    <t>REV-015 - scelta zona non collegata al form</t>
+  </si>
+  <si>
+    <t>La select della zona non era registrata in react-hook-form: era gestita a mano con onChange + setValue. Il valore arrivava al submit, ma il campo restava fuori dal controllo del form, quindi reset() alla chiusura del modal non ripuliva il DOM: riaprendo si vedeva ancora la zona scelta prima mentre il form era tornato a 'nessuna preferenza', e si prenotava credendo di aver scelto una zona. Ora e' un campo registrato come gli altri, con setValueAs che traduce la stringa vuota in null.</t>
+  </si>
+  <si>
+    <t>React Hook Form</t>
+  </si>
+  <si>
+    <t>NEW-001 - modal di modifica prenotazione</t>
+  </si>
+  <si>
+    <t>La modifica esisteva solo lato backend: nessun hook, nessun pulsante, quindi il fix REV-002 (Admin e Staff modificano la prenotazione di un cliente) non era raggiungibile dall'app. Nuovo hook useModificaPrenotazione (PUT update-prenotazione), prop opzionale prenotazione su PrenotazioneModal con precompilazione, pulsante Modifica in colonna Azioni sulle prenotazioni Attive. Nessuna modifica al backend: PrenotazioneDTO esponeva gia' FasciaOrariaId e ZonaId, mancavano solo nei type TypeScript. Le due select si precompilano dopo il caricamento delle rispettive liste, altrimenti il valore cadrebbe a vuoto per assenza delle option.</t>
+  </si>
+  <si>
+    <t>React Query + React Hook Form</t>
+  </si>
+  <si>
+    <t>eslint + tsc + vite</t>
+  </si>
+  <si>
+    <t>Aggiornato: 04/09/2026</t>
+  </si>
+  <si>
+    <t>Bug del frontend (Fase 6)</t>
+  </si>
+  <si>
+    <t>React 19 + React Hook Form + React Query</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 6</t>
+  </si>
+  <si>
+    <t>04-set-26</t>
+  </si>
+  <si>
+    <t>Codice completo, eslint 0 errori, tsc e vite build puliti, backend invariato a 165/165. In attesa della verifica manuale in browser: la fase si chiude quando i sei casi sono provati e su Vercel e' confermata la variabile VITE_API_URL.</t>
+  </si>
+  <si>
+    <t>Nessun pulsante Modifica nelle prenotazioni (solo Conferma/Completa/Annulla): update-prenotazione era una capacita' solo backend e il fix REV-002 non era raggiungibile dall'app. Risolto riusando PrenotazioneModal con prop opzionale prenotazione, nuovo hook useModificaPrenotazione (PUT) e pulsante Modifica sulle prenotazioni Attive. Nessuna modifica al backend.</t>
+  </si>
+  <si>
+    <t>200 Ok - consumato dal frontend dalla Fase 6 (pulsante Modifica, NEW-001)</t>
+  </si>
+  <si>
+    <t>dotnet test 165/165 (erano 74), dotnet build senza errori (restano 5 warning CS8603/CS8602 pre-esistenti, verificati il 04/09: non sono regressioni). Controllo di qualita': rotti temporaneamente due punti del codice (filtro zone disattivate, limite giornaliero) e verificato che solo i test attesi fallissero, poi ripristinato - nessun falso verde. Nessuna migration, nessuna azione richiesta a Fabio (fase solo di test automatici).</t>
+  </si>
+  <si>
+    <t>NEW-004 - eliminazione prenotazione nell'interfaccia</t>
+  </si>
+  <si>
+    <t>L'hook useDeletePrenotazione esisteva in usePrenotazioni.ts ma nessun componente lo usava: eliminare passava solo da Postman. Aggiunto il pulsante Elimina in colonna Azioni, riservato all'Admin (l'endpoint e' Authorize Roles = Admin) e mostrato solo sugli stati che il backend accetta, Attiva e Annullata: fuori da quegli stati il pulsante non compare, invece di far scoprire il limite con un 409. ConfirmDialog ora accetta titolo e testo del pulsante di conferma: prima annullare ed eliminare avrebbero mostrato lo stesso 'Conferma eliminazione / Elimina', due azioni diverse con la stessa faccia.</t>
+  </si>
+  <si>
+    <t>React Query + React 19</t>
+  </si>
+  <si>
+    <t>Schermata bianca da token corrotto, scelta zona scollegata dal form, modal di modifica prenotazione, pulsante di eliminazione per l'Admin, date della dashboard in ora italiana, errore esplicito se manca l'indirizzo del server, scadenza sessione senza reload.</t>
+  </si>
+  <si>
+    <t>Bug del frontend: schermata bianca (REV-014), scelta zona non collegata al form (REV-015), fuso orario della dashboard lato client (REV-016), indirizzo del server mancante (REV-017), scadenza sessione pulita (REV-025), modal di modifica prenotazione (NEW-001), eliminazione prenotazione nell'interfaccia (NEW-004).</t>
+  </si>
+  <si>
+    <t>usePrenotazioni.ts espone useDeletePrenotazione ma nessun componente lo usava: nel frontend c'era solo Annulla, eliminare passava da Postman. Risolto con il pulsante Elimina in colonna Azioni, riservato all'Admin e visibile solo sugli stati Attiva e Annullata, gli unici che il backend accetta. ConfirmDialog ora distingue i due dialoghi (annullamento ed eliminazione), che prima avrebbero avuto lo stesso titolo e lo stesso pulsante.</t>
+  </si>
+  <si>
+    <t>Bug del frontend (REV-014, REV-015, REV-016, REV-017, REV-025, NEW-001, NEW-004)</t>
+  </si>
+  <si>
+    <t>Verifiche di build e test</t>
+  </si>
+  <si>
+    <t>eslint 0 errori (resta il solo warning React Compiler su watch() di RHF, pre-esistente), tsc -b e vite build puliti, dotnet test 168/168 (erano 165: +3 sul profilo di mapping). Nota: la riga di chiusura della Fase 5 diceva 'dotnet build 0 warning' ed e' stata corretta - la build incrementale ne emette 5, una ricompilazione completa 53, tutti pre-esistenti.</t>
+  </si>
+  <si>
+    <t>Verifiche in locale con Playwright</t>
+  </si>
+  <si>
+    <t>Eseguite in browser sull'ambiente locale (backend :5099, frontend :5173) tutte le prove non legate ai dati di produzione: token corrotto, troncato e scaduto (si apre sempre il login, mai pagina bianca); zona che torna a 'Nessuna preferenza' alla riapertura del modal, con controprova sui dati (zona Esterno occupata -&gt; 409, zona Sala -&gt; 201 con tavolo di Sala: se la preferenza si perdesse avrebbe assegnato Sala in entrambi i casi); modal di modifica precompilato e PUT 200; pulsante Elimina assente per Cliente e Staff; date della dashboard in ora italiana; schermata di configurazione mancante; sessione scaduta con toast, ritorno al login e nessun reload (verificato con un marcatore su window che sopravvive alla navigazione).</t>
+  </si>
+  <si>
+    <t>Playwright + Node</t>
+  </si>
+  <si>
+    <t>Difetto 1 - zone invisibili al Cliente</t>
+  </si>
+  <si>
+    <t>Emerso in prova: useZone() chiamava /Zona/get-all-zone, endpoint riservato ad Admin e Staff, quindi per il Cliente la select della zona era sempre vuota (403 ripetuto quattro volte per i retry di React Query). Il campo che REV-015 doveva sistemare, per chi prenota da solo non funzionava affatto. Aggiunto useZoneAttive() su /Zona/get-zone-attive, aperto anche al Cliente e per di piu' la lista corretta: una zona disattivata non e' prenotabile (REV-024 la esclude dall'assegnazione), quindi non ha senso proporla.</t>
+  </si>
+  <si>
+    <t>React Query + RBAC</t>
+  </si>
+  <si>
+    <t>Difetto 2 - ZonaId mai mappato (backend)</t>
+  </si>
+  <si>
+    <t>L'assunzione iniziale era sbagliata a meta': FasciaOrariaId era davvero gia' mappato, ZonaId no. PostazioneAssegnataDTO.ZonaId era dichiarato nel DTO e mai valorizzato, usciva sempre 0 - lo stesso schema di REV-001 (NumeroPosti rimasto a 0). Con zonaId 0 la select non trovava alcuna opzione corrispondente e restava senza selezione. Corretto in PrenotazioneMappingProfile: e' l'unica modifica al backend della Fase 6, nessuna migration. Aggiunto PrenotazioneMappingProfileTests (3 test): il profilo di mapping non era coperto da nulla, ed e' il secondo bug della stessa famiglia. Controprova fatta: rimuovendo il mapping falliscono esattamente i due test attesi. Lato frontend lo 0 e' ora trattato come assenza di zona.</t>
+  </si>
+  <si>
+    <t>AutoMapper + xUnit</t>
+  </si>
+  <si>
+    <t>Difetto 3 - REV-017 lasciava la pagina bianca</t>
+  </si>
+  <si>
+    <t>La prima versione lanciava un throw a livello di modulo in lib/axios.ts: il messaggio finiva in console, ma l'eccezione impediva il caricamento del bundle e la pagina restava bianca - lo stesso sintomo che la fase doveva eliminare, e nessun Error Boundary puo' intercettarlo perche' l'app non arriva a montarsi. Ora la mancanza e' un dato (configurazioneMancante) e main.tsx mostra il componente ConfigurazioneMancante, che spiega a schermo cosa manca e come rimediare in sviluppo e in produzione.</t>
+  </si>
+  <si>
+    <t>Vite env + React</t>
+  </si>
+  <si>
+    <t>Difetto 4 - ErrorBoundary scavalcato da React Router</t>
+  </si>
+  <si>
+    <t>L'ErrorBoundary messo in main.tsx non intercetta gli errori dentro le route: React Router v7 ha un proprio error boundary che li cattura prima e mostra 'Unexpected Application Error!' con lo stack trace in pagina. Copre il caso REV-014 vero (che sta fuori dal router, in AuthProvider) ma non le pagine. Aggiunto router/RouteErrorPage.tsx come errorElement su tutte le route di primo livello; la schermata e' ora condivisa in components/ErrorScreen. Verificato iniettando di proposito un errore in LoginPage e poi rimuovendolo.</t>
+  </si>
+  <si>
+    <t>React Router v7</t>
+  </si>
+  <si>
+    <t>Cosa resta prima di chiudere la fase</t>
+  </si>
+  <si>
+    <t>Da provare in produzione dopo commit, push e merge su main (e' il branch da cui pubblica Vercel): zona, modifica ed eliminazione sui dati reali, piu' la conferma della variabile VITE_API_URL su Vercel (task di Fabio). Il caso REV-017 non va ripetuto in produzione: toglierebbe la variabile al sito pubblico. Restano nel database LOCALE l'utente di prova testfase6 (promosso a Staff con un INSERT diretto in AspNetUserRoles) e una prenotazione di prova del 07/09: la produzione non e' stata toccata.</t>
+  </si>
+  <si>
+    <t>168 test unitari</t>
+  </si>
+  <si>
+    <t>Testing - 168 test OK</t>
+  </si>
+  <si>
+    <t>168 test unitari con xUnit + Moq</t>
+  </si>
+  <si>
+    <t>Token corrotto in localStorage non blocca piu' l'app (parsing difensivo in AuthContext + ErrorBoundary); select della zona registrata in react-hook-form; date della dashboard calcolate in Europe/Rome invece che in UTC; errore esplicito se VITE_API_URL non e' impostata; scadenza sessione con toast e navigazione al posto del reload; modal di modifica prenotazione; pulsante di eliminazione per l'Admin (NEW-004). Verifica manuale in browser ancora da fare. Prove in locale eseguite con Playwright: hanno fatto emergere quattro difetti, tutti corretti (zone invisibili al Cliente, ZonaId mai mappato nel backend, REV-017 che lasciava la pagina bianca, ErrorBoundary scavalcato da React Router). dotnet test 168/168.</t>
   </si>
 </sst>
 </file>
@@ -4698,7 +4851,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>1208</v>
+        <v>1322</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -4733,7 +4886,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>1241</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4856,10 +5009,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1287</v>
+        <v>1357</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1287</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4867,11 +5020,11 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1288</v>
+        <v>1358</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1288</v>
+        <v>1358</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -4891,7 +5044,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>1286</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4899,13 +5052,13 @@
       <c r="B15" s="34"/>
       <c r="C15" s="33"/>
       <c r="D15" s="35" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="37" t="s">
         <v>1134</v>
-      </c>
-      <c r="E15" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>1135</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5165,13 +5318,13 @@
     </row>
     <row r="13" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1273</v>
+        <v>1268</v>
       </c>
       <c r="B13" t="s">
         <v>665</v>
       </c>
       <c r="C13" t="s">
-        <v>1274</v>
+        <v>1269</v>
       </c>
       <c r="D13" t="s">
         <v>653</v>
@@ -5180,27 +5333,27 @@
         <v>437</v>
       </c>
       <c r="F13" t="s">
-        <v>1275</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>1273</v>
+        <v>1268</v>
       </c>
       <c r="B14" t="s">
         <v>651</v>
       </c>
       <c r="C14" t="s">
-        <v>1276</v>
+        <v>1271</v>
       </c>
       <c r="D14" t="s">
-        <v>1277</v>
+        <v>1272</v>
       </c>
       <c r="E14" t="s">
         <v>654</v>
       </c>
       <c r="F14" t="s">
-        <v>1278</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5760,7 +5913,7 @@
         <v>687</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>1272</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5843,7 +5996,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
         <v>354</v>
       </c>
@@ -5860,7 +6013,7 @@
         <v>740</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>693</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -6045,7 +6198,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="56" t="s">
-        <v>1309</v>
+        <v>1300</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
@@ -6564,16 +6717,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C33" t="s">
         <v>1175</v>
       </c>
-      <c r="B33" t="s">
+      <c r="D33" t="s">
         <v>1176</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1177</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1178</v>
       </c>
       <c r="E33" s="27" t="s">
         <v>6</v>
@@ -6581,16 +6734,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B34" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="C34" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="D34" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -6598,16 +6751,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B35" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="C35" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="D35" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -6615,16 +6768,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B36" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="C36" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="D36" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -6632,13 +6785,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B37" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="C37" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="D37" t="s">
         <v>1067</v>
@@ -6649,13 +6802,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B38" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="C38" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="D38" t="s">
         <v>1067</v>
@@ -6669,13 +6822,13 @@
         <v>772</v>
       </c>
       <c r="B39" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1188</v>
+      </c>
+      <c r="D39" t="s">
         <v>1189</v>
-      </c>
-      <c r="C39" t="s">
-        <v>1190</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1191</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -6686,13 +6839,13 @@
         <v>772</v>
       </c>
       <c r="B40" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="C40" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="D40" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -6703,13 +6856,13 @@
         <v>772</v>
       </c>
       <c r="B41" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1193</v>
+      </c>
+      <c r="D41" t="s">
         <v>1194</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1195</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1196</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -6720,13 +6873,13 @@
         <v>772</v>
       </c>
       <c r="B42" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="C42" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="D42" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="E42" s="27" t="s">
         <v>6</v>
@@ -6737,13 +6890,13 @@
         <v>772</v>
       </c>
       <c r="B43" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="C43" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="D43" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>6</v>
@@ -6754,13 +6907,13 @@
         <v>772</v>
       </c>
       <c r="B44" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1200</v>
+      </c>
+      <c r="D44" t="s">
         <v>1201</v>
-      </c>
-      <c r="C44" t="s">
-        <v>1202</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1203</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>6</v>
@@ -6771,13 +6924,13 @@
         <v>772</v>
       </c>
       <c r="B45" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D45" t="s">
         <v>1204</v>
-      </c>
-      <c r="C45" t="s">
-        <v>1205</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1206</v>
       </c>
       <c r="E45" s="27" t="s">
         <v>6</v>
@@ -7160,7 +7313,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H215"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7185,7 +7338,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>1209</v>
+        <v>1322</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -8246,24 +8399,24 @@
     </row>
     <row r="71" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="44" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="B71" s="25" t="s">
-        <v>1226</v>
+        <v>1222</v>
       </c>
       <c r="C71" s="25" t="s">
-        <v>1227</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="44" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="B72" s="25" t="s">
-        <v>1228</v>
+        <v>1224</v>
       </c>
       <c r="C72" s="25" t="s">
-        <v>1229</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -9511,7 +9664,7 @@
         <v>1115</v>
       </c>
       <c r="C157" s="27" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D157" s="27" t="s">
         <v>1116</v>
@@ -9528,10 +9681,10 @@
         <v>6</v>
       </c>
       <c r="B158" s="41" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C158" s="41" t="s">
         <v>1128</v>
-      </c>
-      <c r="C158" s="41" t="s">
-        <v>1129</v>
       </c>
       <c r="D158" s="41" t="s">
         <v>267</v>
@@ -9545,7 +9698,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
@@ -9573,16 +9726,16 @@
         <v>1</v>
       </c>
       <c r="B162" s="27" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C162" s="27" t="s">
         <v>1137</v>
       </c>
-      <c r="C162" s="27" t="s">
+      <c r="D162" s="27" t="s">
         <v>1138</v>
       </c>
-      <c r="D162" s="27" t="s">
+      <c r="E162" s="40" t="s">
         <v>1139</v>
-      </c>
-      <c r="E162" s="40" t="s">
-        <v>1140</v>
       </c>
       <c r="F162" s="27" t="s">
         <v>6</v>
@@ -9593,16 +9746,16 @@
         <v>2</v>
       </c>
       <c r="B163" s="27" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C163" s="27" t="s">
         <v>1141</v>
       </c>
-      <c r="C163" s="27" t="s">
+      <c r="D163" s="27" t="s">
         <v>1142</v>
       </c>
-      <c r="D163" s="27" t="s">
-        <v>1143</v>
-      </c>
       <c r="E163" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F163" s="27" t="s">
         <v>6</v>
@@ -9613,16 +9766,16 @@
         <v>3</v>
       </c>
       <c r="B164" s="27" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C164" s="27" t="s">
         <v>1144</v>
       </c>
-      <c r="C164" s="27" t="s">
+      <c r="D164" s="27" t="s">
         <v>1145</v>
       </c>
-      <c r="D164" s="27" t="s">
-        <v>1146</v>
-      </c>
       <c r="E164" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F164" s="27" t="s">
         <v>6</v>
@@ -9633,16 +9786,16 @@
         <v>4</v>
       </c>
       <c r="B165" s="27" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C165" s="27" t="s">
         <v>1147</v>
       </c>
-      <c r="C165" s="27" t="s">
+      <c r="D165" s="27" t="s">
         <v>1148</v>
       </c>
-      <c r="D165" s="27" t="s">
-        <v>1149</v>
-      </c>
       <c r="E165" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F165" s="27" t="s">
         <v>6</v>
@@ -9653,16 +9806,16 @@
         <v>5</v>
       </c>
       <c r="B166" s="27" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C166" s="27" t="s">
         <v>1150</v>
       </c>
-      <c r="C166" s="27" t="s">
+      <c r="D166" s="27" t="s">
         <v>1151</v>
       </c>
-      <c r="D166" s="27" t="s">
-        <v>1152</v>
-      </c>
       <c r="E166" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F166" s="27" t="s">
         <v>6</v>
@@ -9673,16 +9826,16 @@
         <v>6</v>
       </c>
       <c r="B167" s="27" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C167" s="27" t="s">
         <v>1153</v>
       </c>
-      <c r="C167" s="27" t="s">
+      <c r="D167" s="27" t="s">
         <v>1154</v>
       </c>
-      <c r="D167" s="27" t="s">
-        <v>1155</v>
-      </c>
       <c r="E167" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F167" s="27" t="s">
         <v>6</v>
@@ -9693,16 +9846,16 @@
         <v>7</v>
       </c>
       <c r="B168" s="27" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C168" s="27" t="s">
         <v>1156</v>
-      </c>
-      <c r="C168" s="27" t="s">
-        <v>1157</v>
       </c>
       <c r="D168" s="27" t="s">
         <v>1019</v>
       </c>
       <c r="E168" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F168" s="27" t="s">
         <v>6</v>
@@ -9713,16 +9866,16 @@
         <v>8</v>
       </c>
       <c r="B169" s="27" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C169" s="27" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D169" s="27" t="s">
         <v>1158</v>
       </c>
-      <c r="C169" s="27" t="s">
-        <v>1207</v>
-      </c>
-      <c r="D169" s="27" t="s">
-        <v>1159</v>
-      </c>
       <c r="E169" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F169" s="27" t="s">
         <v>6</v>
@@ -9733,16 +9886,16 @@
         <v>9</v>
       </c>
       <c r="B170" s="27" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C170" s="27" t="s">
         <v>1160</v>
       </c>
-      <c r="C170" s="27" t="s">
+      <c r="D170" s="27" t="s">
         <v>1161</v>
       </c>
-      <c r="D170" s="27" t="s">
-        <v>1162</v>
-      </c>
       <c r="E170" s="40" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="F170" s="27" t="s">
         <v>6</v>
@@ -9750,7 +9903,7 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>1210</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
@@ -9778,16 +9931,16 @@
         <v>1</v>
       </c>
       <c r="B174" s="27" t="s">
-        <v>1211</v>
+        <v>1207</v>
       </c>
       <c r="C174" s="27" t="s">
-        <v>1212</v>
+        <v>1208</v>
       </c>
       <c r="D174" s="27" t="s">
-        <v>1213</v>
+        <v>1209</v>
       </c>
       <c r="E174" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F174" s="27" t="s">
         <v>6</v>
@@ -9798,16 +9951,16 @@
         <v>2</v>
       </c>
       <c r="B175" s="27" t="s">
-        <v>1215</v>
+        <v>1211</v>
       </c>
       <c r="C175" s="27" t="s">
-        <v>1216</v>
+        <v>1212</v>
       </c>
       <c r="D175" s="27" t="s">
-        <v>1217</v>
+        <v>1213</v>
       </c>
       <c r="E175" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F175" s="27" t="s">
         <v>6</v>
@@ -9818,16 +9971,16 @@
         <v>3</v>
       </c>
       <c r="B176" s="27" t="s">
-        <v>1218</v>
+        <v>1214</v>
       </c>
       <c r="C176" s="27" t="s">
-        <v>1219</v>
+        <v>1215</v>
       </c>
       <c r="D176" s="27" t="s">
-        <v>1220</v>
+        <v>1216</v>
       </c>
       <c r="E176" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F176" s="27" t="s">
         <v>6</v>
@@ -9838,19 +9991,19 @@
         <v>4</v>
       </c>
       <c r="B177" s="27" t="s">
-        <v>1221</v>
+        <v>1217</v>
       </c>
       <c r="C177" s="27" t="s">
-        <v>1222</v>
+        <v>1218</v>
       </c>
       <c r="D177" s="27" t="s">
-        <v>1223</v>
+        <v>1219</v>
       </c>
       <c r="E177" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F177" s="43" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
@@ -9858,16 +10011,16 @@
         <v>5</v>
       </c>
       <c r="B178" s="27" t="s">
-        <v>1224</v>
+        <v>1220</v>
       </c>
       <c r="C178" s="27" t="s">
-        <v>1225</v>
+        <v>1221</v>
       </c>
       <c r="D178" s="27" t="s">
         <v>437</v>
       </c>
       <c r="E178" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F178" s="27" t="s">
         <v>6</v>
@@ -9875,7 +10028,7 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>1242</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -9903,16 +10056,16 @@
         <v>1</v>
       </c>
       <c r="B182" s="27" t="s">
-        <v>1243</v>
+        <v>1238</v>
       </c>
       <c r="C182" s="27" t="s">
-        <v>1244</v>
+        <v>1239</v>
       </c>
       <c r="D182" s="27" t="s">
-        <v>1245</v>
+        <v>1240</v>
       </c>
       <c r="E182" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F182" s="27" t="s">
         <v>6</v>
@@ -9923,16 +10076,16 @@
         <v>2</v>
       </c>
       <c r="B183" s="27" t="s">
-        <v>1246</v>
+        <v>1241</v>
       </c>
       <c r="C183" s="27" t="s">
-        <v>1247</v>
+        <v>1242</v>
       </c>
       <c r="D183" s="27" t="s">
-        <v>1248</v>
+        <v>1243</v>
       </c>
       <c r="E183" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F183" s="27" t="s">
         <v>6</v>
@@ -9943,16 +10096,16 @@
         <v>3</v>
       </c>
       <c r="B184" s="27" t="s">
-        <v>1249</v>
+        <v>1244</v>
       </c>
       <c r="C184" s="27" t="s">
-        <v>1250</v>
+        <v>1245</v>
       </c>
       <c r="D184" s="27" t="s">
-        <v>1251</v>
+        <v>1246</v>
       </c>
       <c r="E184" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F184" s="27" t="s">
         <v>6</v>
@@ -9963,16 +10116,16 @@
         <v>4</v>
       </c>
       <c r="B185" s="27" t="s">
-        <v>1252</v>
+        <v>1247</v>
       </c>
       <c r="C185" s="27" t="s">
-        <v>1253</v>
+        <v>1248</v>
       </c>
       <c r="D185" s="27" t="s">
         <v>401</v>
       </c>
       <c r="E185" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F185" s="27" t="s">
         <v>6</v>
@@ -9983,16 +10136,16 @@
         <v>5</v>
       </c>
       <c r="B186" s="27" t="s">
-        <v>1254</v>
+        <v>1249</v>
       </c>
       <c r="C186" s="27" t="s">
-        <v>1255</v>
+        <v>1250</v>
       </c>
       <c r="D186" s="27" t="s">
-        <v>1256</v>
+        <v>1251</v>
       </c>
       <c r="E186" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F186" s="27" t="s">
         <v>6</v>
@@ -10003,16 +10156,16 @@
         <v>6</v>
       </c>
       <c r="B187" s="27" t="s">
-        <v>1257</v>
+        <v>1252</v>
       </c>
       <c r="C187" s="27" t="s">
-        <v>1258</v>
+        <v>1253</v>
       </c>
       <c r="D187" s="27" t="s">
-        <v>1259</v>
+        <v>1254</v>
       </c>
       <c r="E187" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F187" s="27" t="s">
         <v>6</v>
@@ -10023,19 +10176,19 @@
         <v>7</v>
       </c>
       <c r="B188" s="27" t="s">
-        <v>1260</v>
+        <v>1255</v>
       </c>
       <c r="C188" s="27" t="s">
-        <v>1261</v>
+        <v>1256</v>
       </c>
       <c r="D188" s="27" t="s">
         <v>22</v>
       </c>
       <c r="E188" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F188" s="43" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
@@ -10043,16 +10196,16 @@
         <v>8</v>
       </c>
       <c r="B189" s="27" t="s">
-        <v>1279</v>
+        <v>1274</v>
       </c>
       <c r="C189" s="27" t="s">
-        <v>1280</v>
+        <v>1275</v>
       </c>
       <c r="D189" s="27" t="s">
-        <v>1281</v>
+        <v>1276</v>
       </c>
       <c r="E189" s="40" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="F189" s="27" t="s">
         <v>6</v>
@@ -10063,13 +10216,13 @@
         <v>9</v>
       </c>
       <c r="B190" s="27" t="s">
-        <v>1262</v>
+        <v>1257</v>
       </c>
       <c r="C190" s="27" t="s">
-        <v>1289</v>
+        <v>1282</v>
       </c>
       <c r="D190" s="27" t="s">
-        <v>1263</v>
+        <v>1258</v>
       </c>
       <c r="E190" s="40" t="s">
         <v>437</v>
@@ -10080,7 +10233,7 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
-        <v>1290</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
@@ -10108,13 +10261,13 @@
         <v>1</v>
       </c>
       <c r="B193" t="s">
-        <v>1291</v>
+        <v>1284</v>
       </c>
       <c r="C193" t="s">
-        <v>1292</v>
+        <v>1285</v>
       </c>
       <c r="D193" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="E193" s="45">
         <v>46090</v>
@@ -10128,10 +10281,10 @@
         <v>2</v>
       </c>
       <c r="B194" t="s">
-        <v>1293</v>
+        <v>1286</v>
       </c>
       <c r="C194" t="s">
-        <v>1294</v>
+        <v>1287</v>
       </c>
       <c r="D194" t="s">
         <v>74</v>
@@ -10148,13 +10301,13 @@
         <v>3</v>
       </c>
       <c r="B195" t="s">
-        <v>1295</v>
+        <v>1288</v>
       </c>
       <c r="C195" t="s">
-        <v>1296</v>
+        <v>1289</v>
       </c>
       <c r="D195" t="s">
-        <v>1297</v>
+        <v>1290</v>
       </c>
       <c r="E195" s="45">
         <v>46090</v>
@@ -10168,10 +10321,10 @@
         <v>4</v>
       </c>
       <c r="B196" t="s">
-        <v>1298</v>
+        <v>1291</v>
       </c>
       <c r="C196" t="s">
-        <v>1299</v>
+        <v>1292</v>
       </c>
       <c r="D196" t="s">
         <v>74</v>
@@ -10188,13 +10341,13 @@
         <v>5</v>
       </c>
       <c r="B197" t="s">
-        <v>1300</v>
+        <v>1293</v>
       </c>
       <c r="C197" t="s">
-        <v>1301</v>
+        <v>1330</v>
       </c>
       <c r="D197" t="s">
-        <v>1259</v>
+        <v>1254</v>
       </c>
       <c r="E197" s="45">
         <v>46090</v>
@@ -10208,19 +10361,324 @@
         <v>6</v>
       </c>
       <c r="B198" t="s">
-        <v>1302</v>
+        <v>1294</v>
       </c>
       <c r="C198" t="s">
-        <v>1303</v>
+        <v>1295</v>
       </c>
       <c r="D198" t="s">
-        <v>1304</v>
+        <v>1296</v>
       </c>
       <c r="E198" t="s">
         <v>437</v>
       </c>
       <c r="F198" s="38" t="s">
-        <v>979</v>
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B200" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>39</v>
+      </c>
+      <c r="B201" t="s">
+        <v>40</v>
+      </c>
+      <c r="C201" t="s">
+        <v>857</v>
+      </c>
+      <c r="D201" t="s">
+        <v>42</v>
+      </c>
+      <c r="E201" t="s">
+        <v>43</v>
+      </c>
+      <c r="F201" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A202">
+        <v>1</v>
+      </c>
+      <c r="B202" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1304</v>
+      </c>
+      <c r="D202" t="s">
+        <v>1305</v>
+      </c>
+      <c r="E202" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F202" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A203">
+        <v>2</v>
+      </c>
+      <c r="B203" t="s">
+        <v>1306</v>
+      </c>
+      <c r="C203" t="s">
+        <v>1307</v>
+      </c>
+      <c r="D203" t="s">
+        <v>1308</v>
+      </c>
+      <c r="E203" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F203" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A204">
+        <v>3</v>
+      </c>
+      <c r="B204" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C204" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D204" t="s">
+        <v>1311</v>
+      </c>
+      <c r="E204" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F204" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A205">
+        <v>4</v>
+      </c>
+      <c r="B205" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C205" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D205" t="s">
+        <v>1314</v>
+      </c>
+      <c r="E205" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F205" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A206">
+        <v>5</v>
+      </c>
+      <c r="B206" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C206" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D206" t="s">
+        <v>1317</v>
+      </c>
+      <c r="E206" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F206" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A207">
+        <v>6</v>
+      </c>
+      <c r="B207" t="s">
+        <v>1318</v>
+      </c>
+      <c r="C207" t="s">
+        <v>1319</v>
+      </c>
+      <c r="D207" t="s">
+        <v>1320</v>
+      </c>
+      <c r="E207" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F207" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A208">
+        <v>7</v>
+      </c>
+      <c r="B208" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C208" t="s">
+        <v>1332</v>
+      </c>
+      <c r="D208" t="s">
+        <v>1333</v>
+      </c>
+      <c r="E208" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F208" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A209">
+        <v>8</v>
+      </c>
+      <c r="B209" t="s">
+        <v>1338</v>
+      </c>
+      <c r="C209" t="s">
+        <v>1339</v>
+      </c>
+      <c r="D209" t="s">
+        <v>1321</v>
+      </c>
+      <c r="E209" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F209" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A210">
+        <v>8</v>
+      </c>
+      <c r="B210" t="s">
+        <v>1340</v>
+      </c>
+      <c r="C210" t="s">
+        <v>1341</v>
+      </c>
+      <c r="D210" t="s">
+        <v>1342</v>
+      </c>
+      <c r="E210" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F210" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A211">
+        <v>9</v>
+      </c>
+      <c r="B211" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C211" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D211" t="s">
+        <v>1345</v>
+      </c>
+      <c r="E211" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F211" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A212">
+        <v>10</v>
+      </c>
+      <c r="B212" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C212" t="s">
+        <v>1347</v>
+      </c>
+      <c r="D212" t="s">
+        <v>1348</v>
+      </c>
+      <c r="E212" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F212" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A213">
+        <v>11</v>
+      </c>
+      <c r="B213" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C213" t="s">
+        <v>1350</v>
+      </c>
+      <c r="D213" t="s">
+        <v>1351</v>
+      </c>
+      <c r="E213" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F213" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A214">
+        <v>12</v>
+      </c>
+      <c r="B214" t="s">
+        <v>1352</v>
+      </c>
+      <c r="C214" t="s">
+        <v>1353</v>
+      </c>
+      <c r="D214" t="s">
+        <v>1354</v>
+      </c>
+      <c r="E214" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F214" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A215">
+        <v>13</v>
+      </c>
+      <c r="B215" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C215" t="s">
+        <v>1356</v>
+      </c>
+      <c r="D215" t="s">
+        <v>437</v>
+      </c>
+      <c r="E215" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F215" s="38" t="s">
+        <v>1301</v>
       </c>
     </row>
   </sheetData>
@@ -10239,7 +10697,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -10664,7 +11122,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1305</v>
+        <v>1359</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -10729,13 +11187,13 @@
         <v>1043</v>
       </c>
       <c r="B35" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="C35" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D35" t="s">
         <v>1163</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1164</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -10746,16 +11204,33 @@
         <v>1043</v>
       </c>
       <c r="B36" t="s">
-        <v>1264</v>
+        <v>1259</v>
       </c>
       <c r="C36" t="s">
-        <v>1265</v>
+        <v>1260</v>
       </c>
       <c r="D36" t="s">
-        <v>1266</v>
+        <v>1261</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1334</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E37" s="38" t="s">
+        <v>1301</v>
       </c>
     </row>
   </sheetData>
@@ -10772,7 +11247,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -11163,7 +11638,7 @@
         <v>6</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -11171,22 +11646,22 @@
         <v>1008</v>
       </c>
       <c r="B21" s="41" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C21" s="41" t="s">
         <v>1132</v>
       </c>
-      <c r="C21" s="41" t="s">
-        <v>1133</v>
-      </c>
       <c r="D21" s="41" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="E21" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="F21" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -11194,45 +11669,45 @@
         <v>1008</v>
       </c>
       <c r="B22" s="41" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C22" s="41" t="s">
         <v>1166</v>
       </c>
-      <c r="C22" s="41" t="s">
-        <v>1167</v>
-      </c>
       <c r="D22" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="E22" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="F22" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1267</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="41" t="s">
-        <v>1282</v>
+        <v>1277</v>
       </c>
       <c r="B23" s="41" t="s">
-        <v>1283</v>
+        <v>1278</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>1284</v>
+        <v>1279</v>
       </c>
       <c r="D23" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="E23" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="F23" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G23" s="41" t="s">
-        <v>1285</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -11240,22 +11715,43 @@
         <v>1008</v>
       </c>
       <c r="B24" s="41" t="s">
-        <v>1268</v>
+        <v>1263</v>
       </c>
       <c r="C24" s="41" t="s">
-        <v>1269</v>
+        <v>1264</v>
       </c>
       <c r="D24" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="E24" s="41" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="F24" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G24" s="41" t="s">
-        <v>1306</v>
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="41" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B25" s="41" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>1335</v>
+      </c>
+      <c r="D25" s="41" t="s">
+        <v>1326</v>
+      </c>
+      <c r="E25" s="41"/>
+      <c r="F25" s="38" t="s">
+        <v>1301</v>
+      </c>
+      <c r="G25" s="41" t="s">
+        <v>1327</v>
       </c>
     </row>
   </sheetData>
@@ -11269,7 +11765,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -11752,10 +12248,10 @@
         <v>1122</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1174</v>
-      </c>
-      <c r="D39" s="41" t="s">
-        <v>1123</v>
+        <v>1328</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -11763,24 +12259,24 @@
         <v>1121</v>
       </c>
       <c r="B40" s="41" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C40" s="41" t="s">
         <v>1124</v>
       </c>
-      <c r="C40" s="41" t="s">
+      <c r="D40" s="41" t="s">
         <v>1125</v>
-      </c>
-      <c r="D40" s="41" t="s">
-        <v>1126</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="27" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="B41" s="27" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C41" s="27" t="s">
         <v>1168</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>1169</v>
       </c>
       <c r="D41" s="27" t="s">
         <v>6</v>
@@ -11788,27 +12284,27 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="41" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B42" s="41" t="s">
         <v>1170</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="C42" s="41" t="s">
         <v>1171</v>
       </c>
-      <c r="C42" s="41" t="s">
+      <c r="D42" s="43" t="s">
         <v>1172</v>
-      </c>
-      <c r="D42" s="43" t="s">
-        <v>1173</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="41" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="B43" s="41" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="C43" s="41" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
       <c r="D43" s="27" t="s">
         <v>6</v>
@@ -11819,38 +12315,38 @@
         <v>1121</v>
       </c>
       <c r="B44" s="41" t="s">
-        <v>1235</v>
+        <v>1231</v>
       </c>
       <c r="C44" s="41" t="s">
-        <v>1236</v>
-      </c>
-      <c r="D44" s="43" t="s">
-        <v>1123</v>
+        <v>1336</v>
+      </c>
+      <c r="D44" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="41" t="s">
-        <v>1237</v>
+        <v>1232</v>
       </c>
       <c r="B45" s="41" t="s">
-        <v>1238</v>
+        <v>1233</v>
       </c>
       <c r="C45" s="41" t="s">
-        <v>1239</v>
+        <v>1234</v>
       </c>
       <c r="D45" s="43" t="s">
-        <v>1240</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="27" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>1270</v>
+        <v>1265</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>1271</v>
+        <v>1266</v>
       </c>
       <c r="D46" s="27" t="s">
         <v>6</v>
@@ -11858,16 +12354,30 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>1268</v>
+        <v>1263</v>
       </c>
       <c r="B47" t="s">
-        <v>1307</v>
+        <v>1298</v>
       </c>
       <c r="C47" t="s">
-        <v>1308</v>
+        <v>1299</v>
       </c>
       <c r="D47" s="27" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1337</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D48" s="38" t="s">
+        <v>1301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Fase 6 - esiti delle verifiche in locale, difetti corretti e nota di rilascio
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ECFA5CE-5A8F-4DA2-A227-AAB39471C163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAC5BB3-0528-4E84-98AC-33A638026D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2408" uniqueCount="1361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="1363">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -4015,9 +4015,6 @@
     <t>04-set-26</t>
   </si>
   <si>
-    <t>Codice completo, eslint 0 errori, tsc e vite build puliti, backend invariato a 165/165. In attesa della verifica manuale in browser: la fase si chiude quando i sei casi sono provati e su Vercel e' confermata la variabile VITE_API_URL.</t>
-  </si>
-  <si>
     <t>Nessun pulsante Modifica nelle prenotazioni (solo Conferma/Completa/Annulla): update-prenotazione era una capacita' solo backend e il fix REV-002 non era raggiungibile dall'app. Risolto riusando PrenotazioneModal con prop opzionale prenotazione, nuovo hook useModificaPrenotazione (PUT) e pulsante Modifica sulle prenotazioni Attive. Nessuna modifica al backend.</t>
   </si>
   <si>
@@ -4115,6 +4112,15 @@
   </si>
   <si>
     <t>Token corrotto in localStorage non blocca piu' l'app (parsing difensivo in AuthContext + ErrorBoundary); select della zona registrata in react-hook-form; date della dashboard calcolate in Europe/Rome invece che in UTC; errore esplicito se VITE_API_URL non e' impostata; scadenza sessione con toast e navigazione al posto del reload; modal di modifica prenotazione; pulsante di eliminazione per l'Admin (NEW-004). Verifica manuale in browser ancora da fare. Prove in locale eseguite con Playwright: hanno fatto emergere quattro difetti, tutti corretti (zone invisibili al Cliente, ZonaId mai mappato nel backend, REV-017 che lasciava la pagina bianca, ErrorBoundary scavalcato da React Router). dotnet test 168/168.</t>
+  </si>
+  <si>
+    <t>Rilascio del 04/09 - pushato, da verificare</t>
+  </si>
+  <si>
+    <t>Commit c25c66e su dev, merge su main in fast-forward, entrambi pushati (origin/dev e origin/main allineati). Nessun tag, a differenza della v1.0.1: da decidere alla ripresa se creare una v1.0.2 sulla punta di main. Railway e Vercel si ridistribuiscono da soli sul push di main. Nessuna migration: l'unica modifica al backend e' il mapping di ZonaId, che non tocca lo schema. Restano da confermare in produzione: /health Healthy, le prove sui dati reali (zona, modifica, eliminazione con i tre ruoli) e la presenza di VITE_API_URL su Vercel.</t>
+  </si>
+  <si>
+    <t>Codice completo, eslint 0 errori, tsc e vite build puliti, backend invariato a 165/165. In attesa della verifica manuale in browser: la fase si chiude quando i sei casi sono provati e su Vercel e' confermata la variabile VITE_API_URL. Rilasciato il 04/09 con il commit c25c66e (merge dev-&gt;main in fast-forward, pushato, nessun tag). La fase resta In corso finche' non sono confermate le prove in produzione e la variabile VITE_API_URL su Vercel.</t>
   </si>
 </sst>
 </file>
@@ -5009,10 +5015,10 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5020,11 +5026,11 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -6013,7 +6019,7 @@
         <v>740</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -7313,7 +7319,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H215"/>
+  <dimension ref="A1:H216"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -10344,7 +10350,7 @@
         <v>1293</v>
       </c>
       <c r="C197" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="D197" t="s">
         <v>1254</v>
@@ -10526,13 +10532,13 @@
         <v>7</v>
       </c>
       <c r="B208" t="s">
+        <v>1330</v>
+      </c>
+      <c r="C208" t="s">
         <v>1331</v>
       </c>
-      <c r="C208" t="s">
+      <c r="D208" t="s">
         <v>1332</v>
-      </c>
-      <c r="D208" t="s">
-        <v>1333</v>
       </c>
       <c r="E208" s="45">
         <v>46121</v>
@@ -10546,10 +10552,10 @@
         <v>8</v>
       </c>
       <c r="B209" t="s">
+        <v>1337</v>
+      </c>
+      <c r="C209" t="s">
         <v>1338</v>
-      </c>
-      <c r="C209" t="s">
-        <v>1339</v>
       </c>
       <c r="D209" t="s">
         <v>1321</v>
@@ -10566,13 +10572,13 @@
         <v>8</v>
       </c>
       <c r="B210" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C210" t="s">
         <v>1340</v>
       </c>
-      <c r="C210" t="s">
+      <c r="D210" t="s">
         <v>1341</v>
-      </c>
-      <c r="D210" t="s">
-        <v>1342</v>
       </c>
       <c r="E210" s="45">
         <v>46121</v>
@@ -10586,13 +10592,13 @@
         <v>9</v>
       </c>
       <c r="B211" t="s">
+        <v>1342</v>
+      </c>
+      <c r="C211" t="s">
         <v>1343</v>
       </c>
-      <c r="C211" t="s">
+      <c r="D211" t="s">
         <v>1344</v>
-      </c>
-      <c r="D211" t="s">
-        <v>1345</v>
       </c>
       <c r="E211" s="45">
         <v>46121</v>
@@ -10606,13 +10612,13 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
+        <v>1345</v>
+      </c>
+      <c r="C212" t="s">
         <v>1346</v>
       </c>
-      <c r="C212" t="s">
+      <c r="D212" t="s">
         <v>1347</v>
-      </c>
-      <c r="D212" t="s">
-        <v>1348</v>
       </c>
       <c r="E212" s="45">
         <v>46121</v>
@@ -10626,13 +10632,13 @@
         <v>11</v>
       </c>
       <c r="B213" t="s">
+        <v>1348</v>
+      </c>
+      <c r="C213" t="s">
         <v>1349</v>
       </c>
-      <c r="C213" t="s">
+      <c r="D213" t="s">
         <v>1350</v>
-      </c>
-      <c r="D213" t="s">
-        <v>1351</v>
       </c>
       <c r="E213" s="45">
         <v>46121</v>
@@ -10646,13 +10652,13 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
+        <v>1351</v>
+      </c>
+      <c r="C214" t="s">
         <v>1352</v>
       </c>
-      <c r="C214" t="s">
+      <c r="D214" t="s">
         <v>1353</v>
-      </c>
-      <c r="D214" t="s">
-        <v>1354</v>
       </c>
       <c r="E214" s="45">
         <v>46121</v>
@@ -10666,10 +10672,10 @@
         <v>13</v>
       </c>
       <c r="B215" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C215" t="s">
         <v>1355</v>
-      </c>
-      <c r="C215" t="s">
-        <v>1356</v>
       </c>
       <c r="D215" t="s">
         <v>437</v>
@@ -10678,6 +10684,26 @@
         <v>46121</v>
       </c>
       <c r="F215" s="38" t="s">
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A216">
+        <v>14</v>
+      </c>
+      <c r="B216" t="s">
+        <v>1360</v>
+      </c>
+      <c r="C216" t="s">
+        <v>1361</v>
+      </c>
+      <c r="D216" t="s">
+        <v>1276</v>
+      </c>
+      <c r="E216" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F216" s="38" t="s">
         <v>1301</v>
       </c>
     </row>
@@ -11122,7 +11148,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -11224,7 +11250,7 @@
         <v>1323</v>
       </c>
       <c r="C37" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="D37" t="s">
         <v>1324</v>
@@ -11741,7 +11767,7 @@
         <v>1325</v>
       </c>
       <c r="C25" s="41" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="D25" s="41" t="s">
         <v>1326</v>
@@ -11751,7 +11777,7 @@
         <v>1301</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>1327</v>
+        <v>1362</v>
       </c>
     </row>
   </sheetData>
@@ -12248,7 +12274,7 @@
         <v>1122</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D39" s="27" t="s">
         <v>6</v>
@@ -12318,7 +12344,7 @@
         <v>1231</v>
       </c>
       <c r="C44" s="41" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="D44" s="27" t="s">
         <v>6</v>
@@ -12371,10 +12397,10 @@
         <v>1325</v>
       </c>
       <c r="B48" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="C48" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="D48" s="38" t="s">
         <v>1301</v>

</xml_diff>

<commit_message>
feat: Fase 7 - robustezza del backend (REV-018, REV-019, REV-020, REV-021, REV-022,   REV-023, REV-027, REV-028, REV-029, REV-031, REV-032, REV-037, REV-038, REV-039, NEW-003)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAC5BB3-0528-4E84-98AC-33A638026D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4060647A-65E1-41C5-B5BF-7E0E0F3F3981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="1363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="1410">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3550,9 +3550,6 @@
     <t>PostazioneService.UpdateAsync rifiuta l'aggiornamento se HasPrenotazioniAsync trova una qualsiasi riga in PrenotazioniPostazioni, senza distinguere fra prenotazioni future e storiche: dopo la prima prenotazione completata il tavolo non si puo' piu' rinominare, spostare di zona ne' disattivare. Emerso il 02/09 provando a disattivare i tavoli per preparare il test di concorrenza. Il controllo corretto guarda solo le prenotazioni future e non annullate.</t>
   </si>
   <si>
-    <t>Pianificato (Fase 7)</t>
-  </si>
-  <si>
     <t>DbExceptionTranslatorTests</t>
   </si>
   <si>
@@ -3934,9 +3931,6 @@
     <t>PostazioneAssignmentServiceTests ricreato sul metodo reale AssegnaPostazioneDisponibileAsync (16 test), motore puro rinominato in AssegnazioneTavoliTests; +45 test su creazione/modifica prenotazione in PrenotazioniServiceTests; +13 test sui job notturni + nuovo JobsNotturniTests sui gusci Quartz; DashboardServiceTests 1-&gt;17, +3 DisponibilitaService, +7 validator, +6 ruoli (Admin testato per la prima volta), nuovo PrenotazioniRepositoryTests. Controllo di qualita': mutazioni temporanee sul codice per verificare che i test nuovi sappiano davvero fallire. dotnet test 165/165 (erano 74), dotnet build pulita. Nessuna migration.</t>
   </si>
   <si>
-    <t>TEST UNITARI - xUnit + Moq  (Totale: 165 test  |  Tutti OK  |  elenco dettagliato fermo alla Fase 2b/42 test - da Fase 3 in poi il riepilogo per fase e' in ROADMAP_REVISIONE.md e nel foglio Appunti e Step)</t>
-  </si>
-  <si>
     <t>In corso</t>
   </si>
   <si>
@@ -4099,9 +4093,6 @@
     <t>Cosa resta prima di chiudere la fase</t>
   </si>
   <si>
-    <t>Da provare in produzione dopo commit, push e merge su main (e' il branch da cui pubblica Vercel): zona, modifica ed eliminazione sui dati reali, piu' la conferma della variabile VITE_API_URL su Vercel (task di Fabio). Il caso REV-017 non va ripetuto in produzione: toglierebbe la variabile al sito pubblico. Restano nel database LOCALE l'utente di prova testfase6 (promosso a Staff con un INSERT diretto in AspNetUserRoles) e una prenotazione di prova del 07/09: la produzione non e' stata toccata.</t>
-  </si>
-  <si>
     <t>168 test unitari</t>
   </si>
   <si>
@@ -4117,10 +4108,160 @@
     <t>Rilascio del 04/09 - pushato, da verificare</t>
   </si>
   <si>
-    <t>Commit c25c66e su dev, merge su main in fast-forward, entrambi pushati (origin/dev e origin/main allineati). Nessun tag, a differenza della v1.0.1: da decidere alla ripresa se creare una v1.0.2 sulla punta di main. Railway e Vercel si ridistribuiscono da soli sul push di main. Nessuna migration: l'unica modifica al backend e' il mapping di ZonaId, che non tocca lo schema. Restano da confermare in produzione: /health Healthy, le prove sui dati reali (zona, modifica, eliminazione con i tre ruoli) e la presenza di VITE_API_URL su Vercel.</t>
-  </si>
-  <si>
     <t>Codice completo, eslint 0 errori, tsc e vite build puliti, backend invariato a 165/165. In attesa della verifica manuale in browser: la fase si chiude quando i sei casi sono provati e su Vercel e' confermata la variabile VITE_API_URL. Rilasciato il 04/09 con il commit c25c66e (merge dev-&gt;main in fast-forward, pushato, nessun tag). La fase resta In corso finche' non sono confermate le prove in produzione e la variabile VITE_API_URL su Vercel.</t>
+  </si>
+  <si>
+    <t>Chiuso il 04/09/2026. Le prove sui dati reali in produzione sono state eseguite da Fabio e superate: scelta della zona in creazione, modal di modifica, pulsante Elimina con i tre ruoli (visibile solo all'Admin e solo sugli stati Attiva e Annullata). Confermata anche la presenza di VITE_API_URL su Vercel: nel bundle pubblicato la baseURL compare come stringa letterale verso Railway e la schermata ConfigurazioneMancante e' stata eliminata dal tree-shaking, cosa possibile solo se la variabile era impostata al momento della build. Restano nel database LOCALE l'utente di prova testfase6 e una prenotazione del 07/09: la produzione non e' stata toccata.</t>
+  </si>
+  <si>
+    <t>Commit c25c66e su dev, merge su main in fast-forward, entrambi pushati. Verificato in produzione dopo il redeploy: health 200 Healthy, Setup stato con setupCompletato true, get-zone-attive senza token 401, frontend Vercel login 200, bundle Vercel contenente il codice della Fase 6 (Sessione scaduta, Europe Rome, Torna al login, Elimina). Nessuna migration: l'unica modifica al backend e' il mapping di ZonaId, che non tocca lo schema. Tag v1.0.2 creato sulla punta di main. Il commit di documentazione 0fe19b9 resta su dev e verra' portato su main insieme alle modifiche della Fase 7, per non fare un secondo giro di deploy con sola documentazione.</t>
+  </si>
+  <si>
+    <t>200 Ok - consumato dal frontend dalla Fase 6 (pulsante Elimina, NEW-004): visibile solo all'Admin e solo sugli stati Attiva e Annullata</t>
+  </si>
+  <si>
+    <t>Blocco 1 - REV-019 e REV-020: paginazione</t>
+  </si>
+  <si>
+    <t>Page arrivava dalla query string senza controlli: con page=0 il calcolo (Page-1)*PageSize valeva Skip(-20) e faceva fallire la query invece di dare la prima pagina. Ora il valore fuori range rientra nei limiti, come gia' faceva PageSize. REV-020: l'ordinamento era per sola DataPrenotazione, quindi non totale - fra righe dello stesso giorno il database non garantisce alcun ordine e navigando le pagine si vedevano duplicati e si perdevano righe. Aggiunto ThenBy(Id); l'OrderBy veniva inoltre riapplicato dentro ogni ramo del filtro, perdendo i criteri successivi, ed e' stato spostato dopo i Where.</t>
+  </si>
+  <si>
+    <t>EF Core + LINQ</t>
+  </si>
+  <si>
+    <t>Blocco 1 - REV-018: cache delle fasce</t>
+  </si>
+  <si>
+    <t>DeleteAsync invalidava la sola chiave FasceAttive e non quella derivata per giorno: una fascia appena eliminata continuava a comparire in fasce-per-giorno fino alla scadenza naturale della cache (30 minuti) e si poteva provare a prenotare su una fascia inesistente. Era l'unico punto scoperto del service, tutte le altre scritture invalidavano gia' entrambe le chiavi.</t>
+  </si>
+  <si>
+    <t>Blocco 1 - REV-031 e REV-027: contratto degli endpoint</t>
+  </si>
+  <si>
+    <t>Tolti gli ultimi due 404 su collezione vuota (prenotazioni per data e verifica di disponibilita'): un giorno senza prenotazioni o di chiusura e' una risposta, non un errore. Aggiunto il validator mancante sull'unico endpoint pubblico dell'API, che era anche l'unico DTO in ingresso senza validator: stessi limiti del validator di creazione (coperti 1-50, niente date passate) piu' un orizzonte massimo di 365 giorni, perche' senza tetto si potrebbero interrogare date arbitrariamente lontane senza alcun costo per chi chiama.</t>
+  </si>
+  <si>
+    <t>Blocco 1 - REV-099 / NEW-003: tavolo non piu' modificabile</t>
+  </si>
+  <si>
+    <t>Il controllo rispondeva 'si' alla presenza di una qualsiasi riga di prenotazione sul tavolo, storico compreso: dopo la prima prenotazione conclusa quel tavolo non era piu' rinominabile, spostabile di zona ne' disattivabile, e in un locale reale ci si arriva in pochi giorni. Ora si guardano solo gli impegni da oggi in avanti, usando la data denormalizzata sulla riga join. Basta la data perche' l'annullo cancella gia' le righe join (REV-003). L'eliminazione del tavolo resta invece bloccata sull'intero storico, di proposito: eliminarlo distruggerebbe lo storico.</t>
+  </si>
+  <si>
+    <t>EF Core + IClock</t>
+  </si>
+  <si>
+    <t>Blocco 2 - REV-021, REV-022, REV-023: query pesanti</t>
+  </si>
+  <si>
+    <t>Elenco utenti: era una query per ogni utente (i ruoli venivano chiesti dentro il ciclo), ora sono due query fisse con tutte le assegnazioni di ruolo prese in un colpo solo. Job notturni: scrivevano una riga per volta, con una query di ricarica e un salvataggio per ognuna, cioe' 1+2N viaggi al database; ora sono due query in tutto, indipendenti dal numero di righe. Assegnazione del tavolo: il caricamento dello storico e' uscito dal percorso caldo, dove non veniva nemmeno usato.</t>
+  </si>
+  <si>
+    <t>Blocco 3 - REV-029: indirizzo IP reale</t>
+  </si>
+  <si>
+    <t>Registrato per primo il middleware degli header inoltrati, con le liste di proxy noti svuotate (il proxy della piattaforma non e' su loopback) e il limite di catena a 1, che prende solo l'ultimo anello scritto dal proxy e impedisce a un client di falsificare l'header. Oltre all'audit trail, che registrava sempre lo stesso indirizzo, il fix rimette in sesto il rate limit del login: partiziona sull'indirizzo del chiamante, quindi dietro il proxy era di fatto un limite globale di 5 tentativi al minuto per l'intera applicazione, che non fermava chi attacca un singolo account e poteva bloccare gli utenti legittimi.</t>
+  </si>
+  <si>
+    <t>ASP.NET Core middleware</t>
+  </si>
+  <si>
+    <t>Blocco 3 - REV-038: storico protetto dall'eliminazione utente</t>
+  </si>
+  <si>
+    <t>La chiave esterna fra prenotazioni e utenti passa da Cascade a Restrict: eliminare un utente non cancella piu' in silenzio tutto il suo storico, che e' il dato su cui si contano coperti e presenze e che non sarebbe recuperabile. L'endpoint di eliminazione risponde 409 con un messaggio esplicito invece di far affiorare un errore tecnico di chiave esterna. Scelta di prodotto di Fabio del 04/09 fra tre alternative: scartate lo sganciamento delle prenotazioni e la sostituzione dell'eliminazione con una disattivazione, quest'ultima buona per il futuro ma fuori dal perimetro della fase.</t>
+  </si>
+  <si>
+    <t>Blocco 3 - REV-037: audit trail consultabile</t>
+  </si>
+  <si>
+    <t>La tabella del registro attivita' cresce a ogni operazione, non viene mai ripulita e non aveva ne' indici ne' limiti di lunghezza: qualunque lettura era una scansione completa. Aggiunti i limiti di lunghezza e due indici, uno sul momento dell'evento e uno composto su utente e momento, pensato per servire anche l'ordinamento e non solo il filtro. Nuovo controller di sola lettura riservato all'Admin, paginato e filtrabile per utente, intervallo di date e testo dell'azione. Per decisione di Fabio in questa fase solo l'endpoint, nessuna pagina: la consultazione grafica si valuta in Fase 8 o 10.</t>
+  </si>
+  <si>
+    <t>EF Core + ASP.NET Core</t>
+  </si>
+  <si>
+    <t>Blocco 3 - REV-032 residuo: audit log in transazione</t>
+  </si>
+  <si>
+    <t>Nuovo esecutore di transazione condiviso, applicato ai 12 punti di scrittura di Zone, Postazioni e Fasce: prima la scrittura e la registrazione nell'audit trail erano due salvataggi separati, quindi una modifica poteva restare a database senza alcuna traccia di chi l'aveva fatta. La cache si invalida dopo il commit, non dentro il blocco. Il service delle prenotazioni non lo usa: ha gia' il proprio helper, che in piu' traduce la violazione dell'indice univoco sullo slot in un 409 leggibile.</t>
+  </si>
+  <si>
+    <t>EF Core execution strategy</t>
+  </si>
+  <si>
+    <t>Blocco 4 - REV-039 e REV-028</t>
+  </si>
+  <si>
+    <t>I tavoli occupati si contano ora per fascia e non per giornata intera: un tavolo usato a pranzo risultava occupato anche a cena, quindi la sala sembrava piu' piena di quanto fosse mai stata. Il totale di giornata diventa il picco fra le fasce, cioe' il massimo numero di tavoli impegnati nello stesso momento; con una sola fascia i due criteri coincidono. REV-028 non richiede codice: commentato che lo scheduler non e' in cluster mode e cosa succederebbe con piu' repliche, innocuo per il job di completamento e una corsa fra cancellazioni per quello di pulizia.</t>
+  </si>
+  <si>
+    <t>LINQ + Quartz</t>
+  </si>
+  <si>
+    <t>Difetto trovato da un test gia' esistente</t>
+  </si>
+  <si>
+    <t>Calcolando il picco di tavoli occupati a partire dall'elenco delle fasce configurate, le prenotazioni prese su una fascia poi disattivata o eliminata sparivano dal conteggio e la sala risultava libera mentre i tavoli erano occupati. Il picco va calcolato raggruppando le prenotazioni per fascia, non partendo dalle fasce. Il caso e' ora presidiato da un test dedicato.</t>
+  </si>
+  <si>
+    <t>xUnit + EF InMemory</t>
+  </si>
+  <si>
+    <t>Verifiche e controprova sui test</t>
+  </si>
+  <si>
+    <t>224 test verdi su 224 (erano 168), ricompilazione completa senza errori e con 50 warning tutti pre-esistenti. Controprova come in Fase 5: rotti di proposito due punti (l'invalidazione della cache per giorno e il secondo criterio di ordinamento) e verificato che fallissero esattamente i due test attesi, poi ripristinati. Attenzione emersa: cambiando i job da una scrittura per riga a una in blocco, i test negativi che verificavano 'mai chiamato' sul vecchio metodo sarebbero passati sempre, controllando qualcosa che non viene piu' invocato - sono stati riscritti sul metodo nuovo.</t>
+  </si>
+  <si>
+    <t>Cosa resta prima del rilascio</t>
+  </si>
+  <si>
+    <t>C'e' una migration da applicare, in locale e poi in produzione a mano da Fabio. Prima di applicarla va controllato che nessun dato superi i nuovi limiti di lunghezza sulla tabella del registro attivita' (attesi ben sotto 450, 500 e 45 caratteri). Restano poi le prove manuali: elenco utenti dopo il fix delle query, eliminazione di un utente con prenotazioni, lettura del registro con token Admin, dashboard con due fasce nello stesso giorno. Infine, solo dopo il deploy, la verifica che l'audit trail registri l'indirizzo reale del client: dietro il proxy e' l'unica prova possibile che il middleware degli header inoltrati funzioni davvero.</t>
+  </si>
+  <si>
+    <t>Robustezza del backend (Fase 7)</t>
+  </si>
+  <si>
+    <t>Paginazione con ordinamento stabile e numero di pagina validato, cache delle fasce invalidata anche sull'eliminazione, liste vuote al posto degli errori, validator sull'endpoint pubblico, tavolo modificabile finche' non ha impegni futuri, query pesanti alleggerite (elenco utenti e job notturni), indirizzo IP reale nei log e nel rate limit, storico delle prenotazioni protetto dall'eliminazione dell'utente, registro attivita' indicizzato e consultabile, audit log dentro la transazione, tavoli occupati contati per fascia.</t>
+  </si>
+  <si>
+    <t>ASP.NET Core + EF Core + Quartz</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 7</t>
+  </si>
+  <si>
+    <t>Robustezza del backend: REV-018, REV-019, REV-020, REV-021, REV-022, REV-023, REV-027, REV-028, REV-029, REV-031, REV-032 residuo, REV-037, REV-038, REV-039, piu' NEW-003/REV-099. Codice completo e verde in locale; restano la migration e le prove manuali.</t>
+  </si>
+  <si>
+    <t>Robustezza del backend (14 punti)</t>
+  </si>
+  <si>
+    <t>Numero di pagina non validato e ordinamento non deterministico nelle liste paginate; cache delle fasce non invalidata sull'eliminazione; ultimi due 404 su collezione vuota; validator mancante sull'unico endpoint pubblico; tavolo bloccato per sempre dalla prima prenotazione conclusa; query 1+N su elenco utenti e job notturni; caricamento inutile dello storico nel percorso caldo; indirizzo del proxy al posto di quello del client, che rendeva il rate limit del login di fatto globale; eliminazione utente che cancellava a cascata lo storico; registro attivita' senza indici e non consultabile; audit log fuori transazione su Zone, Postazioni e Fasce; tavoli occupati contati per giornata invece che per fascia. Test 224/224. Migration da applicare.</t>
+  </si>
+  <si>
+    <t>TEST UNITARI - xUnit + Moq  (Totale: 224 test  |  Tutti OK  |  elenco dettagliato fermo alla Fase 2b/42 test - da Fase 3 in poi il riepilogo per fase e' in ROADMAP_REVISIONE.md e nel foglio Appunti e Step)</t>
+  </si>
+  <si>
+    <t>224 test unitari</t>
+  </si>
+  <si>
+    <t>Testing - 224 test OK</t>
+  </si>
+  <si>
+    <t>FASE 7 ROADMAP REVISIONE - Robustezza del backend (sessione 04/09/2026)</t>
+  </si>
+  <si>
+    <t>LogActivity</t>
+  </si>
+  <si>
+    <t>get-log</t>
+  </si>
+  <si>
+    <t>userId, da, a, azione, page, pageSize (query, tutti opzionali; pageSize max 200)</t>
+  </si>
+  <si>
+    <t>200 PagedResult di LogActivityDTO, dal piu' recente - REV-037, Fase 7. Lettura dell'audit trail: prima la tabella si scriveva soltanto. userName puo' essere null, la traccia sopravvive all'utente. Nessuna interfaccia frontend.</t>
   </si>
 </sst>
 </file>
@@ -4857,7 +4998,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -4892,7 +5033,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5012,13 +5153,13 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="6" t="s">
-        <v>6</v>
+        <v>1403</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1356</v>
+        <v>1353</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1356</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5026,11 +5167,13 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1357</v>
-      </c>
-      <c r="C13" s="3"/>
+        <v>1404</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>1404</v>
+      </c>
       <c r="D13" s="1" t="s">
-        <v>1357</v>
+        <v>1354</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -5050,7 +5193,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5102,7 +5245,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -5324,13 +5467,13 @@
     </row>
     <row r="13" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="B13" t="s">
         <v>665</v>
       </c>
       <c r="C13" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="D13" t="s">
         <v>653</v>
@@ -5339,27 +5482,27 @@
         <v>437</v>
       </c>
       <c r="F13" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="B14" t="s">
         <v>651</v>
       </c>
       <c r="C14" t="s">
+        <v>1270</v>
+      </c>
+      <c r="D14" t="s">
         <v>1271</v>
-      </c>
-      <c r="D14" t="s">
-        <v>1272</v>
       </c>
       <c r="E14" t="s">
         <v>654</v>
       </c>
       <c r="F14" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5919,7 +6062,7 @@
         <v>687</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6019,10 +6162,10 @@
         <v>740</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>1328</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
         <v>354</v>
       </c>
@@ -6039,7 +6182,7 @@
         <v>669</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>693</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -6180,6 +6323,26 @@
       </c>
       <c r="F55" t="s">
         <v>985</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>1406</v>
+      </c>
+      <c r="B56" t="s">
+        <v>665</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1407</v>
+      </c>
+      <c r="D56" t="s">
+        <v>660</v>
+      </c>
+      <c r="E56" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F56" t="s">
+        <v>1409</v>
       </c>
     </row>
   </sheetData>
@@ -6204,7 +6367,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="56" t="s">
-        <v>1300</v>
+        <v>1402</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
@@ -6723,16 +6886,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B33" t="s">
         <v>1173</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>1174</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>1175</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1176</v>
       </c>
       <c r="E33" s="27" t="s">
         <v>6</v>
@@ -6740,16 +6903,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B34" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C34" t="s">
         <v>1177</v>
       </c>
-      <c r="C34" t="s">
-        <v>1178</v>
-      </c>
       <c r="D34" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="E34" s="27" t="s">
         <v>6</v>
@@ -6757,16 +6920,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B35" t="s">
+        <v>1178</v>
+      </c>
+      <c r="C35" t="s">
         <v>1179</v>
       </c>
-      <c r="C35" t="s">
-        <v>1180</v>
-      </c>
       <c r="D35" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="E35" s="27" t="s">
         <v>6</v>
@@ -6774,16 +6937,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B36" t="s">
+        <v>1180</v>
+      </c>
+      <c r="C36" t="s">
         <v>1181</v>
       </c>
-      <c r="C36" t="s">
-        <v>1182</v>
-      </c>
       <c r="D36" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -6791,13 +6954,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B37" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C37" t="s">
         <v>1183</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1184</v>
       </c>
       <c r="D37" t="s">
         <v>1067</v>
@@ -6808,13 +6971,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B38" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C38" t="s">
         <v>1185</v>
-      </c>
-      <c r="C38" t="s">
-        <v>1186</v>
       </c>
       <c r="D38" t="s">
         <v>1067</v>
@@ -6828,13 +6991,13 @@
         <v>772</v>
       </c>
       <c r="B39" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C39" t="s">
         <v>1187</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>1188</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1189</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -6845,13 +7008,13 @@
         <v>772</v>
       </c>
       <c r="B40" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C40" t="s">
         <v>1190</v>
       </c>
-      <c r="C40" t="s">
-        <v>1191</v>
-      </c>
       <c r="D40" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -6862,13 +7025,13 @@
         <v>772</v>
       </c>
       <c r="B41" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C41" t="s">
         <v>1192</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>1193</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1194</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -6879,13 +7042,13 @@
         <v>772</v>
       </c>
       <c r="B42" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C42" t="s">
         <v>1195</v>
       </c>
-      <c r="C42" t="s">
-        <v>1196</v>
-      </c>
       <c r="D42" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="E42" s="27" t="s">
         <v>6</v>
@@ -6896,13 +7059,13 @@
         <v>772</v>
       </c>
       <c r="B43" t="s">
+        <v>1196</v>
+      </c>
+      <c r="C43" t="s">
         <v>1197</v>
       </c>
-      <c r="C43" t="s">
-        <v>1198</v>
-      </c>
       <c r="D43" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>6</v>
@@ -6913,13 +7076,13 @@
         <v>772</v>
       </c>
       <c r="B44" t="s">
+        <v>1198</v>
+      </c>
+      <c r="C44" t="s">
         <v>1199</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>1200</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1201</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>6</v>
@@ -6930,13 +7093,13 @@
         <v>772</v>
       </c>
       <c r="B45" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C45" t="s">
         <v>1202</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>1203</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1204</v>
       </c>
       <c r="E45" s="27" t="s">
         <v>6</v>
@@ -7319,7 +7482,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H216"/>
+  <dimension ref="A1:H232"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7344,7 +7507,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -8405,24 +8568,24 @@
     </row>
     <row r="71" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="44" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="B71" s="25" t="s">
+        <v>1221</v>
+      </c>
+      <c r="C71" s="25" t="s">
         <v>1222</v>
-      </c>
-      <c r="C71" s="25" t="s">
-        <v>1223</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="44" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="B72" s="25" t="s">
+        <v>1223</v>
+      </c>
+      <c r="C72" s="25" t="s">
         <v>1224</v>
-      </c>
-      <c r="C72" s="25" t="s">
-        <v>1225</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -9875,7 +10038,7 @@
         <v>1157</v>
       </c>
       <c r="C169" s="27" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="D169" s="27" t="s">
         <v>1158</v>
@@ -9909,7 +10072,7 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
@@ -9937,16 +10100,16 @@
         <v>1</v>
       </c>
       <c r="B174" s="27" t="s">
+        <v>1206</v>
+      </c>
+      <c r="C174" s="27" t="s">
         <v>1207</v>
       </c>
-      <c r="C174" s="27" t="s">
+      <c r="D174" s="27" t="s">
         <v>1208</v>
       </c>
-      <c r="D174" s="27" t="s">
+      <c r="E174" s="40" t="s">
         <v>1209</v>
-      </c>
-      <c r="E174" s="40" t="s">
-        <v>1210</v>
       </c>
       <c r="F174" s="27" t="s">
         <v>6</v>
@@ -9957,16 +10120,16 @@
         <v>2</v>
       </c>
       <c r="B175" s="27" t="s">
+        <v>1210</v>
+      </c>
+      <c r="C175" s="27" t="s">
         <v>1211</v>
       </c>
-      <c r="C175" s="27" t="s">
+      <c r="D175" s="27" t="s">
         <v>1212</v>
       </c>
-      <c r="D175" s="27" t="s">
-        <v>1213</v>
-      </c>
       <c r="E175" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F175" s="27" t="s">
         <v>6</v>
@@ -9977,16 +10140,16 @@
         <v>3</v>
       </c>
       <c r="B176" s="27" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C176" s="27" t="s">
         <v>1214</v>
       </c>
-      <c r="C176" s="27" t="s">
+      <c r="D176" s="27" t="s">
         <v>1215</v>
       </c>
-      <c r="D176" s="27" t="s">
-        <v>1216</v>
-      </c>
       <c r="E176" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F176" s="27" t="s">
         <v>6</v>
@@ -9997,16 +10160,16 @@
         <v>4</v>
       </c>
       <c r="B177" s="27" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C177" s="27" t="s">
         <v>1217</v>
       </c>
-      <c r="C177" s="27" t="s">
+      <c r="D177" s="27" t="s">
         <v>1218</v>
       </c>
-      <c r="D177" s="27" t="s">
-        <v>1219</v>
-      </c>
       <c r="E177" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F177" s="43" t="s">
         <v>1129</v>
@@ -10017,16 +10180,16 @@
         <v>5</v>
       </c>
       <c r="B178" s="27" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C178" s="27" t="s">
         <v>1220</v>
-      </c>
-      <c r="C178" s="27" t="s">
-        <v>1221</v>
       </c>
       <c r="D178" s="27" t="s">
         <v>437</v>
       </c>
       <c r="E178" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F178" s="27" t="s">
         <v>6</v>
@@ -10034,7 +10197,7 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -10062,16 +10225,16 @@
         <v>1</v>
       </c>
       <c r="B182" s="27" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C182" s="27" t="s">
         <v>1238</v>
       </c>
-      <c r="C182" s="27" t="s">
+      <c r="D182" s="27" t="s">
         <v>1239</v>
       </c>
-      <c r="D182" s="27" t="s">
-        <v>1240</v>
-      </c>
       <c r="E182" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F182" s="27" t="s">
         <v>6</v>
@@ -10082,16 +10245,16 @@
         <v>2</v>
       </c>
       <c r="B183" s="27" t="s">
+        <v>1240</v>
+      </c>
+      <c r="C183" s="27" t="s">
         <v>1241</v>
       </c>
-      <c r="C183" s="27" t="s">
+      <c r="D183" s="27" t="s">
         <v>1242</v>
       </c>
-      <c r="D183" s="27" t="s">
-        <v>1243</v>
-      </c>
       <c r="E183" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F183" s="27" t="s">
         <v>6</v>
@@ -10102,16 +10265,16 @@
         <v>3</v>
       </c>
       <c r="B184" s="27" t="s">
+        <v>1243</v>
+      </c>
+      <c r="C184" s="27" t="s">
         <v>1244</v>
       </c>
-      <c r="C184" s="27" t="s">
+      <c r="D184" s="27" t="s">
         <v>1245</v>
       </c>
-      <c r="D184" s="27" t="s">
-        <v>1246</v>
-      </c>
       <c r="E184" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F184" s="27" t="s">
         <v>6</v>
@@ -10122,16 +10285,16 @@
         <v>4</v>
       </c>
       <c r="B185" s="27" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C185" s="27" t="s">
         <v>1247</v>
-      </c>
-      <c r="C185" s="27" t="s">
-        <v>1248</v>
       </c>
       <c r="D185" s="27" t="s">
         <v>401</v>
       </c>
       <c r="E185" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F185" s="27" t="s">
         <v>6</v>
@@ -10142,16 +10305,16 @@
         <v>5</v>
       </c>
       <c r="B186" s="27" t="s">
+        <v>1248</v>
+      </c>
+      <c r="C186" s="27" t="s">
         <v>1249</v>
       </c>
-      <c r="C186" s="27" t="s">
+      <c r="D186" s="27" t="s">
         <v>1250</v>
       </c>
-      <c r="D186" s="27" t="s">
-        <v>1251</v>
-      </c>
       <c r="E186" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F186" s="27" t="s">
         <v>6</v>
@@ -10162,16 +10325,16 @@
         <v>6</v>
       </c>
       <c r="B187" s="27" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C187" s="27" t="s">
         <v>1252</v>
       </c>
-      <c r="C187" s="27" t="s">
+      <c r="D187" s="27" t="s">
         <v>1253</v>
       </c>
-      <c r="D187" s="27" t="s">
-        <v>1254</v>
-      </c>
       <c r="E187" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F187" s="27" t="s">
         <v>6</v>
@@ -10182,16 +10345,16 @@
         <v>7</v>
       </c>
       <c r="B188" s="27" t="s">
+        <v>1254</v>
+      </c>
+      <c r="C188" s="27" t="s">
         <v>1255</v>
-      </c>
-      <c r="C188" s="27" t="s">
-        <v>1256</v>
       </c>
       <c r="D188" s="27" t="s">
         <v>22</v>
       </c>
       <c r="E188" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F188" s="43" t="s">
         <v>1129</v>
@@ -10202,16 +10365,16 @@
         <v>8</v>
       </c>
       <c r="B189" s="27" t="s">
+        <v>1273</v>
+      </c>
+      <c r="C189" s="27" t="s">
         <v>1274</v>
       </c>
-      <c r="C189" s="27" t="s">
+      <c r="D189" s="27" t="s">
         <v>1275</v>
       </c>
-      <c r="D189" s="27" t="s">
-        <v>1276</v>
-      </c>
       <c r="E189" s="40" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F189" s="27" t="s">
         <v>6</v>
@@ -10222,13 +10385,13 @@
         <v>9</v>
       </c>
       <c r="B190" s="27" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C190" s="27" t="s">
+        <v>1281</v>
+      </c>
+      <c r="D190" s="27" t="s">
         <v>1257</v>
-      </c>
-      <c r="C190" s="27" t="s">
-        <v>1282</v>
-      </c>
-      <c r="D190" s="27" t="s">
-        <v>1258</v>
       </c>
       <c r="E190" s="40" t="s">
         <v>437</v>
@@ -10239,7 +10402,7 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
@@ -10267,10 +10430,10 @@
         <v>1</v>
       </c>
       <c r="B193" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C193" t="s">
         <v>1284</v>
-      </c>
-      <c r="C193" t="s">
-        <v>1285</v>
       </c>
       <c r="D193" t="s">
         <v>1154</v>
@@ -10287,10 +10450,10 @@
         <v>2</v>
       </c>
       <c r="B194" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C194" t="s">
         <v>1286</v>
-      </c>
-      <c r="C194" t="s">
-        <v>1287</v>
       </c>
       <c r="D194" t="s">
         <v>74</v>
@@ -10307,13 +10470,13 @@
         <v>3</v>
       </c>
       <c r="B195" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C195" t="s">
         <v>1288</v>
       </c>
-      <c r="C195" t="s">
+      <c r="D195" t="s">
         <v>1289</v>
-      </c>
-      <c r="D195" t="s">
-        <v>1290</v>
       </c>
       <c r="E195" s="45">
         <v>46090</v>
@@ -10327,10 +10490,10 @@
         <v>4</v>
       </c>
       <c r="B196" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C196" t="s">
         <v>1291</v>
-      </c>
-      <c r="C196" t="s">
-        <v>1292</v>
       </c>
       <c r="D196" t="s">
         <v>74</v>
@@ -10347,13 +10510,13 @@
         <v>5</v>
       </c>
       <c r="B197" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="C197" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
       <c r="D197" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="E197" s="45">
         <v>46090</v>
@@ -10367,24 +10530,24 @@
         <v>6</v>
       </c>
       <c r="B198" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C198" t="s">
         <v>1294</v>
       </c>
-      <c r="C198" t="s">
+      <c r="D198" t="s">
         <v>1295</v>
-      </c>
-      <c r="D198" t="s">
-        <v>1296</v>
       </c>
       <c r="E198" t="s">
         <v>437</v>
       </c>
       <c r="F198" s="38" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
-        <v>1302</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
@@ -10412,13 +10575,13 @@
         <v>1</v>
       </c>
       <c r="B202" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D202" t="s">
         <v>1303</v>
-      </c>
-      <c r="C202" t="s">
-        <v>1304</v>
-      </c>
-      <c r="D202" t="s">
-        <v>1305</v>
       </c>
       <c r="E202" s="45">
         <v>46121</v>
@@ -10432,13 +10595,13 @@
         <v>2</v>
       </c>
       <c r="B203" t="s">
+        <v>1304</v>
+      </c>
+      <c r="C203" t="s">
+        <v>1305</v>
+      </c>
+      <c r="D203" t="s">
         <v>1306</v>
-      </c>
-      <c r="C203" t="s">
-        <v>1307</v>
-      </c>
-      <c r="D203" t="s">
-        <v>1308</v>
       </c>
       <c r="E203" s="45">
         <v>46121</v>
@@ -10452,13 +10615,13 @@
         <v>3</v>
       </c>
       <c r="B204" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C204" t="s">
+        <v>1308</v>
+      </c>
+      <c r="D204" t="s">
         <v>1309</v>
-      </c>
-      <c r="C204" t="s">
-        <v>1310</v>
-      </c>
-      <c r="D204" t="s">
-        <v>1311</v>
       </c>
       <c r="E204" s="45">
         <v>46121</v>
@@ -10472,13 +10635,13 @@
         <v>4</v>
       </c>
       <c r="B205" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C205" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D205" t="s">
         <v>1312</v>
-      </c>
-      <c r="C205" t="s">
-        <v>1313</v>
-      </c>
-      <c r="D205" t="s">
-        <v>1314</v>
       </c>
       <c r="E205" s="45">
         <v>46121</v>
@@ -10492,13 +10655,13 @@
         <v>5</v>
       </c>
       <c r="B206" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C206" t="s">
+        <v>1314</v>
+      </c>
+      <c r="D206" t="s">
         <v>1315</v>
-      </c>
-      <c r="C206" t="s">
-        <v>1316</v>
-      </c>
-      <c r="D206" t="s">
-        <v>1317</v>
       </c>
       <c r="E206" s="45">
         <v>46121</v>
@@ -10512,13 +10675,13 @@
         <v>6</v>
       </c>
       <c r="B207" t="s">
+        <v>1316</v>
+      </c>
+      <c r="C207" t="s">
+        <v>1317</v>
+      </c>
+      <c r="D207" t="s">
         <v>1318</v>
-      </c>
-      <c r="C207" t="s">
-        <v>1319</v>
-      </c>
-      <c r="D207" t="s">
-        <v>1320</v>
       </c>
       <c r="E207" s="45">
         <v>46121</v>
@@ -10532,13 +10695,13 @@
         <v>7</v>
       </c>
       <c r="B208" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C208" t="s">
+        <v>1329</v>
+      </c>
+      <c r="D208" t="s">
         <v>1330</v>
-      </c>
-      <c r="C208" t="s">
-        <v>1331</v>
-      </c>
-      <c r="D208" t="s">
-        <v>1332</v>
       </c>
       <c r="E208" s="45">
         <v>46121</v>
@@ -10552,13 +10715,13 @@
         <v>8</v>
       </c>
       <c r="B209" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="C209" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="D209" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="E209" s="45">
         <v>46121</v>
@@ -10572,13 +10735,13 @@
         <v>8</v>
       </c>
       <c r="B210" t="s">
+        <v>1337</v>
+      </c>
+      <c r="C210" t="s">
+        <v>1338</v>
+      </c>
+      <c r="D210" t="s">
         <v>1339</v>
-      </c>
-      <c r="C210" t="s">
-        <v>1340</v>
-      </c>
-      <c r="D210" t="s">
-        <v>1341</v>
       </c>
       <c r="E210" s="45">
         <v>46121</v>
@@ -10592,13 +10755,13 @@
         <v>9</v>
       </c>
       <c r="B211" t="s">
+        <v>1340</v>
+      </c>
+      <c r="C211" t="s">
+        <v>1341</v>
+      </c>
+      <c r="D211" t="s">
         <v>1342</v>
-      </c>
-      <c r="C211" t="s">
-        <v>1343</v>
-      </c>
-      <c r="D211" t="s">
-        <v>1344</v>
       </c>
       <c r="E211" s="45">
         <v>46121</v>
@@ -10612,13 +10775,13 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
+        <v>1343</v>
+      </c>
+      <c r="C212" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D212" t="s">
         <v>1345</v>
-      </c>
-      <c r="C212" t="s">
-        <v>1346</v>
-      </c>
-      <c r="D212" t="s">
-        <v>1347</v>
       </c>
       <c r="E212" s="45">
         <v>46121</v>
@@ -10632,13 +10795,13 @@
         <v>11</v>
       </c>
       <c r="B213" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C213" t="s">
+        <v>1347</v>
+      </c>
+      <c r="D213" t="s">
         <v>1348</v>
-      </c>
-      <c r="C213" t="s">
-        <v>1349</v>
-      </c>
-      <c r="D213" t="s">
-        <v>1350</v>
       </c>
       <c r="E213" s="45">
         <v>46121</v>
@@ -10652,13 +10815,13 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C214" t="s">
+        <v>1350</v>
+      </c>
+      <c r="D214" t="s">
         <v>1351</v>
-      </c>
-      <c r="C214" t="s">
-        <v>1352</v>
-      </c>
-      <c r="D214" t="s">
-        <v>1353</v>
       </c>
       <c r="E214" s="45">
         <v>46121</v>
@@ -10672,10 +10835,10 @@
         <v>13</v>
       </c>
       <c r="B215" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
       <c r="C215" t="s">
-        <v>1355</v>
+        <v>1359</v>
       </c>
       <c r="D215" t="s">
         <v>437</v>
@@ -10683,8 +10846,8 @@
       <c r="E215" s="45">
         <v>46121</v>
       </c>
-      <c r="F215" s="38" t="s">
-        <v>1301</v>
+      <c r="F215" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.3">
@@ -10692,19 +10855,304 @@
         <v>14</v>
       </c>
       <c r="B216" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C216" t="s">
         <v>1360</v>
       </c>
-      <c r="C216" t="s">
-        <v>1361</v>
-      </c>
       <c r="D216" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="E216" s="45">
         <v>46121</v>
       </c>
-      <c r="F216" s="38" t="s">
-        <v>1301</v>
+      <c r="F216" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>1405</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>39</v>
+      </c>
+      <c r="B219" t="s">
+        <v>40</v>
+      </c>
+      <c r="C219" t="s">
+        <v>857</v>
+      </c>
+      <c r="D219" t="s">
+        <v>42</v>
+      </c>
+      <c r="E219" t="s">
+        <v>43</v>
+      </c>
+      <c r="F219" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A220">
+        <v>1</v>
+      </c>
+      <c r="B220" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C220" t="s">
+        <v>1363</v>
+      </c>
+      <c r="D220" t="s">
+        <v>1364</v>
+      </c>
+      <c r="E220" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F220" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A221">
+        <v>2</v>
+      </c>
+      <c r="B221" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C221" t="s">
+        <v>1366</v>
+      </c>
+      <c r="D221" t="s">
+        <v>287</v>
+      </c>
+      <c r="E221" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F221" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A222">
+        <v>3</v>
+      </c>
+      <c r="B222" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C222" t="s">
+        <v>1368</v>
+      </c>
+      <c r="D222" t="s">
+        <v>29</v>
+      </c>
+      <c r="E222" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F222" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A223">
+        <v>4</v>
+      </c>
+      <c r="B223" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C223" t="s">
+        <v>1370</v>
+      </c>
+      <c r="D223" t="s">
+        <v>1371</v>
+      </c>
+      <c r="E223" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F223" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A224">
+        <v>5</v>
+      </c>
+      <c r="B224" t="s">
+        <v>1372</v>
+      </c>
+      <c r="C224" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D224" t="s">
+        <v>1364</v>
+      </c>
+      <c r="E224" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F224" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A225">
+        <v>6</v>
+      </c>
+      <c r="B225" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C225" t="s">
+        <v>1375</v>
+      </c>
+      <c r="D225" t="s">
+        <v>1376</v>
+      </c>
+      <c r="E225" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F225" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A226">
+        <v>7</v>
+      </c>
+      <c r="B226" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C226" t="s">
+        <v>1378</v>
+      </c>
+      <c r="D226" t="s">
+        <v>267</v>
+      </c>
+      <c r="E226" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F226" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A227">
+        <v>8</v>
+      </c>
+      <c r="B227" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C227" t="s">
+        <v>1380</v>
+      </c>
+      <c r="D227" t="s">
+        <v>1381</v>
+      </c>
+      <c r="E227" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F227" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A228">
+        <v>9</v>
+      </c>
+      <c r="B228" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C228" t="s">
+        <v>1383</v>
+      </c>
+      <c r="D228" t="s">
+        <v>1384</v>
+      </c>
+      <c r="E228" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F228" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A229">
+        <v>10</v>
+      </c>
+      <c r="B229" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C229" t="s">
+        <v>1386</v>
+      </c>
+      <c r="D229" t="s">
+        <v>1387</v>
+      </c>
+      <c r="E229" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F229" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A230">
+        <v>11</v>
+      </c>
+      <c r="B230" t="s">
+        <v>1388</v>
+      </c>
+      <c r="C230" t="s">
+        <v>1389</v>
+      </c>
+      <c r="D230" t="s">
+        <v>1390</v>
+      </c>
+      <c r="E230" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F230" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A231">
+        <v>12</v>
+      </c>
+      <c r="B231" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C231" t="s">
+        <v>1392</v>
+      </c>
+      <c r="D231" t="s">
+        <v>32</v>
+      </c>
+      <c r="E231" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F231" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A232">
+        <v>13</v>
+      </c>
+      <c r="B232" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C232" t="s">
+        <v>1394</v>
+      </c>
+      <c r="D232" t="s">
+        <v>437</v>
+      </c>
+      <c r="E232" s="45">
+        <v>46121</v>
+      </c>
+      <c r="F232" s="38" t="s">
+        <v>1299</v>
       </c>
     </row>
   </sheetData>
@@ -10723,7 +11171,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -11148,7 +11596,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1358</v>
+        <v>1355</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -11230,13 +11678,13 @@
         <v>1043</v>
       </c>
       <c r="B36" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C36" t="s">
         <v>1259</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>1260</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1261</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -11247,16 +11695,33 @@
         <v>1043</v>
       </c>
       <c r="B37" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
       <c r="C37" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="D37" t="s">
-        <v>1324</v>
-      </c>
-      <c r="E37" s="38" t="s">
-        <v>1301</v>
+        <v>1322</v>
+      </c>
+      <c r="E37" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1396</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1397</v>
+      </c>
+      <c r="E38" s="38" t="s">
+        <v>1299</v>
       </c>
     </row>
   </sheetData>
@@ -11273,7 +11738,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -11681,13 +12146,13 @@
         <v>1164</v>
       </c>
       <c r="E21" s="41" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="41" t="s">
         <v>1226</v>
-      </c>
-      <c r="F21" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="G21" s="41" t="s">
-        <v>1227</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -11701,39 +12166,39 @@
         <v>1166</v>
       </c>
       <c r="D22" s="41" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="E22" s="41" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="F22" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="41" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B23" s="41" t="s">
         <v>1277</v>
       </c>
-      <c r="B23" s="41" t="s">
+      <c r="C23" s="41" t="s">
         <v>1278</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="D23" s="41" t="s">
+        <v>1225</v>
+      </c>
+      <c r="E23" s="41" t="s">
+        <v>1225</v>
+      </c>
+      <c r="F23" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G23" s="41" t="s">
         <v>1279</v>
-      </c>
-      <c r="D23" s="41" t="s">
-        <v>1226</v>
-      </c>
-      <c r="E23" s="41" t="s">
-        <v>1226</v>
-      </c>
-      <c r="F23" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="G23" s="41" t="s">
-        <v>1280</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -11741,22 +12206,22 @@
         <v>1008</v>
       </c>
       <c r="B24" s="41" t="s">
+        <v>1262</v>
+      </c>
+      <c r="C24" s="41" t="s">
         <v>1263</v>
       </c>
-      <c r="C24" s="41" t="s">
-        <v>1264</v>
-      </c>
       <c r="D24" s="41" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="E24" s="41" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="F24" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G24" s="41" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -11764,20 +12229,39 @@
         <v>1008</v>
       </c>
       <c r="B25" s="41" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="C25" s="41" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="D25" s="41" t="s">
-        <v>1326</v>
-      </c>
-      <c r="E25" s="41"/>
-      <c r="F25" s="38" t="s">
-        <v>1301</v>
+        <v>1324</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F25" s="27" t="s">
+        <v>6</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>1362</v>
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1398</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1399</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>1299</v>
       </c>
     </row>
   </sheetData>
@@ -11791,7 +12275,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -12274,7 +12758,7 @@
         <v>1122</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="D39" s="27" t="s">
         <v>6</v>
@@ -12318,19 +12802,19 @@
       <c r="C42" s="41" t="s">
         <v>1171</v>
       </c>
-      <c r="D42" s="43" t="s">
-        <v>1172</v>
+      <c r="D42" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="41" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B43" s="41" t="s">
         <v>1228</v>
       </c>
-      <c r="B43" s="41" t="s">
+      <c r="C43" s="41" t="s">
         <v>1229</v>
-      </c>
-      <c r="C43" s="41" t="s">
-        <v>1230</v>
       </c>
       <c r="D43" s="27" t="s">
         <v>6</v>
@@ -12341,10 +12825,10 @@
         <v>1121</v>
       </c>
       <c r="B44" s="41" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="C44" s="41" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="D44" s="27" t="s">
         <v>6</v>
@@ -12352,16 +12836,16 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="41" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B45" s="41" t="s">
         <v>1232</v>
       </c>
-      <c r="B45" s="41" t="s">
+      <c r="C45" s="41" t="s">
         <v>1233</v>
       </c>
-      <c r="C45" s="41" t="s">
+      <c r="D45" s="43" t="s">
         <v>1234</v>
-      </c>
-      <c r="D45" s="43" t="s">
-        <v>1235</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -12369,10 +12853,10 @@
         <v>1165</v>
       </c>
       <c r="B46" s="27" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C46" s="27" t="s">
         <v>1265</v>
-      </c>
-      <c r="C46" s="27" t="s">
-        <v>1266</v>
       </c>
       <c r="D46" s="27" t="s">
         <v>6</v>
@@ -12380,13 +12864,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="B47" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C47" t="s">
         <v>1298</v>
-      </c>
-      <c r="C47" t="s">
-        <v>1299</v>
       </c>
       <c r="D47" s="27" t="s">
         <v>6</v>
@@ -12394,16 +12878,30 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="B48" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="C48" t="s">
-        <v>1359</v>
-      </c>
-      <c r="D48" s="38" t="s">
-        <v>1301</v>
+        <v>1356</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1400</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1401</v>
+      </c>
+      <c r="D49" s="38" t="s">
+        <v>1299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: chiusura Fase 7 - REV-029 verificato in produzione, tracker e documentazione
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4060647A-65E1-41C5-B5BF-7E0E0F3F3981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D493B661-4ABC-4C93-B19A-F5AF3B3C26DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2493" uniqueCount="1410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="1419">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3994,9 +3994,6 @@
     <t>eslint + tsc + vite</t>
   </si>
   <si>
-    <t>Aggiornato: 04/09/2026</t>
-  </si>
-  <si>
     <t>Bug del frontend (Fase 6)</t>
   </si>
   <si>
@@ -4216,9 +4213,6 @@
     <t>Cosa resta prima del rilascio</t>
   </si>
   <si>
-    <t>C'e' una migration da applicare, in locale e poi in produzione a mano da Fabio. Prima di applicarla va controllato che nessun dato superi i nuovi limiti di lunghezza sulla tabella del registro attivita' (attesi ben sotto 450, 500 e 45 caratteri). Restano poi le prove manuali: elenco utenti dopo il fix delle query, eliminazione di un utente con prenotazioni, lettura del registro con token Admin, dashboard con due fasce nello stesso giorno. Infine, solo dopo il deploy, la verifica che l'audit trail registri l'indirizzo reale del client: dietro il proxy e' l'unica prova possibile che il middleware degli header inoltrati funzioni davvero.</t>
-  </si>
-  <si>
     <t>Robustezza del backend (Fase 7)</t>
   </si>
   <si>
@@ -4240,15 +4234,6 @@
     <t>Numero di pagina non validato e ordinamento non deterministico nelle liste paginate; cache delle fasce non invalidata sull'eliminazione; ultimi due 404 su collezione vuota; validator mancante sull'unico endpoint pubblico; tavolo bloccato per sempre dalla prima prenotazione conclusa; query 1+N su elenco utenti e job notturni; caricamento inutile dello storico nel percorso caldo; indirizzo del proxy al posto di quello del client, che rendeva il rate limit del login di fatto globale; eliminazione utente che cancellava a cascata lo storico; registro attivita' senza indici e non consultabile; audit log fuori transazione su Zone, Postazioni e Fasce; tavoli occupati contati per giornata invece che per fascia. Test 224/224. Migration da applicare.</t>
   </si>
   <si>
-    <t>TEST UNITARI - xUnit + Moq  (Totale: 224 test  |  Tutti OK  |  elenco dettagliato fermo alla Fase 2b/42 test - da Fase 3 in poi il riepilogo per fase e' in ROADMAP_REVISIONE.md e nel foglio Appunti e Step)</t>
-  </si>
-  <si>
-    <t>224 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 224 test OK</t>
-  </si>
-  <si>
     <t>FASE 7 ROADMAP REVISIONE - Robustezza del backend (sessione 04/09/2026)</t>
   </si>
   <si>
@@ -4262,6 +4247,48 @@
   </si>
   <si>
     <t>200 PagedResult di LogActivityDTO, dal piu' recente - REV-037, Fase 7. Lettura dell'audit trail: prima la tabella si scriveva soltanto. userName puo' essere null, la traccia sopravvive all'utente. Nessuna interfaccia frontend.</t>
+  </si>
+  <si>
+    <t>Aggiornato: 07/09/2026</t>
+  </si>
+  <si>
+    <t>Chiuso il 07/09/2026. Migration applicata in locale e in produzione. Sanata anche un'anomalia della Fase 2a: il rename MaxPrenotazioni-&gt;MaxCoperti del 31/08 era stato applicato a mano senza registrare la riga in __EFMigrationsHistory, quindi lo schema era corretto ma EF continuava a considerare la migration da applicare e un futuro update avrebbe tentato di rieseguire il rename. Prove funzionali superate: elenco utenti, eliminazione di un utente con prenotazioni (409 leggibile), lettura del registro attivita' con token Admin e 403 per gli altri ruoli.</t>
+  </si>
+  <si>
+    <t>REV-029 - indirizzo reale del client (chiuso il 07/09)</t>
+  </si>
+  <si>
+    <t>E' costato tre deploy e tre giorni per un errore di metodo. La prima soluzione, il middleware standard con limite di catena a 2, era l'ipotesi giusta ed e' stata scartata perche' la diagnostica mostrava un solo indirizzo nell'header: quel valore era pero' il residuo dopo il passaggio del middleware, che rimuove l'anello che elabora. Leggendo un header gia' consumato sembrava esserci un solo proxy. Solo disattivando il middleware la catena e' tornata visibile per intero e sono comparsi i due anelli: client, proxy di frontiera, e la connessione in arrivo dalla rete interna. Soluzione finale: helper Common/IndirizzoClient che scarta l'anello dell'infrastruttura e prende l'ultimo rimasto - non il primo, che il client puo' falsificare, non l'ultimo, che e' il proxy. Applicato all'audit trail e alla partizione del rate limit del login, che prima era di fatto un limite globale di 5 tentativi al minuto per l'intera applicazione. 13 test unitari sull'helper, su casi prima verificabili solo in produzione. Verificato in produzione: l'audit trail registra l'indirizzo del client, le righe precedenti mostrano ancora quello del proxy. Lezione: quando un comportamento non e' riproducibile in locale, la prima cosa da scrivere e' lo strumento che lo rende osservabile, non la correzione.</t>
+  </si>
+  <si>
+    <t>ASP.NET Core + xUnit</t>
+  </si>
+  <si>
+    <t>07-set-26</t>
+  </si>
+  <si>
+    <t>Backend - Sicurezza e log</t>
+  </si>
+  <si>
+    <t>REV-029: registrato l'indirizzo del proxy al posto di quello del client</t>
+  </si>
+  <si>
+    <t>Oltre a rendere inutile l'audit trail, il difetto rendeva inefficace il rate limit del login, che partiziona sullo stesso valore: dietro il proxy tutti finivano nella stessa partizione, quindi era di fatto un limite globale di 5 tentativi al minuto per l'intera applicazione - non fermava chi attacca un singolo account e poteva bloccare gli utenti legittimi. Risolto con l'helper Common/IndirizzoClient dopo aver misurato la catena reale dei proxy con un endpoint diagnostico dedicato, tenuto in produzione proprio per poterla rimisurare se la piattaforma cambia.</t>
+  </si>
+  <si>
+    <t>diagnostica-inoltro</t>
+  </si>
+  <si>
+    <t>200 con l'indirizzo usato dall'applicazione e gli header di inoltro grezzi della richiesta corrente - REV-029. Serve a rimisurare la catena dei proxy se la piattaforma cambia: in locale quegli header non esistono, quindi e' l'unico modo di osservarla. Mostra solo i dati di chi chiama.</t>
+  </si>
+  <si>
+    <t>TEST UNITARI - xUnit + Moq  (Totale: 237 test  |  Tutti OK  |  elenco dettagliato fermo alla Fase 2b/42 test - da Fase 3 in poi il riepilogo per fase e' in ROADMAP_REVISIONE.md e nel foglio Appunti e Step)</t>
+  </si>
+  <si>
+    <t>237 test unitari</t>
+  </si>
+  <si>
+    <t>Testing - 237 test OK</t>
   </si>
 </sst>
 </file>
@@ -4998,7 +5025,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>1320</v>
+        <v>1405</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -5153,13 +5180,13 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="6" t="s">
-        <v>1403</v>
+        <v>1417</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5167,13 +5194,13 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1404</v>
+        <v>1418</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1404</v>
+        <v>1418</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -5245,7 +5272,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -6162,7 +6189,7 @@
         <v>740</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
@@ -6182,7 +6209,7 @@
         <v>669</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -6327,22 +6354,42 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>1406</v>
+        <v>1401</v>
       </c>
       <c r="B56" t="s">
         <v>665</v>
       </c>
       <c r="C56" t="s">
-        <v>1407</v>
+        <v>1402</v>
       </c>
       <c r="D56" t="s">
         <v>660</v>
       </c>
       <c r="E56" t="s">
-        <v>1408</v>
+        <v>1403</v>
       </c>
       <c r="F56" t="s">
-        <v>1409</v>
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B57" t="s">
+        <v>665</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D57" t="s">
+        <v>660</v>
+      </c>
+      <c r="E57" t="s">
+        <v>437</v>
+      </c>
+      <c r="F57" t="s">
+        <v>1415</v>
       </c>
     </row>
   </sheetData>
@@ -6367,7 +6414,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="56" t="s">
-        <v>1402</v>
+        <v>1416</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
@@ -7482,7 +7529,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H232"/>
+  <dimension ref="A1:H233"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7507,7 +7554,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
-        <v>1320</v>
+        <v>1405</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -10513,7 +10560,7 @@
         <v>1292</v>
       </c>
       <c r="C197" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="D197" t="s">
         <v>1253</v>
@@ -10695,13 +10742,13 @@
         <v>7</v>
       </c>
       <c r="B208" t="s">
+        <v>1327</v>
+      </c>
+      <c r="C208" t="s">
         <v>1328</v>
       </c>
-      <c r="C208" t="s">
+      <c r="D208" t="s">
         <v>1329</v>
-      </c>
-      <c r="D208" t="s">
-        <v>1330</v>
       </c>
       <c r="E208" s="45">
         <v>46121</v>
@@ -10715,10 +10762,10 @@
         <v>8</v>
       </c>
       <c r="B209" t="s">
+        <v>1334</v>
+      </c>
+      <c r="C209" t="s">
         <v>1335</v>
-      </c>
-      <c r="C209" t="s">
-        <v>1336</v>
       </c>
       <c r="D209" t="s">
         <v>1319</v>
@@ -10735,13 +10782,13 @@
         <v>8</v>
       </c>
       <c r="B210" t="s">
+        <v>1336</v>
+      </c>
+      <c r="C210" t="s">
         <v>1337</v>
       </c>
-      <c r="C210" t="s">
+      <c r="D210" t="s">
         <v>1338</v>
-      </c>
-      <c r="D210" t="s">
-        <v>1339</v>
       </c>
       <c r="E210" s="45">
         <v>46121</v>
@@ -10755,13 +10802,13 @@
         <v>9</v>
       </c>
       <c r="B211" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C211" t="s">
         <v>1340</v>
       </c>
-      <c r="C211" t="s">
+      <c r="D211" t="s">
         <v>1341</v>
-      </c>
-      <c r="D211" t="s">
-        <v>1342</v>
       </c>
       <c r="E211" s="45">
         <v>46121</v>
@@ -10775,13 +10822,13 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
+        <v>1342</v>
+      </c>
+      <c r="C212" t="s">
         <v>1343</v>
       </c>
-      <c r="C212" t="s">
+      <c r="D212" t="s">
         <v>1344</v>
-      </c>
-      <c r="D212" t="s">
-        <v>1345</v>
       </c>
       <c r="E212" s="45">
         <v>46121</v>
@@ -10795,13 +10842,13 @@
         <v>11</v>
       </c>
       <c r="B213" t="s">
+        <v>1345</v>
+      </c>
+      <c r="C213" t="s">
         <v>1346</v>
       </c>
-      <c r="C213" t="s">
+      <c r="D213" t="s">
         <v>1347</v>
-      </c>
-      <c r="D213" t="s">
-        <v>1348</v>
       </c>
       <c r="E213" s="45">
         <v>46121</v>
@@ -10815,13 +10862,13 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
+        <v>1348</v>
+      </c>
+      <c r="C214" t="s">
         <v>1349</v>
       </c>
-      <c r="C214" t="s">
+      <c r="D214" t="s">
         <v>1350</v>
-      </c>
-      <c r="D214" t="s">
-        <v>1351</v>
       </c>
       <c r="E214" s="45">
         <v>46121</v>
@@ -10835,10 +10882,10 @@
         <v>13</v>
       </c>
       <c r="B215" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="C215" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="D215" t="s">
         <v>437</v>
@@ -10855,10 +10902,10 @@
         <v>14</v>
       </c>
       <c r="B216" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="C216" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="D216" t="s">
         <v>1275</v>
@@ -10872,7 +10919,7 @@
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
-        <v>1405</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
@@ -10900,13 +10947,13 @@
         <v>1</v>
       </c>
       <c r="B220" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C220" t="s">
         <v>1362</v>
       </c>
-      <c r="C220" t="s">
+      <c r="D220" t="s">
         <v>1363</v>
-      </c>
-      <c r="D220" t="s">
-        <v>1364</v>
       </c>
       <c r="E220" s="45">
         <v>46121</v>
@@ -10920,10 +10967,10 @@
         <v>2</v>
       </c>
       <c r="B221" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C221" t="s">
         <v>1365</v>
-      </c>
-      <c r="C221" t="s">
-        <v>1366</v>
       </c>
       <c r="D221" t="s">
         <v>287</v>
@@ -10940,10 +10987,10 @@
         <v>3</v>
       </c>
       <c r="B222" t="s">
+        <v>1366</v>
+      </c>
+      <c r="C222" t="s">
         <v>1367</v>
-      </c>
-      <c r="C222" t="s">
-        <v>1368</v>
       </c>
       <c r="D222" t="s">
         <v>29</v>
@@ -10960,13 +11007,13 @@
         <v>4</v>
       </c>
       <c r="B223" t="s">
+        <v>1368</v>
+      </c>
+      <c r="C223" t="s">
         <v>1369</v>
       </c>
-      <c r="C223" t="s">
+      <c r="D223" t="s">
         <v>1370</v>
-      </c>
-      <c r="D223" t="s">
-        <v>1371</v>
       </c>
       <c r="E223" s="45">
         <v>46121</v>
@@ -10980,13 +11027,13 @@
         <v>5</v>
       </c>
       <c r="B224" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C224" t="s">
         <v>1372</v>
       </c>
-      <c r="C224" t="s">
-        <v>1373</v>
-      </c>
       <c r="D224" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="E224" s="45">
         <v>46121</v>
@@ -11000,13 +11047,13 @@
         <v>6</v>
       </c>
       <c r="B225" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C225" t="s">
         <v>1374</v>
       </c>
-      <c r="C225" t="s">
+      <c r="D225" t="s">
         <v>1375</v>
-      </c>
-      <c r="D225" t="s">
-        <v>1376</v>
       </c>
       <c r="E225" s="45">
         <v>46121</v>
@@ -11020,10 +11067,10 @@
         <v>7</v>
       </c>
       <c r="B226" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C226" t="s">
         <v>1377</v>
-      </c>
-      <c r="C226" t="s">
-        <v>1378</v>
       </c>
       <c r="D226" t="s">
         <v>267</v>
@@ -11040,13 +11087,13 @@
         <v>8</v>
       </c>
       <c r="B227" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C227" t="s">
         <v>1379</v>
       </c>
-      <c r="C227" t="s">
+      <c r="D227" t="s">
         <v>1380</v>
-      </c>
-      <c r="D227" t="s">
-        <v>1381</v>
       </c>
       <c r="E227" s="45">
         <v>46121</v>
@@ -11060,13 +11107,13 @@
         <v>9</v>
       </c>
       <c r="B228" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C228" t="s">
         <v>1382</v>
       </c>
-      <c r="C228" t="s">
+      <c r="D228" t="s">
         <v>1383</v>
-      </c>
-      <c r="D228" t="s">
-        <v>1384</v>
       </c>
       <c r="E228" s="45">
         <v>46121</v>
@@ -11080,13 +11127,13 @@
         <v>10</v>
       </c>
       <c r="B229" t="s">
+        <v>1384</v>
+      </c>
+      <c r="C229" t="s">
         <v>1385</v>
       </c>
-      <c r="C229" t="s">
+      <c r="D229" t="s">
         <v>1386</v>
-      </c>
-      <c r="D229" t="s">
-        <v>1387</v>
       </c>
       <c r="E229" s="45">
         <v>46121</v>
@@ -11100,13 +11147,13 @@
         <v>11</v>
       </c>
       <c r="B230" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C230" t="s">
         <v>1388</v>
       </c>
-      <c r="C230" t="s">
+      <c r="D230" t="s">
         <v>1389</v>
-      </c>
-      <c r="D230" t="s">
-        <v>1390</v>
       </c>
       <c r="E230" s="45">
         <v>46121</v>
@@ -11120,10 +11167,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
+        <v>1390</v>
+      </c>
+      <c r="C231" t="s">
         <v>1391</v>
-      </c>
-      <c r="C231" t="s">
-        <v>1392</v>
       </c>
       <c r="D231" t="s">
         <v>32</v>
@@ -11140,19 +11187,39 @@
         <v>13</v>
       </c>
       <c r="B232" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="C232" t="s">
-        <v>1394</v>
+        <v>1406</v>
       </c>
       <c r="D232" t="s">
         <v>437</v>
       </c>
       <c r="E232" s="45">
-        <v>46121</v>
-      </c>
-      <c r="F232" s="38" t="s">
-        <v>1299</v>
+        <v>46212</v>
+      </c>
+      <c r="F232" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A233">
+        <v>14</v>
+      </c>
+      <c r="B233" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C233" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D233" t="s">
+        <v>1409</v>
+      </c>
+      <c r="E233" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F233" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -11596,7 +11663,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -11695,13 +11762,13 @@
         <v>1043</v>
       </c>
       <c r="B37" t="s">
+        <v>1320</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1330</v>
+      </c>
+      <c r="D37" t="s">
         <v>1321</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1331</v>
-      </c>
-      <c r="D37" t="s">
-        <v>1322</v>
       </c>
       <c r="E37" s="27" t="s">
         <v>6</v>
@@ -11712,16 +11779,16 @@
         <v>1043</v>
       </c>
       <c r="B38" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1394</v>
+      </c>
+      <c r="D38" t="s">
         <v>1395</v>
       </c>
-      <c r="C38" t="s">
-        <v>1396</v>
-      </c>
-      <c r="D38" t="s">
-        <v>1397</v>
-      </c>
-      <c r="E38" s="38" t="s">
-        <v>1299</v>
+      <c r="E38" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -12229,22 +12296,22 @@
         <v>1008</v>
       </c>
       <c r="B25" s="41" t="s">
+        <v>1322</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>1331</v>
+      </c>
+      <c r="D25" s="41" t="s">
         <v>1323</v>
       </c>
-      <c r="C25" s="41" t="s">
-        <v>1332</v>
-      </c>
-      <c r="D25" s="41" t="s">
-        <v>1324</v>
-      </c>
       <c r="E25" s="41" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="F25" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -12252,16 +12319,19 @@
         <v>1008</v>
       </c>
       <c r="B26" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="C26" t="s">
-        <v>1399</v>
+        <v>1397</v>
       </c>
       <c r="D26" t="s">
-        <v>1324</v>
-      </c>
-      <c r="F26" s="38" t="s">
-        <v>1299</v>
+        <v>1323</v>
+      </c>
+      <c r="E26" t="s">
+        <v>1410</v>
+      </c>
+      <c r="F26" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -12275,7 +12345,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -12758,7 +12828,7 @@
         <v>1122</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="D39" s="27" t="s">
         <v>6</v>
@@ -12828,7 +12898,7 @@
         <v>1230</v>
       </c>
       <c r="C44" s="41" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="D44" s="27" t="s">
         <v>6</v>
@@ -12878,13 +12948,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="B48" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="C48" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="D48" s="27" t="s">
         <v>6</v>
@@ -12892,16 +12962,30 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B49" t="s">
         <v>1398</v>
       </c>
-      <c r="B49" t="s">
-        <v>1400</v>
-      </c>
       <c r="C49" t="s">
-        <v>1401</v>
-      </c>
-      <c r="D49" s="38" t="s">
-        <v>1299</v>
+        <v>1399</v>
+      </c>
+      <c r="D49" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1413</v>
+      </c>
+      <c r="D50" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Fase 9.0.1 - pulizia del codice (dead code, duplicazioni, refusi, npm audit)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22779ED0-8016-4D88-A8DF-9B44CAFD4CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6243A2-60D6-4814-8BFD-3E2E395B6383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2624" uniqueCount="1495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2716" uniqueCount="1546">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3868,9 +3868,6 @@
     <t>Fast-forward, commit 66e7f5c. Nessuna migration. Verificato in produzione: /health Healthy, /api/Setup/stato setupCompletato true, seed-admin 404. Railway e Vercel ridistribuiti sul push.</t>
   </si>
   <si>
-    <t>Railway - PostgreSQL + .NET, health check /health - in produzione v1.0.1 (03/09/2026)</t>
-  </si>
-  <si>
     <t>Test del backend: copertura del flusso di prenotazione (REV-051 creazione e modifica, REV-052 assegnazione reale del tavolo, REV-053 disponibilita' dashboard e ruoli, REV-054 job notturni). La release intermedia v1.0.1 e' stata decisa e fatta lo stesso giorno (vedi riga precedente).</t>
   </si>
   <si>
@@ -4402,9 +4399,6 @@
     <t>Prossimo passo - Fase 9</t>
   </si>
   <si>
-    <t>Pulizia: cartelle vuote e codice morto (REV-055, REV-077), costruttore fantasma di PrenotazioniService (REV-010), nome di 'fascia oraria' scritto in quattro modi (REV-056), duplicazioni e costanti ripetute (REV-058/059/060/061), implementazioni che lanciano solo NotImplementedException (REV-030), refusi e nomi troncati (REV-067, REV-068), path degli endpoint centralizzati (REV-082), formattazione automatica (REV-078). Nessun task per Fabio.</t>
-  </si>
-  <si>
     <t>Robustezza del frontend (Fase 8)</t>
   </si>
   <si>
@@ -4517,6 +4511,165 @@
   </si>
   <si>
     <t>FASE 8 CHIUSA 07/09/2026. Nessuna modifica al backend, nessuna migration, dotnet test invariato a 237/237. Introdotti i primi test del frontend: 26 verdi con Vitest + Testing Library. strict di TypeScript attivato senza un solo errore da correggere. Due difetti emersi lavorando e non previsti dalla roadmap: la policy password del frontend era piu' permissiva di quella del backend su registrazione e creazione utente, e uno dei test nuovi era vacuo (scoperto con la controprova). Prova manuale eseguita in locale: server irraggiungibile -&gt; toast dedicato, REV-041 confermato end-to-end. Le altre quattro prove (paginazione, notifica singola, doppio clic, password nel form) non sono state eseguite, nessuna bloccante. Emerso e registrato NEW-006 per la Fase 10. Da provare in produzione dopo il merge: paginazione su un elenco lungo e assenza dei devtools.</t>
+  </si>
+  <si>
+    <t>RILASCIO v1.0.4</t>
+  </si>
+  <si>
+    <t>Commit 923202d su dev, merge su main in fast-forward (main era antenato diretto, nessun conflitto possibile), entrambi pushati. Vercel ridistribuito sul push; Railway non toccato, il backend non e' cambiato e non c'e' migration, quindi deploy di solo frontend senza backup ne' finestra di manutenzione. Tag v1.0.4 annotato creato da Visual Studio sulla punta di main e pubblicato: verificato con git ls-remote che punti a 923202d, lo stesso commit di main remoto. 35 file nel commit (24 modificati + 11 nuovi), contati prima di confermare per non ripetere l'incidente del 04/09.</t>
+  </si>
+  <si>
+    <t>Git + Vercel</t>
+  </si>
+  <si>
+    <t>Pulizia: cartelle vuote e codice morto (REV-055, REV-077), costruttore fantasma di PrenotazioniService (REV-010), nome di 'fascia oraria' scritto in quattro modi (REV-056), duplicazioni e costanti ripetute (REV-058/059/060/061), implementazioni che lanciano solo NotImplementedException (REV-030), refusi e nomi troncati (REV-067, REV-068), path degli endpoint centralizzati (REV-082), formattazione automatica (REV-078), piu' i DateTime.Now scritti a mano nei messaggi di log che mostrano un orario diverso da quello di Serilog per lo stesso evento. Nessun task per Fabio.</t>
+  </si>
+  <si>
+    <t>v1.0.4</t>
+  </si>
+  <si>
+    <t>Merge dev -&gt; main della Fase 8 con tag v1.0.4</t>
+  </si>
+  <si>
+    <t>Fast-forward, commit 923202d, tag annotato v1.0.4 pubblicato da Visual Studio e verificato sul remoto. Deploy di solo frontend: Vercel ridistribuito sul push, Railway non toccato (backend invariato, nessuna migration). Deploy riuscito. Restano non eseguite quattro prove manuali non bloccanti (paginazione, notifica singola, doppio clic, password nel form): la logica e' coperta dai 26 test automatici.</t>
+  </si>
+  <si>
+    <t>Railway - PostgreSQL + .NET, health check /health. In produzione: backend v1.0.3 (Fase 7), frontend Vercel v1.0.4 (Fase 8, 07/09/2026)</t>
+  </si>
+  <si>
+    <t>FASE 9 ROADMAP REVISIONE - Pulizia (sessione 07/09/2026)</t>
+  </si>
+  <si>
+    <t>REV-055 / REV-010 - codice morto</t>
+  </si>
+  <si>
+    <t>Cartelle vuote Services/FasciaOraria e Repositories/FasciaOraria, residuo del rename al plurale della Fase 7. In PrenotazioniService rimossi i campi object1..object7 e il secondo costruttore fantasma (8 parametri mai assegnati): se il DI lo avesse scelto, il service sarebbe partito con tutte le dipendenze null.</t>
+  </si>
+  <si>
+    <t>REV-030 - throw solo per soddisfare un'interfaccia</t>
+  </si>
+  <si>
+    <t>IFasciaOrariaService e IPostazioneService non ereditano piu' IService&lt;T&gt;: il generico imponeva una firma diversa da quella reale (GetByIdAsync restituiva l'entita', non il DTO), e i due service avevano una seconda implementazione esplicita che si limitava a un throw NotImplementedException. GetAllQueryableAsync spostato da IRepository&lt;T&gt; a IPrenotazioniRepository, l'unico a usarlo davvero: ZonaRepository non porta piu' l'implementazione fittizia.</t>
+  </si>
+  <si>
+    <t>C# - interfacce</t>
+  </si>
+  <si>
+    <t>REV-067 / REV-068 - refusi</t>
+  </si>
+  <si>
+    <t>File di test rinominato FasciaOrariaServiceTe.cs -&gt; FasciaOrariaServiceTests.cs (la classe al suo interno era gia' corretta). Email di contatto in Swagger corretta (outloo.com -&gt; outlook.com).</t>
+  </si>
+  <si>
+    <t>REV-059 - id utente e IP duplicati</t>
+  </si>
+  <si>
+    <t>GetAuthenticatedUserId()/GetIpAddress() erano copiati identici in 4 service (FasciaOrariaService, PostazioneService, ZonaService, PrenotazioniService) e 2 controller (AuthenticationUserController, SetupController). Centralizzati in Extensions/HttpContextExtensions.cs, sopra i due helper che facevano gia' il lavoro vero (ClaimsPrincipalExtensions, Common/IndirizzoClient).</t>
+  </si>
+  <si>
+    <t>ASP.NET Core - extension methods</t>
+  </si>
+  <si>
+    <t>REV-060 - proiezione FasciaOraria duplicata</t>
+  </si>
+  <si>
+    <t>La stessa proiezione FasciaOraria -&gt; FasciaOrariaDTO era scritta identica in 4 metodi di FasciaOrariaService. Estratta in un unico MapToDto privato.</t>
+  </si>
+  <si>
+    <t>C#</t>
+  </si>
+  <si>
+    <t>REV-061 - costanti ripetute</t>
+  </si>
+  <si>
+    <t>CacheDuration (30 minuti) era la stessa costante ripetuta in 3 service: spostata in CacheKeys.Durata. CapienzaConsentita {2,4,8} in PostazioneService non era piu' referenziata da nessuno (il vincolo era gia' stato tolto dai validator nel checkpoint 2b) ed e' stata rimossa. La retention di 6 mesi delle prenotazioni completate, scritta come -6 in mezzo al metodo di pulizia, e' ora la costante nominata MesiRetentionCompletate.</t>
+  </si>
+  <si>
+    <t>Residuo REV-092 - doppio timestamp nei log</t>
+  </si>
+  <si>
+    <t>31 DateTime.Now/DateTime.UtcNow scritti a mano nei messaggi di log di 5 controller duplicavano il timestamp che Serilog scrive gia' per ogni riga (lo stesso difetto gia' documentato sui log di dominio: due orari diversi per lo stesso evento). Rimossi i parametri e i placeholder {Data}/{Timestamp} corrispondenti. Lasciati intatti i {Data} legittimi in DashboardController: li' e' la data richiesta in query, un parametro di dominio, non un timestamp.</t>
+  </si>
+  <si>
+    <t>REV-077 - codice morto nel frontend</t>
+  </si>
+  <si>
+    <t>App.tsx, App.css e src/assets/* (hero.png, react.svg, vite.svg) erano residui dello scaffold iniziale, senza alcun riferimento nel codice ne' nel favicon (che usa public/favicon.svg). L'hook useUpdateStatoZona esisteva ma nessuna pagina lo chiamava.</t>
+  </si>
+  <si>
+    <t>React + Vite</t>
+  </si>
+  <si>
+    <t>REV-082 - path degli endpoint sparsi</t>
+  </si>
+  <si>
+    <t>24 chiamate ad apiClient in 8 hook piu' LoginPage e RegisterPage scrivevano il path dell'endpoint inline, spesso ripetuto identico fra query e mutation dello stesso modulo. Creato lib/endpoints.ts, un unico oggetto Endpoints raggruppato per area (auth, setup, dashboard, zona, fasciaOraria, postazione, prenotazione) con lo stesso raggruppamento del backend.</t>
+  </si>
+  <si>
+    <t>GIORNI_SETTIMANA duplicata</t>
+  </si>
+  <si>
+    <t>L'elenco dei giorni della settimana era scritto identico in FasciaOrariaModal e FasciaOrariaPage. Estratto in lib/giorni.ts.</t>
+  </si>
+  <si>
+    <t>REV-078 - formattazione mai applicata</t>
+  </si>
+  <si>
+    <t>Prettier era configurato dalla Fase 8 ma non era mai stato eseguito su tutto il progetto: 3 pagine usavano indentazione a 4 spazi contro il tabWidth 2 configurato. Il file .prettierrc stesso aveva un'indentazione fuori posto. Eseguito 'prettier --write' su tutto src/: nessuna riga di logica toccata, solo spaziatura, virgolette e a-capo.</t>
+  </si>
+  <si>
+    <t>Prettier</t>
+  </si>
+  <si>
+    <t>npm audit - 18 vulnerabilita'</t>
+  </si>
+  <si>
+    <t>npm audit' segnalava 18 vulnerabilita' lasciate in sospeso dalla Fase 8 (3 basse, 3 medie, 12 alte), fra cui axios, react-router-dom e vite come dipendenze dirette. 'npm audit fix' senza --force le ha risolte tutte restando dentro i range semver gia' dichiarati in package.json (nessun major bump, package.json invariato, solo package-lock.json aggiornato). 0 vulnerabilita' residue.</t>
+  </si>
+  <si>
+    <t>npm audit</t>
+  </si>
+  <si>
+    <t>Backend: dotnet build 0 errori (27 warning preesistenti, invariati), dotnet test 237/237 (invariato). Frontend: tsc -b --force 0 errori, npm test 26/26 (invariato), npm run build pulita, eslint 0 errori (il solo warning preesistente su watch() di react-hook-form). Nessuna migration.</t>
+  </si>
+  <si>
+    <t>dotnet test + Vitest + tsc + eslint</t>
+  </si>
+  <si>
+    <t>REV-056 rimandato di proposito</t>
+  </si>
+  <si>
+    <t>Allineare del tutto il naming di 'fascia oraria' avrebbe richiesto di rinominare FasceOrarieController e la sua route (/api/FasceOrarie): un cambio di contratto che avrebbe rotto tutti gli hook del frontend gia' aggiornati in questa stessa fase, per un guadagno di sola leggibilita'. Deciso con Fabio di sistemare solo cartelle e namespace (gia' fatto con REV-055) e lasciare la route com'e'.</t>
+  </si>
+  <si>
+    <t>Decisione di prodotto</t>
+  </si>
+  <si>
+    <t>Prossimo passo - Fase 10</t>
+  </si>
+  <si>
+    <t>Esperienza d'uso: layout adattivo da telefono (REV-071), messaggi per le liste vuote (REV-073), messaggio vero sugli errori di caricamento invece di 'Errore nel caricamento' uguale per tutti i casi (NEW-006), caricamento parziale al posto del 'Caricamento...' a schermo intero (REV-074), stile uniforme dei pulsanti (REV-075), accessibilita' di base (REV-072), nome/ruolo utente e pagina attiva nel menu (REV-081), link di ritorno da /unauthorized (REV-080), titolo/lingua/icona del sito (REV-079). Pannello disponibilita' nel form di creazione (NEW-002) da confermare, e' opzionale.</t>
+  </si>
+  <si>
+    <t>Pulizia del codice (Fase 9)</t>
+  </si>
+  <si>
+    <t>Cartelle vuote e costruttore fantasma rimossi (REV-055, REV-010), interfacce che imponevano un throw NotImplementedException solo per compatibilita' (REV-030), id utente/IP e proiezione FasciaOraria-&gt;DTO centralizzati (REV-059, REV-060), costanti duplicate accorpate (REV-061), refusi corretti (REV-067, REV-068), doppio timestamp nei log dei controller rimosso (residuo REV-092), codice morto e path degli endpoint sparsi nel frontend (REV-077, REV-082), formattazione uniforme (REV-078), 18 vulnerabilita' npm risolte.</t>
+  </si>
+  <si>
+    <t>C# + TypeScript + Prettier + npm audit</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 9</t>
+  </si>
+  <si>
+    <t>Pulizia: codice morto, duplicazioni, refusi, costanti ripetute, path degli endpoint centralizzati, formattazione uniforme, vulnerabilita' npm (REV-010, REV-030, REV-055, REV-059, REV-060, REV-061, REV-067, REV-068, REV-077, REV-078, REV-082). Nessuna migration, nessun task per Fabio.</t>
+  </si>
+  <si>
+    <t>Pulizia (REV-010, REV-030, REV-055, REV-059, REV-060, REV-061, REV-067, REV-068, REV-077, REV-078, REV-082)</t>
+  </si>
+  <si>
+    <t>Cartelle vuote e costruttore fantasma di PrenotazioniService rimossi; le interfacce di FasciaOrariaService e PostazioneService non impongono piu' un throw solo per compatibilita' con IService&lt;T&gt;; GetAuthenticatedUserId/GetIpAddress centralizzati in Extensions/HttpContextExtensions (prima duplicati in 4 service e 2 controller); proiezione FasciaOraria-&gt;DTO unificata; CacheDuration/CapienzaConsentita/retention accorpate in costanti nominate; file di test rinominato e refuso email Swagger corretto; rimossi i timestamp scritti a mano nei log dei controller, doppioni di quelli di Serilog. Lato frontend: rimosso codice morto (App.tsx, assets, hook inutilizzato), creato lib/endpoints.ts per i path prima sparsi in 8 hook, GIORNI_SETTIMANA centralizzato, Prettier applicato a tutto il progetto, 18 vulnerabilita' npm risolte con npm audit fix senza --force. dotnet test 237/237 invariato, npm test 26/26 invariato, build e typecheck puliti su entrambi. Nessuna migration.</t>
   </si>
 </sst>
 </file>
@@ -4789,7 +4942,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4935,6 +5088,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -5260,7 +5414,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="47" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="B2" s="48"/>
       <c r="C2" s="48"/>
@@ -5415,13 +5569,13 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="6" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5429,13 +5583,13 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>6</v>
@@ -5455,7 +5609,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>1278</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -6344,7 +6498,7 @@
         <v>731</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>1467</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6384,7 +6538,7 @@
         <v>437</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>1468</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6424,7 +6578,7 @@
         <v>739</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
@@ -6444,7 +6598,7 @@
         <v>669</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -6589,33 +6743,33 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="B56" t="s">
         <v>665</v>
       </c>
       <c r="C56" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="D56" t="s">
         <v>660</v>
       </c>
       <c r="E56" t="s">
+        <v>1400</v>
+      </c>
+      <c r="F56" t="s">
         <v>1401</v>
-      </c>
-      <c r="F56" t="s">
-        <v>1402</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="B57" t="s">
         <v>665</v>
       </c>
       <c r="C57" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="D57" t="s">
         <v>660</v>
@@ -6624,7 +6778,7 @@
         <v>437</v>
       </c>
       <c r="F57" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
     </row>
   </sheetData>
@@ -6649,7 +6803,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="57" t="s">
-        <v>1469</v>
+        <v>1467</v>
       </c>
       <c r="B1" s="48"/>
       <c r="C1" s="48"/>
@@ -7389,16 +7543,16 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1469</v>
+      </c>
+      <c r="C47" t="s">
         <v>1470</v>
       </c>
-      <c r="B47" t="s">
+      <c r="D47" t="s">
         <v>1471</v>
-      </c>
-      <c r="C47" t="s">
-        <v>1472</v>
-      </c>
-      <c r="D47" t="s">
-        <v>1473</v>
       </c>
       <c r="E47" s="27" t="s">
         <v>6</v>
@@ -7406,16 +7560,16 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C48" t="s">
         <v>1474</v>
       </c>
-      <c r="B48" t="s">
+      <c r="D48" t="s">
         <v>1475</v>
-      </c>
-      <c r="C48" t="s">
-        <v>1476</v>
-      </c>
-      <c r="D48" t="s">
-        <v>1477</v>
       </c>
       <c r="E48" s="27" t="s">
         <v>6</v>
@@ -7423,16 +7577,16 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>1476</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C49" t="s">
         <v>1478</v>
       </c>
-      <c r="B49" t="s">
+      <c r="D49" t="s">
         <v>1479</v>
-      </c>
-      <c r="C49" t="s">
-        <v>1480</v>
-      </c>
-      <c r="D49" t="s">
-        <v>1481</v>
       </c>
       <c r="E49" s="27" t="s">
         <v>6</v>
@@ -7440,16 +7594,16 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1481</v>
+      </c>
+      <c r="C50" t="s">
         <v>1482</v>
       </c>
-      <c r="B50" t="s">
+      <c r="D50" t="s">
         <v>1483</v>
-      </c>
-      <c r="C50" t="s">
-        <v>1484</v>
-      </c>
-      <c r="D50" t="s">
-        <v>1485</v>
       </c>
       <c r="E50" s="27" t="s">
         <v>6</v>
@@ -7832,7 +7986,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H252"/>
+  <dimension ref="A1:H271"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7857,7 +8011,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="47" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="B2" s="48"/>
       <c r="C2" s="48"/>
@@ -10738,7 +10892,7 @@
         <v>1254</v>
       </c>
       <c r="C190" s="27" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="D190" s="27" t="s">
         <v>1255</v>
@@ -10752,7 +10906,7 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
@@ -10780,10 +10934,10 @@
         <v>1</v>
       </c>
       <c r="B193" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C193" t="s">
         <v>1281</v>
-      </c>
-      <c r="C193" t="s">
-        <v>1282</v>
       </c>
       <c r="D193" t="s">
         <v>1152</v>
@@ -10800,10 +10954,10 @@
         <v>2</v>
       </c>
       <c r="B194" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C194" t="s">
         <v>1283</v>
-      </c>
-      <c r="C194" t="s">
-        <v>1284</v>
       </c>
       <c r="D194" t="s">
         <v>74</v>
@@ -10820,13 +10974,13 @@
         <v>3</v>
       </c>
       <c r="B195" t="s">
+        <v>1284</v>
+      </c>
+      <c r="C195" t="s">
         <v>1285</v>
       </c>
-      <c r="C195" t="s">
+      <c r="D195" t="s">
         <v>1286</v>
-      </c>
-      <c r="D195" t="s">
-        <v>1287</v>
       </c>
       <c r="E195" s="45">
         <v>46090</v>
@@ -10840,10 +10994,10 @@
         <v>4</v>
       </c>
       <c r="B196" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C196" t="s">
         <v>1288</v>
-      </c>
-      <c r="C196" t="s">
-        <v>1289</v>
       </c>
       <c r="D196" t="s">
         <v>74</v>
@@ -10860,10 +11014,10 @@
         <v>5</v>
       </c>
       <c r="B197" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="C197" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="D197" t="s">
         <v>1251</v>
@@ -10880,24 +11034,24 @@
         <v>6</v>
       </c>
       <c r="B198" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C198" t="s">
         <v>1291</v>
       </c>
-      <c r="C198" t="s">
+      <c r="D198" t="s">
         <v>1292</v>
-      </c>
-      <c r="D198" t="s">
-        <v>1293</v>
       </c>
       <c r="E198" t="s">
         <v>437</v>
       </c>
       <c r="F198" s="38" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
@@ -10925,13 +11079,13 @@
         <v>1</v>
       </c>
       <c r="B202" t="s">
+        <v>1298</v>
+      </c>
+      <c r="C202" t="s">
         <v>1299</v>
       </c>
-      <c r="C202" t="s">
+      <c r="D202" t="s">
         <v>1300</v>
-      </c>
-      <c r="D202" t="s">
-        <v>1301</v>
       </c>
       <c r="E202" s="45">
         <v>46121</v>
@@ -10945,13 +11099,13 @@
         <v>2</v>
       </c>
       <c r="B203" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C203" t="s">
         <v>1302</v>
       </c>
-      <c r="C203" t="s">
+      <c r="D203" t="s">
         <v>1303</v>
-      </c>
-      <c r="D203" t="s">
-        <v>1304</v>
       </c>
       <c r="E203" s="45">
         <v>46121</v>
@@ -10965,13 +11119,13 @@
         <v>3</v>
       </c>
       <c r="B204" t="s">
+        <v>1304</v>
+      </c>
+      <c r="C204" t="s">
         <v>1305</v>
       </c>
-      <c r="C204" t="s">
+      <c r="D204" t="s">
         <v>1306</v>
-      </c>
-      <c r="D204" t="s">
-        <v>1307</v>
       </c>
       <c r="E204" s="45">
         <v>46121</v>
@@ -10985,13 +11139,13 @@
         <v>4</v>
       </c>
       <c r="B205" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C205" t="s">
         <v>1308</v>
       </c>
-      <c r="C205" t="s">
+      <c r="D205" t="s">
         <v>1309</v>
-      </c>
-      <c r="D205" t="s">
-        <v>1310</v>
       </c>
       <c r="E205" s="45">
         <v>46121</v>
@@ -11005,13 +11159,13 @@
         <v>5</v>
       </c>
       <c r="B206" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C206" t="s">
         <v>1311</v>
       </c>
-      <c r="C206" t="s">
+      <c r="D206" t="s">
         <v>1312</v>
-      </c>
-      <c r="D206" t="s">
-        <v>1313</v>
       </c>
       <c r="E206" s="45">
         <v>46121</v>
@@ -11025,13 +11179,13 @@
         <v>6</v>
       </c>
       <c r="B207" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C207" t="s">
         <v>1314</v>
       </c>
-      <c r="C207" t="s">
+      <c r="D207" t="s">
         <v>1315</v>
-      </c>
-      <c r="D207" t="s">
-        <v>1316</v>
       </c>
       <c r="E207" s="45">
         <v>46121</v>
@@ -11045,13 +11199,13 @@
         <v>7</v>
       </c>
       <c r="B208" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C208" t="s">
         <v>1325</v>
       </c>
-      <c r="C208" t="s">
+      <c r="D208" t="s">
         <v>1326</v>
-      </c>
-      <c r="D208" t="s">
-        <v>1327</v>
       </c>
       <c r="E208" s="45">
         <v>46121</v>
@@ -11065,13 +11219,13 @@
         <v>8</v>
       </c>
       <c r="B209" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C209" t="s">
         <v>1332</v>
       </c>
-      <c r="C209" t="s">
-        <v>1333</v>
-      </c>
       <c r="D209" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="E209" s="45">
         <v>46121</v>
@@ -11085,13 +11239,13 @@
         <v>8</v>
       </c>
       <c r="B210" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C210" t="s">
         <v>1334</v>
       </c>
-      <c r="C210" t="s">
+      <c r="D210" t="s">
         <v>1335</v>
-      </c>
-      <c r="D210" t="s">
-        <v>1336</v>
       </c>
       <c r="E210" s="45">
         <v>46121</v>
@@ -11105,13 +11259,13 @@
         <v>9</v>
       </c>
       <c r="B211" t="s">
+        <v>1336</v>
+      </c>
+      <c r="C211" t="s">
         <v>1337</v>
       </c>
-      <c r="C211" t="s">
+      <c r="D211" t="s">
         <v>1338</v>
-      </c>
-      <c r="D211" t="s">
-        <v>1339</v>
       </c>
       <c r="E211" s="45">
         <v>46121</v>
@@ -11125,13 +11279,13 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C212" t="s">
         <v>1340</v>
       </c>
-      <c r="C212" t="s">
+      <c r="D212" t="s">
         <v>1341</v>
-      </c>
-      <c r="D212" t="s">
-        <v>1342</v>
       </c>
       <c r="E212" s="45">
         <v>46121</v>
@@ -11145,13 +11299,13 @@
         <v>11</v>
       </c>
       <c r="B213" t="s">
+        <v>1342</v>
+      </c>
+      <c r="C213" t="s">
         <v>1343</v>
       </c>
-      <c r="C213" t="s">
+      <c r="D213" t="s">
         <v>1344</v>
-      </c>
-      <c r="D213" t="s">
-        <v>1345</v>
       </c>
       <c r="E213" s="45">
         <v>46121</v>
@@ -11165,13 +11319,13 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
+        <v>1345</v>
+      </c>
+      <c r="C214" t="s">
         <v>1346</v>
       </c>
-      <c r="C214" t="s">
+      <c r="D214" t="s">
         <v>1347</v>
-      </c>
-      <c r="D214" t="s">
-        <v>1348</v>
       </c>
       <c r="E214" s="45">
         <v>46121</v>
@@ -11185,10 +11339,10 @@
         <v>13</v>
       </c>
       <c r="B215" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="C215" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="D215" t="s">
         <v>437</v>
@@ -11205,10 +11359,10 @@
         <v>14</v>
       </c>
       <c r="B216" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="C216" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="D216" t="s">
         <v>1273</v>
@@ -11222,7 +11376,7 @@
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
@@ -11250,13 +11404,13 @@
         <v>1</v>
       </c>
       <c r="B220" t="s">
+        <v>1358</v>
+      </c>
+      <c r="C220" t="s">
         <v>1359</v>
       </c>
-      <c r="C220" t="s">
+      <c r="D220" t="s">
         <v>1360</v>
-      </c>
-      <c r="D220" t="s">
-        <v>1361</v>
       </c>
       <c r="E220" s="45">
         <v>46121</v>
@@ -11270,10 +11424,10 @@
         <v>2</v>
       </c>
       <c r="B221" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C221" t="s">
         <v>1362</v>
-      </c>
-      <c r="C221" t="s">
-        <v>1363</v>
       </c>
       <c r="D221" t="s">
         <v>287</v>
@@ -11290,10 +11444,10 @@
         <v>3</v>
       </c>
       <c r="B222" t="s">
+        <v>1363</v>
+      </c>
+      <c r="C222" t="s">
         <v>1364</v>
-      </c>
-      <c r="C222" t="s">
-        <v>1365</v>
       </c>
       <c r="D222" t="s">
         <v>29</v>
@@ -11310,13 +11464,13 @@
         <v>4</v>
       </c>
       <c r="B223" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C223" t="s">
         <v>1366</v>
       </c>
-      <c r="C223" t="s">
+      <c r="D223" t="s">
         <v>1367</v>
-      </c>
-      <c r="D223" t="s">
-        <v>1368</v>
       </c>
       <c r="E223" s="45">
         <v>46121</v>
@@ -11330,13 +11484,13 @@
         <v>5</v>
       </c>
       <c r="B224" t="s">
+        <v>1368</v>
+      </c>
+      <c r="C224" t="s">
         <v>1369</v>
       </c>
-      <c r="C224" t="s">
-        <v>1370</v>
-      </c>
       <c r="D224" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="E224" s="45">
         <v>46121</v>
@@ -11350,13 +11504,13 @@
         <v>6</v>
       </c>
       <c r="B225" t="s">
+        <v>1370</v>
+      </c>
+      <c r="C225" t="s">
         <v>1371</v>
       </c>
-      <c r="C225" t="s">
+      <c r="D225" t="s">
         <v>1372</v>
-      </c>
-      <c r="D225" t="s">
-        <v>1373</v>
       </c>
       <c r="E225" s="45">
         <v>46121</v>
@@ -11370,10 +11524,10 @@
         <v>7</v>
       </c>
       <c r="B226" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C226" t="s">
         <v>1374</v>
-      </c>
-      <c r="C226" t="s">
-        <v>1375</v>
       </c>
       <c r="D226" t="s">
         <v>267</v>
@@ -11390,13 +11544,13 @@
         <v>8</v>
       </c>
       <c r="B227" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C227" t="s">
         <v>1376</v>
       </c>
-      <c r="C227" t="s">
+      <c r="D227" t="s">
         <v>1377</v>
-      </c>
-      <c r="D227" t="s">
-        <v>1378</v>
       </c>
       <c r="E227" s="45">
         <v>46121</v>
@@ -11410,13 +11564,13 @@
         <v>9</v>
       </c>
       <c r="B228" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C228" t="s">
         <v>1379</v>
       </c>
-      <c r="C228" t="s">
+      <c r="D228" t="s">
         <v>1380</v>
-      </c>
-      <c r="D228" t="s">
-        <v>1381</v>
       </c>
       <c r="E228" s="45">
         <v>46121</v>
@@ -11430,13 +11584,13 @@
         <v>10</v>
       </c>
       <c r="B229" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C229" t="s">
         <v>1382</v>
       </c>
-      <c r="C229" t="s">
+      <c r="D229" t="s">
         <v>1383</v>
-      </c>
-      <c r="D229" t="s">
-        <v>1384</v>
       </c>
       <c r="E229" s="45">
         <v>46121</v>
@@ -11450,13 +11604,13 @@
         <v>11</v>
       </c>
       <c r="B230" t="s">
+        <v>1384</v>
+      </c>
+      <c r="C230" t="s">
         <v>1385</v>
       </c>
-      <c r="C230" t="s">
+      <c r="D230" t="s">
         <v>1386</v>
-      </c>
-      <c r="D230" t="s">
-        <v>1387</v>
       </c>
       <c r="E230" s="45">
         <v>46121</v>
@@ -11470,10 +11624,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C231" t="s">
         <v>1388</v>
-      </c>
-      <c r="C231" t="s">
-        <v>1389</v>
       </c>
       <c r="D231" t="s">
         <v>32</v>
@@ -11490,10 +11644,10 @@
         <v>13</v>
       </c>
       <c r="B232" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
       <c r="C232" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="D232" t="s">
         <v>437</v>
@@ -11510,13 +11664,13 @@
         <v>14</v>
       </c>
       <c r="B233" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C233" t="s">
         <v>1405</v>
       </c>
-      <c r="C233" t="s">
+      <c r="D233" t="s">
         <v>1406</v>
-      </c>
-      <c r="D233" t="s">
-        <v>1407</v>
       </c>
       <c r="E233" s="45">
         <v>46212</v>
@@ -11527,7 +11681,7 @@
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="236" spans="1:6" x14ac:dyDescent="0.3">
@@ -11555,13 +11709,13 @@
         <v>1</v>
       </c>
       <c r="B237" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C237" t="s">
         <v>1417</v>
       </c>
-      <c r="C237" t="s">
+      <c r="D237" t="s">
         <v>1418</v>
-      </c>
-      <c r="D237" t="s">
-        <v>1419</v>
       </c>
       <c r="E237" s="45">
         <v>46212</v>
@@ -11575,13 +11729,13 @@
         <v>2</v>
       </c>
       <c r="B238" t="s">
+        <v>1419</v>
+      </c>
+      <c r="C238" t="s">
         <v>1420</v>
       </c>
-      <c r="C238" t="s">
+      <c r="D238" t="s">
         <v>1421</v>
-      </c>
-      <c r="D238" t="s">
-        <v>1422</v>
       </c>
       <c r="E238" s="45">
         <v>46212</v>
@@ -11595,13 +11749,13 @@
         <v>3</v>
       </c>
       <c r="B239" t="s">
+        <v>1422</v>
+      </c>
+      <c r="C239" t="s">
         <v>1423</v>
       </c>
-      <c r="C239" t="s">
+      <c r="D239" t="s">
         <v>1424</v>
-      </c>
-      <c r="D239" t="s">
-        <v>1425</v>
       </c>
       <c r="E239" s="45">
         <v>46212</v>
@@ -11615,13 +11769,13 @@
         <v>4</v>
       </c>
       <c r="B240" t="s">
+        <v>1425</v>
+      </c>
+      <c r="C240" t="s">
         <v>1426</v>
       </c>
-      <c r="C240" t="s">
+      <c r="D240" t="s">
         <v>1427</v>
-      </c>
-      <c r="D240" t="s">
-        <v>1428</v>
       </c>
       <c r="E240" s="45">
         <v>46212</v>
@@ -11635,13 +11789,13 @@
         <v>5</v>
       </c>
       <c r="B241" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C241" t="s">
         <v>1429</v>
       </c>
-      <c r="C241" t="s">
+      <c r="D241" t="s">
         <v>1430</v>
-      </c>
-      <c r="D241" t="s">
-        <v>1431</v>
       </c>
       <c r="E241" s="45">
         <v>46212</v>
@@ -11655,13 +11809,13 @@
         <v>6</v>
       </c>
       <c r="B242" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C242" t="s">
         <v>1432</v>
       </c>
-      <c r="C242" t="s">
+      <c r="D242" t="s">
         <v>1433</v>
-      </c>
-      <c r="D242" t="s">
-        <v>1434</v>
       </c>
       <c r="E242" s="45">
         <v>46212</v>
@@ -11675,13 +11829,13 @@
         <v>7</v>
       </c>
       <c r="B243" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C243" t="s">
         <v>1435</v>
       </c>
-      <c r="C243" t="s">
+      <c r="D243" t="s">
         <v>1436</v>
-      </c>
-      <c r="D243" t="s">
-        <v>1437</v>
       </c>
       <c r="E243" s="45">
         <v>46212</v>
@@ -11695,13 +11849,13 @@
         <v>8</v>
       </c>
       <c r="B244" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C244" t="s">
         <v>1438</v>
       </c>
-      <c r="C244" t="s">
+      <c r="D244" t="s">
         <v>1439</v>
-      </c>
-      <c r="D244" t="s">
-        <v>1440</v>
       </c>
       <c r="E244" s="45">
         <v>46212</v>
@@ -11715,13 +11869,13 @@
         <v>9</v>
       </c>
       <c r="B245" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C245" t="s">
         <v>1441</v>
       </c>
-      <c r="C245" t="s">
+      <c r="D245" t="s">
         <v>1442</v>
-      </c>
-      <c r="D245" t="s">
-        <v>1443</v>
       </c>
       <c r="E245" s="45">
         <v>46212</v>
@@ -11735,13 +11889,13 @@
         <v>10</v>
       </c>
       <c r="B246" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C246" t="s">
         <v>1444</v>
       </c>
-      <c r="C246" t="s">
+      <c r="D246" t="s">
         <v>1445</v>
-      </c>
-      <c r="D246" t="s">
-        <v>1446</v>
       </c>
       <c r="E246" s="45">
         <v>46212</v>
@@ -11755,10 +11909,10 @@
         <v>11</v>
       </c>
       <c r="B247" t="s">
+        <v>1446</v>
+      </c>
+      <c r="C247" t="s">
         <v>1447</v>
-      </c>
-      <c r="C247" t="s">
-        <v>1448</v>
       </c>
       <c r="D247" t="s">
         <v>437</v>
@@ -11775,13 +11929,13 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C248" t="s">
         <v>1449</v>
       </c>
-      <c r="C248" t="s">
+      <c r="D248" t="s">
         <v>1450</v>
-      </c>
-      <c r="D248" t="s">
-        <v>1451</v>
       </c>
       <c r="E248" s="45">
         <v>46212</v>
@@ -11795,13 +11949,13 @@
         <v>13</v>
       </c>
       <c r="B249" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C249" t="s">
         <v>1452</v>
       </c>
-      <c r="C249" t="s">
+      <c r="D249" t="s">
         <v>1453</v>
-      </c>
-      <c r="D249" t="s">
-        <v>1454</v>
       </c>
       <c r="E249" s="45">
         <v>46212</v>
@@ -11815,13 +11969,13 @@
         <v>14</v>
       </c>
       <c r="B250" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C250" t="s">
+        <v>1488</v>
+      </c>
+      <c r="D250" t="s">
         <v>1489</v>
-      </c>
-      <c r="C250" t="s">
-        <v>1490</v>
-      </c>
-      <c r="D250" t="s">
-        <v>1491</v>
       </c>
       <c r="E250" s="45">
         <v>46212</v>
@@ -11835,13 +11989,13 @@
         <v>15</v>
       </c>
       <c r="B251" t="s">
-        <v>1492</v>
+        <v>1490</v>
       </c>
       <c r="C251" t="s">
-        <v>1493</v>
+        <v>1491</v>
       </c>
       <c r="D251" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="E251" s="45">
         <v>46212</v>
@@ -11855,20 +12009,361 @@
         <v>16</v>
       </c>
       <c r="B252" t="s">
-        <v>1455</v>
+        <v>1493</v>
       </c>
       <c r="C252" t="s">
-        <v>1456</v>
+        <v>1494</v>
       </c>
       <c r="D252" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E252" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F252" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A253">
+        <v>17</v>
+      </c>
+      <c r="B253" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C253" t="s">
+        <v>1496</v>
+      </c>
+      <c r="D253" t="s">
         <v>437</v>
       </c>
-      <c r="E252" t="s">
+      <c r="E253" t="s">
         <v>437</v>
       </c>
-      <c r="F252" s="46" t="s">
+      <c r="F253" s="46" t="s">
         <v>977</v>
       </c>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A255" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A256" t="s">
+        <v>39</v>
+      </c>
+      <c r="B256" t="s">
+        <v>40</v>
+      </c>
+      <c r="C256" t="s">
+        <v>856</v>
+      </c>
+      <c r="D256" t="s">
+        <v>42</v>
+      </c>
+      <c r="E256" t="s">
+        <v>43</v>
+      </c>
+      <c r="F256" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A257">
+        <v>1</v>
+      </c>
+      <c r="B257" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C257" t="s">
+        <v>1503</v>
+      </c>
+      <c r="D257" t="s">
+        <v>3</v>
+      </c>
+      <c r="E257" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F257" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A258">
+        <v>2</v>
+      </c>
+      <c r="B258" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C258" t="s">
+        <v>1505</v>
+      </c>
+      <c r="D258" t="s">
+        <v>1506</v>
+      </c>
+      <c r="E258" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F258" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A259">
+        <v>3</v>
+      </c>
+      <c r="B259" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C259" t="s">
+        <v>1508</v>
+      </c>
+      <c r="D259" t="s">
+        <v>437</v>
+      </c>
+      <c r="E259" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F259" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A260">
+        <v>4</v>
+      </c>
+      <c r="B260" t="s">
+        <v>1509</v>
+      </c>
+      <c r="C260" t="s">
+        <v>1510</v>
+      </c>
+      <c r="D260" t="s">
+        <v>1511</v>
+      </c>
+      <c r="E260" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F260" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A261">
+        <v>5</v>
+      </c>
+      <c r="B261" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C261" t="s">
+        <v>1513</v>
+      </c>
+      <c r="D261" t="s">
+        <v>1514</v>
+      </c>
+      <c r="E261" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F261" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="262" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A262">
+        <v>6</v>
+      </c>
+      <c r="B262" t="s">
+        <v>1515</v>
+      </c>
+      <c r="C262" t="s">
+        <v>1516</v>
+      </c>
+      <c r="D262" t="s">
+        <v>1514</v>
+      </c>
+      <c r="E262" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F262" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A263">
+        <v>7</v>
+      </c>
+      <c r="B263" t="s">
+        <v>1517</v>
+      </c>
+      <c r="C263" t="s">
+        <v>1518</v>
+      </c>
+      <c r="D263" t="s">
+        <v>22</v>
+      </c>
+      <c r="E263" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F263" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A264">
+        <v>8</v>
+      </c>
+      <c r="B264" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C264" t="s">
+        <v>1520</v>
+      </c>
+      <c r="D264" t="s">
+        <v>1521</v>
+      </c>
+      <c r="E264" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F264" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A265">
+        <v>9</v>
+      </c>
+      <c r="B265" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C265" t="s">
+        <v>1523</v>
+      </c>
+      <c r="D265" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E265" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F265" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A266">
+        <v>10</v>
+      </c>
+      <c r="B266" t="s">
+        <v>1524</v>
+      </c>
+      <c r="C266" t="s">
+        <v>1525</v>
+      </c>
+      <c r="D266" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E266" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F266" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A267">
+        <v>11</v>
+      </c>
+      <c r="B267" t="s">
+        <v>1526</v>
+      </c>
+      <c r="C267" t="s">
+        <v>1527</v>
+      </c>
+      <c r="D267" t="s">
+        <v>1528</v>
+      </c>
+      <c r="E267" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F267" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A268">
+        <v>12</v>
+      </c>
+      <c r="B268" t="s">
+        <v>1529</v>
+      </c>
+      <c r="C268" s="59" t="s">
+        <v>1530</v>
+      </c>
+      <c r="D268" t="s">
+        <v>1531</v>
+      </c>
+      <c r="E268" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F268" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A269">
+        <v>13</v>
+      </c>
+      <c r="B269" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C269" t="s">
+        <v>1532</v>
+      </c>
+      <c r="D269" t="s">
+        <v>1533</v>
+      </c>
+      <c r="E269" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F269" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A270">
+        <v>14</v>
+      </c>
+      <c r="B270" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C270" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D270" t="s">
+        <v>1536</v>
+      </c>
+      <c r="E270" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F270" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="271" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A271">
+        <v>15</v>
+      </c>
+      <c r="B271" t="s">
+        <v>1537</v>
+      </c>
+      <c r="C271" t="s">
+        <v>1538</v>
+      </c>
+      <c r="D271" t="s">
+        <v>437</v>
+      </c>
+      <c r="E271" s="45"/>
+      <c r="F271" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -11886,7 +12381,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -12311,7 +12806,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -12410,13 +12905,13 @@
         <v>1041</v>
       </c>
       <c r="B37" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1327</v>
+      </c>
+      <c r="D37" t="s">
         <v>1318</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1328</v>
-      </c>
-      <c r="D37" t="s">
-        <v>1319</v>
       </c>
       <c r="E37" s="27" t="s">
         <v>6</v>
@@ -12427,13 +12922,13 @@
         <v>1041</v>
       </c>
       <c r="B38" t="s">
+        <v>1390</v>
+      </c>
+      <c r="C38" t="s">
         <v>1391</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>1392</v>
-      </c>
-      <c r="D38" t="s">
-        <v>1393</v>
       </c>
       <c r="E38" s="27" t="s">
         <v>6</v>
@@ -12444,15 +12939,32 @@
         <v>1041</v>
       </c>
       <c r="B39" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1456</v>
+      </c>
+      <c r="D39" t="s">
         <v>1457</v>
       </c>
-      <c r="C39" t="s">
-        <v>1458</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1459</v>
-      </c>
       <c r="E39" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1541</v>
+      </c>
+      <c r="E40" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -12470,7 +12982,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -12953,7 +13465,7 @@
         <v>6</v>
       </c>
       <c r="G24" s="41" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -12961,22 +13473,22 @@
         <v>1006</v>
       </c>
       <c r="B25" s="41" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>1328</v>
+      </c>
+      <c r="D25" s="41" t="s">
         <v>1320</v>
       </c>
-      <c r="C25" s="41" t="s">
-        <v>1329</v>
-      </c>
-      <c r="D25" s="41" t="s">
-        <v>1321</v>
-      </c>
       <c r="E25" s="41" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="F25" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -12984,16 +13496,16 @@
         <v>1006</v>
       </c>
       <c r="B26" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C26" t="s">
         <v>1394</v>
       </c>
-      <c r="C26" t="s">
-        <v>1395</v>
-      </c>
       <c r="D26" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="E26" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="F26" s="27" t="s">
         <v>6</v>
@@ -13004,22 +13516,65 @@
         <v>1006</v>
       </c>
       <c r="B27" t="s">
-        <v>1460</v>
+        <v>1458</v>
       </c>
       <c r="C27" t="s">
-        <v>1461</v>
+        <v>1459</v>
       </c>
       <c r="D27" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="E27" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="F27" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G27" t="s">
-        <v>1494</v>
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1498</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1407</v>
+      </c>
+      <c r="E28" t="s">
+        <v>1407</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1542</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1543</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1407</v>
+      </c>
+      <c r="E29" t="s">
+        <v>1407</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -13033,7 +13588,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -13516,7 +14071,7 @@
         <v>1120</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="D39" s="27" t="s">
         <v>6</v>
@@ -13586,7 +14141,7 @@
         <v>1228</v>
       </c>
       <c r="C44" s="41" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="D44" s="27" t="s">
         <v>6</v>
@@ -13625,10 +14180,10 @@
         <v>1260</v>
       </c>
       <c r="B47" t="s">
+        <v>1294</v>
+      </c>
+      <c r="C47" t="s">
         <v>1295</v>
-      </c>
-      <c r="C47" t="s">
-        <v>1296</v>
       </c>
       <c r="D47" s="27" t="s">
         <v>6</v>
@@ -13636,13 +14191,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="B48" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="C48" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="D48" s="27" t="s">
         <v>6</v>
@@ -13650,13 +14205,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="B49" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C49" t="s">
         <v>1396</v>
-      </c>
-      <c r="C49" t="s">
-        <v>1397</v>
       </c>
       <c r="D49" s="27" t="s">
         <v>6</v>
@@ -13664,13 +14219,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>1408</v>
+      </c>
+      <c r="B50" t="s">
         <v>1409</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>1410</v>
-      </c>
-      <c r="C50" t="s">
-        <v>1411</v>
       </c>
       <c r="D50" s="27" t="s">
         <v>6</v>
@@ -13678,13 +14233,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B51" t="s">
         <v>1460</v>
       </c>
-      <c r="B51" t="s">
-        <v>1462</v>
-      </c>
       <c r="C51" t="s">
-        <v>1463</v>
+        <v>1461</v>
       </c>
       <c r="D51" s="27" t="s">
         <v>6</v>
@@ -13692,13 +14247,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1463</v>
+      </c>
+      <c r="C52" t="s">
         <v>1464</v>
-      </c>
-      <c r="B52" t="s">
-        <v>1465</v>
-      </c>
-      <c r="C52" t="s">
-        <v>1466</v>
       </c>
       <c r="D52" s="27" t="s">
         <v>6</v>
@@ -13706,16 +14261,30 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C53" t="s">
         <v>1486</v>
-      </c>
-      <c r="B53" t="s">
-        <v>1487</v>
-      </c>
-      <c r="C53" t="s">
-        <v>1488</v>
       </c>
       <c r="D53" s="41" t="s">
         <v>1123</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1544</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1545</v>
+      </c>
+      <c r="D54" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 10 - esperienza d'uso (responsive, accessibilità, stati onesti, semaforo disponibilità)
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6243A2-60D6-4814-8BFD-3E2E395B6383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16921961-69B3-4829-967B-27F6CC713C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2716" uniqueCount="1546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2781" uniqueCount="1582">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -4670,6 +4670,114 @@
   </si>
   <si>
     <t>Cartelle vuote e costruttore fantasma di PrenotazioniService rimossi; le interfacce di FasciaOrariaService e PostazioneService non impongono piu' un throw solo per compatibilita' con IService&lt;T&gt;; GetAuthenticatedUserId/GetIpAddress centralizzati in Extensions/HttpContextExtensions (prima duplicati in 4 service e 2 controller); proiezione FasciaOraria-&gt;DTO unificata; CacheDuration/CapienzaConsentita/retention accorpate in costanti nominate; file di test rinominato e refuso email Swagger corretto; rimossi i timestamp scritti a mano nei log dei controller, doppioni di quelli di Serilog. Lato frontend: rimosso codice morto (App.tsx, assets, hook inutilizzato), creato lib/endpoints.ts per i path prima sparsi in 8 hook, GIORNI_SETTIMANA centralizzato, Prettier applicato a tutto il progetto, 18 vulnerabilita' npm risolte con npm audit fix senza --force. dotnet test 237/237 invariato, npm test 26/26 invariato, build e typecheck puliti su entrambi. Nessuna migration.</t>
+  </si>
+  <si>
+    <t>FASE 10 ROADMAP REVISIONE - Esperienza d'uso (sessione 07/09/2026)</t>
+  </si>
+  <si>
+    <t>REV-079 - titolo, lingua e meta description</t>
+  </si>
+  <si>
+    <t>index.html aveva lang='en' su un'app in italiano, title 'gestora-frontend' (il nome della cartella, non del prodotto) e nessuna meta description. Corretti tutti e tre.</t>
+  </si>
+  <si>
+    <t>HTML</t>
+  </si>
+  <si>
+    <t>REV-080 - /unauthorized senza via d'uscita</t>
+  </si>
+  <si>
+    <t>Era un vicolo cieco: l'unico modo per uscirne era modificare l'URL a mano. Aggiunto un pulsante di ritorno, verso la Dashboard per Staff/Admin e verso Prenotazioni per il Cliente (che alla Dashboard non ha comunque accesso).</t>
+  </si>
+  <si>
+    <t>React Router</t>
+  </si>
+  <si>
+    <t>REV-081 - nessuna indicazione di chi sei e dove sei</t>
+  </si>
+  <si>
+    <t>L'header mostrava solo l'email, senza il ruolo: a colpo d'occhio non si distingueva un Cliente da uno Staff. La sidebar non segnalava la pagina attiva. Aggiunto il ruolo sotto l'email nell'header e lo stile attivo sui link della sidebar con NavLink.</t>
+  </si>
+  <si>
+    <t>REV-071 - zero responsive</t>
+  </si>
+  <si>
+    <t>Sidebar fissa a 264px sempre a schermo e 7 tabelle senza scorrimento orizzontale: da smartphone l'app era inutilizzabile, la sidebar da sola occupava piu' della meta' dello schermo. Sidebar richiudibile sotto la soglia md (pannello a scomparsa apribile dall'header), tutte le tabelle avvolte in un contenitore con scorrimento orizzontale proprio, le card della Dashboard passano da 4 a 2 colonne sotto la soglia md.</t>
+  </si>
+  <si>
+    <t>Tailwind CSS</t>
+  </si>
+  <si>
+    <t>REV-075 - stile dei pulsanti incoerente</t>
+  </si>
+  <si>
+    <t>Meta' app usava &lt;Button&gt; di shadcn, l'altra meta' &lt;button&gt; scritti a mano con bg-blue-500/bg-green-500, colori fuori dalla palette del tema. Migrati tutti i pulsanti d'azione (Zone, Postazioni, Fasce Orarie, Prenotazioni, Paginazione, i tre modal CRUD) a &lt;Button&gt;, con una sola eccezione voluta: il link 'Logout' nell'header resta testo semplice, non e' il tipo di incoerenza segnalata.</t>
+  </si>
+  <si>
+    <t>shadcn/ui</t>
+  </si>
+  <si>
+    <t>REV-072 - accessibilita' di base</t>
+  </si>
+  <si>
+    <t>Nessun htmlFor/id collegava le &lt;label&gt; ai campi in tutto il progetto (12 form), i tre checkbox 'Attiva' usavano uno &lt;span&gt; al posto di una &lt;label&gt;, e PrenotazioneModal era l'unico modal con un overlay fatto a mano invece di Radix: senza focus trap ne' chiusura con ESC. htmlFor/id aggiunti ovunque (label visibili sui form del backoffice, sr-only su Login/Registrazione dove il design usa solo il placeholder), PrenotazioneModal migrato su Dialog di Radix come gli altri quattro.</t>
+  </si>
+  <si>
+    <t>Radix UI</t>
+  </si>
+  <si>
+    <t>REV-073 - liste vuote senza spiegazione</t>
+  </si>
+  <si>
+    <t>Zone, Postazioni, Fasce Orarie, Prenotazioni e Utenti mostravano solo l'intestazione della tabella quando l'elenco era vuoto: sembrava un errore, non uno stato normale. Su Postazioni in particolare, prima di scegliere una zona, la tabella vuota non aveva alcuna spiegazione. Nuovo componente EmptyState (una riga con colSpan e un messaggio) su tutte e cinque; su Postazioni aggiunto anche un messaggio esplicito per lo stato 'nessuna zona ancora scelta', diverso da 'zona scelta ma senza postazioni'.</t>
+  </si>
+  <si>
+    <t>React</t>
+  </si>
+  <si>
+    <t>REV-074 + NEW-006 - caricamento a pagina intera ed errori tutti uguali</t>
+  </si>
+  <si>
+    <t>6 pagine sostituivano l'intera vista con &lt;div&gt;Caricamento...&lt;/div&gt; durante il primo caricamento, facendo sparire anche intestazione, filtri e pulsante 'Aggiungi'; gli errori di caricamento dicevano tutti 'Errore nel caricamento' a prescindere dalla causa (server spento, permessi mancanti, database in errore). Nuovo componente condiviso PageState (PageLoading + PageError), quest'ultimo basato su messaggioErroreCaricamento (nuova funzione in lib/apiError, riusa messaggioErrore gia' scritto e testato in Fase 8/9): ora solo il contenuto della pagina si sostituisce, intestazione e filtri restano a schermo.</t>
+  </si>
+  <si>
+    <t>NEW-002 - semaforo di disponibilita' nel form di prenotazione</t>
+  </si>
+  <si>
+    <t>Prima si scopriva che una fascia non aveva piu' posto solo dopo aver premuto Salva. check-disponibilita (pubblico, gia' esistente) risponde con tutte le fasce del giorno gia' valutate: una sola chiamata per (data, coperti) basta per l'intera select. Nuovo hook useCheckDisponibilita (modulo separato da usePrenotazioni.ts apposta, che nei test di REV-047 e' mockato per intero) mostra 'esaurita' sulle option non disponibili e il motivo del rifiuto sotto la select quando si sceglie comunque una fascia piena.</t>
+  </si>
+  <si>
+    <t>tsc -b --force 0 errori, npm test 26/26 (invariato, piu' l'aggiornamento dei test di REV-047 da container.querySelector a screen.getByLabelText - reso possibile proprio da REV-072), npm run build pulita, eslint 0 errori (corretto anche un errore nuovo di React Compiler su una setState sincrona in un effetto, risolto con l'aggiornamento di stato durante il render invece che in un effetto). Nessuna modifica al backend, nessuna migration.</t>
+  </si>
+  <si>
+    <t>Vitest + tsc + eslint</t>
+  </si>
+  <si>
+    <t>Prossimo passo - Fase 11</t>
+  </si>
+  <si>
+    <t>Chiusura del progetto: ultimo giro di revisione, pulizia dei dati di test rimasti in produzione (NEW-005), verifica finale su dispositivo reale.</t>
+  </si>
+  <si>
+    <t>Esperienza d'uso (Fase 10)</t>
+  </si>
+  <si>
+    <t>App utilizzabile da smartphone (sidebar richiudibile, tabelle scorrevoli, card responsive), titolo/lingua/meta corretti, /unauthorized con via d'uscita, ruolo utente e pagina attiva visibili, liste vuote spiegate invece di sembrare un errore, caricamento ed errori parziali (con causa distinta, non piu' un messaggio unico), form accessibili (label collegate, PrenotazioneModal su Radix con ESC e focus trap), semaforo di disponibilita' nel form di prenotazione (NEW-002).</t>
+  </si>
+  <si>
+    <t>React 19 + Tailwind + Radix UI + React Query</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 10</t>
+  </si>
+  <si>
+    <t>Esperienza d'uso: responsive (REV-071), accessibilita' (REV-072), liste vuote (REV-073), caricamento/errori parziali (REV-074, NEW-006), stile pulsanti uniforme (REV-075), titolo/lingua/meta (REV-079), via d'uscita da /unauthorized (REV-080), ruolo utente e pagina attiva (REV-081), semaforo di disponibilita' nel form di prenotazione (NEW-002). Nessuna migration. Un giro di prova da telefono sui tre ruoli ancora da fare (task Fabio).</t>
+  </si>
+  <si>
+    <t>Esperienza d'uso (REV-071, REV-072, REV-073, REV-074, REV-075, REV-079, REV-080, REV-081, NEW-002, NEW-006)</t>
+  </si>
+  <si>
+    <t>Sidebar richiudibile sotto la soglia tablet e tabelle con scorrimento orizzontale proprio (prima l'app era inutilizzabile da smartphone); pulsanti custom con colori fuori palette migrati a &lt;Button&gt; di shadcn ovunque tranne il link Logout; htmlFor/id aggiunti a tutti i form e PrenotazioneModal migrato su Dialog di Radix (era l'unico overlay fatto a mano, senza ESC ne' focus trap); nuovo componente EmptyState sulle cinque liste che prima mostravano solo l'intestazione; nuovo componente PageState (loading ed errore) che lascia intestazione e filtri a schermo durante il caricamento e mostra la causa reale dell'errore (nuova funzione messaggioErroreCaricamento in lib/apiError, riusa quella delle mutation); index.html con lingua italiana, titolo e meta description; /unauthorized con un pulsante di ritorno alla home del ruolo; header con ruolo oltre all'email, sidebar con la voce attiva evidenziata; semaforo di disponibilita' nel form di prenotazione tramite l'endpoint pubblico check-disponibilita, gia' esistente. tsc -b --force 0 errori, npm test 26/26 invariato (test di REV-047 aggiornati per il nuovo Dialog di Radix), build ed eslint puliti. Nessuna migration, backend non toccato.</t>
   </si>
 </sst>
 </file>
@@ -5058,6 +5166,7 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5088,7 +5197,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -5403,36 +5511,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="48" t="s">
         <v>1402</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="51" t="s">
+      <c r="B4" s="53"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="F4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="54"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -5627,24 +5735,24 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="54" t="s">
+      <c r="A16" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="53"/>
+      <c r="B16" s="53"/>
+      <c r="C16" s="53"/>
+      <c r="D16" s="53"/>
+      <c r="E16" s="53"/>
+      <c r="F16" s="54"/>
     </row>
     <row r="17" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="49" t="s">
+      <c r="A17" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -5672,14 +5780,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>643</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -6802,13 +6910,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>1467</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7628,11 +7736,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>794</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
     </row>
     <row r="3" spans="1:3" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7898,14 +8006,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>840</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -7986,7 +8094,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H271"/>
+  <dimension ref="A1:H285"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -7998,40 +8106,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="48" t="s">
         <v>1402</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="53"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="54"/>
     </row>
     <row r="5" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -8354,16 +8462,16 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="51" t="s">
+      <c r="A22" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="53"/>
+      <c r="B22" s="53"/>
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="54"/>
     </row>
     <row r="23" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
@@ -8586,16 +8694,16 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="55" t="s">
+      <c r="A35" s="56" t="s">
         <v>134</v>
       </c>
-      <c r="B35" s="52"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
-      <c r="H35" s="53"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="54"/>
     </row>
     <row r="36" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
@@ -8778,16 +8886,16 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="56" t="s">
+      <c r="A46" s="57" t="s">
         <v>173</v>
       </c>
-      <c r="B46" s="52"/>
-      <c r="C46" s="52"/>
-      <c r="D46" s="52"/>
-      <c r="E46" s="52"/>
-      <c r="F46" s="52"/>
-      <c r="G46" s="52"/>
-      <c r="H46" s="53"/>
+      <c r="B46" s="53"/>
+      <c r="C46" s="53"/>
+      <c r="D46" s="53"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="53"/>
+      <c r="G46" s="53"/>
+      <c r="H46" s="54"/>
     </row>
     <row r="47" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
@@ -8850,16 +8958,16 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="54" t="s">
+      <c r="A51" s="55" t="s">
         <v>185</v>
       </c>
-      <c r="B51" s="52"/>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="52"/>
-      <c r="H51" s="53"/>
+      <c r="B51" s="53"/>
+      <c r="C51" s="53"/>
+      <c r="D51" s="53"/>
+      <c r="E51" s="53"/>
+      <c r="F51" s="53"/>
+      <c r="G51" s="53"/>
+      <c r="H51" s="54"/>
     </row>
     <row r="52" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
@@ -12296,7 +12404,7 @@
       <c r="B268" t="s">
         <v>1529</v>
       </c>
-      <c r="C268" s="59" t="s">
+      <c r="C268" s="47" t="s">
         <v>1530</v>
       </c>
       <c r="D268" t="s">
@@ -12364,6 +12472,247 @@
       </c>
       <c r="E271" s="45"/>
       <c r="F271" s="27"/>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A273" t="s">
+        <v>1546</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A274" t="s">
+        <v>39</v>
+      </c>
+      <c r="B274" t="s">
+        <v>40</v>
+      </c>
+      <c r="C274" t="s">
+        <v>856</v>
+      </c>
+      <c r="D274" t="s">
+        <v>42</v>
+      </c>
+      <c r="E274" t="s">
+        <v>43</v>
+      </c>
+      <c r="F274" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A275">
+        <v>1</v>
+      </c>
+      <c r="B275" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C275" t="s">
+        <v>1548</v>
+      </c>
+      <c r="D275" t="s">
+        <v>1549</v>
+      </c>
+      <c r="E275" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F275" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="276" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A276">
+        <v>2</v>
+      </c>
+      <c r="B276" t="s">
+        <v>1550</v>
+      </c>
+      <c r="C276" t="s">
+        <v>1551</v>
+      </c>
+      <c r="D276" t="s">
+        <v>1552</v>
+      </c>
+      <c r="E276" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F276" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="277" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A277">
+        <v>3</v>
+      </c>
+      <c r="B277" t="s">
+        <v>1553</v>
+      </c>
+      <c r="C277" t="s">
+        <v>1554</v>
+      </c>
+      <c r="D277" t="s">
+        <v>1552</v>
+      </c>
+      <c r="E277" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F277" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A278">
+        <v>4</v>
+      </c>
+      <c r="B278" t="s">
+        <v>1555</v>
+      </c>
+      <c r="C278" t="s">
+        <v>1556</v>
+      </c>
+      <c r="D278" t="s">
+        <v>1557</v>
+      </c>
+      <c r="E278" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F278" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="279" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A279">
+        <v>5</v>
+      </c>
+      <c r="B279" t="s">
+        <v>1558</v>
+      </c>
+      <c r="C279" t="s">
+        <v>1559</v>
+      </c>
+      <c r="D279" t="s">
+        <v>1560</v>
+      </c>
+      <c r="E279" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F279" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="280" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A280">
+        <v>6</v>
+      </c>
+      <c r="B280" t="s">
+        <v>1561</v>
+      </c>
+      <c r="C280" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D280" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E280" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F280" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="281" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A281">
+        <v>7</v>
+      </c>
+      <c r="B281" t="s">
+        <v>1564</v>
+      </c>
+      <c r="C281" t="s">
+        <v>1565</v>
+      </c>
+      <c r="D281" t="s">
+        <v>1566</v>
+      </c>
+      <c r="E281" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F281" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="282" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A282">
+        <v>8</v>
+      </c>
+      <c r="B282" t="s">
+        <v>1567</v>
+      </c>
+      <c r="C282" t="s">
+        <v>1568</v>
+      </c>
+      <c r="D282" t="s">
+        <v>1439</v>
+      </c>
+      <c r="E282" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F282" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="283" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A283">
+        <v>9</v>
+      </c>
+      <c r="B283" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C283" t="s">
+        <v>1570</v>
+      </c>
+      <c r="D283" t="s">
+        <v>1439</v>
+      </c>
+      <c r="E283" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F283" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="284" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A284">
+        <v>10</v>
+      </c>
+      <c r="B284" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C284" t="s">
+        <v>1571</v>
+      </c>
+      <c r="D284" t="s">
+        <v>1572</v>
+      </c>
+      <c r="E284" s="45">
+        <v>46212</v>
+      </c>
+      <c r="F284" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="285" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A285">
+        <v>11</v>
+      </c>
+      <c r="B285" t="s">
+        <v>1573</v>
+      </c>
+      <c r="C285" t="s">
+        <v>1574</v>
+      </c>
+      <c r="D285" t="s">
+        <v>437</v>
+      </c>
+      <c r="E285" s="45"/>
+      <c r="F285" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -12381,7 +12730,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -12392,24 +12741,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="59" t="s">
         <v>221</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="53"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="54"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -12497,14 +12846,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="54" t="s">
+      <c r="A10" s="55" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="52"/>
-      <c r="C10" s="52"/>
-      <c r="D10" s="52"/>
-      <c r="E10" s="52"/>
-      <c r="F10" s="53"/>
+      <c r="B10" s="53"/>
+      <c r="C10" s="53"/>
+      <c r="D10" s="53"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="54"/>
     </row>
     <row r="11" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -12592,14 +12941,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="51" t="s">
+      <c r="A17" s="52" t="s">
         <v>255</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="53"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="54"/>
     </row>
     <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -12721,14 +13070,14 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="51" t="s">
+      <c r="A26" s="52" t="s">
         <v>279</v>
       </c>
-      <c r="B26" s="52"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="53"/>
+      <c r="B26" s="53"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="54"/>
     </row>
     <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -12965,6 +13314,23 @@
         <v>1541</v>
       </c>
       <c r="E40" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1576</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1577</v>
+      </c>
+      <c r="E41" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -12982,7 +13348,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -12994,26 +13360,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="55" t="s">
         <v>289</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="53"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="54"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -13574,6 +13940,26 @@
         <v>1407</v>
       </c>
       <c r="F29" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1579</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1407</v>
+      </c>
+      <c r="E30" t="s">
+        <v>1407</v>
+      </c>
+      <c r="F30" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -13588,7 +13974,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -13598,24 +13984,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>346</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="52" t="s">
         <v>347</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="53"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="54"/>
     </row>
     <row r="4" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
@@ -13800,14 +14186,14 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="58" t="s">
+      <c r="A18" s="59" t="s">
         <v>379</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="53"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="53"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="53"/>
+      <c r="F18" s="54"/>
     </row>
     <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -13914,14 +14300,14 @@
       <c r="D26" s="30"/>
     </row>
     <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="54" t="s">
+      <c r="A28" s="55" t="s">
         <v>392</v>
       </c>
-      <c r="B28" s="52"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="53"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="53"/>
+      <c r="D28" s="53"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="54"/>
     </row>
     <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
@@ -14284,6 +14670,20 @@
         <v>1545</v>
       </c>
       <c r="D54" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>1578</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1580</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1581</v>
+      </c>
+      <c r="D55" s="27" t="s">
         <v>6</v>
       </c>
     </row>
@@ -14311,14 +14711,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>404</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -14495,14 +14895,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>427</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="3" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -15105,13 +15505,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>503</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -15508,13 +15908,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="58" t="s">
         <v>582</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="3" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">

</xml_diff>

<commit_message>
fix: Fase 11 - controllo sovrapposizione fasce non aggirabile in creazione
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1660C9-4CD9-4090-8409-875860D294DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608014CF-9C00-4218-9F7F-0E7E35811A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2818" uniqueCount="1603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2850" uniqueCount="1621">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -3721,12 +3721,6 @@
     <t>NEW-005: pulizia generale del database di produzione a fine progetto</t>
   </si>
   <si>
-    <t>La produzione e' usata anche come ambiente di test, quindi i dati di prova non vengono cancellati man mano (zona Test concorrenza, tavolo da 2, prenotazione del 09/09 e quanto si accumulera' nei prossimi giri). A fine progetto va fatta una pulizia generale prima della consegna. Ordine vincolante per via di NEW-003/REV-099: prima le prenotazioni, poi le postazioni, poi le zone.</t>
-  </si>
-  <si>
-    <t>Pianificato (fine progetto)</t>
-  </si>
-  <si>
     <t>Login, Register, Token JWT - primo avvio via /api/Setup (REV-007), seed-admin rimosso</t>
   </si>
   <si>
@@ -4075,12 +4069,6 @@
     <t>Cosa resta prima di chiudere la fase</t>
   </si>
   <si>
-    <t>168 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 168 test OK</t>
-  </si>
-  <si>
     <t>168 test unitari con xUnit + Moq</t>
   </si>
   <si>
@@ -4264,12 +4252,6 @@
     <t>200 con l'indirizzo usato dall'applicazione e gli header di inoltro grezzi della richiesta corrente - REV-029. Serve a rimisurare la catena dei proxy se la piattaforma cambia: in locale quegli header non esistono, quindi e' l'unico modo di osservarla. Mostra solo i dati di chi chiama.</t>
   </si>
   <si>
-    <t>237 test unitari</t>
-  </si>
-  <si>
-    <t>Testing - 237 backend + 26 frontend</t>
-  </si>
-  <si>
     <t>FASE 8 ROADMAP REVISIONE - Robustezza del frontend (sessione 07/09/2026)</t>
   </si>
   <si>
@@ -4525,9 +4507,6 @@
     <t>Fast-forward, commit 923202d, tag annotato v1.0.4 pubblicato da Visual Studio e verificato sul remoto. Deploy di solo frontend: Vercel ridistribuito sul push, Railway non toccato (backend invariato, nessuna migration). Deploy riuscito. Restano non eseguite quattro prove manuali non bloccanti (paginazione, notifica singola, doppio clic, password nel form): la logica e' coperta dai 26 test automatici.</t>
   </si>
   <si>
-    <t>Railway - PostgreSQL + .NET, health check /health. In produzione: backend v1.0.3 (Fase 7), frontend Vercel v1.0.4 (Fase 8, 07/09/2026)</t>
-  </si>
-  <si>
     <t>FASE 9 ROADMAP REVISIONE - Pulizia (sessione 07/09/2026)</t>
   </si>
   <si>
@@ -4810,9 +4789,6 @@
     <t>C# - FluentValidation / service layer</t>
   </si>
   <si>
-    <t>NEW-007 chiuso, la Fase 11 non e' piu' bloccata. Resta da fare il commit della Fase 10, ancora non committata (un solo commit, tutte modifiche frontend). Poi Fase 11: chiusura del progetto, pulizia dei dati di test rimasti in produzione (NEW-005) e in locale (utente testfase6), piu' il buco di FasciaOrariaService.AddAsync qui sopra.</t>
-  </si>
-  <si>
     <t>Unique index sullo slot (tavolo + data + fascia) con colonne denormalizzate sulla join, scritture in transazione dentro l'execution strategy, violazione 23505 tradotta in 409 leggibile Garanzia verificata sui dati di produzione il 08/09/2026 durante l'indagine NEW-007: indice presente con la definizione esatta del codice, nessuna coppia (tavolo, data, fascia) duplicata.</t>
   </si>
   <si>
@@ -4822,9 +4798,6 @@
     <t>Verifica in produzione della doppia occupazione tavolo segnalata il 07/09: esito falso allarme</t>
   </si>
   <si>
-    <t>Nessuna modifica al codice. Indice UX_PrenotazionePostazione_Slot verificato integro in produzione e nessun duplicato in tutto il database. Aperta una nuova riga in Fix e Bug sul controllo di sovrapposizione delle fasce. Fase 11 sbloccata; resta da committare la Fase 10.</t>
-  </si>
-  <si>
     <t>Falso allarme, verificato sui dati di produzione il 08/09/2026. L'indice UX_PrenotazionePostazione_Slot esiste in produzione con la definizione esatta del codice (nessuno schema drift) e in tutto il database non c'e' una sola coppia (PostazioneId, DataPrenotazione, FasciaOrariaId) duplicata. Sul tavolo 4 del 09/09 le due prenotazioni sono in fasce diverse e non sovrapposte: la 31 sulla fascia 4 (20:00-21:30) e la 30 sulla fascia 10 (21:30-23:30), cioe' il riuso corretto del tavolo nel secondo turno. Nessuna prenotazione usa una fascia di un giorno della settimana diverso dalla propria data. La lettura sbagliata nasce dal numero 21:30, fine dell'una e inizio dell'altra, piu' le sette fasce 20:00-21:30 con etichetta identica (una per giorno). Anche i due utenti diversi sono apparenti: le tre prenotazioni hanno lo stesso UserId (admin), 'Raro' e' il campo NomeCliente. Verificata anche la catena di visualizzazione (Include della FasciaOraria, mapping su OraInizio/OraFine, stampa diretta in PrenotazionePage): non puo' mostrare un orario sbagliato, al massimo vuoto. Nessuna modifica al codice, Fase 11 sbloccata.</t>
   </si>
   <si>
@@ -4834,13 +4807,94 @@
     <t>Controllo di sovrapposizione aggirabile in creazione (emerso indagando NEW-007)</t>
   </si>
   <si>
-    <t>In FasciaOrariaService.AddAsync il controllo GuardSovrapposizioneAsync riceve dto.Id come id da escludere dal confronto. In creazione quel campo dovrebbe valere 0, ma arriva dal client: chi invia un Id uguale a quello di una fascia esistente si fa escludere proprio quella dal controllo e crea una fascia sovrapposta sullo stesso giorno. Oggi non risulta sfruttato - la configurazione in produzione e' pulita, 10 fasce senza sovrapposizioni - ma e' il tipo di difetto che si nota solo quando ha gia' prodotto dati incoerenti, e le fasce sono la base su cui poggia l'unicita' dello slot. Correzione proposta: ignorare dto.Id in creazione (passare 0) e usarlo solo in UpdateAsync, dove escludere la fascia che si sta modificando e' corretto. Da valutare in Fase 11.</t>
-  </si>
-  <si>
     <t>NEW-007 - segnalazione di doppia occupazione dello stesso tavolo (falso allarme)</t>
   </si>
   <si>
     <t>08-set-26</t>
+  </si>
+  <si>
+    <t>In FasciaOrariaService.AddAsync il controllo GuardSovrapposizioneAsync riceve dto.Id come id da escludere dal confronto. In creazione quel campo dovrebbe valere 0, ma arriva dal client: chi invia un Id uguale a quello di una fascia esistente si fa escludere proprio quella dal controllo e crea una fascia sovrapposta sullo stesso giorno. Oggi non risulta sfruttato - la configurazione in produzione e' pulita, 10 fasce senza sovrapposizioni - ma e' il tipo di difetto che si nota solo quando ha gia' prodotto dati incoerenti, e le fasce sono la base su cui poggia l'unicita' dello slot. Correzione proposta: ignorare dto.Id in creazione (passare 0) e usarlo solo in UpdateAsync, dove escludere la fascia che si sta modificando e' corretto. Da valutare in Fase 11. CHIUSO in Fase 11 (08/09/2026): il difetto era doppio. Oltre al guard, dto.Id veniva copiato anche sull'entita' inserita (Id = dto.Id), quindi un Id inviato dal client tentava pure di forzare la chiave primaria, che genera il database. In AddAsync ora si passa 0 al controllo di sovrapposizione e l'Id del DTO non finisce sull'entita'; UpdateAsync resta invariato, li' escludere dal confronto la fascia che si sta modificando e' corretto ed e' un Id verificato, perche' l'entita' viene caricata prima. Due test nuovi in FasciaOrariaServiceTests, scritti prima del fix e visti fallire per il motivo giusto (la fascia sovrapposta veniva creata senza alcuna eccezione): dotnet test 239/239, erano 237. Nessuna migration, nessun cambio di contratto per il frontend.</t>
+  </si>
+  <si>
+    <t>Backlog - appunti d'uso</t>
+  </si>
+  <si>
+    <t>Migliorie d'uso raccolte da Fabio - da formalizzare in una fase dedicata (riga segnaposto)</t>
+  </si>
+  <si>
+    <t>Fabio tiene un file di appunti personale con i miglioramenti minori che emergono usando l'app tutti i giorni (fra questi: etichette delle fasce orarie difficili da distinguere, turno da mostrare accanto all'orario in tabella Prenotazioni, coperti per tavolo - il campo NumeroPosti esiste gia' nel database ma non esce nell'API - e ordinamento delle liste). Per decisione dell'08/09/2026 il file NON viene aperto in Fase 11, che resta una fase di sola chiusura: sara' letto e formalizzato punto per punto, con ID e priorita', in una fase separata successiva. Questa riga esiste solo perche' il backlog non resti invisibile a chi rilegge il tracker.</t>
+  </si>
+  <si>
+    <t>Nessuna modifica al codice. Indice UX_PrenotazionePostazione_Slot verificato integro in produzione e nessun duplicato in tutto il database. Aperta una nuova riga in Fix e Bug sul controllo di sovrapposizione delle fasce, chiusa poi in Fase 11. Fase 11 sbloccata. Fase 10 committata, pushata e mergiata su main l'08/09.</t>
+  </si>
+  <si>
+    <t>v1.0.5</t>
+  </si>
+  <si>
+    <t>Tag della Fase 10, in produzione ma non versionata</t>
+  </si>
+  <si>
+    <t>Tag v1.0.5 su 45ad335, la punta di main: versiona esattamente cio' che gira in produzione. Pubblicato PRIMA di aprire la Fase 11, per non doverla poi taggare insieme alla Fase 10 e perdere la distinzione fra le due. Nessun deploy: il tag non cambia codice, e' solo un riferimento sulla storia. La Fase 9 resta non taggata per scelta, era solo refactoring interno.</t>
+  </si>
+  <si>
+    <t>Roadmap revisione - Fase 11</t>
+  </si>
+  <si>
+    <t>Testing - 239 backend + 26 frontend</t>
+  </si>
+  <si>
+    <t>Railway - PostgreSQL + .NET, health check /health. In produzione: backend allineato a main (Fase 9, non taggata), frontend Vercel v1.0.5 (Fase 10, taggata l'08/09/2026)</t>
+  </si>
+  <si>
+    <t>NEW-007 chiuso, Fase 10 committata e pushata, tag v1.0.5 pubblicato: la Fase 11 e' partita l'08/09/2026 come fase di sola chiusura, vedi sezione successiva. Le migliorie raccolte nel file di appunti d'uso di Fabio non entrano in questa fase: saranno formalizzate in una fase separata.</t>
+  </si>
+  <si>
+    <t>FASE 11 ROADMAP REVISIONE - Chiusura del progetto (sessione 08/09/2026)</t>
+  </si>
+  <si>
+    <t>Blocco 0 - igiene: tag v1.0.5 e stato allineato</t>
+  </si>
+  <si>
+    <t>La Fase 10 era in produzione ma non versionata, e l'aggiornamento di stato dell'08/09 (chiusura NEW-007) era scritto in CLAUDE.md ma mai committato: il working tree non era pulito come sembrava. Tag v1.0.5 pubblicato su 45ad335 prima di aprire la fase, cosi' versiona esattamente cio' che gira in produzione invece di finire mescolato alla Fase 11. Poi commit della documentazione (bff0c3c). Pulizia dell'ambiente locale (utente testfase6) spostata nel blocco di chiusura.</t>
+  </si>
+  <si>
+    <t>Git - tag annotato</t>
+  </si>
+  <si>
+    <t>Blocco A - controllo di sovrapposizione delle fasce aggirabile in creazione</t>
+  </si>
+  <si>
+    <t>Il difetto trovato indagando NEW-007 era piu' largo di come era stato registrato: dto.Id non finiva solo in GuardSovrapposizioneAsync, dove faceva escludere dal confronto proprio la fascia con cui ci si sovrappone, ma veniva anche copiato sull'entita' inserita, tentando di forzare una chiave primaria che genera il database. Corretti entrambi i punti: 0 al guard in creazione, Id non copiato, UpdateAsync invariato. Fatto in TDD: prima i due test, visti fallire per il motivo giusto (la fascia sovrapposta veniva creata, nessuna eccezione), poi il fix. dotnet test 239/239, erano 237. Nessuna migration, nessun cambio di contratto per il frontend.</t>
+  </si>
+  <si>
+    <t>C# - service layer + xUnit (TDD)</t>
+  </si>
+  <si>
+    <t>Test automatici</t>
+  </si>
+  <si>
+    <t>239 test backend (xUnit + Moq) + 26 frontend (Vitest)</t>
+  </si>
+  <si>
+    <t>RBAC e ruoli</t>
+  </si>
+  <si>
+    <t>La produzione e' usata anche come ambiente di test, quindi i dati di prova non vengono cancellati man mano (zona Test concorrenza, tavolo da 2, prenotazione del 09/09 e quanto si accumulera' nei prossimi giri). A fine progetto va fatta una pulizia generale prima della consegna. Ordine vincolante per via di NEW-003/REV-099: prima le prenotazioni, poi le postazioni, poi le zone. DECISIONE 08/09/2026 (Fase 11): al posto della cancellazione mirata riga per riga si fara' un RESET COMPLETO di entrambi i database, locale e produzione, quando tutte le implementazioni e i fix saranno chiusi. Motivo pratico: la cancellazione mirata si blocca sulle prenotazioni gia' Completata, che le API non permettono ne' di eliminare (409 su qualsiasi stato diverso da Attiva/Annullata) ne' di annullare, e la loro riga in PrenotazioniPostazioni rende poi non eliminabile anche il tavolo e, a cascata, la zona. Il reset evita del tutto il vicolo cieco. Da ricordare per quando si fara': le tabelle QRTZ_ non stanno nelle migration EF, va rieseguito Scripts/quartz_postgres.sql o l'app non parte; il primo Admin si ricrea da POST /api/Setup/admin, che si riapre da solo quando non esiste nessun Admin; sparisce anche l'audit trail (tabella Logging), che e' una conseguenza voluta e non un effetto collaterale.</t>
+  </si>
+  <si>
+    <t>Blocco D - chiusura (pulizia dati rimandata al reset finale)</t>
+  </si>
+  <si>
+    <t>La pulizia mirata dei dati di test (NEW-005 in produzione e utente testfase6 in locale) NON e' stata eseguita: per decisione di Fabio dell'08/09/2026 si fara' un reset completo di entrambi i database a implementazioni e fix conclusi, invece di cancellare riga per riga. La cancellazione mirata si sarebbe comunque bloccata sulle prenotazioni gia' Completata, che le API non lasciano ne' eliminare ne' annullare e che tengono in vita la riga di collegamento, rendendo non eliminabili tavolo e zona. Del Blocco D restano quindi solo il merge, il tag di chiusura e l'aggiornamento della documentazione.</t>
+  </si>
+  <si>
+    <t>Git + documentazione</t>
+  </si>
+  <si>
+    <t>Chiusura del progetto: controllo di sovrapposizione delle fasce aggirabile in creazione (Fix e Bug riga 57). La pulizia dei dati di test esce dalla fase: sara' un reset completo dei due database a fine progetto (NEW-005 aggiornato). Le migliorie d'uso raccolte da Fabio restano volutamente fuori: fase separata.</t>
+  </si>
+  <si>
+    <t>Blocco A chiuso: fix in TDD, test scritti prima e visti fallire, dotnet test 239/239 (erano 237). Nessuna migration, frontend non toccato. Pulizia dati rimandata al reset finale dei database. Resta la chiusura formale: merge e tag.</t>
   </si>
 </sst>
 </file>
@@ -5592,7 +5646,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="49" t="s">
-        <v>1580</v>
+        <v>1573</v>
       </c>
       <c r="B2" s="50"/>
       <c r="C2" s="50"/>
@@ -5627,7 +5681,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5747,13 +5801,13 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="6" t="s">
-        <v>1410</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>1347</v>
+        <v>1612</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>6</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>1347</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5761,15 +5815,13 @@
         <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1411</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>1411</v>
-      </c>
+        <v>1602</v>
+      </c>
+      <c r="C13" s="3"/>
       <c r="D13" s="1" t="s">
-        <v>1348</v>
-      </c>
-      <c r="E13" s="4" t="s">
+        <v>1614</v>
+      </c>
+      <c r="E13" s="30" t="s">
         <v>6</v>
       </c>
       <c r="F13" s="5" t="s">
@@ -5787,7 +5839,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>1497</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5801,7 +5853,7 @@
         <v>6</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>1581</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -6061,13 +6113,13 @@
     </row>
     <row r="13" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
       <c r="B13" t="s">
         <v>665</v>
       </c>
       <c r="C13" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="D13" t="s">
         <v>653</v>
@@ -6076,27 +6128,27 @@
         <v>437</v>
       </c>
       <c r="F13" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
       <c r="B14" t="s">
         <v>651</v>
       </c>
       <c r="C14" t="s">
-        <v>1266</v>
+        <v>1264</v>
       </c>
       <c r="D14" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="E14" t="s">
         <v>654</v>
       </c>
       <c r="F14" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6656,7 +6708,7 @@
         <v>687</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6676,7 +6728,7 @@
         <v>731</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6716,7 +6768,7 @@
         <v>437</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>1463</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6756,7 +6808,7 @@
         <v>739</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
@@ -6776,7 +6828,7 @@
         <v>669</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>1355</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -6921,33 +6973,33 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>1396</v>
+        <v>1392</v>
       </c>
       <c r="B56" t="s">
         <v>665</v>
       </c>
       <c r="C56" t="s">
-        <v>1397</v>
+        <v>1393</v>
       </c>
       <c r="D56" t="s">
         <v>660</v>
       </c>
       <c r="E56" t="s">
-        <v>1398</v>
+        <v>1394</v>
       </c>
       <c r="F56" t="s">
-        <v>1399</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>1396</v>
+        <v>1392</v>
       </c>
       <c r="B57" t="s">
         <v>665</v>
       </c>
       <c r="C57" t="s">
-        <v>1408</v>
+        <v>1404</v>
       </c>
       <c r="D57" t="s">
         <v>660</v>
@@ -6956,7 +7008,7 @@
         <v>437</v>
       </c>
       <c r="F57" t="s">
-        <v>1409</v>
+        <v>1405</v>
       </c>
     </row>
   </sheetData>
@@ -6981,7 +7033,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="59" t="s">
-        <v>1464</v>
+        <v>1458</v>
       </c>
       <c r="B1" s="50"/>
       <c r="C1" s="50"/>
@@ -7721,16 +7773,16 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>1465</v>
+        <v>1459</v>
       </c>
       <c r="B47" t="s">
-        <v>1466</v>
+        <v>1460</v>
       </c>
       <c r="C47" t="s">
-        <v>1467</v>
+        <v>1461</v>
       </c>
       <c r="D47" t="s">
-        <v>1468</v>
+        <v>1462</v>
       </c>
       <c r="E47" s="27" t="s">
         <v>6</v>
@@ -7738,16 +7790,16 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1469</v>
+        <v>1463</v>
       </c>
       <c r="B48" t="s">
-        <v>1470</v>
+        <v>1464</v>
       </c>
       <c r="C48" t="s">
-        <v>1471</v>
+        <v>1465</v>
       </c>
       <c r="D48" t="s">
-        <v>1472</v>
+        <v>1466</v>
       </c>
       <c r="E48" s="27" t="s">
         <v>6</v>
@@ -7755,16 +7807,16 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>1473</v>
+        <v>1467</v>
       </c>
       <c r="B49" t="s">
-        <v>1474</v>
+        <v>1468</v>
       </c>
       <c r="C49" t="s">
-        <v>1475</v>
+        <v>1469</v>
       </c>
       <c r="D49" t="s">
-        <v>1476</v>
+        <v>1470</v>
       </c>
       <c r="E49" s="27" t="s">
         <v>6</v>
@@ -7772,16 +7824,16 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>1477</v>
+        <v>1471</v>
       </c>
       <c r="B50" t="s">
-        <v>1478</v>
+        <v>1472</v>
       </c>
       <c r="C50" t="s">
-        <v>1479</v>
+        <v>1473</v>
       </c>
       <c r="D50" t="s">
-        <v>1480</v>
+        <v>1474</v>
       </c>
       <c r="E50" s="27" t="s">
         <v>6</v>
@@ -8164,7 +8216,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H292"/>
+  <dimension ref="A1:H298"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -8189,7 +8241,7 @@
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="49" t="s">
-        <v>1580</v>
+        <v>1573</v>
       </c>
       <c r="B2" s="50"/>
       <c r="C2" s="50"/>
@@ -10879,7 +10931,7 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>1232</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -10907,13 +10959,13 @@
         <v>1</v>
       </c>
       <c r="B182" s="27" t="s">
+        <v>1231</v>
+      </c>
+      <c r="C182" s="27" t="s">
+        <v>1232</v>
+      </c>
+      <c r="D182" s="27" t="s">
         <v>1233</v>
-      </c>
-      <c r="C182" s="27" t="s">
-        <v>1234</v>
-      </c>
-      <c r="D182" s="27" t="s">
-        <v>1235</v>
       </c>
       <c r="E182" s="40" t="s">
         <v>1205</v>
@@ -10927,13 +10979,13 @@
         <v>2</v>
       </c>
       <c r="B183" s="27" t="s">
+        <v>1234</v>
+      </c>
+      <c r="C183" s="27" t="s">
+        <v>1235</v>
+      </c>
+      <c r="D183" s="27" t="s">
         <v>1236</v>
-      </c>
-      <c r="C183" s="27" t="s">
-        <v>1237</v>
-      </c>
-      <c r="D183" s="27" t="s">
-        <v>1238</v>
       </c>
       <c r="E183" s="40" t="s">
         <v>1205</v>
@@ -10947,13 +10999,13 @@
         <v>3</v>
       </c>
       <c r="B184" s="27" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C184" s="27" t="s">
+        <v>1238</v>
+      </c>
+      <c r="D184" s="27" t="s">
         <v>1239</v>
-      </c>
-      <c r="C184" s="27" t="s">
-        <v>1240</v>
-      </c>
-      <c r="D184" s="27" t="s">
-        <v>1241</v>
       </c>
       <c r="E184" s="40" t="s">
         <v>1205</v>
@@ -10967,10 +11019,10 @@
         <v>4</v>
       </c>
       <c r="B185" s="27" t="s">
-        <v>1242</v>
+        <v>1240</v>
       </c>
       <c r="C185" s="27" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="D185" s="27" t="s">
         <v>401</v>
@@ -10987,13 +11039,13 @@
         <v>5</v>
       </c>
       <c r="B186" s="27" t="s">
+        <v>1242</v>
+      </c>
+      <c r="C186" s="27" t="s">
+        <v>1243</v>
+      </c>
+      <c r="D186" s="27" t="s">
         <v>1244</v>
-      </c>
-      <c r="C186" s="27" t="s">
-        <v>1245</v>
-      </c>
-      <c r="D186" s="27" t="s">
-        <v>1246</v>
       </c>
       <c r="E186" s="40" t="s">
         <v>1205</v>
@@ -11007,13 +11059,13 @@
         <v>6</v>
       </c>
       <c r="B187" s="27" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C187" s="27" t="s">
+        <v>1246</v>
+      </c>
+      <c r="D187" s="27" t="s">
         <v>1247</v>
-      </c>
-      <c r="C187" s="27" t="s">
-        <v>1248</v>
-      </c>
-      <c r="D187" s="27" t="s">
-        <v>1249</v>
       </c>
       <c r="E187" s="40" t="s">
         <v>1205</v>
@@ -11027,10 +11079,10 @@
         <v>7</v>
       </c>
       <c r="B188" s="27" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
       <c r="C188" s="27" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="D188" s="27" t="s">
         <v>22</v>
@@ -11047,13 +11099,13 @@
         <v>8</v>
       </c>
       <c r="B189" s="27" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C189" s="27" t="s">
+        <v>1268</v>
+      </c>
+      <c r="D189" s="27" t="s">
         <v>1269</v>
-      </c>
-      <c r="C189" s="27" t="s">
-        <v>1270</v>
-      </c>
-      <c r="D189" s="27" t="s">
-        <v>1271</v>
       </c>
       <c r="E189" s="40" t="s">
         <v>1205</v>
@@ -11067,13 +11119,13 @@
         <v>9</v>
       </c>
       <c r="B190" s="27" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
       <c r="C190" s="27" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
       <c r="D190" s="27" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="E190" s="40" t="s">
         <v>437</v>
@@ -11084,7 +11136,7 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
@@ -11112,10 +11164,10 @@
         <v>1</v>
       </c>
       <c r="B193" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="C193" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="D193" t="s">
         <v>1151</v>
@@ -11132,10 +11184,10 @@
         <v>2</v>
       </c>
       <c r="B194" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
       <c r="C194" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="D194" t="s">
         <v>74</v>
@@ -11152,13 +11204,13 @@
         <v>3</v>
       </c>
       <c r="B195" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C195" t="s">
+        <v>1281</v>
+      </c>
+      <c r="D195" t="s">
         <v>1282</v>
-      </c>
-      <c r="C195" t="s">
-        <v>1283</v>
-      </c>
-      <c r="D195" t="s">
-        <v>1284</v>
       </c>
       <c r="E195" s="45">
         <v>46090</v>
@@ -11172,10 +11224,10 @@
         <v>4</v>
       </c>
       <c r="B196" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
       <c r="C196" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="D196" t="s">
         <v>74</v>
@@ -11192,13 +11244,13 @@
         <v>5</v>
       </c>
       <c r="B197" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="C197" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="D197" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="E197" s="45">
         <v>46090</v>
@@ -11212,24 +11264,24 @@
         <v>6</v>
       </c>
       <c r="B198" t="s">
+        <v>1286</v>
+      </c>
+      <c r="C198" t="s">
+        <v>1287</v>
+      </c>
+      <c r="D198" t="s">
         <v>1288</v>
-      </c>
-      <c r="C198" t="s">
-        <v>1289</v>
-      </c>
-      <c r="D198" t="s">
-        <v>1290</v>
       </c>
       <c r="E198" t="s">
         <v>437</v>
       </c>
       <c r="F198" s="38" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
@@ -11257,13 +11309,13 @@
         <v>1</v>
       </c>
       <c r="B202" t="s">
+        <v>1294</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1295</v>
+      </c>
+      <c r="D202" t="s">
         <v>1296</v>
-      </c>
-      <c r="C202" t="s">
-        <v>1297</v>
-      </c>
-      <c r="D202" t="s">
-        <v>1298</v>
       </c>
       <c r="E202" s="45">
         <v>46121</v>
@@ -11277,13 +11329,13 @@
         <v>2</v>
       </c>
       <c r="B203" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C203" t="s">
+        <v>1298</v>
+      </c>
+      <c r="D203" t="s">
         <v>1299</v>
-      </c>
-      <c r="C203" t="s">
-        <v>1300</v>
-      </c>
-      <c r="D203" t="s">
-        <v>1301</v>
       </c>
       <c r="E203" s="45">
         <v>46121</v>
@@ -11297,13 +11349,13 @@
         <v>3</v>
       </c>
       <c r="B204" t="s">
+        <v>1300</v>
+      </c>
+      <c r="C204" t="s">
+        <v>1301</v>
+      </c>
+      <c r="D204" t="s">
         <v>1302</v>
-      </c>
-      <c r="C204" t="s">
-        <v>1303</v>
-      </c>
-      <c r="D204" t="s">
-        <v>1304</v>
       </c>
       <c r="E204" s="45">
         <v>46121</v>
@@ -11317,13 +11369,13 @@
         <v>4</v>
       </c>
       <c r="B205" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C205" t="s">
+        <v>1304</v>
+      </c>
+      <c r="D205" t="s">
         <v>1305</v>
-      </c>
-      <c r="C205" t="s">
-        <v>1306</v>
-      </c>
-      <c r="D205" t="s">
-        <v>1307</v>
       </c>
       <c r="E205" s="45">
         <v>46121</v>
@@ -11337,13 +11389,13 @@
         <v>5</v>
       </c>
       <c r="B206" t="s">
+        <v>1306</v>
+      </c>
+      <c r="C206" t="s">
+        <v>1307</v>
+      </c>
+      <c r="D206" t="s">
         <v>1308</v>
-      </c>
-      <c r="C206" t="s">
-        <v>1309</v>
-      </c>
-      <c r="D206" t="s">
-        <v>1310</v>
       </c>
       <c r="E206" s="45">
         <v>46121</v>
@@ -11357,13 +11409,13 @@
         <v>6</v>
       </c>
       <c r="B207" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C207" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D207" t="s">
         <v>1311</v>
-      </c>
-      <c r="C207" t="s">
-        <v>1312</v>
-      </c>
-      <c r="D207" t="s">
-        <v>1313</v>
       </c>
       <c r="E207" s="45">
         <v>46121</v>
@@ -11377,13 +11429,13 @@
         <v>7</v>
       </c>
       <c r="B208" t="s">
+        <v>1320</v>
+      </c>
+      <c r="C208" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D208" t="s">
         <v>1322</v>
-      </c>
-      <c r="C208" t="s">
-        <v>1323</v>
-      </c>
-      <c r="D208" t="s">
-        <v>1324</v>
       </c>
       <c r="E208" s="45">
         <v>46121</v>
@@ -11397,13 +11449,13 @@
         <v>8</v>
       </c>
       <c r="B209" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
       <c r="C209" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="D209" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
       <c r="E209" s="45">
         <v>46121</v>
@@ -11417,13 +11469,13 @@
         <v>8</v>
       </c>
       <c r="B210" t="s">
+        <v>1329</v>
+      </c>
+      <c r="C210" t="s">
+        <v>1330</v>
+      </c>
+      <c r="D210" t="s">
         <v>1331</v>
-      </c>
-      <c r="C210" t="s">
-        <v>1332</v>
-      </c>
-      <c r="D210" t="s">
-        <v>1333</v>
       </c>
       <c r="E210" s="45">
         <v>46121</v>
@@ -11437,13 +11489,13 @@
         <v>9</v>
       </c>
       <c r="B211" t="s">
+        <v>1332</v>
+      </c>
+      <c r="C211" t="s">
+        <v>1333</v>
+      </c>
+      <c r="D211" t="s">
         <v>1334</v>
-      </c>
-      <c r="C211" t="s">
-        <v>1335</v>
-      </c>
-      <c r="D211" t="s">
-        <v>1336</v>
       </c>
       <c r="E211" s="45">
         <v>46121</v>
@@ -11457,13 +11509,13 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
+        <v>1335</v>
+      </c>
+      <c r="C212" t="s">
+        <v>1336</v>
+      </c>
+      <c r="D212" t="s">
         <v>1337</v>
-      </c>
-      <c r="C212" t="s">
-        <v>1338</v>
-      </c>
-      <c r="D212" t="s">
-        <v>1339</v>
       </c>
       <c r="E212" s="45">
         <v>46121</v>
@@ -11477,13 +11529,13 @@
         <v>11</v>
       </c>
       <c r="B213" t="s">
+        <v>1338</v>
+      </c>
+      <c r="C213" t="s">
+        <v>1339</v>
+      </c>
+      <c r="D213" t="s">
         <v>1340</v>
-      </c>
-      <c r="C213" t="s">
-        <v>1341</v>
-      </c>
-      <c r="D213" t="s">
-        <v>1342</v>
       </c>
       <c r="E213" s="45">
         <v>46121</v>
@@ -11497,13 +11549,13 @@
         <v>12</v>
       </c>
       <c r="B214" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C214" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D214" t="s">
         <v>1343</v>
-      </c>
-      <c r="C214" t="s">
-        <v>1344</v>
-      </c>
-      <c r="D214" t="s">
-        <v>1345</v>
       </c>
       <c r="E214" s="45">
         <v>46121</v>
@@ -11517,10 +11569,10 @@
         <v>13</v>
       </c>
       <c r="B215" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="C215" t="s">
-        <v>1353</v>
+        <v>1349</v>
       </c>
       <c r="D215" t="s">
         <v>437</v>
@@ -11537,13 +11589,13 @@
         <v>14</v>
       </c>
       <c r="B216" t="s">
-        <v>1351</v>
+        <v>1347</v>
       </c>
       <c r="C216" t="s">
-        <v>1354</v>
+        <v>1350</v>
       </c>
       <c r="D216" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="E216" s="45">
         <v>46121</v>
@@ -11554,7 +11606,7 @@
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
@@ -11582,13 +11634,13 @@
         <v>1</v>
       </c>
       <c r="B220" t="s">
-        <v>1356</v>
+        <v>1352</v>
       </c>
       <c r="C220" t="s">
-        <v>1357</v>
+        <v>1353</v>
       </c>
       <c r="D220" t="s">
-        <v>1358</v>
+        <v>1354</v>
       </c>
       <c r="E220" s="45">
         <v>46121</v>
@@ -11602,10 +11654,10 @@
         <v>2</v>
       </c>
       <c r="B221" t="s">
-        <v>1359</v>
+        <v>1355</v>
       </c>
       <c r="C221" t="s">
-        <v>1360</v>
+        <v>1356</v>
       </c>
       <c r="D221" t="s">
         <v>287</v>
@@ -11622,10 +11674,10 @@
         <v>3</v>
       </c>
       <c r="B222" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="C222" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="D222" t="s">
         <v>29</v>
@@ -11642,13 +11694,13 @@
         <v>4</v>
       </c>
       <c r="B223" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
       <c r="C223" t="s">
-        <v>1364</v>
+        <v>1360</v>
       </c>
       <c r="D223" t="s">
-        <v>1365</v>
+        <v>1361</v>
       </c>
       <c r="E223" s="45">
         <v>46121</v>
@@ -11662,13 +11714,13 @@
         <v>5</v>
       </c>
       <c r="B224" t="s">
-        <v>1366</v>
+        <v>1362</v>
       </c>
       <c r="C224" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
       <c r="D224" t="s">
-        <v>1358</v>
+        <v>1354</v>
       </c>
       <c r="E224" s="45">
         <v>46121</v>
@@ -11682,13 +11734,13 @@
         <v>6</v>
       </c>
       <c r="B225" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="C225" t="s">
-        <v>1369</v>
+        <v>1365</v>
       </c>
       <c r="D225" t="s">
-        <v>1370</v>
+        <v>1366</v>
       </c>
       <c r="E225" s="45">
         <v>46121</v>
@@ -11702,10 +11754,10 @@
         <v>7</v>
       </c>
       <c r="B226" t="s">
-        <v>1371</v>
+        <v>1367</v>
       </c>
       <c r="C226" t="s">
-        <v>1372</v>
+        <v>1368</v>
       </c>
       <c r="D226" t="s">
         <v>267</v>
@@ -11722,13 +11774,13 @@
         <v>8</v>
       </c>
       <c r="B227" t="s">
-        <v>1373</v>
+        <v>1369</v>
       </c>
       <c r="C227" t="s">
-        <v>1374</v>
+        <v>1370</v>
       </c>
       <c r="D227" t="s">
-        <v>1375</v>
+        <v>1371</v>
       </c>
       <c r="E227" s="45">
         <v>46121</v>
@@ -11742,13 +11794,13 @@
         <v>9</v>
       </c>
       <c r="B228" t="s">
-        <v>1376</v>
+        <v>1372</v>
       </c>
       <c r="C228" t="s">
-        <v>1377</v>
+        <v>1373</v>
       </c>
       <c r="D228" t="s">
-        <v>1378</v>
+        <v>1374</v>
       </c>
       <c r="E228" s="45">
         <v>46121</v>
@@ -11762,13 +11814,13 @@
         <v>10</v>
       </c>
       <c r="B229" t="s">
-        <v>1379</v>
+        <v>1375</v>
       </c>
       <c r="C229" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="D229" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
       <c r="E229" s="45">
         <v>46121</v>
@@ -11782,13 +11834,13 @@
         <v>11</v>
       </c>
       <c r="B230" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="C230" t="s">
-        <v>1383</v>
+        <v>1379</v>
       </c>
       <c r="D230" t="s">
-        <v>1384</v>
+        <v>1380</v>
       </c>
       <c r="E230" s="45">
         <v>46121</v>
@@ -11802,10 +11854,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
-        <v>1385</v>
+        <v>1381</v>
       </c>
       <c r="C231" t="s">
-        <v>1386</v>
+        <v>1382</v>
       </c>
       <c r="D231" t="s">
         <v>32</v>
@@ -11822,10 +11874,10 @@
         <v>13</v>
       </c>
       <c r="B232" t="s">
-        <v>1387</v>
+        <v>1383</v>
       </c>
       <c r="C232" t="s">
-        <v>1400</v>
+        <v>1396</v>
       </c>
       <c r="D232" t="s">
         <v>437</v>
@@ -11842,13 +11894,13 @@
         <v>14</v>
       </c>
       <c r="B233" t="s">
-        <v>1401</v>
+        <v>1397</v>
       </c>
       <c r="C233" t="s">
-        <v>1402</v>
+        <v>1398</v>
       </c>
       <c r="D233" t="s">
-        <v>1403</v>
+        <v>1399</v>
       </c>
       <c r="E233" s="45">
         <v>46212</v>
@@ -11859,7 +11911,7 @@
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
-        <v>1412</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="236" spans="1:6" x14ac:dyDescent="0.3">
@@ -11887,13 +11939,13 @@
         <v>1</v>
       </c>
       <c r="B237" t="s">
-        <v>1413</v>
+        <v>1407</v>
       </c>
       <c r="C237" t="s">
-        <v>1414</v>
+        <v>1408</v>
       </c>
       <c r="D237" t="s">
-        <v>1415</v>
+        <v>1409</v>
       </c>
       <c r="E237" s="45">
         <v>46212</v>
@@ -11907,13 +11959,13 @@
         <v>2</v>
       </c>
       <c r="B238" t="s">
-        <v>1416</v>
+        <v>1410</v>
       </c>
       <c r="C238" t="s">
-        <v>1417</v>
+        <v>1411</v>
       </c>
       <c r="D238" t="s">
-        <v>1418</v>
+        <v>1412</v>
       </c>
       <c r="E238" s="45">
         <v>46212</v>
@@ -11927,13 +11979,13 @@
         <v>3</v>
       </c>
       <c r="B239" t="s">
-        <v>1419</v>
+        <v>1413</v>
       </c>
       <c r="C239" t="s">
-        <v>1420</v>
+        <v>1414</v>
       </c>
       <c r="D239" t="s">
-        <v>1421</v>
+        <v>1415</v>
       </c>
       <c r="E239" s="45">
         <v>46212</v>
@@ -11947,13 +11999,13 @@
         <v>4</v>
       </c>
       <c r="B240" t="s">
-        <v>1422</v>
+        <v>1416</v>
       </c>
       <c r="C240" t="s">
-        <v>1423</v>
+        <v>1417</v>
       </c>
       <c r="D240" t="s">
-        <v>1424</v>
+        <v>1418</v>
       </c>
       <c r="E240" s="45">
         <v>46212</v>
@@ -11967,13 +12019,13 @@
         <v>5</v>
       </c>
       <c r="B241" t="s">
-        <v>1425</v>
+        <v>1419</v>
       </c>
       <c r="C241" t="s">
-        <v>1426</v>
+        <v>1420</v>
       </c>
       <c r="D241" t="s">
-        <v>1427</v>
+        <v>1421</v>
       </c>
       <c r="E241" s="45">
         <v>46212</v>
@@ -11987,13 +12039,13 @@
         <v>6</v>
       </c>
       <c r="B242" t="s">
-        <v>1428</v>
+        <v>1422</v>
       </c>
       <c r="C242" t="s">
-        <v>1429</v>
+        <v>1423</v>
       </c>
       <c r="D242" t="s">
-        <v>1430</v>
+        <v>1424</v>
       </c>
       <c r="E242" s="45">
         <v>46212</v>
@@ -12007,13 +12059,13 @@
         <v>7</v>
       </c>
       <c r="B243" t="s">
-        <v>1431</v>
+        <v>1425</v>
       </c>
       <c r="C243" t="s">
-        <v>1432</v>
+        <v>1426</v>
       </c>
       <c r="D243" t="s">
-        <v>1433</v>
+        <v>1427</v>
       </c>
       <c r="E243" s="45">
         <v>46212</v>
@@ -12027,13 +12079,13 @@
         <v>8</v>
       </c>
       <c r="B244" t="s">
-        <v>1434</v>
+        <v>1428</v>
       </c>
       <c r="C244" t="s">
-        <v>1435</v>
+        <v>1429</v>
       </c>
       <c r="D244" t="s">
-        <v>1436</v>
+        <v>1430</v>
       </c>
       <c r="E244" s="45">
         <v>46212</v>
@@ -12047,13 +12099,13 @@
         <v>9</v>
       </c>
       <c r="B245" t="s">
-        <v>1437</v>
+        <v>1431</v>
       </c>
       <c r="C245" t="s">
-        <v>1438</v>
+        <v>1432</v>
       </c>
       <c r="D245" t="s">
-        <v>1439</v>
+        <v>1433</v>
       </c>
       <c r="E245" s="45">
         <v>46212</v>
@@ -12067,13 +12119,13 @@
         <v>10</v>
       </c>
       <c r="B246" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
       <c r="C246" t="s">
-        <v>1441</v>
+        <v>1435</v>
       </c>
       <c r="D246" t="s">
-        <v>1442</v>
+        <v>1436</v>
       </c>
       <c r="E246" s="45">
         <v>46212</v>
@@ -12087,10 +12139,10 @@
         <v>11</v>
       </c>
       <c r="B247" t="s">
-        <v>1443</v>
+        <v>1437</v>
       </c>
       <c r="C247" t="s">
-        <v>1444</v>
+        <v>1438</v>
       </c>
       <c r="D247" t="s">
         <v>437</v>
@@ -12107,13 +12159,13 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
-        <v>1445</v>
+        <v>1439</v>
       </c>
       <c r="C248" t="s">
-        <v>1446</v>
+        <v>1440</v>
       </c>
       <c r="D248" t="s">
-        <v>1447</v>
+        <v>1441</v>
       </c>
       <c r="E248" s="45">
         <v>46212</v>
@@ -12127,13 +12179,13 @@
         <v>13</v>
       </c>
       <c r="B249" t="s">
-        <v>1448</v>
+        <v>1442</v>
       </c>
       <c r="C249" t="s">
-        <v>1449</v>
+        <v>1443</v>
       </c>
       <c r="D249" t="s">
-        <v>1450</v>
+        <v>1444</v>
       </c>
       <c r="E249" s="45">
         <v>46212</v>
@@ -12147,13 +12199,13 @@
         <v>14</v>
       </c>
       <c r="B250" t="s">
-        <v>1484</v>
+        <v>1478</v>
       </c>
       <c r="C250" t="s">
-        <v>1485</v>
+        <v>1479</v>
       </c>
       <c r="D250" t="s">
-        <v>1486</v>
+        <v>1480</v>
       </c>
       <c r="E250" s="45">
         <v>46212</v>
@@ -12167,13 +12219,13 @@
         <v>15</v>
       </c>
       <c r="B251" t="s">
-        <v>1487</v>
+        <v>1481</v>
       </c>
       <c r="C251" t="s">
-        <v>1488</v>
+        <v>1482</v>
       </c>
       <c r="D251" t="s">
-        <v>1436</v>
+        <v>1430</v>
       </c>
       <c r="E251" s="45">
         <v>46212</v>
@@ -12187,13 +12239,13 @@
         <v>16</v>
       </c>
       <c r="B252" t="s">
-        <v>1490</v>
+        <v>1484</v>
       </c>
       <c r="C252" t="s">
-        <v>1491</v>
+        <v>1485</v>
       </c>
       <c r="D252" t="s">
-        <v>1492</v>
+        <v>1486</v>
       </c>
       <c r="E252" s="45">
         <v>46212</v>
@@ -12207,10 +12259,10 @@
         <v>17</v>
       </c>
       <c r="B253" t="s">
-        <v>1451</v>
+        <v>1445</v>
       </c>
       <c r="C253" t="s">
-        <v>1493</v>
+        <v>1487</v>
       </c>
       <c r="D253" t="s">
         <v>437</v>
@@ -12224,7 +12276,7 @@
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
-        <v>1498</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.3">
@@ -12252,10 +12304,10 @@
         <v>1</v>
       </c>
       <c r="B257" t="s">
-        <v>1499</v>
+        <v>1492</v>
       </c>
       <c r="C257" t="s">
-        <v>1500</v>
+        <v>1493</v>
       </c>
       <c r="D257" t="s">
         <v>3</v>
@@ -12272,13 +12324,13 @@
         <v>2</v>
       </c>
       <c r="B258" t="s">
-        <v>1501</v>
+        <v>1494</v>
       </c>
       <c r="C258" t="s">
-        <v>1502</v>
+        <v>1495</v>
       </c>
       <c r="D258" t="s">
-        <v>1503</v>
+        <v>1496</v>
       </c>
       <c r="E258" s="45">
         <v>46212</v>
@@ -12292,10 +12344,10 @@
         <v>3</v>
       </c>
       <c r="B259" t="s">
-        <v>1504</v>
+        <v>1497</v>
       </c>
       <c r="C259" t="s">
-        <v>1505</v>
+        <v>1498</v>
       </c>
       <c r="D259" t="s">
         <v>437</v>
@@ -12312,13 +12364,13 @@
         <v>4</v>
       </c>
       <c r="B260" t="s">
-        <v>1506</v>
+        <v>1499</v>
       </c>
       <c r="C260" t="s">
-        <v>1507</v>
+        <v>1500</v>
       </c>
       <c r="D260" t="s">
-        <v>1508</v>
+        <v>1501</v>
       </c>
       <c r="E260" s="45">
         <v>46212</v>
@@ -12332,13 +12384,13 @@
         <v>5</v>
       </c>
       <c r="B261" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="C261" t="s">
-        <v>1510</v>
+        <v>1503</v>
       </c>
       <c r="D261" t="s">
-        <v>1511</v>
+        <v>1504</v>
       </c>
       <c r="E261" s="45">
         <v>46212</v>
@@ -12352,13 +12404,13 @@
         <v>6</v>
       </c>
       <c r="B262" t="s">
-        <v>1512</v>
+        <v>1505</v>
       </c>
       <c r="C262" t="s">
-        <v>1513</v>
+        <v>1506</v>
       </c>
       <c r="D262" t="s">
-        <v>1511</v>
+        <v>1504</v>
       </c>
       <c r="E262" s="45">
         <v>46212</v>
@@ -12372,10 +12424,10 @@
         <v>7</v>
       </c>
       <c r="B263" t="s">
-        <v>1514</v>
+        <v>1507</v>
       </c>
       <c r="C263" t="s">
-        <v>1515</v>
+        <v>1508</v>
       </c>
       <c r="D263" t="s">
         <v>22</v>
@@ -12392,13 +12444,13 @@
         <v>8</v>
       </c>
       <c r="B264" t="s">
-        <v>1516</v>
+        <v>1509</v>
       </c>
       <c r="C264" t="s">
-        <v>1517</v>
+        <v>1510</v>
       </c>
       <c r="D264" t="s">
-        <v>1518</v>
+        <v>1511</v>
       </c>
       <c r="E264" s="45">
         <v>46212</v>
@@ -12412,13 +12464,13 @@
         <v>9</v>
       </c>
       <c r="B265" t="s">
-        <v>1519</v>
+        <v>1512</v>
       </c>
       <c r="C265" t="s">
-        <v>1520</v>
+        <v>1513</v>
       </c>
       <c r="D265" t="s">
-        <v>1439</v>
+        <v>1433</v>
       </c>
       <c r="E265" s="45">
         <v>46212</v>
@@ -12432,13 +12484,13 @@
         <v>10</v>
       </c>
       <c r="B266" t="s">
-        <v>1521</v>
+        <v>1514</v>
       </c>
       <c r="C266" t="s">
-        <v>1522</v>
+        <v>1515</v>
       </c>
       <c r="D266" t="s">
-        <v>1439</v>
+        <v>1433</v>
       </c>
       <c r="E266" s="45">
         <v>46212</v>
@@ -12452,13 +12504,13 @@
         <v>11</v>
       </c>
       <c r="B267" t="s">
-        <v>1523</v>
+        <v>1516</v>
       </c>
       <c r="C267" t="s">
-        <v>1524</v>
+        <v>1517</v>
       </c>
       <c r="D267" t="s">
-        <v>1525</v>
+        <v>1518</v>
       </c>
       <c r="E267" s="45">
         <v>46212</v>
@@ -12472,13 +12524,13 @@
         <v>12</v>
       </c>
       <c r="B268" t="s">
-        <v>1526</v>
+        <v>1519</v>
       </c>
       <c r="C268" s="47" t="s">
-        <v>1527</v>
+        <v>1520</v>
       </c>
       <c r="D268" t="s">
-        <v>1528</v>
+        <v>1521</v>
       </c>
       <c r="E268" s="45">
         <v>46212</v>
@@ -12492,13 +12544,13 @@
         <v>13</v>
       </c>
       <c r="B269" t="s">
-        <v>1448</v>
+        <v>1442</v>
       </c>
       <c r="C269" t="s">
-        <v>1529</v>
+        <v>1522</v>
       </c>
       <c r="D269" t="s">
-        <v>1530</v>
+        <v>1523</v>
       </c>
       <c r="E269" s="45">
         <v>46212</v>
@@ -12512,13 +12564,13 @@
         <v>14</v>
       </c>
       <c r="B270" t="s">
-        <v>1531</v>
+        <v>1524</v>
       </c>
       <c r="C270" t="s">
-        <v>1532</v>
+        <v>1525</v>
       </c>
       <c r="D270" t="s">
-        <v>1533</v>
+        <v>1526</v>
       </c>
       <c r="E270" s="45">
         <v>46212</v>
@@ -12532,10 +12584,10 @@
         <v>15</v>
       </c>
       <c r="B271" t="s">
-        <v>1534</v>
+        <v>1527</v>
       </c>
       <c r="C271" t="s">
-        <v>1535</v>
+        <v>1528</v>
       </c>
       <c r="D271" t="s">
         <v>437</v>
@@ -12545,7 +12597,7 @@
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
-        <v>1543</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="274" spans="1:6" x14ac:dyDescent="0.3">
@@ -12573,13 +12625,13 @@
         <v>1</v>
       </c>
       <c r="B275" t="s">
-        <v>1544</v>
+        <v>1537</v>
       </c>
       <c r="C275" t="s">
-        <v>1545</v>
+        <v>1538</v>
       </c>
       <c r="D275" t="s">
-        <v>1546</v>
+        <v>1539</v>
       </c>
       <c r="E275" s="45">
         <v>46212</v>
@@ -12593,13 +12645,13 @@
         <v>2</v>
       </c>
       <c r="B276" t="s">
-        <v>1547</v>
+        <v>1540</v>
       </c>
       <c r="C276" t="s">
-        <v>1548</v>
+        <v>1541</v>
       </c>
       <c r="D276" t="s">
-        <v>1549</v>
+        <v>1542</v>
       </c>
       <c r="E276" s="45">
         <v>46212</v>
@@ -12613,13 +12665,13 @@
         <v>3</v>
       </c>
       <c r="B277" t="s">
-        <v>1550</v>
+        <v>1543</v>
       </c>
       <c r="C277" t="s">
-        <v>1551</v>
+        <v>1544</v>
       </c>
       <c r="D277" t="s">
-        <v>1549</v>
+        <v>1542</v>
       </c>
       <c r="E277" s="45">
         <v>46212</v>
@@ -12633,13 +12685,13 @@
         <v>4</v>
       </c>
       <c r="B278" t="s">
-        <v>1552</v>
+        <v>1545</v>
       </c>
       <c r="C278" t="s">
-        <v>1553</v>
+        <v>1546</v>
       </c>
       <c r="D278" t="s">
-        <v>1554</v>
+        <v>1547</v>
       </c>
       <c r="E278" s="45">
         <v>46212</v>
@@ -12653,13 +12705,13 @@
         <v>5</v>
       </c>
       <c r="B279" t="s">
-        <v>1555</v>
+        <v>1548</v>
       </c>
       <c r="C279" t="s">
-        <v>1556</v>
+        <v>1549</v>
       </c>
       <c r="D279" t="s">
-        <v>1557</v>
+        <v>1550</v>
       </c>
       <c r="E279" s="45">
         <v>46212</v>
@@ -12673,13 +12725,13 @@
         <v>6</v>
       </c>
       <c r="B280" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="C280" t="s">
-        <v>1559</v>
+        <v>1552</v>
       </c>
       <c r="D280" t="s">
-        <v>1560</v>
+        <v>1553</v>
       </c>
       <c r="E280" s="45">
         <v>46212</v>
@@ -12693,13 +12745,13 @@
         <v>7</v>
       </c>
       <c r="B281" t="s">
-        <v>1561</v>
+        <v>1554</v>
       </c>
       <c r="C281" t="s">
-        <v>1562</v>
+        <v>1555</v>
       </c>
       <c r="D281" t="s">
-        <v>1563</v>
+        <v>1556</v>
       </c>
       <c r="E281" s="45">
         <v>46212</v>
@@ -12713,13 +12765,13 @@
         <v>8</v>
       </c>
       <c r="B282" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="C282" t="s">
-        <v>1565</v>
+        <v>1558</v>
       </c>
       <c r="D282" t="s">
-        <v>1436</v>
+        <v>1430</v>
       </c>
       <c r="E282" s="45">
         <v>46212</v>
@@ -12733,13 +12785,13 @@
         <v>9</v>
       </c>
       <c r="B283" t="s">
-        <v>1566</v>
+        <v>1559</v>
       </c>
       <c r="C283" t="s">
-        <v>1567</v>
+        <v>1560</v>
       </c>
       <c r="D283" t="s">
-        <v>1436</v>
+        <v>1430</v>
       </c>
       <c r="E283" s="45">
         <v>46212</v>
@@ -12753,13 +12805,13 @@
         <v>10</v>
       </c>
       <c r="B284" t="s">
-        <v>1448</v>
+        <v>1442</v>
       </c>
       <c r="C284" t="s">
-        <v>1568</v>
+        <v>1561</v>
       </c>
       <c r="D284" t="s">
-        <v>1569</v>
+        <v>1562</v>
       </c>
       <c r="E284" s="45">
         <v>46212</v>
@@ -12773,10 +12825,10 @@
         <v>11</v>
       </c>
       <c r="B285" t="s">
-        <v>1570</v>
+        <v>1563</v>
       </c>
       <c r="C285" t="s">
-        <v>1571</v>
+        <v>1564</v>
       </c>
       <c r="D285" t="s">
         <v>437</v>
@@ -12786,7 +12838,7 @@
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
-        <v>1582</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="288" spans="1:6" x14ac:dyDescent="0.3">
@@ -12814,13 +12866,13 @@
         <v>1</v>
       </c>
       <c r="B289" t="s">
-        <v>1583</v>
+        <v>1576</v>
       </c>
       <c r="C289" t="s">
-        <v>1584</v>
+        <v>1577</v>
       </c>
       <c r="D289" t="s">
-        <v>1585</v>
+        <v>1578</v>
       </c>
       <c r="E289" s="45">
         <v>46273</v>
@@ -12834,13 +12886,13 @@
         <v>2</v>
       </c>
       <c r="B290" t="s">
-        <v>1586</v>
+        <v>1579</v>
       </c>
       <c r="C290" t="s">
-        <v>1587</v>
+        <v>1580</v>
       </c>
       <c r="D290" t="s">
-        <v>1588</v>
+        <v>1581</v>
       </c>
       <c r="E290" s="45">
         <v>46273</v>
@@ -12854,19 +12906,19 @@
         <v>3</v>
       </c>
       <c r="B291" t="s">
-        <v>1589</v>
+        <v>1582</v>
       </c>
       <c r="C291" t="s">
-        <v>1590</v>
+        <v>1583</v>
       </c>
       <c r="D291" t="s">
-        <v>1591</v>
+        <v>1584</v>
       </c>
       <c r="E291" s="45">
         <v>46273</v>
       </c>
-      <c r="F291" s="38" t="s">
-        <v>977</v>
+      <c r="F291" s="27" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.3">
@@ -12874,16 +12926,101 @@
         <v>4</v>
       </c>
       <c r="B292" t="s">
-        <v>1570</v>
+        <v>1563</v>
       </c>
       <c r="C292" t="s">
-        <v>1592</v>
+        <v>1604</v>
       </c>
       <c r="D292" t="s">
         <v>437</v>
       </c>
       <c r="E292" s="45"/>
       <c r="F292" s="27"/>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A294" t="s">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A295" t="s">
+        <v>39</v>
+      </c>
+      <c r="B295" t="s">
+        <v>40</v>
+      </c>
+      <c r="C295" t="s">
+        <v>856</v>
+      </c>
+      <c r="D295" t="s">
+        <v>42</v>
+      </c>
+      <c r="E295" t="s">
+        <v>43</v>
+      </c>
+      <c r="F295" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A296">
+        <v>1</v>
+      </c>
+      <c r="B296" t="s">
+        <v>1606</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1607</v>
+      </c>
+      <c r="D296" t="s">
+        <v>1608</v>
+      </c>
+      <c r="E296" s="45">
+        <v>46273</v>
+      </c>
+      <c r="F296" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A297">
+        <v>2</v>
+      </c>
+      <c r="B297" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C297" t="s">
+        <v>1610</v>
+      </c>
+      <c r="D297" t="s">
+        <v>1611</v>
+      </c>
+      <c r="E297" s="45">
+        <v>46273</v>
+      </c>
+      <c r="F297" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A298">
+        <v>3</v>
+      </c>
+      <c r="B298" t="s">
+        <v>1616</v>
+      </c>
+      <c r="C298" t="s">
+        <v>1617</v>
+      </c>
+      <c r="D298" t="s">
+        <v>1618</v>
+      </c>
+      <c r="E298" s="45">
+        <v>46273</v>
+      </c>
+      <c r="F298" s="38" t="s">
+        <v>1292</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -13326,7 +13463,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1349</v>
+        <v>1345</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>74</v>
@@ -13394,7 +13531,7 @@
         <v>1131</v>
       </c>
       <c r="C35" t="s">
-        <v>1593</v>
+        <v>1585</v>
       </c>
       <c r="D35" t="s">
         <v>1159</v>
@@ -13408,13 +13545,13 @@
         <v>1041</v>
       </c>
       <c r="B36" t="s">
+        <v>1252</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1253</v>
+      </c>
+      <c r="D36" t="s">
         <v>1254</v>
-      </c>
-      <c r="C36" t="s">
-        <v>1255</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1256</v>
       </c>
       <c r="E36" s="27" t="s">
         <v>6</v>
@@ -13425,13 +13562,13 @@
         <v>1041</v>
       </c>
       <c r="B37" t="s">
-        <v>1315</v>
+        <v>1313</v>
       </c>
       <c r="C37" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="D37" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
       <c r="E37" s="27" t="s">
         <v>6</v>
@@ -13442,13 +13579,13 @@
         <v>1041</v>
       </c>
       <c r="B38" t="s">
-        <v>1388</v>
+        <v>1384</v>
       </c>
       <c r="C38" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
       <c r="D38" t="s">
-        <v>1390</v>
+        <v>1386</v>
       </c>
       <c r="E38" s="27" t="s">
         <v>6</v>
@@ -13459,13 +13596,13 @@
         <v>1041</v>
       </c>
       <c r="B39" t="s">
-        <v>1452</v>
+        <v>1446</v>
       </c>
       <c r="C39" t="s">
-        <v>1453</v>
+        <v>1447</v>
       </c>
       <c r="D39" t="s">
-        <v>1454</v>
+        <v>1448</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>6</v>
@@ -13476,13 +13613,13 @@
         <v>1041</v>
       </c>
       <c r="B40" t="s">
-        <v>1536</v>
+        <v>1529</v>
       </c>
       <c r="C40" t="s">
-        <v>1537</v>
+        <v>1530</v>
       </c>
       <c r="D40" t="s">
-        <v>1538</v>
+        <v>1531</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>6</v>
@@ -13493,13 +13630,13 @@
         <v>1041</v>
       </c>
       <c r="B41" t="s">
-        <v>1572</v>
+        <v>1565</v>
       </c>
       <c r="C41" t="s">
-        <v>1573</v>
+        <v>1566</v>
       </c>
       <c r="D41" t="s">
-        <v>1574</v>
+        <v>1567</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>6</v>
@@ -13519,7 +13656,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -13956,18 +14093,18 @@
         <v>6</v>
       </c>
       <c r="G22" s="41" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="41" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B23" s="41" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C23" s="41" t="s">
         <v>1272</v>
-      </c>
-      <c r="B23" s="41" t="s">
-        <v>1273</v>
-      </c>
-      <c r="C23" s="41" t="s">
-        <v>1274</v>
       </c>
       <c r="D23" s="41" t="s">
         <v>1221</v>
@@ -13979,7 +14116,7 @@
         <v>6</v>
       </c>
       <c r="G23" s="41" t="s">
-        <v>1275</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -13987,10 +14124,10 @@
         <v>1006</v>
       </c>
       <c r="B24" s="41" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="C24" s="41" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="D24" s="41" t="s">
         <v>1221</v>
@@ -14002,7 +14139,7 @@
         <v>6</v>
       </c>
       <c r="G24" s="41" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -14010,22 +14147,22 @@
         <v>1006</v>
       </c>
       <c r="B25" s="41" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="C25" s="41" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
       <c r="D25" s="41" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="E25" s="41" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="F25" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>1352</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -14033,16 +14170,16 @@
         <v>1006</v>
       </c>
       <c r="B26" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
       <c r="C26" t="s">
-        <v>1392</v>
+        <v>1388</v>
       </c>
       <c r="D26" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="E26" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="F26" s="27" t="s">
         <v>6</v>
@@ -14053,45 +14190,45 @@
         <v>1006</v>
       </c>
       <c r="B27" t="s">
-        <v>1455</v>
+        <v>1449</v>
       </c>
       <c r="C27" t="s">
-        <v>1456</v>
+        <v>1450</v>
       </c>
       <c r="D27" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="E27" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="F27" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G27" t="s">
-        <v>1489</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
       <c r="B28" t="s">
-        <v>1494</v>
+        <v>1488</v>
       </c>
       <c r="C28" t="s">
-        <v>1495</v>
+        <v>1489</v>
       </c>
       <c r="D28" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="E28" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="F28" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G28" t="s">
-        <v>1496</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -14099,16 +14236,16 @@
         <v>1006</v>
       </c>
       <c r="B29" t="s">
-        <v>1539</v>
+        <v>1532</v>
       </c>
       <c r="C29" t="s">
-        <v>1540</v>
+        <v>1533</v>
       </c>
       <c r="D29" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="E29" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="F29" s="27" t="s">
         <v>6</v>
@@ -14119,16 +14256,16 @@
         <v>1006</v>
       </c>
       <c r="B30" t="s">
-        <v>1575</v>
+        <v>1568</v>
       </c>
       <c r="C30" t="s">
-        <v>1578</v>
+        <v>1571</v>
       </c>
       <c r="D30" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="E30" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="F30" s="27" t="s">
         <v>6</v>
@@ -14139,22 +14276,65 @@
         <v>1006</v>
       </c>
       <c r="B31" t="s">
-        <v>1594</v>
+        <v>1586</v>
       </c>
       <c r="C31" t="s">
-        <v>1595</v>
+        <v>1587</v>
       </c>
       <c r="D31" t="s">
-        <v>1602</v>
+        <v>1592</v>
       </c>
       <c r="E31" t="s">
-        <v>1602</v>
+        <v>1592</v>
       </c>
       <c r="F31" s="27" t="s">
         <v>6</v>
       </c>
       <c r="G31" t="s">
-        <v>1596</v>
+        <v>1597</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1599</v>
+      </c>
+      <c r="D32" s="45">
+        <v>46273</v>
+      </c>
+      <c r="E32" s="45">
+        <v>46273</v>
+      </c>
+      <c r="F32" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="G32" t="s">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1619</v>
+      </c>
+      <c r="D33" s="45">
+        <v>46273</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>1292</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1620</v>
       </c>
     </row>
   </sheetData>
@@ -14168,7 +14348,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14651,7 +14831,7 @@
         <v>1120</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="D39" s="27" t="s">
         <v>6</v>
@@ -14721,7 +14901,7 @@
         <v>1226</v>
       </c>
       <c r="C44" s="41" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="D44" s="27" t="s">
         <v>6</v>
@@ -14735,10 +14915,10 @@
         <v>1228</v>
       </c>
       <c r="C45" s="41" t="s">
-        <v>1229</v>
-      </c>
-      <c r="D45" s="43" t="s">
-        <v>1230</v>
+        <v>1615</v>
+      </c>
+      <c r="D45" s="41" t="s">
+        <v>1127</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -14746,10 +14926,10 @@
         <v>1161</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>1261</v>
+        <v>1259</v>
       </c>
       <c r="D46" s="27" t="s">
         <v>6</v>
@@ -14757,13 +14937,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="B47" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
       <c r="C47" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
       <c r="D47" s="27" t="s">
         <v>6</v>
@@ -14771,13 +14951,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="B48" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
       <c r="C48" t="s">
-        <v>1350</v>
+        <v>1346</v>
       </c>
       <c r="D48" s="27" t="s">
         <v>6</v>
@@ -14785,13 +14965,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
       <c r="B49" t="s">
-        <v>1393</v>
+        <v>1389</v>
       </c>
       <c r="C49" t="s">
-        <v>1394</v>
+        <v>1390</v>
       </c>
       <c r="D49" s="27" t="s">
         <v>6</v>
@@ -14799,13 +14979,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
       <c r="B50" t="s">
-        <v>1406</v>
+        <v>1402</v>
       </c>
       <c r="C50" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
       <c r="D50" s="27" t="s">
         <v>6</v>
@@ -14813,13 +14993,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>1455</v>
+        <v>1449</v>
       </c>
       <c r="B51" t="s">
-        <v>1457</v>
+        <v>1451</v>
       </c>
       <c r="C51" t="s">
-        <v>1458</v>
+        <v>1452</v>
       </c>
       <c r="D51" s="27" t="s">
         <v>6</v>
@@ -14827,13 +15007,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>1459</v>
+        <v>1453</v>
       </c>
       <c r="B52" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="C52" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="D52" s="27" t="s">
         <v>6</v>
@@ -14841,13 +15021,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>1481</v>
+        <v>1475</v>
       </c>
       <c r="B53" t="s">
-        <v>1482</v>
+        <v>1476</v>
       </c>
       <c r="C53" t="s">
-        <v>1483</v>
+        <v>1477</v>
       </c>
       <c r="D53" s="41" t="s">
         <v>1123</v>
@@ -14855,13 +15035,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>1539</v>
+        <v>1532</v>
       </c>
       <c r="B54" t="s">
-        <v>1541</v>
+        <v>1534</v>
       </c>
       <c r="C54" t="s">
-        <v>1542</v>
+        <v>1535</v>
       </c>
       <c r="D54" s="27" t="s">
         <v>6</v>
@@ -14869,13 +15049,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>1575</v>
+        <v>1568</v>
       </c>
       <c r="B55" t="s">
-        <v>1576</v>
+        <v>1569</v>
       </c>
       <c r="C55" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="D55" s="27" t="s">
         <v>6</v>
@@ -14883,13 +15063,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>1579</v>
+        <v>1572</v>
       </c>
       <c r="B56" t="s">
-        <v>1601</v>
+        <v>1591</v>
       </c>
       <c r="C56" t="s">
-        <v>1597</v>
+        <v>1588</v>
       </c>
       <c r="D56" s="48" t="s">
         <v>109</v>
@@ -14897,16 +15077,30 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>1598</v>
+        <v>1589</v>
       </c>
       <c r="B57" t="s">
-        <v>1599</v>
+        <v>1590</v>
       </c>
       <c r="C57" t="s">
-        <v>1600</v>
-      </c>
-      <c r="D57" s="38" t="s">
-        <v>977</v>
+        <v>1593</v>
+      </c>
+      <c r="D57" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>1594</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1595</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1596</v>
+      </c>
+      <c r="D58" s="41" t="s">
+        <v>1127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: nuovo tracker v2 e programma per la v1.1
</commit_message>
<xml_diff>
--- a/TrackAttività_Gestora.xlsx
+++ b/TrackAttività_Gestora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Taranto\Progetti_Tech\Personali\Gestora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3CE426-C7AB-4634-AD73-BF526B9C75D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F36633E-B1B9-4AD8-85CD-5BECB7ACEA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="1920" windowWidth="30960" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3153" uniqueCount="1812">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3154" uniqueCount="1813">
   <si>
     <t>GESTORA WEB API — CRUSCOTTO PROGETTO</t>
   </si>
@@ -5469,13 +5469,16 @@
   </si>
   <si>
     <t>Fabio usa l'app e segna difetti e migliorie prima del rilascio, con la checklist in GestoraDocs/verifica-redesign.md. In parallelo applica CAP-001 (tre punti in BACKLOG.md): tetto dei coperti garantito sotto concorrenza, validazione dentro la transazione anche in modifica, e sforamento mostrato invece che schiacciato.</t>
+  </si>
+  <si>
+    <t>CONGELATO il 09/09/2026 — archivio storico, non si aggiorna piu'. Tracker attivo: TrackGestora_v2.xlsx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5567,6 +5570,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -5747,7 +5758,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -5906,6 +5917,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -6239,6 +6251,11 @@
       <c r="E2" s="56"/>
       <c r="F2" s="56"/>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="68" t="s">
+        <v>1812</v>
+      </c>
+    </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="62" t="s">
         <v>1</v>

</xml_diff>